<commit_message>
House search data from run 101
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$167</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W169"/>
+  <dimension ref="A1:W167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2336,10 +2336,10 @@
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>1868</v>
+        <v>1350</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="7" t="n">
         <v>1</v>
@@ -2351,23 +2351,21 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>Union Road, Bristol</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="n">
-        <v>524</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="n"/>
       <c r="J22" s="7" t="n"/>
       <c r="K22" s="7" t="n"/>
       <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
       <c r="N22" s="7" t="n">
-        <v>11632</v>
+        <v>20080</v>
       </c>
       <c r="O22" s="7" t="n">
         <v>0</v>
@@ -2375,12 +2373,12 @@
       <c r="P22" s="7" t="n"/>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S22" s="8" t="inlineStr">
@@ -2401,7 +2399,7 @@
       <c r="V22" s="6" t="inlineStr"/>
       <c r="W22" s="7" t="inlineStr">
         <is>
-          <t>76680a66dec4a621e595dd1a625ea2323ba7dfc6</t>
+          <t>120a391700629cb94d575b3211bbdf9c0218d349</t>
         </is>
       </c>
     </row>
@@ -2415,10 +2413,10 @@
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>1350</v>
+        <v>1400</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>1</v>
@@ -2430,21 +2428,23 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Union Road, Bristol</t>
+          <t>Harbourside, The Crescent, BS1 5LQ</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>603</v>
+      </c>
       <c r="J23" s="7" t="n"/>
       <c r="K23" s="7" t="n"/>
       <c r="L23" s="7" t="n"/>
       <c r="M23" s="7" t="n"/>
       <c r="N23" s="7" t="n">
-        <v>20080</v>
+        <v>16724</v>
       </c>
       <c r="O23" s="7" t="n">
         <v>0</v>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="R23" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S23" s="8" t="inlineStr">
@@ -2478,7 +2478,7 @@
       <c r="V23" s="6" t="inlineStr"/>
       <c r="W23" s="7" t="inlineStr">
         <is>
-          <t>120a391700629cb94d575b3211bbdf9c0218d349</t>
+          <t>7a10ed41d917a52d904d0556bbba8459de456473</t>
         </is>
       </c>
     </row>
@@ -2492,13 +2492,13 @@
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1400</v>
+        <v>1775</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, The Crescent, BS1 5LQ</t>
+          <t>Twine House, Redcliff Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
@@ -2516,14 +2516,14 @@
         </is>
       </c>
       <c r="I24" s="7" t="n">
-        <v>603</v>
+        <v>767</v>
       </c>
       <c r="J24" s="7" t="n"/>
       <c r="K24" s="7" t="n"/>
       <c r="L24" s="7" t="n"/>
       <c r="M24" s="7" t="n"/>
       <c r="N24" s="7" t="n">
-        <v>16724</v>
+        <v>20888</v>
       </c>
       <c r="O24" s="7" t="n">
         <v>0</v>
@@ -2531,12 +2531,12 @@
       <c r="P24" s="7" t="n"/>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S24" s="8" t="inlineStr">
@@ -2557,7 +2557,7 @@
       <c r="V24" s="6" t="inlineStr"/>
       <c r="W24" s="7" t="inlineStr">
         <is>
-          <t>7a10ed41d917a52d904d0556bbba8459de456473</t>
+          <t>27c0f9ce89d081b8d1914ffcc561e9aa878d6d99</t>
         </is>
       </c>
     </row>
@@ -2571,13 +2571,13 @@
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>1775</v>
+        <v>1700</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -2586,23 +2586,21 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Twine House, Redcliff Street, Redcliff, Bristol, Bristol City</t>
+          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="n">
-        <v>767</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n"/>
       <c r="J25" s="7" t="n"/>
       <c r="K25" s="7" t="n"/>
       <c r="L25" s="7" t="n"/>
       <c r="M25" s="7" t="n"/>
       <c r="N25" s="7" t="n">
-        <v>20888</v>
+        <v>4892</v>
       </c>
       <c r="O25" s="7" t="n">
         <v>0</v>
@@ -2610,12 +2608,12 @@
       <c r="P25" s="7" t="n"/>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S25" s="8" t="inlineStr">
@@ -2636,7 +2634,7 @@
       <c r="V25" s="6" t="inlineStr"/>
       <c r="W25" s="7" t="inlineStr">
         <is>
-          <t>27c0f9ce89d081b8d1914ffcc561e9aa878d6d99</t>
+          <t>916b8e1db731f908cd8ba08a69c2e9978e66cd1c</t>
         </is>
       </c>
     </row>
@@ -2650,10 +2648,10 @@
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>1700</v>
+        <v>1823</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>1</v>
@@ -2665,21 +2663,23 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I26" s="7" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>524</v>
+      </c>
       <c r="J26" s="7" t="n"/>
       <c r="K26" s="7" t="n"/>
       <c r="L26" s="7" t="n"/>
       <c r="M26" s="7" t="n"/>
       <c r="N26" s="7" t="n">
-        <v>4892</v>
+        <v>11632</v>
       </c>
       <c r="O26" s="7" t="n">
         <v>0</v>
@@ -2687,12 +2687,12 @@
       <c r="P26" s="7" t="n"/>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R26" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S26" s="8" t="inlineStr">
@@ -2713,7 +2713,7 @@
       <c r="V26" s="6" t="inlineStr"/>
       <c r="W26" s="7" t="inlineStr">
         <is>
-          <t>916b8e1db731f908cd8ba08a69c2e9978e66cd1c</t>
+          <t>96f4c09e794ccdc0fe9190c623669e365937c4d3</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>1823</v>
+        <v>1500</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>1</v>
@@ -2742,23 +2742,23 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>St. David Mews, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I27" s="7" t="n">
-        <v>524</v>
+        <v>560</v>
       </c>
       <c r="J27" s="7" t="n"/>
       <c r="K27" s="7" t="n"/>
       <c r="L27" s="7" t="n"/>
       <c r="M27" s="7" t="n"/>
       <c r="N27" s="7" t="n">
-        <v>11632</v>
+        <v>18292</v>
       </c>
       <c r="O27" s="7" t="n">
         <v>0</v>
@@ -2766,12 +2766,12 @@
       <c r="P27" s="7" t="n"/>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S27" s="8" t="inlineStr">
@@ -2792,7 +2792,7 @@
       <c r="V27" s="6" t="inlineStr"/>
       <c r="W27" s="7" t="inlineStr">
         <is>
-          <t>96f4c09e794ccdc0fe9190c623669e365937c4d3</t>
+          <t>acc3c4682d6bc0b232ebba18bc6c42d125641e52</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="C28" s="9" t="n">
-        <v>1650</v>
+        <v>1868</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>1</v>
@@ -2821,21 +2821,23 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I28" s="7" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>524</v>
+      </c>
       <c r="J28" s="7" t="n"/>
       <c r="K28" s="7" t="n"/>
       <c r="L28" s="7" t="n"/>
       <c r="M28" s="7" t="n"/>
       <c r="N28" s="7" t="n">
-        <v>21996</v>
+        <v>11632</v>
       </c>
       <c r="O28" s="7" t="n">
         <v>0</v>
@@ -2843,17 +2845,17 @@
       <c r="P28" s="7" t="n"/>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S28" s="8" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T28" s="10" t="inlineStr">
@@ -2869,7 +2871,7 @@
       <c r="V28" s="6" t="inlineStr"/>
       <c r="W28" s="7" t="inlineStr">
         <is>
-          <t>48fa0ece469b09f31eb9d082a42a7c6ed00c6aac</t>
+          <t>76680a66dec4a621e595dd1a625ea2323ba7dfc6</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2885,7 @@
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>1450</v>
+        <v>1650</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>1</v>
@@ -2898,12 +2900,12 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>Norfolk House, Norfolk Avenue, St Paul's, BS2</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I29" s="7" t="n"/>
@@ -2912,25 +2914,25 @@
       <c r="L29" s="7" t="n"/>
       <c r="M29" s="7" t="n"/>
       <c r="N29" s="7" t="n">
-        <v>14016</v>
+        <v>21996</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P29" s="7" t="n"/>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R29" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S29" s="8" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T29" s="10" t="inlineStr">
@@ -2946,7 +2948,7 @@
       <c r="V29" s="6" t="inlineStr"/>
       <c r="W29" s="7" t="inlineStr">
         <is>
-          <t>a6e3aa5da01b2c2d03e0168a413f098ce4121aa0</t>
+          <t>48fa0ece469b09f31eb9d082a42a7c6ed00c6aac</t>
         </is>
       </c>
     </row>
@@ -2960,7 +2962,7 @@
         </is>
       </c>
       <c r="C30" s="9" t="n">
-        <v>1823</v>
+        <v>1450</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>1</v>
@@ -2975,23 +2977,21 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>Norfolk House, Norfolk Avenue, St Paul's, BS2</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I30" s="7" t="n">
-        <v>524</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="n"/>
       <c r="J30" s="7" t="n"/>
       <c r="K30" s="7" t="n"/>
       <c r="L30" s="7" t="n"/>
       <c r="M30" s="7" t="n"/>
       <c r="N30" s="7" t="n">
-        <v>11632</v>
+        <v>14016</v>
       </c>
       <c r="O30" s="7" t="n">
         <v>1</v>
@@ -2999,12 +2999,12 @@
       <c r="P30" s="7" t="n"/>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S30" s="8" t="inlineStr">
@@ -3025,7 +3025,7 @@
       <c r="V30" s="6" t="inlineStr"/>
       <c r="W30" s="7" t="inlineStr">
         <is>
-          <t>e0b7eeddf14c3f69bac6d7087896295a39a16c3f</t>
+          <t>a6e3aa5da01b2c2d03e0168a413f098ce4121aa0</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>1665</v>
+        <v>1823</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>1</v>
@@ -3054,23 +3054,23 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I31" s="7" t="n">
-        <v>547</v>
+        <v>524</v>
       </c>
       <c r="J31" s="7" t="n"/>
       <c r="K31" s="7" t="n"/>
       <c r="L31" s="7" t="n"/>
       <c r="M31" s="7" t="n"/>
       <c r="N31" s="7" t="n">
-        <v>13408</v>
+        <v>11632</v>
       </c>
       <c r="O31" s="7" t="n">
         <v>1</v>
@@ -3078,12 +3078,12 @@
       <c r="P31" s="7" t="n"/>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S31" s="8" t="inlineStr">
@@ -3104,7 +3104,7 @@
       <c r="V31" s="6" t="inlineStr"/>
       <c r="W31" s="7" t="inlineStr">
         <is>
-          <t>880b3fa3b06517eb65b3a604c4cde6e6ec04898f</t>
+          <t>e0b7eeddf14c3f69bac6d7087896295a39a16c3f</t>
         </is>
       </c>
     </row>
@@ -3118,10 +3118,10 @@
         </is>
       </c>
       <c r="C32" s="9" t="n">
-        <v>1550</v>
+        <v>1665</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>1</v>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>City Road, St Pauls, Bristol, BS2</t>
+          <t>Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -3142,14 +3142,14 @@
         </is>
       </c>
       <c r="I32" s="7" t="n">
-        <v>872</v>
+        <v>547</v>
       </c>
       <c r="J32" s="7" t="n"/>
       <c r="K32" s="7" t="n"/>
       <c r="L32" s="7" t="n"/>
       <c r="M32" s="7" t="n"/>
       <c r="N32" s="7" t="n">
-        <v>13004</v>
+        <v>13408</v>
       </c>
       <c r="O32" s="7" t="n">
         <v>1</v>
@@ -3157,17 +3157,17 @@
       <c r="P32" s="7" t="n"/>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="R32" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S32" s="8" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T32" s="10" t="inlineStr">
@@ -3183,7 +3183,7 @@
       <c r="V32" s="6" t="inlineStr"/>
       <c r="W32" s="7" t="inlineStr">
         <is>
-          <t>f0084682d29703f51fa0be542fd382e673d76549</t>
+          <t>880b3fa3b06517eb65b3a604c4cde6e6ec04898f</t>
         </is>
       </c>
     </row>
@@ -3197,10 +3197,10 @@
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>1400</v>
+        <v>1550</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>1</v>
@@ -3212,23 +3212,23 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Great Western House, BS1 6GN</t>
+          <t>City Road, St Pauls, Bristol, BS2</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I33" s="7" t="n">
-        <v>538</v>
+        <v>872</v>
       </c>
       <c r="J33" s="7" t="n"/>
       <c r="K33" s="7" t="n"/>
       <c r="L33" s="7" t="n"/>
       <c r="M33" s="7" t="n"/>
       <c r="N33" s="7" t="n">
-        <v>14412</v>
+        <v>13004</v>
       </c>
       <c r="O33" s="7" t="n">
         <v>1</v>
@@ -3236,17 +3236,17 @@
       <c r="P33" s="7" t="n"/>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S33" s="8" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T33" s="10" t="inlineStr">
@@ -3262,7 +3262,7 @@
       <c r="V33" s="6" t="inlineStr"/>
       <c r="W33" s="7" t="inlineStr">
         <is>
-          <t>4ec2700ca7d475b941e223f1b5c74e8cd5be890b</t>
+          <t>f0084682d29703f51fa0be542fd382e673d76549</t>
         </is>
       </c>
     </row>
@@ -3276,13 +3276,13 @@
         </is>
       </c>
       <c r="C34" s="9" t="n">
-        <v>2050</v>
+        <v>1400</v>
       </c>
       <c r="D34" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
@@ -3291,36 +3291,36 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>421 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>Harbourside, Great Western House, BS1 6GN</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I34" s="7" t="n">
-        <v>802</v>
+        <v>538</v>
       </c>
       <c r="J34" s="7" t="n"/>
       <c r="K34" s="7" t="n"/>
       <c r="L34" s="7" t="n"/>
       <c r="M34" s="7" t="n"/>
       <c r="N34" s="7" t="n">
-        <v>13408</v>
+        <v>14412</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P34" s="7" t="n"/>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R34" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S34" s="8" t="inlineStr">
@@ -3341,7 +3341,7 @@
       <c r="V34" s="6" t="inlineStr"/>
       <c r="W34" s="7" t="inlineStr">
         <is>
-          <t>b7d86b41b199aaf040e0304048e519e961081fd2</t>
+          <t>4ec2700ca7d475b941e223f1b5c74e8cd5be890b</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>1795</v>
+        <v>2050</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>2</v>
@@ -3370,36 +3370,36 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>421 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I35" s="7" t="n">
-        <v>647</v>
+        <v>802</v>
       </c>
       <c r="J35" s="7" t="n"/>
       <c r="K35" s="7" t="n"/>
       <c r="L35" s="7" t="n"/>
       <c r="M35" s="7" t="n"/>
       <c r="N35" s="7" t="n">
-        <v>21476</v>
+        <v>13408</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P35" s="7" t="n"/>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R35" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S35" s="8" t="inlineStr">
@@ -3420,7 +3420,7 @@
       <c r="V35" s="6" t="inlineStr"/>
       <c r="W35" s="7" t="inlineStr">
         <is>
-          <t>53eb1a881a4e0138c82c0a97c88cad4df5dbd397</t>
+          <t>b7d86b41b199aaf040e0304048e519e961081fd2</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3434,7 @@
         </is>
       </c>
       <c r="C36" s="9" t="n">
-        <v>2850</v>
+        <v>1795</v>
       </c>
       <c r="D36" s="7" t="n">
         <v>2</v>
@@ -3449,23 +3449,23 @@
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>Capricorn Place, Hotwells, BS8</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>BS8</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I36" s="7" t="n">
-        <v>1615</v>
+        <v>647</v>
       </c>
       <c r="J36" s="7" t="n"/>
       <c r="K36" s="7" t="n"/>
       <c r="L36" s="7" t="n"/>
       <c r="M36" s="7" t="n"/>
       <c r="N36" s="7" t="n">
-        <v>15260</v>
+        <v>21476</v>
       </c>
       <c r="O36" s="7" t="n">
         <v>1</v>
@@ -3473,12 +3473,12 @@
       <c r="P36" s="7" t="n"/>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R36" s="7" t="inlineStr">
         <is>
-          <t>Sarah Kenny Residential Lettings, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S36" s="8" t="inlineStr">
@@ -3499,7 +3499,7 @@
       <c r="V36" s="6" t="inlineStr"/>
       <c r="W36" s="7" t="inlineStr">
         <is>
-          <t>11c93771b8963d430763c083c575b56042e71418</t>
+          <t>53eb1a881a4e0138c82c0a97c88cad4df5dbd397</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>2000</v>
+        <v>2850</v>
       </c>
       <c r="D37" s="7" t="n">
         <v>2</v>
@@ -3528,36 +3528,36 @@
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>Chatfield House, Marsh Street, Bristol</t>
+          <t>Capricorn Place, Hotwells, BS8</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS8</t>
         </is>
       </c>
       <c r="I37" s="7" t="n">
-        <v>705</v>
+        <v>1615</v>
       </c>
       <c r="J37" s="7" t="n"/>
       <c r="K37" s="7" t="n"/>
       <c r="L37" s="7" t="n"/>
       <c r="M37" s="7" t="n"/>
       <c r="N37" s="7" t="n">
-        <v>20932</v>
+        <v>15260</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P37" s="7" t="n"/>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr">
         <is>
-          <t>Mariana Real Estate, London</t>
+          <t>Sarah Kenny Residential Lettings, Bristol</t>
         </is>
       </c>
       <c r="S37" s="8" t="inlineStr">
@@ -3578,7 +3578,7 @@
       <c r="V37" s="6" t="inlineStr"/>
       <c r="W37" s="7" t="inlineStr">
         <is>
-          <t>be4fdd18faf2bcf44d894da42e9c874b7d868fbe</t>
+          <t>11c93771b8963d430763c083c575b56042e71418</t>
         </is>
       </c>
     </row>
@@ -3592,13 +3592,13 @@
         </is>
       </c>
       <c r="C38" s="9" t="n">
-        <v>1600</v>
+        <v>2000</v>
       </c>
       <c r="D38" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>St. Stephens Street, Bristol, BS1</t>
+          <t>Chatfield House, Marsh Street, Bristol</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -3615,13 +3615,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I38" s="7" t="n"/>
+      <c r="I38" s="7" t="n">
+        <v>705</v>
+      </c>
       <c r="J38" s="7" t="n"/>
       <c r="K38" s="7" t="n"/>
       <c r="L38" s="7" t="n"/>
       <c r="M38" s="7" t="n"/>
       <c r="N38" s="7" t="n">
-        <v>13940</v>
+        <v>20932</v>
       </c>
       <c r="O38" s="7" t="n">
         <v>0</v>
@@ -3634,7 +3636,7 @@
       </c>
       <c r="R38" s="7" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>Mariana Real Estate, London</t>
         </is>
       </c>
       <c r="S38" s="8" t="inlineStr">
@@ -3655,7 +3657,7 @@
       <c r="V38" s="6" t="inlineStr"/>
       <c r="W38" s="7" t="inlineStr">
         <is>
-          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
+          <t>be4fdd18faf2bcf44d894da42e9c874b7d868fbe</t>
         </is>
       </c>
     </row>
@@ -3669,10 +3671,10 @@
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>1758</v>
+        <v>1600</v>
       </c>
       <c r="D39" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>1</v>
@@ -3684,23 +3686,21 @@
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>St. Stephens Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="n">
-        <v>524</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="n"/>
       <c r="J39" s="7" t="n"/>
       <c r="K39" s="7" t="n"/>
       <c r="L39" s="7" t="n"/>
       <c r="M39" s="7" t="n"/>
       <c r="N39" s="7" t="n">
-        <v>11632</v>
+        <v>13940</v>
       </c>
       <c r="O39" s="7" t="n">
         <v>0</v>
@@ -3708,12 +3708,12 @@
       <c r="P39" s="7" t="n"/>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S39" s="8" t="inlineStr">
@@ -3734,7 +3734,7 @@
       <c r="V39" s="6" t="inlineStr"/>
       <c r="W39" s="7" t="inlineStr">
         <is>
-          <t>c89d3936db6998bf29cb9eaaa090ca063504a042</t>
+          <t>cd770dd603af2e6f4f23a72c9685c7468c731a6d</t>
         </is>
       </c>
     </row>
@@ -3748,12 +3748,14 @@
         </is>
       </c>
       <c r="C40" s="9" t="n">
-        <v>1400</v>
+        <v>1758</v>
       </c>
       <c r="D40" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="7" t="n"/>
+      <c r="E40" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -3761,21 +3763,23 @@
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Millennium Promenade, Bristol, BS1</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I40" s="7" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>524</v>
+      </c>
       <c r="J40" s="7" t="n"/>
       <c r="K40" s="7" t="n"/>
       <c r="L40" s="7" t="n"/>
       <c r="M40" s="7" t="n"/>
       <c r="N40" s="7" t="n">
-        <v>16168</v>
+        <v>11632</v>
       </c>
       <c r="O40" s="7" t="n">
         <v>0</v>
@@ -3783,12 +3787,12 @@
       <c r="P40" s="7" t="n"/>
       <c r="Q40" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R40" s="7" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S40" s="8" t="inlineStr">
@@ -3809,7 +3813,7 @@
       <c r="V40" s="6" t="inlineStr"/>
       <c r="W40" s="7" t="inlineStr">
         <is>
-          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
+          <t>c89d3936db6998bf29cb9eaaa090ca063504a042</t>
         </is>
       </c>
     </row>
@@ -3823,14 +3827,12 @@
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>1900</v>
+        <v>1400</v>
       </c>
       <c r="D41" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E41" s="7" t="n"/>
       <c r="F41" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -3838,7 +3840,7 @@
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>Deanery Road, BRISTOL</t>
+          <t>Millennium Promenade, Bristol, BS1</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -3852,7 +3854,7 @@
       <c r="L41" s="7" t="n"/>
       <c r="M41" s="7" t="n"/>
       <c r="N41" s="7" t="n">
-        <v>11916</v>
+        <v>16168</v>
       </c>
       <c r="O41" s="7" t="n">
         <v>0</v>
@@ -3860,12 +3862,12 @@
       <c r="P41" s="7" t="n"/>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R41" s="7" t="inlineStr">
         <is>
-          <t>Allen &amp; Harris, Clifton</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S41" s="8" t="inlineStr">
@@ -3886,7 +3888,7 @@
       <c r="V41" s="6" t="inlineStr"/>
       <c r="W41" s="7" t="inlineStr">
         <is>
-          <t>7de28a016a4c688c515861dbb81f78d510e563cb</t>
+          <t>5ec68f33756a2f8f7606ead5febd7f33ed18c280</t>
         </is>
       </c>
     </row>
@@ -3900,13 +3902,13 @@
         </is>
       </c>
       <c r="C42" s="9" t="n">
-        <v>1758</v>
+        <v>1900</v>
       </c>
       <c r="D42" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -3915,23 +3917,21 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>Deanery Road, BRISTOL</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I42" s="7" t="n">
-        <v>524</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="n"/>
       <c r="J42" s="7" t="n"/>
       <c r="K42" s="7" t="n"/>
       <c r="L42" s="7" t="n"/>
       <c r="M42" s="7" t="n"/>
       <c r="N42" s="7" t="n">
-        <v>11632</v>
+        <v>11916</v>
       </c>
       <c r="O42" s="7" t="n">
         <v>0</v>
@@ -3939,12 +3939,12 @@
       <c r="P42" s="7" t="n"/>
       <c r="Q42" s="7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R42" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>Allen &amp; Harris, Clifton</t>
         </is>
       </c>
       <c r="S42" s="8" t="inlineStr">
@@ -3965,7 +3965,7 @@
       <c r="V42" s="6" t="inlineStr"/>
       <c r="W42" s="7" t="inlineStr">
         <is>
-          <t>2a07769bc6317adeb6dd550e1e056ddeac2ac129</t>
+          <t>7de28a016a4c688c515861dbb81f78d510e563cb</t>
         </is>
       </c>
     </row>
@@ -3979,22 +3979,22 @@
         </is>
       </c>
       <c r="C43" s="9" t="n">
-        <v>1800</v>
+        <v>1758</v>
       </c>
       <c r="D43" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>Osborne Road, Southville, Bristol, BS3</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -4002,13 +4002,15 @@
           <t>BS3</t>
         </is>
       </c>
-      <c r="I43" s="7" t="n"/>
+      <c r="I43" s="7" t="n">
+        <v>524</v>
+      </c>
       <c r="J43" s="7" t="n"/>
       <c r="K43" s="7" t="n"/>
       <c r="L43" s="7" t="n"/>
       <c r="M43" s="7" t="n"/>
       <c r="N43" s="7" t="n">
-        <v>14028</v>
+        <v>11632</v>
       </c>
       <c r="O43" s="7" t="n">
         <v>0</v>
@@ -4016,17 +4018,17 @@
       <c r="P43" s="7" t="n"/>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R43" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Southville</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S43" s="8" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T43" s="10" t="inlineStr">
@@ -4042,7 +4044,7 @@
       <c r="V43" s="6" t="inlineStr"/>
       <c r="W43" s="7" t="inlineStr">
         <is>
-          <t>69ee3b35f8d9109c2a36a94ae5b3d0b237a035bd</t>
+          <t>2a07769bc6317adeb6dd550e1e056ddeac2ac129</t>
         </is>
       </c>
     </row>
@@ -4056,27 +4058,27 @@
         </is>
       </c>
       <c r="C44" s="9" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="D44" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
+          <t>Osborne Road, Southville, Bristol, BS3</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I44" s="7" t="n"/>
@@ -4085,7 +4087,7 @@
       <c r="L44" s="7" t="n"/>
       <c r="M44" s="7" t="n"/>
       <c r="N44" s="7" t="n">
-        <v>5244</v>
+        <v>14028</v>
       </c>
       <c r="O44" s="7" t="n">
         <v>0</v>
@@ -4093,17 +4095,17 @@
       <c r="P44" s="7" t="n"/>
       <c r="Q44" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R44" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Clifton</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S44" s="8" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T44" s="10" t="inlineStr">
@@ -4119,7 +4121,7 @@
       <c r="V44" s="6" t="inlineStr"/>
       <c r="W44" s="7" t="inlineStr">
         <is>
-          <t>1df0f6132fa2c969b5e48b842f8a67e797952b7e</t>
+          <t>69ee3b35f8d9109c2a36a94ae5b3d0b237a035bd</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4135,7 @@
         </is>
       </c>
       <c r="C45" s="9" t="n">
-        <v>1450</v>
+        <v>1650</v>
       </c>
       <c r="D45" s="7" t="n">
         <v>1</v>
@@ -4148,12 +4150,12 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>The Crescent, Bristol, BS1</t>
+          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I45" s="7" t="n"/>
@@ -4162,7 +4164,7 @@
       <c r="L45" s="7" t="n"/>
       <c r="M45" s="7" t="n"/>
       <c r="N45" s="7" t="n">
-        <v>16792</v>
+        <v>5244</v>
       </c>
       <c r="O45" s="7" t="n">
         <v>0</v>
@@ -4170,12 +4172,12 @@
       <c r="P45" s="7" t="n"/>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S45" s="8" t="inlineStr">
@@ -4196,7 +4198,7 @@
       <c r="V45" s="6" t="inlineStr"/>
       <c r="W45" s="7" t="inlineStr">
         <is>
-          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
+          <t>1df0f6132fa2c969b5e48b842f8a67e797952b7e</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4212,7 @@
         </is>
       </c>
       <c r="C46" s="9" t="n">
-        <v>1758</v>
+        <v>1450</v>
       </c>
       <c r="D46" s="7" t="n">
         <v>1</v>
@@ -4225,23 +4227,21 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>The Crescent, Bristol, BS1</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I46" s="7" t="n">
-        <v>524</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="n"/>
       <c r="J46" s="7" t="n"/>
       <c r="K46" s="7" t="n"/>
       <c r="L46" s="7" t="n"/>
       <c r="M46" s="7" t="n"/>
       <c r="N46" s="7" t="n">
-        <v>11632</v>
+        <v>16792</v>
       </c>
       <c r="O46" s="7" t="n">
         <v>0</v>
@@ -4249,12 +4249,12 @@
       <c r="P46" s="7" t="n"/>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S46" s="8" t="inlineStr">
@@ -4275,7 +4275,7 @@
       <c r="V46" s="6" t="inlineStr"/>
       <c r="W46" s="7" t="inlineStr">
         <is>
-          <t>cb7836e81328c8e3f4365c151c332c5f761e9d2b</t>
+          <t>d447d1158e90abd2c82eb7828f8a98e7f5fbe2bd</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="C47" s="9" t="n">
-        <v>1225</v>
+        <v>1758</v>
       </c>
       <c r="D47" s="7" t="n">
         <v>1</v>
@@ -4304,21 +4304,23 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>New Walls, Totterdown, BS4</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I47" s="7" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="n">
+        <v>524</v>
+      </c>
       <c r="J47" s="7" t="n"/>
       <c r="K47" s="7" t="n"/>
       <c r="L47" s="7" t="n"/>
       <c r="M47" s="7" t="n"/>
       <c r="N47" s="7" t="n">
-        <v>8540</v>
+        <v>11632</v>
       </c>
       <c r="O47" s="7" t="n">
         <v>0</v>
@@ -4326,12 +4328,12 @@
       <c r="P47" s="7" t="n"/>
       <c r="Q47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R47" s="7" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S47" s="8" t="inlineStr">
@@ -4352,7 +4354,7 @@
       <c r="V47" s="6" t="inlineStr"/>
       <c r="W47" s="7" t="inlineStr">
         <is>
-          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
+          <t>cb7836e81328c8e3f4365c151c332c5f761e9d2b</t>
         </is>
       </c>
     </row>
@@ -4366,13 +4368,13 @@
         </is>
       </c>
       <c r="C48" s="9" t="n">
-        <v>2000</v>
+        <v>1225</v>
       </c>
       <c r="D48" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -4381,12 +4383,12 @@
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>Caledonian Road, Bristol, BS1</t>
+          <t>New Walls, Totterdown, BS4</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I48" s="7" t="n"/>
@@ -4395,7 +4397,7 @@
       <c r="L48" s="7" t="n"/>
       <c r="M48" s="7" t="n"/>
       <c r="N48" s="7" t="n">
-        <v>14632</v>
+        <v>8540</v>
       </c>
       <c r="O48" s="7" t="n">
         <v>0</v>
@@ -4403,12 +4405,12 @@
       <c r="P48" s="7" t="n"/>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S48" s="8" t="inlineStr">
@@ -4429,7 +4431,7 @@
       <c r="V48" s="6" t="inlineStr"/>
       <c r="W48" s="7" t="inlineStr">
         <is>
-          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
+          <t>ff7cade97c52dbe0ee822ce3951fd4f71c9b4146</t>
         </is>
       </c>
     </row>
@@ -4443,13 +4445,13 @@
         </is>
       </c>
       <c r="C49" s="9" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
@@ -4458,7 +4460,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>The Crescent, Harbourside, BS1</t>
+          <t>Caledonian Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -4472,7 +4474,7 @@
       <c r="L49" s="7" t="n"/>
       <c r="M49" s="7" t="n"/>
       <c r="N49" s="7" t="n">
-        <v>16368</v>
+        <v>14632</v>
       </c>
       <c r="O49" s="7" t="n">
         <v>0</v>
@@ -4480,12 +4482,12 @@
       <c r="P49" s="7" t="n"/>
       <c r="Q49" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R49" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S49" s="8" t="inlineStr">
@@ -4506,7 +4508,7 @@
       <c r="V49" s="6" t="inlineStr"/>
       <c r="W49" s="7" t="inlineStr">
         <is>
-          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
+          <t>9a270cf54e31627246aef21daa26a60bb5f977ad</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4522,7 @@
         </is>
       </c>
       <c r="C50" s="9" t="n">
-        <v>1200</v>
+        <v>1400</v>
       </c>
       <c r="D50" s="7" t="n">
         <v>1</v>
@@ -4535,12 +4537,12 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Union Road, Bristol BS2 0FN</t>
+          <t>The Crescent, Harbourside, BS1</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I50" s="7" t="n"/>
@@ -4549,7 +4551,7 @@
       <c r="L50" s="7" t="n"/>
       <c r="M50" s="7" t="n"/>
       <c r="N50" s="7" t="n">
-        <v>20144</v>
+        <v>16368</v>
       </c>
       <c r="O50" s="7" t="n">
         <v>0</v>
@@ -4557,12 +4559,12 @@
       <c r="P50" s="7" t="n"/>
       <c r="Q50" s="7" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R50" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S50" s="8" t="inlineStr">
@@ -4583,7 +4585,7 @@
       <c r="V50" s="6" t="inlineStr"/>
       <c r="W50" s="7" t="inlineStr">
         <is>
-          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
+          <t>59af10441dff618517a35c62d6a67a8485c2f2fa</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4599,7 @@
         </is>
       </c>
       <c r="C51" s="9" t="n">
-        <v>1758</v>
+        <v>1200</v>
       </c>
       <c r="D51" s="7" t="n">
         <v>1</v>
@@ -4612,23 +4614,21 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>Union Road, Bristol BS2 0FN</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I51" s="7" t="n">
-        <v>524</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="n"/>
       <c r="J51" s="7" t="n"/>
       <c r="K51" s="7" t="n"/>
       <c r="L51" s="7" t="n"/>
       <c r="M51" s="7" t="n"/>
       <c r="N51" s="7" t="n">
-        <v>11632</v>
+        <v>20144</v>
       </c>
       <c r="O51" s="7" t="n">
         <v>0</v>
@@ -4636,12 +4636,12 @@
       <c r="P51" s="7" t="n"/>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="R51" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S51" s="8" t="inlineStr">
@@ -4662,7 +4662,7 @@
       <c r="V51" s="6" t="inlineStr"/>
       <c r="W51" s="7" t="inlineStr">
         <is>
-          <t>e01353518e32ee855b640499d951960a537bb160</t>
+          <t>2b2295e0c22bd50658835eb43d2eb433f6d1cd1b</t>
         </is>
       </c>
     </row>
@@ -4676,13 +4676,13 @@
         </is>
       </c>
       <c r="C52" s="9" t="n">
-        <v>1900</v>
+        <v>1758</v>
       </c>
       <c r="D52" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
@@ -4691,21 +4691,23 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>51.02 - St James Barton</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I52" s="7" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>524</v>
+      </c>
       <c r="J52" s="7" t="n"/>
       <c r="K52" s="7" t="n"/>
       <c r="L52" s="7" t="n"/>
       <c r="M52" s="7" t="n"/>
       <c r="N52" s="7" t="n">
-        <v>22132</v>
+        <v>11632</v>
       </c>
       <c r="O52" s="7" t="n">
         <v>0</v>
@@ -4713,12 +4715,12 @@
       <c r="P52" s="7" t="n"/>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S52" s="8" t="inlineStr">
@@ -4739,7 +4741,7 @@
       <c r="V52" s="6" t="inlineStr"/>
       <c r="W52" s="7" t="inlineStr">
         <is>
-          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
+          <t>e01353518e32ee855b640499d951960a537bb160</t>
         </is>
       </c>
     </row>
@@ -4753,7 +4755,7 @@
         </is>
       </c>
       <c r="C53" s="9" t="n">
-        <v>1850</v>
+        <v>1900</v>
       </c>
       <c r="D53" s="7" t="n">
         <v>2</v>
@@ -4768,7 +4770,7 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>51.02 - St James Barton</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -4782,7 +4784,7 @@
       <c r="L53" s="7" t="n"/>
       <c r="M53" s="7" t="n"/>
       <c r="N53" s="7" t="n">
-        <v>22020</v>
+        <v>22132</v>
       </c>
       <c r="O53" s="7" t="n">
         <v>0</v>
@@ -4790,7 +4792,7 @@
       <c r="P53" s="7" t="n"/>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R53" s="7" t="inlineStr">
@@ -4800,7 +4802,7 @@
       </c>
       <c r="S53" s="8" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T53" s="10" t="inlineStr">
@@ -4816,7 +4818,7 @@
       <c r="V53" s="6" t="inlineStr"/>
       <c r="W53" s="7" t="inlineStr">
         <is>
-          <t>dcc16fa39cff678f7a157aec0c52e4b6b97a0fb3</t>
+          <t>1d421f07eb2d142471d3e293f8cb751813656c56</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4832,7 @@
         </is>
       </c>
       <c r="C54" s="9" t="n">
-        <v>2300</v>
+        <v>1850</v>
       </c>
       <c r="D54" s="7" t="n">
         <v>2</v>
@@ -4845,7 +4847,7 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Electricity House, Bristol, BS1</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -4859,7 +4861,7 @@
       <c r="L54" s="7" t="n"/>
       <c r="M54" s="7" t="n"/>
       <c r="N54" s="7" t="n">
-        <v>21876</v>
+        <v>22020</v>
       </c>
       <c r="O54" s="7" t="n">
         <v>0</v>
@@ -4867,17 +4869,17 @@
       <c r="P54" s="7" t="n"/>
       <c r="Q54" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R54" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S54" s="8" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T54" s="10" t="inlineStr">
@@ -4893,7 +4895,7 @@
       <c r="V54" s="6" t="inlineStr"/>
       <c r="W54" s="7" t="inlineStr">
         <is>
-          <t>35ca98fa51e87bf8bad5117293380e1cb3a5cc07</t>
+          <t>dcc16fa39cff678f7a157aec0c52e4b6b97a0fb3</t>
         </is>
       </c>
     </row>
@@ -4907,13 +4909,13 @@
         </is>
       </c>
       <c r="C55" s="9" t="n">
-        <v>1500</v>
+        <v>2300</v>
       </c>
       <c r="D55" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
@@ -4922,7 +4924,7 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Horizon - City Centre</t>
+          <t>Electricity House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
@@ -4936,7 +4938,7 @@
       <c r="L55" s="7" t="n"/>
       <c r="M55" s="7" t="n"/>
       <c r="N55" s="7" t="n">
-        <v>22020</v>
+        <v>21876</v>
       </c>
       <c r="O55" s="7" t="n">
         <v>0</v>
@@ -4944,17 +4946,17 @@
       <c r="P55" s="7" t="n"/>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R55" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S55" s="8" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>parking</t>
         </is>
       </c>
       <c r="T55" s="10" t="inlineStr">
@@ -4970,7 +4972,7 @@
       <c r="V55" s="6" t="inlineStr"/>
       <c r="W55" s="7" t="inlineStr">
         <is>
-          <t>25fbd71b098a83412bb2a614282b6fb33b9a3c90</t>
+          <t>35ca98fa51e87bf8bad5117293380e1cb3a5cc07</t>
         </is>
       </c>
     </row>
@@ -4984,10 +4986,10 @@
         </is>
       </c>
       <c r="C56" s="9" t="n">
-        <v>1550</v>
+        <v>1500</v>
       </c>
       <c r="D56" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E56" s="7" t="n">
         <v>1</v>
@@ -4999,12 +5001,12 @@
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Beaufort Street, Stapleton, Bristol</t>
+          <t>Horizon - City Centre</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I56" s="7" t="n"/>
@@ -5013,7 +5015,7 @@
       <c r="L56" s="7" t="n"/>
       <c r="M56" s="7" t="n"/>
       <c r="N56" s="7" t="n">
-        <v>19400</v>
+        <v>22020</v>
       </c>
       <c r="O56" s="7" t="n">
         <v>0</v>
@@ -5021,17 +5023,17 @@
       <c r="P56" s="7" t="n"/>
       <c r="Q56" s="7" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R56" s="7" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bradley Stoke</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S56" s="8" t="inlineStr">
         <is>
-          <t>parking</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="T56" s="10" t="inlineStr">
@@ -5047,7 +5049,7 @@
       <c r="V56" s="6" t="inlineStr"/>
       <c r="W56" s="7" t="inlineStr">
         <is>
-          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
+          <t>25fbd71b098a83412bb2a614282b6fb33b9a3c90</t>
         </is>
       </c>
     </row>
@@ -5061,12 +5063,14 @@
         </is>
       </c>
       <c r="C57" s="9" t="n">
-        <v>2100</v>
+        <v>1550</v>
       </c>
       <c r="D57" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E57" s="7" t="n"/>
+      <c r="E57" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -5074,23 +5078,21 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>Beaufort Street, Stapleton, Bristol</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I57" s="7" t="n">
-        <v>800</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="n"/>
       <c r="J57" s="7" t="n"/>
       <c r="K57" s="7" t="n"/>
       <c r="L57" s="7" t="n"/>
       <c r="M57" s="7" t="n"/>
       <c r="N57" s="7" t="n">
-        <v>20800</v>
+        <v>19400</v>
       </c>
       <c r="O57" s="7" t="n">
         <v>0</v>
@@ -5098,12 +5100,12 @@
       <c r="P57" s="7" t="n"/>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Taylors Lettings, Bradley Stoke</t>
         </is>
       </c>
       <c r="S57" s="8" t="inlineStr">
@@ -5124,7 +5126,7 @@
       <c r="V57" s="6" t="inlineStr"/>
       <c r="W57" s="7" t="inlineStr">
         <is>
-          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
+          <t>81712a02a3a8827c0a71232c3b582e0d2b990a2a</t>
         </is>
       </c>
     </row>
@@ -5138,14 +5140,12 @@
         </is>
       </c>
       <c r="C58" s="9" t="n">
-        <v>2120</v>
+        <v>2100</v>
       </c>
       <c r="D58" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E58" s="7" t="n">
-        <v>2</v>
-      </c>
+      <c r="E58" s="7" t="n"/>
       <c r="F58" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>526 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="I58" s="7" t="n">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="J58" s="7" t="n"/>
       <c r="K58" s="7" t="n"/>
@@ -5203,7 +5203,7 @@
       <c r="V58" s="6" t="inlineStr"/>
       <c r="W58" s="7" t="inlineStr">
         <is>
-          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
+          <t>74d41470c07849b906ad0a12b07a1745551d8e6f</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
         </is>
       </c>
       <c r="C59" s="9" t="n">
-        <v>2150</v>
+        <v>2120</v>
       </c>
       <c r="D59" s="7" t="n">
         <v>2</v>
@@ -5232,7 +5232,7 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>522 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -5241,7 +5241,7 @@
         </is>
       </c>
       <c r="I59" s="7" t="n">
-        <v>809</v>
+        <v>799</v>
       </c>
       <c r="J59" s="7" t="n"/>
       <c r="K59" s="7" t="n"/>
@@ -5282,7 +5282,7 @@
       <c r="V59" s="6" t="inlineStr"/>
       <c r="W59" s="7" t="inlineStr">
         <is>
-          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
+          <t>4a3dbf2b76e61d3a02d3b62cb6a5a56affeadff0</t>
         </is>
       </c>
     </row>
@@ -5296,10 +5296,10 @@
         </is>
       </c>
       <c r="C60" s="9" t="n">
-        <v>2830</v>
+        <v>2150</v>
       </c>
       <c r="D60" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E60" s="7" t="n">
         <v>2</v>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>802 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
@@ -5320,7 +5320,7 @@
         </is>
       </c>
       <c r="I60" s="7" t="n">
-        <v>1120</v>
+        <v>809</v>
       </c>
       <c r="J60" s="7" t="n"/>
       <c r="K60" s="7" t="n"/>
@@ -5335,7 +5335,7 @@
       <c r="P60" s="7" t="n"/>
       <c r="Q60" s="7" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R60" s="7" t="inlineStr">
@@ -5361,7 +5361,7 @@
       <c r="V60" s="6" t="inlineStr"/>
       <c r="W60" s="7" t="inlineStr">
         <is>
-          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
+          <t>fcdcdd1da915be6f6b065ad9cbeea66062d00301</t>
         </is>
       </c>
     </row>
@@ -5375,13 +5375,13 @@
         </is>
       </c>
       <c r="C61" s="9" t="n">
-        <v>1680</v>
+        <v>2830</v>
       </c>
       <c r="D61" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
@@ -5390,7 +5390,7 @@
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
+          <t>315 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -5399,7 +5399,7 @@
         </is>
       </c>
       <c r="I61" s="7" t="n">
-        <v>557</v>
+        <v>1120</v>
       </c>
       <c r="J61" s="7" t="n"/>
       <c r="K61" s="7" t="n"/>
@@ -5414,7 +5414,7 @@
       <c r="P61" s="7" t="n"/>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="R61" s="7" t="inlineStr">
@@ -5440,7 +5440,7 @@
       <c r="V61" s="6" t="inlineStr"/>
       <c r="W61" s="7" t="inlineStr">
         <is>
-          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
+          <t>e4f6deef9389498e73820b4056b013ac2b6ff363</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5454,7 @@
         </is>
       </c>
       <c r="C62" s="9" t="n">
-        <v>1715</v>
+        <v>1680</v>
       </c>
       <c r="D62" s="7" t="n">
         <v>1</v>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>904 Dovetail, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
@@ -5478,7 +5478,7 @@
         </is>
       </c>
       <c r="I62" s="7" t="n">
-        <v>547</v>
+        <v>557</v>
       </c>
       <c r="J62" s="7" t="n"/>
       <c r="K62" s="7" t="n"/>
@@ -5519,7 +5519,7 @@
       <c r="V62" s="6" t="inlineStr"/>
       <c r="W62" s="7" t="inlineStr">
         <is>
-          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
+          <t>3d5fce4a62f2bd2b3bbd100f6bd7598155b266f2</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5533,7 @@
         </is>
       </c>
       <c r="C63" s="9" t="n">
-        <v>1655</v>
+        <v>1715</v>
       </c>
       <c r="D63" s="7" t="n">
         <v>1</v>
@@ -5548,7 +5548,7 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>1006 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
@@ -5572,7 +5572,7 @@
       <c r="P63" s="7" t="n"/>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R63" s="7" t="inlineStr">
@@ -5598,7 +5598,7 @@
       <c r="V63" s="6" t="inlineStr"/>
       <c r="W63" s="7" t="inlineStr">
         <is>
-          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
+          <t>baed14f153217bbfa48df27148f4a5b45559a145</t>
         </is>
       </c>
     </row>
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="C64" s="9" t="n">
-        <v>1665</v>
+        <v>1655</v>
       </c>
       <c r="D64" s="7" t="n">
         <v>1</v>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
+          <t>712 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
@@ -5636,7 +5636,7 @@
         </is>
       </c>
       <c r="I64" s="7" t="n">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="J64" s="7" t="n"/>
       <c r="K64" s="7" t="n"/>
@@ -5677,7 +5677,7 @@
       <c r="V64" s="6" t="inlineStr"/>
       <c r="W64" s="7" t="inlineStr">
         <is>
-          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
+          <t>219bc0a98e52a6b4cd0d3939d181df307abb678d</t>
         </is>
       </c>
     </row>
@@ -5691,13 +5691,13 @@
         </is>
       </c>
       <c r="C65" s="9" t="n">
-        <v>2400</v>
+        <v>1665</v>
       </c>
       <c r="D65" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
@@ -5706,21 +5706,23 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Gaol Ferry Steps, Bristol, BS1</t>
+          <t>425 Rosewood, New Kingsley Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I65" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="n">
+        <v>548</v>
+      </c>
       <c r="J65" s="7" t="n"/>
       <c r="K65" s="7" t="n"/>
       <c r="L65" s="7" t="n"/>
       <c r="M65" s="7" t="n"/>
       <c r="N65" s="7" t="n">
-        <v>16416</v>
+        <v>20800</v>
       </c>
       <c r="O65" s="7" t="n">
         <v>0</v>
@@ -5728,12 +5730,12 @@
       <c r="P65" s="7" t="n"/>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S65" s="8" t="inlineStr">
@@ -5754,7 +5756,7 @@
       <c r="V65" s="6" t="inlineStr"/>
       <c r="W65" s="7" t="inlineStr">
         <is>
-          <t>80580eaf8f14d71d98570c27e868e28d7528cf0d</t>
+          <t>51bc0e8bb190437e4c5c4710bf40ee90758a79f0</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6573,7 @@
         </is>
       </c>
       <c r="C77" s="9" t="n">
-        <v>2000</v>
+        <v>3200</v>
       </c>
       <c r="D77" s="7" t="n">
         <v>2</v>
@@ -6586,7 +6588,7 @@
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>Protheroes House, Hobbs Lane, BS1</t>
+          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
@@ -6600,7 +6602,7 @@
       <c r="L77" s="7" t="n"/>
       <c r="M77" s="7" t="n"/>
       <c r="N77" s="7" t="n">
-        <v>13584</v>
+        <v>16416</v>
       </c>
       <c r="O77" s="7" t="n">
         <v>0</v>
@@ -6613,7 +6615,7 @@
       </c>
       <c r="R77" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>LettingaProperty.com, Nationwide - Lettings</t>
         </is>
       </c>
       <c r="S77" s="8" t="inlineStr"/>
@@ -6630,7 +6632,7 @@
       <c r="V77" s="6" t="inlineStr"/>
       <c r="W77" s="7" t="inlineStr">
         <is>
-          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
+          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
         </is>
       </c>
     </row>
@@ -6644,13 +6646,13 @@
         </is>
       </c>
       <c r="C78" s="9" t="n">
-        <v>3200</v>
+        <v>1600</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E78" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
@@ -6659,7 +6661,7 @@
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
@@ -6673,7 +6675,7 @@
       <c r="L78" s="7" t="n"/>
       <c r="M78" s="7" t="n"/>
       <c r="N78" s="7" t="n">
-        <v>16416</v>
+        <v>21996</v>
       </c>
       <c r="O78" s="7" t="n">
         <v>0</v>
@@ -6686,7 +6688,7 @@
       </c>
       <c r="R78" s="7" t="inlineStr">
         <is>
-          <t>LettingaProperty.com, Nationwide - Lettings</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S78" s="8" t="inlineStr"/>
@@ -6703,7 +6705,7 @@
       <c r="V78" s="6" t="inlineStr"/>
       <c r="W78" s="7" t="inlineStr">
         <is>
-          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
+          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
         </is>
       </c>
     </row>
@@ -6717,36 +6719,38 @@
         </is>
       </c>
       <c r="C79" s="9" t="n">
-        <v>1600</v>
+        <v>2250</v>
       </c>
       <c r="D79" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Newfoundland Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I79" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I79" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J79" s="7" t="n"/>
       <c r="K79" s="7" t="n"/>
       <c r="L79" s="7" t="n"/>
       <c r="M79" s="7" t="n"/>
       <c r="N79" s="7" t="n">
-        <v>21996</v>
+        <v>19800</v>
       </c>
       <c r="O79" s="7" t="n">
         <v>0</v>
@@ -6754,12 +6758,12 @@
       <c r="P79" s="7" t="n"/>
       <c r="Q79" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R79" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Lets Rent Bristol, Bristol</t>
         </is>
       </c>
       <c r="S79" s="8" t="inlineStr"/>
@@ -6776,7 +6780,7 @@
       <c r="V79" s="6" t="inlineStr"/>
       <c r="W79" s="7" t="inlineStr">
         <is>
-          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
+          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
         </is>
       </c>
     </row>
@@ -6790,38 +6794,36 @@
         </is>
       </c>
       <c r="C80" s="9" t="n">
-        <v>2250</v>
+        <v>1400</v>
       </c>
       <c r="D80" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E80" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Newfoundland Road, Bristol, BS2</t>
+          <t>Invicta, Millenium Promenade, BS1</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I80" s="7" t="n">
-        <v>980</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I80" s="7" t="n"/>
       <c r="J80" s="7" t="n"/>
       <c r="K80" s="7" t="n"/>
       <c r="L80" s="7" t="n"/>
       <c r="M80" s="7" t="n"/>
       <c r="N80" s="7" t="n">
-        <v>19800</v>
+        <v>17344</v>
       </c>
       <c r="O80" s="7" t="n">
         <v>0</v>
@@ -6834,7 +6836,7 @@
       </c>
       <c r="R80" s="7" t="inlineStr">
         <is>
-          <t>Lets Rent Bristol, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S80" s="8" t="inlineStr"/>
@@ -6851,7 +6853,7 @@
       <c r="V80" s="6" t="inlineStr"/>
       <c r="W80" s="7" t="inlineStr">
         <is>
-          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
+          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6867,7 @@
         </is>
       </c>
       <c r="C81" s="9" t="n">
-        <v>1400</v>
+        <v>1600</v>
       </c>
       <c r="D81" s="7" t="n">
         <v>1</v>
@@ -6880,7 +6882,7 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>Invicta, Millenium Promenade, BS1</t>
+          <t>Central Quay North, Bristol, BS1</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
@@ -6894,7 +6896,7 @@
       <c r="L81" s="7" t="n"/>
       <c r="M81" s="7" t="n"/>
       <c r="N81" s="7" t="n">
-        <v>17344</v>
+        <v>13404</v>
       </c>
       <c r="O81" s="7" t="n">
         <v>0</v>
@@ -6907,7 +6909,7 @@
       </c>
       <c r="R81" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S81" s="8" t="inlineStr"/>
@@ -6924,7 +6926,7 @@
       <c r="V81" s="6" t="inlineStr"/>
       <c r="W81" s="7" t="inlineStr">
         <is>
-          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
+          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
         </is>
       </c>
     </row>
@@ -6938,7 +6940,7 @@
         </is>
       </c>
       <c r="C82" s="9" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="D82" s="7" t="n">
         <v>1</v>
@@ -6953,7 +6955,7 @@
       </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol, BS1</t>
+          <t>Eclipse, Broad Weir, Bristol</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
@@ -6967,7 +6969,7 @@
       <c r="L82" s="7" t="n"/>
       <c r="M82" s="7" t="n"/>
       <c r="N82" s="7" t="n">
-        <v>13404</v>
+        <v>22164</v>
       </c>
       <c r="O82" s="7" t="n">
         <v>0</v>
@@ -6980,7 +6982,7 @@
       </c>
       <c r="R82" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Martin &amp; Co, Bath</t>
         </is>
       </c>
       <c r="S82" s="8" t="inlineStr"/>
@@ -6997,7 +6999,7 @@
       <c r="V82" s="6" t="inlineStr"/>
       <c r="W82" s="7" t="inlineStr">
         <is>
-          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
+          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7013,7 @@
         </is>
       </c>
       <c r="C83" s="9" t="n">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="D83" s="7" t="n">
         <v>1</v>
@@ -7026,7 +7028,7 @@
       </c>
       <c r="G83" s="8" t="inlineStr">
         <is>
-          <t>Eclipse, Broad Weir, Bristol</t>
+          <t>Broad Weir, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
@@ -7034,13 +7036,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I83" s="7" t="n"/>
+      <c r="I83" s="7" t="n">
+        <v>474</v>
+      </c>
       <c r="J83" s="7" t="n"/>
       <c r="K83" s="7" t="n"/>
       <c r="L83" s="7" t="n"/>
       <c r="M83" s="7" t="n"/>
       <c r="N83" s="7" t="n">
-        <v>22164</v>
+        <v>22080</v>
       </c>
       <c r="O83" s="7" t="n">
         <v>0</v>
@@ -7048,12 +7052,12 @@
       <c r="P83" s="7" t="n"/>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R83" s="7" t="inlineStr">
         <is>
-          <t>Martin &amp; Co, Bath</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S83" s="8" t="inlineStr"/>
@@ -7070,7 +7074,7 @@
       <c r="V83" s="6" t="inlineStr"/>
       <c r="W83" s="7" t="inlineStr">
         <is>
-          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
+          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
         </is>
       </c>
     </row>
@@ -7084,7 +7088,7 @@
         </is>
       </c>
       <c r="C84" s="9" t="n">
-        <v>1800</v>
+        <v>1605</v>
       </c>
       <c r="D84" s="7" t="n">
         <v>1</v>
@@ -7099,7 +7103,7 @@
       </c>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t>Broad Weir, City Centre, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
@@ -7108,14 +7112,14 @@
         </is>
       </c>
       <c r="I84" s="7" t="n">
-        <v>474</v>
+        <v>487</v>
       </c>
       <c r="J84" s="7" t="n"/>
       <c r="K84" s="7" t="n"/>
       <c r="L84" s="7" t="n"/>
       <c r="M84" s="7" t="n"/>
       <c r="N84" s="7" t="n">
-        <v>22080</v>
+        <v>13860</v>
       </c>
       <c r="O84" s="7" t="n">
         <v>0</v>
@@ -7123,12 +7127,12 @@
       <c r="P84" s="7" t="n"/>
       <c r="Q84" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R84" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Clifton</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S84" s="8" t="inlineStr"/>
@@ -7145,7 +7149,7 @@
       <c r="V84" s="6" t="inlineStr"/>
       <c r="W84" s="7" t="inlineStr">
         <is>
-          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
+          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
         </is>
       </c>
     </row>
@@ -7159,13 +7163,13 @@
         </is>
       </c>
       <c r="C85" s="9" t="n">
-        <v>1605</v>
+        <v>2185</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
@@ -7183,7 +7187,7 @@
         </is>
       </c>
       <c r="I85" s="7" t="n">
-        <v>487</v>
+        <v>721</v>
       </c>
       <c r="J85" s="7" t="n"/>
       <c r="K85" s="7" t="n"/>
@@ -7220,7 +7224,7 @@
       <c r="V85" s="6" t="inlineStr"/>
       <c r="W85" s="7" t="inlineStr">
         <is>
-          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
+          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
         </is>
       </c>
     </row>
@@ -7234,13 +7238,13 @@
         </is>
       </c>
       <c r="C86" s="9" t="n">
-        <v>2185</v>
+        <v>1650</v>
       </c>
       <c r="D86" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E86" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" s="7" t="inlineStr">
         <is>
@@ -7249,23 +7253,21 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Crown &amp; Anchor House, Bristol, BS2</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I86" s="7" t="n">
-        <v>721</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I86" s="7" t="n"/>
       <c r="J86" s="7" t="n"/>
       <c r="K86" s="7" t="n"/>
       <c r="L86" s="7" t="n"/>
       <c r="M86" s="7" t="n"/>
       <c r="N86" s="7" t="n">
-        <v>13860</v>
+        <v>20472</v>
       </c>
       <c r="O86" s="7" t="n">
         <v>0</v>
@@ -7273,12 +7275,12 @@
       <c r="P86" s="7" t="n"/>
       <c r="Q86" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R86" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S86" s="8" t="inlineStr"/>
@@ -7295,7 +7297,7 @@
       <c r="V86" s="6" t="inlineStr"/>
       <c r="W86" s="7" t="inlineStr">
         <is>
-          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
+          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
         </is>
       </c>
     </row>
@@ -7309,10 +7311,10 @@
         </is>
       </c>
       <c r="C87" s="9" t="n">
-        <v>1650</v>
+        <v>1640</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E87" s="7" t="n">
         <v>1</v>
@@ -7324,21 +7326,23 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>Crown &amp; Anchor House, Bristol, BS2</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I87" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I87" s="7" t="n">
+        <v>484</v>
+      </c>
       <c r="J87" s="7" t="n"/>
       <c r="K87" s="7" t="n"/>
       <c r="L87" s="7" t="n"/>
       <c r="M87" s="7" t="n"/>
       <c r="N87" s="7" t="n">
-        <v>20472</v>
+        <v>13860</v>
       </c>
       <c r="O87" s="7" t="n">
         <v>0</v>
@@ -7351,7 +7355,7 @@
       </c>
       <c r="R87" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S87" s="8" t="inlineStr"/>
@@ -7368,7 +7372,7 @@
       <c r="V87" s="6" t="inlineStr"/>
       <c r="W87" s="7" t="inlineStr">
         <is>
-          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
+          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
         </is>
       </c>
     </row>
@@ -7382,13 +7386,13 @@
         </is>
       </c>
       <c r="C88" s="9" t="n">
-        <v>1640</v>
+        <v>1650</v>
       </c>
       <c r="D88" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E88" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
@@ -7397,7 +7401,7 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Harbourside, Harris Lofts, BS1 4BB</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
@@ -7406,14 +7410,14 @@
         </is>
       </c>
       <c r="I88" s="7" t="n">
-        <v>484</v>
+        <v>667</v>
       </c>
       <c r="J88" s="7" t="n"/>
       <c r="K88" s="7" t="n"/>
       <c r="L88" s="7" t="n"/>
       <c r="M88" s="7" t="n"/>
       <c r="N88" s="7" t="n">
-        <v>13860</v>
+        <v>20088</v>
       </c>
       <c r="O88" s="7" t="n">
         <v>0</v>
@@ -7421,12 +7425,12 @@
       <c r="P88" s="7" t="n"/>
       <c r="Q88" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R88" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S88" s="8" t="inlineStr"/>
@@ -7443,7 +7447,7 @@
       <c r="V88" s="6" t="inlineStr"/>
       <c r="W88" s="7" t="inlineStr">
         <is>
-          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
+          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
         </is>
       </c>
     </row>
@@ -7460,10 +7464,10 @@
         <v>1650</v>
       </c>
       <c r="D89" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
@@ -7472,7 +7476,7 @@
       </c>
       <c r="G89" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Harris Lofts, BS1 4BB</t>
+          <t>Central Quey North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
@@ -7480,15 +7484,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I89" s="7" t="n">
-        <v>667</v>
-      </c>
+      <c r="I89" s="7" t="n"/>
       <c r="J89" s="7" t="n"/>
       <c r="K89" s="7" t="n"/>
       <c r="L89" s="7" t="n"/>
       <c r="M89" s="7" t="n"/>
       <c r="N89" s="7" t="n">
-        <v>20088</v>
+        <v>20768</v>
       </c>
       <c r="O89" s="7" t="n">
         <v>0</v>
@@ -7501,7 +7503,7 @@
       </c>
       <c r="R89" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S89" s="8" t="inlineStr"/>
@@ -7518,7 +7520,7 @@
       <c r="V89" s="6" t="inlineStr"/>
       <c r="W89" s="7" t="inlineStr">
         <is>
-          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
+          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
         </is>
       </c>
     </row>
@@ -7532,13 +7534,13 @@
         </is>
       </c>
       <c r="C90" s="9" t="n">
-        <v>1650</v>
+        <v>1450</v>
       </c>
       <c r="D90" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F90" s="7" t="inlineStr">
         <is>
@@ -7547,21 +7549,23 @@
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>Central Quey North, Broad Quay, BS1</t>
+          <t>Woodbridge Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I90" s="7" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I90" s="7" t="n">
+        <v>678</v>
+      </c>
       <c r="J90" s="7" t="n"/>
       <c r="K90" s="7" t="n"/>
       <c r="L90" s="7" t="n"/>
       <c r="M90" s="7" t="n"/>
       <c r="N90" s="7" t="n">
-        <v>20768</v>
+        <v>5700</v>
       </c>
       <c r="O90" s="7" t="n">
         <v>0</v>
@@ -7574,7 +7578,7 @@
       </c>
       <c r="R90" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S90" s="8" t="inlineStr"/>
@@ -7591,7 +7595,7 @@
       <c r="V90" s="6" t="inlineStr"/>
       <c r="W90" s="7" t="inlineStr">
         <is>
-          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
+          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
         </is>
       </c>
     </row>
@@ -7605,10 +7609,10 @@
         </is>
       </c>
       <c r="C91" s="9" t="n">
-        <v>1450</v>
+        <v>2010</v>
       </c>
       <c r="D91" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E91" s="7" t="n">
         <v>2</v>
@@ -7620,23 +7624,23 @@
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>Woodbridge Road, Bristol, BS4</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I91" s="7" t="n">
-        <v>678</v>
+        <v>722</v>
       </c>
       <c r="J91" s="7" t="n"/>
       <c r="K91" s="7" t="n"/>
       <c r="L91" s="7" t="n"/>
       <c r="M91" s="7" t="n"/>
       <c r="N91" s="7" t="n">
-        <v>5700</v>
+        <v>13860</v>
       </c>
       <c r="O91" s="7" t="n">
         <v>0</v>
@@ -7644,12 +7648,12 @@
       <c r="P91" s="7" t="n"/>
       <c r="Q91" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R91" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S91" s="8" t="inlineStr"/>
@@ -7666,7 +7670,7 @@
       <c r="V91" s="6" t="inlineStr"/>
       <c r="W91" s="7" t="inlineStr">
         <is>
-          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
+          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
         </is>
       </c>
     </row>
@@ -7680,13 +7684,13 @@
         </is>
       </c>
       <c r="C92" s="9" t="n">
-        <v>2010</v>
+        <v>1630</v>
       </c>
       <c r="D92" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E92" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F92" s="7" t="inlineStr">
         <is>
@@ -7704,7 +7708,7 @@
         </is>
       </c>
       <c r="I92" s="7" t="n">
-        <v>722</v>
+        <v>486</v>
       </c>
       <c r="J92" s="7" t="n"/>
       <c r="K92" s="7" t="n"/>
@@ -7741,7 +7745,7 @@
       <c r="V92" s="6" t="inlineStr"/>
       <c r="W92" s="7" t="inlineStr">
         <is>
-          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
+          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7759,7 @@
         </is>
       </c>
       <c r="C93" s="9" t="n">
-        <v>1630</v>
+        <v>1635</v>
       </c>
       <c r="D93" s="7" t="n">
         <v>1</v>
@@ -7770,7 +7774,7 @@
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
@@ -7779,14 +7783,14 @@
         </is>
       </c>
       <c r="I93" s="7" t="n">
-        <v>486</v>
+        <v>560</v>
       </c>
       <c r="J93" s="7" t="n"/>
       <c r="K93" s="7" t="n"/>
       <c r="L93" s="7" t="n"/>
       <c r="M93" s="7" t="n"/>
       <c r="N93" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O93" s="7" t="n">
         <v>0</v>
@@ -7799,7 +7803,7 @@
       </c>
       <c r="R93" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S93" s="8" t="inlineStr"/>
@@ -7816,7 +7820,7 @@
       <c r="V93" s="6" t="inlineStr"/>
       <c r="W93" s="7" t="inlineStr">
         <is>
-          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
+          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
         </is>
       </c>
     </row>
@@ -7830,7 +7834,7 @@
         </is>
       </c>
       <c r="C94" s="9" t="n">
-        <v>1635</v>
+        <v>1665</v>
       </c>
       <c r="D94" s="7" t="n">
         <v>1</v>
@@ -7845,7 +7849,7 @@
       </c>
       <c r="G94" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
@@ -7854,14 +7858,14 @@
         </is>
       </c>
       <c r="I94" s="7" t="n">
-        <v>560</v>
+        <v>434</v>
       </c>
       <c r="J94" s="7" t="n"/>
       <c r="K94" s="7" t="n"/>
       <c r="L94" s="7" t="n"/>
       <c r="M94" s="7" t="n"/>
       <c r="N94" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O94" s="7" t="n">
         <v>0</v>
@@ -7874,7 +7878,7 @@
       </c>
       <c r="R94" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S94" s="8" t="inlineStr"/>
@@ -7891,7 +7895,7 @@
       <c r="V94" s="6" t="inlineStr"/>
       <c r="W94" s="7" t="inlineStr">
         <is>
-          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
+          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
         </is>
       </c>
     </row>
@@ -7905,7 +7909,7 @@
         </is>
       </c>
       <c r="C95" s="9" t="n">
-        <v>1665</v>
+        <v>1400</v>
       </c>
       <c r="D95" s="7" t="n">
         <v>1</v>
@@ -7920,7 +7924,7 @@
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>The Atrium, Redcliffe Street, BS1</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
@@ -7928,15 +7932,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I95" s="7" t="n">
-        <v>434</v>
-      </c>
+      <c r="I95" s="7" t="n"/>
       <c r="J95" s="7" t="n"/>
       <c r="K95" s="7" t="n"/>
       <c r="L95" s="7" t="n"/>
       <c r="M95" s="7" t="n"/>
       <c r="N95" s="7" t="n">
-        <v>13964</v>
+        <v>20292</v>
       </c>
       <c r="O95" s="7" t="n">
         <v>0</v>
@@ -7949,7 +7951,7 @@
       </c>
       <c r="R95" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S95" s="8" t="inlineStr"/>
@@ -7966,7 +7968,7 @@
       <c r="V95" s="6" t="inlineStr"/>
       <c r="W95" s="7" t="inlineStr">
         <is>
-          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
+          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
         </is>
       </c>
     </row>
@@ -7980,7 +7982,7 @@
         </is>
       </c>
       <c r="C96" s="9" t="n">
-        <v>1400</v>
+        <v>1460</v>
       </c>
       <c r="D96" s="7" t="n">
         <v>1</v>
@@ -7995,7 +7997,7 @@
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>The Atrium, Redcliffe Street, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
@@ -8003,13 +8005,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I96" s="7" t="n"/>
+      <c r="I96" s="7" t="n">
+        <v>473</v>
+      </c>
       <c r="J96" s="7" t="n"/>
       <c r="K96" s="7" t="n"/>
       <c r="L96" s="7" t="n"/>
       <c r="M96" s="7" t="n"/>
       <c r="N96" s="7" t="n">
-        <v>20292</v>
+        <v>21476</v>
       </c>
       <c r="O96" s="7" t="n">
         <v>0</v>
@@ -8017,12 +8021,12 @@
       <c r="P96" s="7" t="n"/>
       <c r="Q96" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R96" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S96" s="8" t="inlineStr"/>
@@ -8039,7 +8043,7 @@
       <c r="V96" s="6" t="inlineStr"/>
       <c r="W96" s="7" t="inlineStr">
         <is>
-          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
+          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
         </is>
       </c>
     </row>
@@ -8053,13 +8057,13 @@
         </is>
       </c>
       <c r="C97" s="9" t="n">
-        <v>1460</v>
+        <v>1990</v>
       </c>
       <c r="D97" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E97" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
@@ -8077,14 +8081,14 @@
         </is>
       </c>
       <c r="I97" s="7" t="n">
-        <v>473</v>
+        <v>682</v>
       </c>
       <c r="J97" s="7" t="n"/>
       <c r="K97" s="7" t="n"/>
       <c r="L97" s="7" t="n"/>
       <c r="M97" s="7" t="n"/>
       <c r="N97" s="7" t="n">
-        <v>21476</v>
+        <v>13964</v>
       </c>
       <c r="O97" s="7" t="n">
         <v>0</v>
@@ -8114,7 +8118,7 @@
       <c r="V97" s="6" t="inlineStr"/>
       <c r="W97" s="7" t="inlineStr">
         <is>
-          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
+          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
         </is>
       </c>
     </row>
@@ -8128,13 +8132,13 @@
         </is>
       </c>
       <c r="C98" s="9" t="n">
-        <v>1990</v>
+        <v>1640</v>
       </c>
       <c r="D98" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E98" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
@@ -8143,7 +8147,7 @@
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
@@ -8152,14 +8156,14 @@
         </is>
       </c>
       <c r="I98" s="7" t="n">
-        <v>682</v>
+        <v>487</v>
       </c>
       <c r="J98" s="7" t="n"/>
       <c r="K98" s="7" t="n"/>
       <c r="L98" s="7" t="n"/>
       <c r="M98" s="7" t="n"/>
       <c r="N98" s="7" t="n">
-        <v>13964</v>
+        <v>13356</v>
       </c>
       <c r="O98" s="7" t="n">
         <v>0</v>
@@ -8172,7 +8176,7 @@
       </c>
       <c r="R98" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S98" s="8" t="inlineStr"/>
@@ -8189,7 +8193,7 @@
       <c r="V98" s="6" t="inlineStr"/>
       <c r="W98" s="7" t="inlineStr">
         <is>
-          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
+          <t>ecc803f25866be367a83778bda0456688426a26e</t>
         </is>
       </c>
     </row>
@@ -8203,7 +8207,7 @@
         </is>
       </c>
       <c r="C99" s="9" t="n">
-        <v>1640</v>
+        <v>1300</v>
       </c>
       <c r="D99" s="7" t="n">
         <v>1</v>
@@ -8218,7 +8222,7 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>City Centre, Deanery Road, BS1 5AF</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
@@ -8227,14 +8231,14 @@
         </is>
       </c>
       <c r="I99" s="7" t="n">
-        <v>487</v>
+        <v>570</v>
       </c>
       <c r="J99" s="7" t="n"/>
       <c r="K99" s="7" t="n"/>
       <c r="L99" s="7" t="n"/>
       <c r="M99" s="7" t="n"/>
       <c r="N99" s="7" t="n">
-        <v>13356</v>
+        <v>19300</v>
       </c>
       <c r="O99" s="7" t="n">
         <v>0</v>
@@ -8247,7 +8251,7 @@
       </c>
       <c r="R99" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S99" s="8" t="inlineStr"/>
@@ -8264,7 +8268,7 @@
       <c r="V99" s="6" t="inlineStr"/>
       <c r="W99" s="7" t="inlineStr">
         <is>
-          <t>ecc803f25866be367a83778bda0456688426a26e</t>
+          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
         </is>
       </c>
     </row>
@@ -8278,7 +8282,7 @@
         </is>
       </c>
       <c r="C100" s="9" t="n">
-        <v>1300</v>
+        <v>1995</v>
       </c>
       <c r="D100" s="7" t="n">
         <v>1</v>
@@ -8293,7 +8297,7 @@
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Deanery Road, BS1 5AF</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr">
@@ -8301,15 +8305,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I100" s="7" t="n">
-        <v>570</v>
-      </c>
+      <c r="I100" s="7" t="n"/>
       <c r="J100" s="7" t="n"/>
       <c r="K100" s="7" t="n"/>
       <c r="L100" s="7" t="n"/>
       <c r="M100" s="7" t="n"/>
       <c r="N100" s="7" t="n">
-        <v>19300</v>
+        <v>21196</v>
       </c>
       <c r="O100" s="7" t="n">
         <v>0</v>
@@ -8322,7 +8324,7 @@
       </c>
       <c r="R100" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S100" s="8" t="inlineStr"/>
@@ -8339,7 +8341,7 @@
       <c r="V100" s="6" t="inlineStr"/>
       <c r="W100" s="7" t="inlineStr">
         <is>
-          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
+          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
         </is>
       </c>
     </row>
@@ -8353,7 +8355,7 @@
         </is>
       </c>
       <c r="C101" s="9" t="n">
-        <v>1995</v>
+        <v>1395</v>
       </c>
       <c r="D101" s="7" t="n">
         <v>1</v>
@@ -8368,7 +8370,7 @@
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
@@ -8382,7 +8384,7 @@
       <c r="L101" s="7" t="n"/>
       <c r="M101" s="7" t="n"/>
       <c r="N101" s="7" t="n">
-        <v>21196</v>
+        <v>20524</v>
       </c>
       <c r="O101" s="7" t="n">
         <v>0</v>
@@ -8390,7 +8392,7 @@
       <c r="P101" s="7" t="n"/>
       <c r="Q101" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R101" s="7" t="inlineStr">
@@ -8412,7 +8414,7 @@
       <c r="V101" s="6" t="inlineStr"/>
       <c r="W101" s="7" t="inlineStr">
         <is>
-          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
@@ -8426,13 +8428,13 @@
         </is>
       </c>
       <c r="C102" s="9" t="n">
-        <v>1395</v>
+        <v>2085</v>
       </c>
       <c r="D102" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E102" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F102" s="7" t="inlineStr">
         <is>
@@ -8441,7 +8443,7 @@
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr">
@@ -8449,13 +8451,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I102" s="7" t="n"/>
+      <c r="I102" s="7" t="n">
+        <v>722</v>
+      </c>
       <c r="J102" s="7" t="n"/>
       <c r="K102" s="7" t="n"/>
       <c r="L102" s="7" t="n"/>
       <c r="M102" s="7" t="n"/>
       <c r="N102" s="7" t="n">
-        <v>20524</v>
+        <v>13860</v>
       </c>
       <c r="O102" s="7" t="n">
         <v>0</v>
@@ -8468,7 +8472,7 @@
       </c>
       <c r="R102" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S102" s="8" t="inlineStr"/>
@@ -8485,7 +8489,7 @@
       <c r="V102" s="6" t="inlineStr"/>
       <c r="W102" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
         </is>
       </c>
     </row>
@@ -8499,13 +8503,13 @@
         </is>
       </c>
       <c r="C103" s="9" t="n">
-        <v>2085</v>
+        <v>1485</v>
       </c>
       <c r="D103" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E103" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
@@ -8514,7 +8518,7 @@
       </c>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr">
@@ -8523,14 +8527,14 @@
         </is>
       </c>
       <c r="I103" s="7" t="n">
-        <v>722</v>
+        <v>470</v>
       </c>
       <c r="J103" s="7" t="n"/>
       <c r="K103" s="7" t="n"/>
       <c r="L103" s="7" t="n"/>
       <c r="M103" s="7" t="n"/>
       <c r="N103" s="7" t="n">
-        <v>13860</v>
+        <v>21476</v>
       </c>
       <c r="O103" s="7" t="n">
         <v>0</v>
@@ -8543,7 +8547,7 @@
       </c>
       <c r="R103" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S103" s="8" t="inlineStr"/>
@@ -8560,7 +8564,7 @@
       <c r="V103" s="6" t="inlineStr"/>
       <c r="W103" s="7" t="inlineStr">
         <is>
-          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
+          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
         </is>
       </c>
     </row>
@@ -8574,7 +8578,7 @@
         </is>
       </c>
       <c r="C104" s="9" t="n">
-        <v>1485</v>
+        <v>1650</v>
       </c>
       <c r="D104" s="7" t="n">
         <v>1</v>
@@ -8589,7 +8593,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr">
@@ -8598,14 +8602,14 @@
         </is>
       </c>
       <c r="I104" s="7" t="n">
-        <v>470</v>
+        <v>553</v>
       </c>
       <c r="J104" s="7" t="n"/>
       <c r="K104" s="7" t="n"/>
       <c r="L104" s="7" t="n"/>
       <c r="M104" s="7" t="n"/>
       <c r="N104" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O104" s="7" t="n">
         <v>0</v>
@@ -8618,7 +8622,7 @@
       </c>
       <c r="R104" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S104" s="8" t="inlineStr"/>
@@ -8635,7 +8639,7 @@
       <c r="V104" s="6" t="inlineStr"/>
       <c r="W104" s="7" t="inlineStr">
         <is>
-          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
+          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
         </is>
       </c>
     </row>
@@ -8652,10 +8656,10 @@
         <v>1650</v>
       </c>
       <c r="D105" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E105" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
@@ -8664,7 +8668,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr">
@@ -8672,15 +8676,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I105" s="7" t="n">
-        <v>553</v>
-      </c>
+      <c r="I105" s="7" t="n"/>
       <c r="J105" s="7" t="n"/>
       <c r="K105" s="7" t="n"/>
       <c r="L105" s="7" t="n"/>
       <c r="M105" s="7" t="n"/>
       <c r="N105" s="7" t="n">
-        <v>13356</v>
+        <v>20880</v>
       </c>
       <c r="O105" s="7" t="n">
         <v>0</v>
@@ -8688,12 +8690,12 @@
       <c r="P105" s="7" t="n"/>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R105" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S105" s="8" t="inlineStr"/>
@@ -8710,7 +8712,7 @@
       <c r="V105" s="6" t="inlineStr"/>
       <c r="W105" s="7" t="inlineStr">
         <is>
-          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
+          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
         </is>
       </c>
     </row>
@@ -8724,7 +8726,7 @@
         </is>
       </c>
       <c r="C106" s="9" t="n">
-        <v>1650</v>
+        <v>1900</v>
       </c>
       <c r="D106" s="7" t="n">
         <v>2</v>
@@ -8739,7 +8741,7 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Waverley House, BS1</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr">
@@ -8753,7 +8755,7 @@
       <c r="L106" s="7" t="n"/>
       <c r="M106" s="7" t="n"/>
       <c r="N106" s="7" t="n">
-        <v>20880</v>
+        <v>17956</v>
       </c>
       <c r="O106" s="7" t="n">
         <v>0</v>
@@ -8766,7 +8768,7 @@
       </c>
       <c r="R106" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S106" s="8" t="inlineStr"/>
@@ -8783,7 +8785,7 @@
       <c r="V106" s="6" t="inlineStr"/>
       <c r="W106" s="7" t="inlineStr">
         <is>
-          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
+          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8799,7 @@
         </is>
       </c>
       <c r="C107" s="9" t="n">
-        <v>1900</v>
+        <v>2000</v>
       </c>
       <c r="D107" s="7" t="n">
         <v>2</v>
@@ -8812,7 +8814,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>Waverley House, BS1</t>
+          <t>Protheroes House, Hobbs Lane, BS1</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr">
@@ -8826,7 +8828,7 @@
       <c r="L107" s="7" t="n"/>
       <c r="M107" s="7" t="n"/>
       <c r="N107" s="7" t="n">
-        <v>17956</v>
+        <v>13584</v>
       </c>
       <c r="O107" s="7" t="n">
         <v>0</v>
@@ -8834,12 +8836,12 @@
       <c r="P107" s="7" t="n"/>
       <c r="Q107" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R107" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S107" s="8" t="inlineStr"/>
@@ -8856,7 +8858,7 @@
       <c r="V107" s="6" t="inlineStr"/>
       <c r="W107" s="7" t="inlineStr">
         <is>
-          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
+          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
         </is>
       </c>
     </row>
@@ -13312,156 +13314,10 @@
         </is>
       </c>
     </row>
-    <row r="168">
-      <c r="A168" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B168" s="8" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C168" s="9" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D168" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E168" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F168" s="7" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G168" s="8" t="inlineStr">
-        <is>
-          <t>Talavera Close, Bristol</t>
-        </is>
-      </c>
-      <c r="H168" s="7" t="inlineStr">
-        <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I168" s="7" t="n"/>
-      <c r="J168" s="7" t="n"/>
-      <c r="K168" s="7" t="n"/>
-      <c r="L168" s="7" t="n"/>
-      <c r="M168" s="7" t="n"/>
-      <c r="N168" s="7" t="n">
-        <v>19980</v>
-      </c>
-      <c r="O168" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P168" s="7" t="n"/>
-      <c r="Q168" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="R168" s="7" t="inlineStr">
-        <is>
-          <t>Campions Property Lettings &amp; Management Ltd, National</t>
-        </is>
-      </c>
-      <c r="S168" s="8" t="inlineStr"/>
-      <c r="T168" s="10" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U168" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V168" s="6" t="inlineStr"/>
-      <c r="W168" s="7" t="inlineStr">
-        <is>
-          <t>e0a93f8e75c81900b60248c526509a97c04a5289</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B169" s="8" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C169" s="9" t="n">
-        <v>2300</v>
-      </c>
-      <c r="D169" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E169" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F169" s="7" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G169" s="8" t="inlineStr">
-        <is>
-          <t>Mill Lane, Bedminster, Bristol, BS3</t>
-        </is>
-      </c>
-      <c r="H169" s="7" t="inlineStr">
-        <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I169" s="7" t="n"/>
-      <c r="J169" s="7" t="n"/>
-      <c r="K169" s="7" t="n"/>
-      <c r="L169" s="7" t="n"/>
-      <c r="M169" s="7" t="n"/>
-      <c r="N169" s="7" t="n">
-        <v>11524</v>
-      </c>
-      <c r="O169" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P169" s="7" t="n"/>
-      <c r="Q169" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="R169" s="7" t="inlineStr">
-        <is>
-          <t>Howard, Bristol</t>
-        </is>
-      </c>
-      <c r="S169" s="8" t="inlineStr"/>
-      <c r="T169" s="10" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U169" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V169" s="6" t="inlineStr"/>
-      <c r="W169" s="7" t="inlineStr">
-        <is>
-          <t>955f1495a28b861e234b64739033e0312fd2b568</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W169"/>
+  <autoFilter ref="A1:W167"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -13632,8 +13488,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T165" r:id="rId164"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T166" r:id="rId165"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T167" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T168" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T169" r:id="rId168"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 102
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -1895,7 +1895,7 @@
       <c r="L16" s="7" t="n"/>
       <c r="M16" s="7" t="n"/>
       <c r="N16" s="7" t="n">
-        <v>21152</v>
+        <v>21140</v>
       </c>
       <c r="O16" s="7" t="n">
         <v>0</v>
@@ -1974,7 +1974,7 @@
       <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="n"/>
       <c r="N17" s="7" t="n">
-        <v>13408</v>
+        <v>20780</v>
       </c>
       <c r="O17" s="7" t="n">
         <v>0</v>
@@ -2053,7 +2053,7 @@
       <c r="L18" s="7" t="n"/>
       <c r="M18" s="7" t="n"/>
       <c r="N18" s="7" t="n">
-        <v>21152</v>
+        <v>21140</v>
       </c>
       <c r="O18" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
House search data from run 105
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W164"/>
+  <dimension ref="A1:W163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1090,10 +1090,10 @@
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2830</v>
+        <v>1850</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>2</v>
@@ -1105,23 +1105,21 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>315 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>The Laureate, Charles Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>1120</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7" t="n"/>
       <c r="N6" s="7" t="n">
-        <v>21152</v>
+        <v>21912</v>
       </c>
       <c r="O6" s="7" t="n">
         <v>0</v>
@@ -1129,12 +1127,12 @@
       <c r="P6" s="7" t="n"/>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S6" s="8" t="inlineStr">
@@ -1155,7 +1153,7 @@
       <c r="V6" s="6" t="inlineStr"/>
       <c r="W6" s="7" t="inlineStr">
         <is>
-          <t>b70e24d9417674d7a16e52abd8d5a34b925d04ea</t>
+          <t>8d6d721187298dcfb94d30d9172f6f10952dc87d</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1167,7 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>1850</v>
+        <v>2000</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>2</v>
@@ -1184,7 +1182,7 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>The Laureate, Charles Street, Bristol, BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1198,7 +1196,7 @@
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="n"/>
       <c r="N7" s="7" t="n">
-        <v>21912</v>
+        <v>16644</v>
       </c>
       <c r="O7" s="7" t="n">
         <v>0</v>
@@ -1211,7 +1209,7 @@
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S7" s="8" t="inlineStr">
@@ -1232,7 +1230,7 @@
       <c r="V7" s="6" t="inlineStr"/>
       <c r="W7" s="7" t="inlineStr">
         <is>
-          <t>8d6d721187298dcfb94d30d9172f6f10952dc87d</t>
+          <t>1e517b09a4d3bd665354a55c719f877b837af199</t>
         </is>
       </c>
     </row>
@@ -1246,27 +1244,27 @@
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>2000</v>
+        <v>2600</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol</t>
+          <t>Norfolk Heights, BS2</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I8" s="7" t="n"/>
@@ -1275,7 +1273,7 @@
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n">
-        <v>16644</v>
+        <v>21800</v>
       </c>
       <c r="O8" s="7" t="n">
         <v>0</v>
@@ -1288,7 +1286,7 @@
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol</t>
         </is>
       </c>
       <c r="S8" s="8" t="inlineStr">
@@ -1309,7 +1307,7 @@
       <c r="V8" s="6" t="inlineStr"/>
       <c r="W8" s="7" t="inlineStr">
         <is>
-          <t>1e517b09a4d3bd665354a55c719f877b837af199</t>
+          <t>2c2a0756e18994fc5ddb57fd3f3b4e46f6b18829</t>
         </is>
       </c>
     </row>
@@ -1323,27 +1321,27 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>2600</v>
+        <v>1600</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Norfolk Heights, BS2</t>
+          <t>Magdalena Court, Redcliffe, Bristol City Centre</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I9" s="7" t="n"/>
@@ -1352,7 +1350,7 @@
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="n"/>
       <c r="N9" s="7" t="n">
-        <v>21800</v>
+        <v>18672</v>
       </c>
       <c r="O9" s="7" t="n">
         <v>0</v>
@@ -1360,7 +1358,7 @@
       <c r="P9" s="7" t="n"/>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
@@ -1386,7 +1384,7 @@
       <c r="V9" s="6" t="inlineStr"/>
       <c r="W9" s="7" t="inlineStr">
         <is>
-          <t>2c2a0756e18994fc5ddb57fd3f3b4e46f6b18829</t>
+          <t>d1a94a3de68ac71225d3643c6e5ec331fbc7261e</t>
         </is>
       </c>
     </row>
@@ -1400,13 +1398,13 @@
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -1415,7 +1413,7 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Magdalena Court, Redcliffe, Bristol City Centre</t>
+          <t>The Panoramic, Park Row, BS1</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1429,7 +1427,7 @@
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7" t="n"/>
       <c r="N10" s="7" t="n">
-        <v>18672</v>
+        <v>20940</v>
       </c>
       <c r="O10" s="7" t="n">
         <v>0</v>
@@ -1437,12 +1435,12 @@
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S10" s="8" t="inlineStr">
@@ -1463,7 +1461,7 @@
       <c r="V10" s="6" t="inlineStr"/>
       <c r="W10" s="7" t="inlineStr">
         <is>
-          <t>d1a94a3de68ac71225d3643c6e5ec331fbc7261e</t>
+          <t>454917a7536fb9944c891f2559e33e66404388a1</t>
         </is>
       </c>
     </row>
@@ -1477,13 +1475,13 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>1800</v>
+        <v>1200</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
@@ -1492,12 +1490,12 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>The Panoramic, Park Row, BS1</t>
+          <t>Union Road, Bristol</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I11" s="7" t="n"/>
@@ -1506,7 +1504,7 @@
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="n"/>
       <c r="N11" s="7" t="n">
-        <v>20940</v>
+        <v>20080</v>
       </c>
       <c r="O11" s="7" t="n">
         <v>0</v>
@@ -1514,12 +1512,12 @@
       <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S11" s="8" t="inlineStr">
@@ -1540,7 +1538,7 @@
       <c r="V11" s="6" t="inlineStr"/>
       <c r="W11" s="7" t="inlineStr">
         <is>
-          <t>454917a7536fb9944c891f2559e33e66404388a1</t>
+          <t>4558d8edbc8cb892b2ba019e5ce18d84db095b71</t>
         </is>
       </c>
     </row>
@@ -1554,13 +1552,13 @@
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>1200</v>
+        <v>2695</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -1569,21 +1567,23 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Union Road, Bristol</t>
+          <t>Guinea Street, Bristol, Somerset, BS1</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>935</v>
+      </c>
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7" t="n"/>
       <c r="N12" s="7" t="n">
-        <v>20080</v>
+        <v>18508</v>
       </c>
       <c r="O12" s="7" t="n">
         <v>0</v>
@@ -1591,12 +1591,12 @@
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Savills Lettings, Clifton</t>
         </is>
       </c>
       <c r="S12" s="8" t="inlineStr">
@@ -1617,7 +1617,7 @@
       <c r="V12" s="6" t="inlineStr"/>
       <c r="W12" s="7" t="inlineStr">
         <is>
-          <t>4558d8edbc8cb892b2ba019e5ce18d84db095b71</t>
+          <t>2e2a5701906948994c2a2e41c1281a602dad764c</t>
         </is>
       </c>
     </row>
@@ -1631,13 +1631,13 @@
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
+          <t>Marsh House, Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I13" s="7" t="n"/>
@@ -1660,7 +1660,7 @@
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7" t="n"/>
       <c r="N13" s="7" t="n">
-        <v>5244</v>
+        <v>20788</v>
       </c>
       <c r="O13" s="7" t="n">
         <v>0</v>
@@ -1668,12 +1668,12 @@
       <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Kingswood</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S13" s="8" t="inlineStr">
@@ -1694,7 +1694,7 @@
       <c r="V13" s="6" t="inlineStr"/>
       <c r="W13" s="7" t="inlineStr">
         <is>
-          <t>6b42638cf55169ff2e715f3f1db70e5db21111f3</t>
+          <t>8056582dfefc0ed6bd89dfe9a286f4e11c283370</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>2695</v>
+        <v>2000</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>2</v>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Guinea Street, Bristol, Somerset, BS1</t>
+          <t>Lower Park Row - City Centre</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1731,15 +1731,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I14" s="7" t="n">
-        <v>935</v>
-      </c>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7" t="n"/>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7" t="n"/>
       <c r="N14" s="7" t="n">
-        <v>18508</v>
+        <v>21532</v>
       </c>
       <c r="O14" s="7" t="n">
         <v>0</v>
@@ -1747,12 +1745,12 @@
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, Clifton</t>
+          <t>Ocean, Clifton</t>
         </is>
       </c>
       <c r="S14" s="8" t="inlineStr">
@@ -1773,7 +1771,7 @@
       <c r="V14" s="6" t="inlineStr"/>
       <c r="W14" s="7" t="inlineStr">
         <is>
-          <t>2e2a5701906948994c2a2e41c1281a602dad764c</t>
+          <t>8c589025b84fb12583a29c490c3882a26aca2559</t>
         </is>
       </c>
     </row>
@@ -1787,13 +1785,13 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>1800</v>
+        <v>1300</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
@@ -1802,21 +1800,23 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Marsh House, Marsh Street, Bristol, BS1</t>
+          <t>St. Paul Street, Bristol, BS2</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>441</v>
+      </c>
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
       <c r="M15" s="7" t="n"/>
       <c r="N15" s="7" t="n">
-        <v>20788</v>
+        <v>14016</v>
       </c>
       <c r="O15" s="7" t="n">
         <v>0</v>
@@ -1824,12 +1824,12 @@
       <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Southville</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S15" s="8" t="inlineStr">
@@ -1850,7 +1850,7 @@
       <c r="V15" s="6" t="inlineStr"/>
       <c r="W15" s="7" t="inlineStr">
         <is>
-          <t>8056582dfefc0ed6bd89dfe9a286f4e11c283370</t>
+          <t>9d32516da14aa47e9697f1f28aa43d03320187fe</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>2060</v>
+        <v>2125</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>2</v>
@@ -1879,23 +1879,23 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>The Quays, Cumberland Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I16" s="7" t="n">
-        <v>806</v>
+        <v>1081</v>
       </c>
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
       <c r="M16" s="7" t="n"/>
       <c r="N16" s="7" t="n">
-        <v>21152</v>
+        <v>16680</v>
       </c>
       <c r="O16" s="7" t="n">
         <v>0</v>
@@ -1903,12 +1903,12 @@
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>Savills Lettings, Clifton</t>
         </is>
       </c>
       <c r="S16" s="8" t="inlineStr">
@@ -1929,7 +1929,7 @@
       <c r="V16" s="6" t="inlineStr"/>
       <c r="W16" s="7" t="inlineStr">
         <is>
-          <t>ebe11a3ee06d602469bbb264eb9fb9a1bd399d3b</t>
+          <t>1005199ebd289ea67528d7b4b89c9cff3289e53b</t>
         </is>
       </c>
     </row>
@@ -1943,13 +1943,13 @@
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>2050</v>
+        <v>1350</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>Union Road, Bristol</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1966,15 +1966,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I17" s="7" t="n">
-        <v>802</v>
-      </c>
+      <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
       <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="n"/>
       <c r="N17" s="7" t="n">
-        <v>13408</v>
+        <v>20080</v>
       </c>
       <c r="O17" s="7" t="n">
         <v>0</v>
@@ -1982,12 +1980,12 @@
       <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S17" s="8" t="inlineStr">
@@ -2008,7 +2006,7 @@
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="7" t="inlineStr">
         <is>
-          <t>c2e87dbf92e1efc8f86ddd31b7364facadbd36d2</t>
+          <t>120a391700629cb94d575b3211bbdf9c0218d349</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2020,7 @@
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>1620</v>
+        <v>1400</v>
       </c>
       <c r="D18" s="7" t="n">
         <v>1</v>
@@ -2037,23 +2035,23 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>Harbourside, The Crescent, BS1 5LQ</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I18" s="7" t="n">
-        <v>557</v>
+        <v>603</v>
       </c>
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
       <c r="L18" s="7" t="n"/>
       <c r="M18" s="7" t="n"/>
       <c r="N18" s="7" t="n">
-        <v>21152</v>
+        <v>16724</v>
       </c>
       <c r="O18" s="7" t="n">
         <v>0</v>
@@ -2061,12 +2059,12 @@
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S18" s="8" t="inlineStr">
@@ -2087,7 +2085,7 @@
       <c r="V18" s="6" t="inlineStr"/>
       <c r="W18" s="7" t="inlineStr">
         <is>
-          <t>165ffd90b6b9a1057c6dca2ebd6ed6293b55dac8</t>
+          <t>7a10ed41d917a52d904d0556bbba8459de456473</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2099,7 @@
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>2000</v>
+        <v>1775</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>2</v>
@@ -2116,7 +2114,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Lower Park Row - City Centre</t>
+          <t>Twine House, Redcliff Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -2124,13 +2122,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I19" s="7" t="n"/>
+      <c r="I19" s="7" t="n">
+        <v>767</v>
+      </c>
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7" t="n"/>
       <c r="L19" s="7" t="n"/>
       <c r="M19" s="7" t="n"/>
       <c r="N19" s="7" t="n">
-        <v>21532</v>
+        <v>20888</v>
       </c>
       <c r="O19" s="7" t="n">
         <v>0</v>
@@ -2138,12 +2138,12 @@
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Clifton</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S19" s="8" t="inlineStr">
@@ -2164,7 +2164,7 @@
       <c r="V19" s="6" t="inlineStr"/>
       <c r="W19" s="7" t="inlineStr">
         <is>
-          <t>8c589025b84fb12583a29c490c3882a26aca2559</t>
+          <t>27c0f9ce89d081b8d1914ffcc561e9aa878d6d99</t>
         </is>
       </c>
     </row>
@@ -2178,10 +2178,10 @@
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>1300</v>
+        <v>1700</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>1</v>
@@ -2193,23 +2193,21 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>St. Paul Street, Bristol, BS2</t>
+          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>441</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n"/>
       <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n">
-        <v>14016</v>
+        <v>4892</v>
       </c>
       <c r="O20" s="7" t="n">
         <v>0</v>
@@ -2217,12 +2215,12 @@
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S20" s="8" t="inlineStr">
@@ -2243,7 +2241,7 @@
       <c r="V20" s="6" t="inlineStr"/>
       <c r="W20" s="7" t="inlineStr">
         <is>
-          <t>9d32516da14aa47e9697f1f28aa43d03320187fe</t>
+          <t>916b8e1db731f908cd8ba08a69c2e9978e66cd1c</t>
         </is>
       </c>
     </row>
@@ -2257,13 +2255,13 @@
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>2125</v>
+        <v>1823</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -2272,23 +2270,23 @@
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>The Quays, Cumberland Road, Bristol, BS1</t>
+          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I21" s="7" t="n">
-        <v>1081</v>
+        <v>524</v>
       </c>
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
       <c r="L21" s="7" t="n"/>
       <c r="M21" s="7" t="n"/>
       <c r="N21" s="7" t="n">
-        <v>16680</v>
+        <v>11632</v>
       </c>
       <c r="O21" s="7" t="n">
         <v>0</v>
@@ -2296,12 +2294,12 @@
       <c r="P21" s="7" t="n"/>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, Clifton</t>
+          <t>CompassRock International, Stafford Yard</t>
         </is>
       </c>
       <c r="S21" s="8" t="inlineStr">
@@ -2322,7 +2320,7 @@
       <c r="V21" s="6" t="inlineStr"/>
       <c r="W21" s="7" t="inlineStr">
         <is>
-          <t>1005199ebd289ea67528d7b4b89c9cff3289e53b</t>
+          <t>96f4c09e794ccdc0fe9190c623669e365937c4d3</t>
         </is>
       </c>
     </row>
@@ -2336,10 +2334,10 @@
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>1350</v>
+        <v>1500</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" s="7" t="n">
         <v>1</v>
@@ -2351,21 +2349,23 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Union Road, Bristol</t>
+          <t>St. David Mews, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>560</v>
+      </c>
       <c r="J22" s="7" t="n"/>
       <c r="K22" s="7" t="n"/>
       <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
       <c r="N22" s="7" t="n">
-        <v>20080</v>
+        <v>18292</v>
       </c>
       <c r="O22" s="7" t="n">
         <v>0</v>
@@ -2373,12 +2373,12 @@
       <c r="P22" s="7" t="n"/>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S22" s="8" t="inlineStr">
@@ -2399,7 +2399,7 @@
       <c r="V22" s="6" t="inlineStr"/>
       <c r="W22" s="7" t="inlineStr">
         <is>
-          <t>120a391700629cb94d575b3211bbdf9c0218d349</t>
+          <t>acc3c4682d6bc0b232ebba18bc6c42d125641e52</t>
         </is>
       </c>
     </row>
@@ -2413,13 +2413,13 @@
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>1400</v>
+        <v>2110</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -2428,23 +2428,23 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, The Crescent, BS1 5LQ</t>
+          <t>507 Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I23" s="7" t="n">
-        <v>603</v>
+        <v>803</v>
       </c>
       <c r="J23" s="7" t="n"/>
       <c r="K23" s="7" t="n"/>
       <c r="L23" s="7" t="n"/>
       <c r="M23" s="7" t="n"/>
       <c r="N23" s="7" t="n">
-        <v>16724</v>
+        <v>20780</v>
       </c>
       <c r="O23" s="7" t="n">
         <v>0</v>
@@ -2452,12 +2452,12 @@
       <c r="P23" s="7" t="n"/>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S23" s="8" t="inlineStr">
@@ -2478,7 +2478,7 @@
       <c r="V23" s="6" t="inlineStr"/>
       <c r="W23" s="7" t="inlineStr">
         <is>
-          <t>7a10ed41d917a52d904d0556bbba8459de456473</t>
+          <t>893e6113f15b08871107b7b3c0648cb534424a90</t>
         </is>
       </c>
     </row>
@@ -2492,13 +2492,13 @@
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1775</v>
+        <v>1645</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
@@ -2507,23 +2507,23 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Twine House, Redcliff Street, Redcliff, Bristol, Bristol City</t>
+          <t>705 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I24" s="7" t="n">
-        <v>767</v>
+        <v>538</v>
       </c>
       <c r="J24" s="7" t="n"/>
       <c r="K24" s="7" t="n"/>
       <c r="L24" s="7" t="n"/>
       <c r="M24" s="7" t="n"/>
       <c r="N24" s="7" t="n">
-        <v>20888</v>
+        <v>21152</v>
       </c>
       <c r="O24" s="7" t="n">
         <v>0</v>
@@ -2531,12 +2531,12 @@
       <c r="P24" s="7" t="n"/>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S24" s="8" t="inlineStr">
@@ -2557,7 +2557,7 @@
       <c r="V24" s="6" t="inlineStr"/>
       <c r="W24" s="7" t="inlineStr">
         <is>
-          <t>27c0f9ce89d081b8d1914ffcc561e9aa878d6d99</t>
+          <t>303852d12f30a1bf3d6ef265921d3ee8a77897e6</t>
         </is>
       </c>
     </row>
@@ -2571,13 +2571,13 @@
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>1700</v>
+        <v>2060</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -2586,21 +2586,23 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
+          <t>702 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>806</v>
+      </c>
       <c r="J25" s="7" t="n"/>
       <c r="K25" s="7" t="n"/>
       <c r="L25" s="7" t="n"/>
       <c r="M25" s="7" t="n"/>
       <c r="N25" s="7" t="n">
-        <v>4892</v>
+        <v>21152</v>
       </c>
       <c r="O25" s="7" t="n">
         <v>0</v>
@@ -2608,12 +2610,12 @@
       <c r="P25" s="7" t="n"/>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S25" s="8" t="inlineStr">
@@ -2634,7 +2636,7 @@
       <c r="V25" s="6" t="inlineStr"/>
       <c r="W25" s="7" t="inlineStr">
         <is>
-          <t>916b8e1db731f908cd8ba08a69c2e9978e66cd1c</t>
+          <t>58b4cd7c991d7cdd8dab09c103fa87d8124bce04</t>
         </is>
       </c>
     </row>
@@ -2648,13 +2650,13 @@
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>1823</v>
+        <v>2050</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
@@ -2663,23 +2665,23 @@
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Stafford Yard, Stafford Street, Bedminster, Bristol, Bristol City</t>
+          <t>421 Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I26" s="7" t="n">
-        <v>524</v>
+        <v>802</v>
       </c>
       <c r="J26" s="7" t="n"/>
       <c r="K26" s="7" t="n"/>
       <c r="L26" s="7" t="n"/>
       <c r="M26" s="7" t="n"/>
       <c r="N26" s="7" t="n">
-        <v>11632</v>
+        <v>20780</v>
       </c>
       <c r="O26" s="7" t="n">
         <v>0</v>
@@ -2687,12 +2689,12 @@
       <c r="P26" s="7" t="n"/>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="R26" s="7" t="inlineStr">
         <is>
-          <t>CompassRock International, Stafford Yard</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S26" s="8" t="inlineStr">
@@ -2713,7 +2715,7 @@
       <c r="V26" s="6" t="inlineStr"/>
       <c r="W26" s="7" t="inlineStr">
         <is>
-          <t>96f4c09e794ccdc0fe9190c623669e365937c4d3</t>
+          <t>c47e481c7dd90aac76ea9c8c662ba108d03efd56</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2729,7 @@
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>1500</v>
+        <v>1620</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>1</v>
@@ -2742,23 +2744,23 @@
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>St. David Mews, City Centre, Bristol, BS1</t>
+          <t>204 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I27" s="7" t="n">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="J27" s="7" t="n"/>
       <c r="K27" s="7" t="n"/>
       <c r="L27" s="7" t="n"/>
       <c r="M27" s="7" t="n"/>
       <c r="N27" s="7" t="n">
-        <v>18292</v>
+        <v>21152</v>
       </c>
       <c r="O27" s="7" t="n">
         <v>0</v>
@@ -2766,12 +2768,12 @@
       <c r="P27" s="7" t="n"/>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Clifton</t>
+          <t>urbanbubble, Box Makers Yard</t>
         </is>
       </c>
       <c r="S27" s="8" t="inlineStr">
@@ -2792,7 +2794,7 @@
       <c r="V27" s="6" t="inlineStr"/>
       <c r="W27" s="7" t="inlineStr">
         <is>
-          <t>acc3c4682d6bc0b232ebba18bc6c42d125641e52</t>
+          <t>75a7b799dc05caec9f24132d32f937ce8a9830ec</t>
         </is>
       </c>
     </row>
@@ -2806,10 +2808,10 @@
         </is>
       </c>
       <c r="C28" s="9" t="n">
-        <v>2110</v>
+        <v>2830</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>2</v>
@@ -2821,7 +2823,7 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>507 Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>315 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
@@ -2830,15 +2832,13 @@
         </is>
       </c>
       <c r="I28" s="7" t="n">
-        <v>803</v>
+        <v>1120</v>
       </c>
       <c r="J28" s="7" t="n"/>
       <c r="K28" s="7" t="n"/>
       <c r="L28" s="7" t="n"/>
       <c r="M28" s="7" t="n"/>
-      <c r="N28" s="7" t="n">
-        <v>13408</v>
-      </c>
+      <c r="N28" s="7" t="n"/>
       <c r="O28" s="7" t="n">
         <v>0</v>
       </c>
@@ -2871,7 +2871,7 @@
       <c r="V28" s="6" t="inlineStr"/>
       <c r="W28" s="7" t="inlineStr">
         <is>
-          <t>893e6113f15b08871107b7b3c0648cb534424a90</t>
+          <t>9d79544e8a6ed02af10383bd3d053236bec757b5</t>
         </is>
       </c>
     </row>
@@ -2885,13 +2885,13 @@
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>1645</v>
+        <v>2830</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>705 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>315 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -2909,7 +2909,7 @@
         </is>
       </c>
       <c r="I29" s="7" t="n">
-        <v>538</v>
+        <v>1120</v>
       </c>
       <c r="J29" s="7" t="n"/>
       <c r="K29" s="7" t="n"/>
@@ -2924,7 +2924,7 @@
       <c r="P29" s="7" t="n"/>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="R29" s="7" t="inlineStr">
@@ -2950,7 +2950,7 @@
       <c r="V29" s="6" t="inlineStr"/>
       <c r="W29" s="7" t="inlineStr">
         <is>
-          <t>303852d12f30a1bf3d6ef265921d3ee8a77897e6</t>
+          <t>b70e24d9417674d7a16e52abd8d5a34b925d04ea</t>
         </is>
       </c>
     </row>
@@ -2964,13 +2964,13 @@
         </is>
       </c>
       <c r="C30" s="9" t="n">
-        <v>2060</v>
+        <v>1650</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -2979,23 +2979,21 @@
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>702 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>Paintworks, Arnos Vale, Bristol, BS4</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I30" s="7" t="n">
-        <v>806</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="n"/>
       <c r="J30" s="7" t="n"/>
       <c r="K30" s="7" t="n"/>
       <c r="L30" s="7" t="n"/>
       <c r="M30" s="7" t="n"/>
       <c r="N30" s="7" t="n">
-        <v>21152</v>
+        <v>5244</v>
       </c>
       <c r="O30" s="7" t="n">
         <v>0</v>
@@ -3003,12 +3001,12 @@
       <c r="P30" s="7" t="n"/>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>urbanbubble, Box Makers Yard</t>
+          <t>CJ Hole, Kingswood</t>
         </is>
       </c>
       <c r="S30" s="8" t="inlineStr">
@@ -3029,7 +3027,7 @@
       <c r="V30" s="6" t="inlineStr"/>
       <c r="W30" s="7" t="inlineStr">
         <is>
-          <t>58b4cd7c991d7cdd8dab09c103fa87d8124bce04</t>
+          <t>6b42638cf55169ff2e715f3f1db70e5db21111f3</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3041,7 @@
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>2050</v>
+        <v>2060</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>2</v>
@@ -3058,7 +3056,7 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>421 Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -3067,14 +3065,14 @@
         </is>
       </c>
       <c r="I31" s="7" t="n">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="J31" s="7" t="n"/>
       <c r="K31" s="7" t="n"/>
       <c r="L31" s="7" t="n"/>
       <c r="M31" s="7" t="n"/>
       <c r="N31" s="7" t="n">
-        <v>13408</v>
+        <v>21152</v>
       </c>
       <c r="O31" s="7" t="n">
         <v>0</v>
@@ -3082,7 +3080,7 @@
       <c r="P31" s="7" t="n"/>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
@@ -3108,7 +3106,7 @@
       <c r="V31" s="6" t="inlineStr"/>
       <c r="W31" s="7" t="inlineStr">
         <is>
-          <t>c47e481c7dd90aac76ea9c8c662ba108d03efd56</t>
+          <t>ebe11a3ee06d602469bbb264eb9fb9a1bd399d3b</t>
         </is>
       </c>
     </row>
@@ -3122,13 +3120,13 @@
         </is>
       </c>
       <c r="C32" s="9" t="n">
-        <v>1620</v>
+        <v>2050</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
@@ -3137,7 +3135,7 @@
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>204 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>Rosewood, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -3146,14 +3144,14 @@
         </is>
       </c>
       <c r="I32" s="7" t="n">
-        <v>557</v>
+        <v>802</v>
       </c>
       <c r="J32" s="7" t="n"/>
       <c r="K32" s="7" t="n"/>
       <c r="L32" s="7" t="n"/>
       <c r="M32" s="7" t="n"/>
       <c r="N32" s="7" t="n">
-        <v>21152</v>
+        <v>13408</v>
       </c>
       <c r="O32" s="7" t="n">
         <v>0</v>
@@ -3161,7 +3159,7 @@
       <c r="P32" s="7" t="n"/>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="R32" s="7" t="inlineStr">
@@ -3187,7 +3185,7 @@
       <c r="V32" s="6" t="inlineStr"/>
       <c r="W32" s="7" t="inlineStr">
         <is>
-          <t>75a7b799dc05caec9f24132d32f937ce8a9830ec</t>
+          <t>c2e87dbf92e1efc8f86ddd31b7364facadbd36d2</t>
         </is>
       </c>
     </row>
@@ -3201,13 +3199,13 @@
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>2830</v>
+        <v>1620</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
@@ -3216,7 +3214,7 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>315 Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
+          <t>Dovetail, New Kingsley Road, St Philips, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -3225,20 +3223,22 @@
         </is>
       </c>
       <c r="I33" s="7" t="n">
-        <v>1120</v>
+        <v>557</v>
       </c>
       <c r="J33" s="7" t="n"/>
       <c r="K33" s="7" t="n"/>
       <c r="L33" s="7" t="n"/>
       <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
+      <c r="N33" s="7" t="n">
+        <v>21152</v>
+      </c>
       <c r="O33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P33" s="7" t="n"/>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr">
@@ -3264,7 +3264,7 @@
       <c r="V33" s="6" t="inlineStr"/>
       <c r="W33" s="7" t="inlineStr">
         <is>
-          <t>9d79544e8a6ed02af10383bd3d053236bec757b5</t>
+          <t>165ffd90b6b9a1057c6dca2ebd6ed6293b55dac8</t>
         </is>
       </c>
     </row>
@@ -5535,12 +5535,14 @@
         </is>
       </c>
       <c r="C63" s="9" t="n">
-        <v>1450</v>
+        <v>1325</v>
       </c>
       <c r="D63" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -5548,12 +5550,12 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Broad Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I63" s="7" t="n"/>
@@ -5562,7 +5564,7 @@
       <c r="L63" s="7" t="n"/>
       <c r="M63" s="7" t="n"/>
       <c r="N63" s="7" t="n">
-        <v>19488</v>
+        <v>21788</v>
       </c>
       <c r="O63" s="7" t="n">
         <v>1</v>
@@ -5570,12 +5572,12 @@
       <c r="P63" s="7" t="n"/>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="R63" s="7" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S63" s="8" t="inlineStr"/>
@@ -5592,7 +5594,7 @@
       <c r="V63" s="6" t="inlineStr"/>
       <c r="W63" s="7" t="inlineStr">
         <is>
-          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
+          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
         </is>
       </c>
     </row>
@@ -5606,7 +5608,7 @@
         </is>
       </c>
       <c r="C64" s="9" t="n">
-        <v>1325</v>
+        <v>1200</v>
       </c>
       <c r="D64" s="7" t="n">
         <v>1</v>
@@ -5621,12 +5623,12 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Broad Street, Bristol, BS1</t>
+          <t>Bushy Park, The Bank Bushy Park, BS4</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I64" s="7" t="n"/>
@@ -5635,7 +5637,7 @@
       <c r="L64" s="7" t="n"/>
       <c r="M64" s="7" t="n"/>
       <c r="N64" s="7" t="n">
-        <v>21788</v>
+        <v>7216</v>
       </c>
       <c r="O64" s="7" t="n">
         <v>1</v>
@@ -5643,12 +5645,12 @@
       <c r="P64" s="7" t="n"/>
       <c r="Q64" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="R64" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S64" s="8" t="inlineStr"/>
@@ -5665,7 +5667,7 @@
       <c r="V64" s="6" t="inlineStr"/>
       <c r="W64" s="7" t="inlineStr">
         <is>
-          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
+          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
         </is>
       </c>
     </row>
@@ -5679,27 +5681,27 @@
         </is>
       </c>
       <c r="C65" s="9" t="n">
-        <v>1200</v>
+        <v>1950</v>
       </c>
       <c r="D65" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E65" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Bushy Park, The Bank Bushy Park, BS4</t>
+          <t>Webb Street, Bristol, BS5</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I65" s="7" t="n"/>
@@ -5708,20 +5710,20 @@
       <c r="L65" s="7" t="n"/>
       <c r="M65" s="7" t="n"/>
       <c r="N65" s="7" t="n">
-        <v>7216</v>
+        <v>19580</v>
       </c>
       <c r="O65" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P65" s="7" t="n"/>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S65" s="8" t="inlineStr"/>
@@ -5738,7 +5740,7 @@
       <c r="V65" s="6" t="inlineStr"/>
       <c r="W65" s="7" t="inlineStr">
         <is>
-          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
+          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
         </is>
       </c>
     </row>
@@ -5752,13 +5754,13 @@
         </is>
       </c>
       <c r="C66" s="9" t="n">
-        <v>1950</v>
+        <v>3800</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E66" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
@@ -5767,12 +5769,12 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Webb Street, Bristol, BS5</t>
+          <t>Barton Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I66" s="7" t="n"/>
@@ -5781,7 +5783,7 @@
       <c r="L66" s="7" t="n"/>
       <c r="M66" s="7" t="n"/>
       <c r="N66" s="7" t="n">
-        <v>19580</v>
+        <v>19720</v>
       </c>
       <c r="O66" s="7" t="n">
         <v>0</v>
@@ -5789,7 +5791,7 @@
       <c r="P66" s="7" t="n"/>
       <c r="Q66" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R66" s="7" t="inlineStr">
@@ -5811,7 +5813,7 @@
       <c r="V66" s="6" t="inlineStr"/>
       <c r="W66" s="7" t="inlineStr">
         <is>
-          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
+          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
         </is>
       </c>
     </row>
@@ -5825,27 +5827,27 @@
         </is>
       </c>
       <c r="C67" s="9" t="n">
-        <v>3800</v>
+        <v>2200</v>
       </c>
       <c r="D67" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>Barton Road, Bristol, BS2</t>
+          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I67" s="7" t="n"/>
@@ -5854,7 +5856,7 @@
       <c r="L67" s="7" t="n"/>
       <c r="M67" s="7" t="n"/>
       <c r="N67" s="7" t="n">
-        <v>19720</v>
+        <v>16788</v>
       </c>
       <c r="O67" s="7" t="n">
         <v>0</v>
@@ -5862,12 +5864,12 @@
       <c r="P67" s="7" t="n"/>
       <c r="Q67" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R67" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S67" s="8" t="inlineStr"/>
@@ -5884,7 +5886,7 @@
       <c r="V67" s="6" t="inlineStr"/>
       <c r="W67" s="7" t="inlineStr">
         <is>
-          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
+          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
         </is>
       </c>
     </row>
@@ -5898,7 +5900,7 @@
         </is>
       </c>
       <c r="C68" s="9" t="n">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="D68" s="7" t="n">
         <v>2</v>
@@ -5913,7 +5915,7 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
+          <t>Colston Avenue, Bristol, BS1</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
@@ -5927,7 +5929,7 @@
       <c r="L68" s="7" t="n"/>
       <c r="M68" s="7" t="n"/>
       <c r="N68" s="7" t="n">
-        <v>16788</v>
+        <v>14108</v>
       </c>
       <c r="O68" s="7" t="n">
         <v>0</v>
@@ -5935,12 +5937,12 @@
       <c r="P68" s="7" t="n"/>
       <c r="Q68" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R68" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S68" s="8" t="inlineStr"/>
@@ -5957,7 +5959,7 @@
       <c r="V68" s="6" t="inlineStr"/>
       <c r="W68" s="7" t="inlineStr">
         <is>
-          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
+          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
         </is>
       </c>
     </row>
@@ -5971,13 +5973,13 @@
         </is>
       </c>
       <c r="C69" s="9" t="n">
-        <v>2400</v>
+        <v>1450</v>
       </c>
       <c r="D69" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
@@ -5986,21 +5988,23 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Colston Avenue, Bristol, BS1</t>
+          <t>East Street, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I69" s="7" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="n">
+        <v>560</v>
+      </c>
       <c r="J69" s="7" t="n"/>
       <c r="K69" s="7" t="n"/>
       <c r="L69" s="7" t="n"/>
       <c r="M69" s="7" t="n"/>
       <c r="N69" s="7" t="n">
-        <v>14108</v>
+        <v>14176</v>
       </c>
       <c r="O69" s="7" t="n">
         <v>0</v>
@@ -6013,7 +6017,7 @@
       </c>
       <c r="R69" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Xeno Property, Bristol</t>
         </is>
       </c>
       <c r="S69" s="8" t="inlineStr"/>
@@ -6030,7 +6034,7 @@
       <c r="V69" s="6" t="inlineStr"/>
       <c r="W69" s="7" t="inlineStr">
         <is>
-          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
+          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
         </is>
       </c>
     </row>
@@ -6044,13 +6048,13 @@
         </is>
       </c>
       <c r="C70" s="9" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
@@ -6059,12 +6063,12 @@
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I70" s="7" t="n"/>
@@ -6073,7 +6077,7 @@
       <c r="L70" s="7" t="n"/>
       <c r="M70" s="7" t="n"/>
       <c r="N70" s="7" t="n">
-        <v>20768</v>
+        <v>21360</v>
       </c>
       <c r="O70" s="7" t="n">
         <v>0</v>
@@ -6081,12 +6085,12 @@
       <c r="P70" s="7" t="n"/>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R70" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S70" s="8" t="inlineStr"/>
@@ -6103,7 +6107,7 @@
       <c r="V70" s="6" t="inlineStr"/>
       <c r="W70" s="7" t="inlineStr">
         <is>
-          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
+          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
         </is>
       </c>
     </row>
@@ -6117,13 +6121,13 @@
         </is>
       </c>
       <c r="C71" s="9" t="n">
-        <v>1450</v>
+        <v>3200</v>
       </c>
       <c r="D71" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
@@ -6132,7 +6136,7 @@
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol</t>
+          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -6146,7 +6150,7 @@
       <c r="L71" s="7" t="n"/>
       <c r="M71" s="7" t="n"/>
       <c r="N71" s="7" t="n">
-        <v>13668</v>
+        <v>16664</v>
       </c>
       <c r="O71" s="7" t="n">
         <v>0</v>
@@ -6154,12 +6158,12 @@
       <c r="P71" s="7" t="n"/>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R71" s="7" t="inlineStr">
         <is>
-          <t>Wildheart Residential Management Limited, Epsom</t>
+          <t>LettingaProperty.com, Nationwide - Lettings</t>
         </is>
       </c>
       <c r="S71" s="8" t="inlineStr"/>
@@ -6176,7 +6180,7 @@
       <c r="V71" s="6" t="inlineStr"/>
       <c r="W71" s="7" t="inlineStr">
         <is>
-          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
+          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6194,7 @@
         </is>
       </c>
       <c r="C72" s="9" t="n">
-        <v>1450</v>
+        <v>1600</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>1</v>
@@ -6205,23 +6209,21 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>East Street, Bedminster, BS3</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I72" s="7" t="n">
-        <v>560</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I72" s="7" t="n"/>
       <c r="J72" s="7" t="n"/>
       <c r="K72" s="7" t="n"/>
       <c r="L72" s="7" t="n"/>
       <c r="M72" s="7" t="n"/>
       <c r="N72" s="7" t="n">
-        <v>14176</v>
+        <v>21996</v>
       </c>
       <c r="O72" s="7" t="n">
         <v>0</v>
@@ -6229,12 +6231,12 @@
       <c r="P72" s="7" t="n"/>
       <c r="Q72" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R72" s="7" t="inlineStr">
         <is>
-          <t>Xeno Property, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S72" s="8" t="inlineStr"/>
@@ -6251,7 +6253,7 @@
       <c r="V72" s="6" t="inlineStr"/>
       <c r="W72" s="7" t="inlineStr">
         <is>
-          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
+          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
         </is>
       </c>
     </row>
@@ -6265,13 +6267,13 @@
         </is>
       </c>
       <c r="C73" s="9" t="n">
-        <v>2500</v>
+        <v>1400</v>
       </c>
       <c r="D73" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E73" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
@@ -6280,12 +6282,12 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>Invicta, Millenium Promenade, BS1</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I73" s="7" t="n"/>
@@ -6294,7 +6296,7 @@
       <c r="L73" s="7" t="n"/>
       <c r="M73" s="7" t="n"/>
       <c r="N73" s="7" t="n">
-        <v>21360</v>
+        <v>17344</v>
       </c>
       <c r="O73" s="7" t="n">
         <v>0</v>
@@ -6302,12 +6304,12 @@
       <c r="P73" s="7" t="n"/>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R73" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S73" s="8" t="inlineStr"/>
@@ -6324,7 +6326,7 @@
       <c r="V73" s="6" t="inlineStr"/>
       <c r="W73" s="7" t="inlineStr">
         <is>
-          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
+          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
         </is>
       </c>
     </row>
@@ -6338,13 +6340,13 @@
         </is>
       </c>
       <c r="C74" s="9" t="n">
-        <v>3200</v>
+        <v>1600</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E74" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
@@ -6353,7 +6355,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
+          <t>Central Quay North, Bristol, BS1</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
@@ -6367,7 +6369,7 @@
       <c r="L74" s="7" t="n"/>
       <c r="M74" s="7" t="n"/>
       <c r="N74" s="7" t="n">
-        <v>16416</v>
+        <v>13404</v>
       </c>
       <c r="O74" s="7" t="n">
         <v>0</v>
@@ -6375,12 +6377,12 @@
       <c r="P74" s="7" t="n"/>
       <c r="Q74" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R74" s="7" t="inlineStr">
         <is>
-          <t>LettingaProperty.com, Nationwide - Lettings</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S74" s="8" t="inlineStr"/>
@@ -6397,7 +6399,7 @@
       <c r="V74" s="6" t="inlineStr"/>
       <c r="W74" s="7" t="inlineStr">
         <is>
-          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
+          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6413,7 @@
         </is>
       </c>
       <c r="C75" s="9" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="D75" s="7" t="n">
         <v>1</v>
@@ -6426,7 +6428,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Eclipse, Broad Weir, Bristol</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
@@ -6440,7 +6442,7 @@
       <c r="L75" s="7" t="n"/>
       <c r="M75" s="7" t="n"/>
       <c r="N75" s="7" t="n">
-        <v>21996</v>
+        <v>22164</v>
       </c>
       <c r="O75" s="7" t="n">
         <v>0</v>
@@ -6448,12 +6450,12 @@
       <c r="P75" s="7" t="n"/>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R75" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Martin &amp; Co, Bath</t>
         </is>
       </c>
       <c r="S75" s="8" t="inlineStr"/>
@@ -6470,7 +6472,7 @@
       <c r="V75" s="6" t="inlineStr"/>
       <c r="W75" s="7" t="inlineStr">
         <is>
-          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
+          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
         </is>
       </c>
     </row>
@@ -6484,38 +6486,38 @@
         </is>
       </c>
       <c r="C76" s="9" t="n">
-        <v>2250</v>
+        <v>1800</v>
       </c>
       <c r="D76" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Newfoundland Road, Bristol, BS2</t>
+          <t>Broad Weir, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I76" s="7" t="n">
-        <v>980</v>
+        <v>474</v>
       </c>
       <c r="J76" s="7" t="n"/>
       <c r="K76" s="7" t="n"/>
       <c r="L76" s="7" t="n"/>
       <c r="M76" s="7" t="n"/>
       <c r="N76" s="7" t="n">
-        <v>19800</v>
+        <v>22080</v>
       </c>
       <c r="O76" s="7" t="n">
         <v>0</v>
@@ -6523,12 +6525,12 @@
       <c r="P76" s="7" t="n"/>
       <c r="Q76" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R76" s="7" t="inlineStr">
         <is>
-          <t>Lets Rent Bristol, Bristol</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S76" s="8" t="inlineStr"/>
@@ -6545,7 +6547,7 @@
       <c r="V76" s="6" t="inlineStr"/>
       <c r="W76" s="7" t="inlineStr">
         <is>
-          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
+          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
         </is>
       </c>
     </row>
@@ -6559,7 +6561,7 @@
         </is>
       </c>
       <c r="C77" s="9" t="n">
-        <v>1400</v>
+        <v>1605</v>
       </c>
       <c r="D77" s="7" t="n">
         <v>1</v>
@@ -6574,7 +6576,7 @@
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>Invicta, Millenium Promenade, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
@@ -6582,13 +6584,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I77" s="7" t="n"/>
+      <c r="I77" s="7" t="n">
+        <v>487</v>
+      </c>
       <c r="J77" s="7" t="n"/>
       <c r="K77" s="7" t="n"/>
       <c r="L77" s="7" t="n"/>
       <c r="M77" s="7" t="n"/>
       <c r="N77" s="7" t="n">
-        <v>17344</v>
+        <v>13860</v>
       </c>
       <c r="O77" s="7" t="n">
         <v>0</v>
@@ -6596,12 +6600,12 @@
       <c r="P77" s="7" t="n"/>
       <c r="Q77" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R77" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S77" s="8" t="inlineStr"/>
@@ -6618,7 +6622,7 @@
       <c r="V77" s="6" t="inlineStr"/>
       <c r="W77" s="7" t="inlineStr">
         <is>
-          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
+          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
         </is>
       </c>
     </row>
@@ -6632,13 +6636,13 @@
         </is>
       </c>
       <c r="C78" s="9" t="n">
-        <v>1600</v>
+        <v>2185</v>
       </c>
       <c r="D78" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E78" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
@@ -6647,7 +6651,7 @@
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
@@ -6655,13 +6659,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I78" s="7" t="n"/>
+      <c r="I78" s="7" t="n">
+        <v>721</v>
+      </c>
       <c r="J78" s="7" t="n"/>
       <c r="K78" s="7" t="n"/>
       <c r="L78" s="7" t="n"/>
       <c r="M78" s="7" t="n"/>
       <c r="N78" s="7" t="n">
-        <v>13404</v>
+        <v>13860</v>
       </c>
       <c r="O78" s="7" t="n">
         <v>0</v>
@@ -6669,12 +6675,12 @@
       <c r="P78" s="7" t="n"/>
       <c r="Q78" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R78" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S78" s="8" t="inlineStr"/>
@@ -6691,7 +6697,7 @@
       <c r="V78" s="6" t="inlineStr"/>
       <c r="W78" s="7" t="inlineStr">
         <is>
-          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
+          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
         </is>
       </c>
     </row>
@@ -6705,10 +6711,10 @@
         </is>
       </c>
       <c r="C79" s="9" t="n">
-        <v>1500</v>
+        <v>1650</v>
       </c>
       <c r="D79" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E79" s="7" t="n">
         <v>1</v>
@@ -6720,12 +6726,12 @@
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>Eclipse, Broad Weir, Bristol</t>
+          <t>Crown &amp; Anchor House, Bristol, BS2</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I79" s="7" t="n"/>
@@ -6734,7 +6740,7 @@
       <c r="L79" s="7" t="n"/>
       <c r="M79" s="7" t="n"/>
       <c r="N79" s="7" t="n">
-        <v>22164</v>
+        <v>20472</v>
       </c>
       <c r="O79" s="7" t="n">
         <v>0</v>
@@ -6742,12 +6748,12 @@
       <c r="P79" s="7" t="n"/>
       <c r="Q79" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R79" s="7" t="inlineStr">
         <is>
-          <t>Martin &amp; Co, Bath</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S79" s="8" t="inlineStr"/>
@@ -6764,7 +6770,7 @@
       <c r="V79" s="6" t="inlineStr"/>
       <c r="W79" s="7" t="inlineStr">
         <is>
-          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
+          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
         </is>
       </c>
     </row>
@@ -6778,7 +6784,7 @@
         </is>
       </c>
       <c r="C80" s="9" t="n">
-        <v>1800</v>
+        <v>1640</v>
       </c>
       <c r="D80" s="7" t="n">
         <v>1</v>
@@ -6793,7 +6799,7 @@
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Broad Weir, City Centre, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
@@ -6802,14 +6808,14 @@
         </is>
       </c>
       <c r="I80" s="7" t="n">
-        <v>474</v>
+        <v>484</v>
       </c>
       <c r="J80" s="7" t="n"/>
       <c r="K80" s="7" t="n"/>
       <c r="L80" s="7" t="n"/>
       <c r="M80" s="7" t="n"/>
       <c r="N80" s="7" t="n">
-        <v>22080</v>
+        <v>13860</v>
       </c>
       <c r="O80" s="7" t="n">
         <v>0</v>
@@ -6817,12 +6823,12 @@
       <c r="P80" s="7" t="n"/>
       <c r="Q80" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R80" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Clifton</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S80" s="8" t="inlineStr"/>
@@ -6839,7 +6845,7 @@
       <c r="V80" s="6" t="inlineStr"/>
       <c r="W80" s="7" t="inlineStr">
         <is>
-          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
+          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
         </is>
       </c>
     </row>
@@ -6853,13 +6859,13 @@
         </is>
       </c>
       <c r="C81" s="9" t="n">
-        <v>1605</v>
+        <v>1650</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
@@ -6868,7 +6874,7 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Harbourside, Harris Lofts, BS1 4BB</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
@@ -6877,14 +6883,14 @@
         </is>
       </c>
       <c r="I81" s="7" t="n">
-        <v>487</v>
+        <v>667</v>
       </c>
       <c r="J81" s="7" t="n"/>
       <c r="K81" s="7" t="n"/>
       <c r="L81" s="7" t="n"/>
       <c r="M81" s="7" t="n"/>
       <c r="N81" s="7" t="n">
-        <v>13860</v>
+        <v>20088</v>
       </c>
       <c r="O81" s="7" t="n">
         <v>0</v>
@@ -6892,12 +6898,12 @@
       <c r="P81" s="7" t="n"/>
       <c r="Q81" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R81" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S81" s="8" t="inlineStr"/>
@@ -6914,7 +6920,7 @@
       <c r="V81" s="6" t="inlineStr"/>
       <c r="W81" s="7" t="inlineStr">
         <is>
-          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
+          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
         </is>
       </c>
     </row>
@@ -6928,13 +6934,13 @@
         </is>
       </c>
       <c r="C82" s="9" t="n">
-        <v>2185</v>
+        <v>1650</v>
       </c>
       <c r="D82" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E82" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
@@ -6943,7 +6949,7 @@
       </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Central Quey North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
@@ -6951,15 +6957,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I82" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I82" s="7" t="n"/>
       <c r="J82" s="7" t="n"/>
       <c r="K82" s="7" t="n"/>
       <c r="L82" s="7" t="n"/>
       <c r="M82" s="7" t="n"/>
       <c r="N82" s="7" t="n">
-        <v>13860</v>
+        <v>20768</v>
       </c>
       <c r="O82" s="7" t="n">
         <v>0</v>
@@ -6967,12 +6971,12 @@
       <c r="P82" s="7" t="n"/>
       <c r="Q82" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R82" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S82" s="8" t="inlineStr"/>
@@ -6989,7 +6993,7 @@
       <c r="V82" s="6" t="inlineStr"/>
       <c r="W82" s="7" t="inlineStr">
         <is>
-          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
+          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
         </is>
       </c>
     </row>
@@ -7003,13 +7007,13 @@
         </is>
       </c>
       <c r="C83" s="9" t="n">
-        <v>1650</v>
+        <v>1450</v>
       </c>
       <c r="D83" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
@@ -7018,21 +7022,23 @@
       </c>
       <c r="G83" s="8" t="inlineStr">
         <is>
-          <t>Crown &amp; Anchor House, Bristol, BS2</t>
+          <t>Woodbridge Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I83" s="7" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I83" s="7" t="n">
+        <v>678</v>
+      </c>
       <c r="J83" s="7" t="n"/>
       <c r="K83" s="7" t="n"/>
       <c r="L83" s="7" t="n"/>
       <c r="M83" s="7" t="n"/>
       <c r="N83" s="7" t="n">
-        <v>20472</v>
+        <v>5700</v>
       </c>
       <c r="O83" s="7" t="n">
         <v>0</v>
@@ -7040,12 +7046,12 @@
       <c r="P83" s="7" t="n"/>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R83" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S83" s="8" t="inlineStr"/>
@@ -7062,7 +7068,7 @@
       <c r="V83" s="6" t="inlineStr"/>
       <c r="W83" s="7" t="inlineStr">
         <is>
-          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
+          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
         </is>
       </c>
     </row>
@@ -7076,13 +7082,13 @@
         </is>
       </c>
       <c r="C84" s="9" t="n">
-        <v>1640</v>
+        <v>2010</v>
       </c>
       <c r="D84" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
@@ -7100,7 +7106,7 @@
         </is>
       </c>
       <c r="I84" s="7" t="n">
-        <v>484</v>
+        <v>722</v>
       </c>
       <c r="J84" s="7" t="n"/>
       <c r="K84" s="7" t="n"/>
@@ -7115,7 +7121,7 @@
       <c r="P84" s="7" t="n"/>
       <c r="Q84" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R84" s="7" t="inlineStr">
@@ -7137,7 +7143,7 @@
       <c r="V84" s="6" t="inlineStr"/>
       <c r="W84" s="7" t="inlineStr">
         <is>
-          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
+          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
         </is>
       </c>
     </row>
@@ -7151,13 +7157,13 @@
         </is>
       </c>
       <c r="C85" s="9" t="n">
-        <v>1650</v>
+        <v>1630</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
@@ -7166,7 +7172,7 @@
       </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Harris Lofts, BS1 4BB</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
@@ -7175,14 +7181,14 @@
         </is>
       </c>
       <c r="I85" s="7" t="n">
-        <v>667</v>
+        <v>486</v>
       </c>
       <c r="J85" s="7" t="n"/>
       <c r="K85" s="7" t="n"/>
       <c r="L85" s="7" t="n"/>
       <c r="M85" s="7" t="n"/>
       <c r="N85" s="7" t="n">
-        <v>20088</v>
+        <v>13860</v>
       </c>
       <c r="O85" s="7" t="n">
         <v>0</v>
@@ -7190,12 +7196,12 @@
       <c r="P85" s="7" t="n"/>
       <c r="Q85" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R85" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S85" s="8" t="inlineStr"/>
@@ -7212,7 +7218,7 @@
       <c r="V85" s="6" t="inlineStr"/>
       <c r="W85" s="7" t="inlineStr">
         <is>
-          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
+          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
         </is>
       </c>
     </row>
@@ -7226,7 +7232,7 @@
         </is>
       </c>
       <c r="C86" s="9" t="n">
-        <v>1650</v>
+        <v>1635</v>
       </c>
       <c r="D86" s="7" t="n">
         <v>1</v>
@@ -7241,7 +7247,7 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>Central Quey North, Broad Quay, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
@@ -7249,13 +7255,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I86" s="7" t="n"/>
+      <c r="I86" s="7" t="n">
+        <v>560</v>
+      </c>
       <c r="J86" s="7" t="n"/>
       <c r="K86" s="7" t="n"/>
       <c r="L86" s="7" t="n"/>
       <c r="M86" s="7" t="n"/>
       <c r="N86" s="7" t="n">
-        <v>20768</v>
+        <v>13356</v>
       </c>
       <c r="O86" s="7" t="n">
         <v>0</v>
@@ -7263,12 +7271,12 @@
       <c r="P86" s="7" t="n"/>
       <c r="Q86" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R86" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S86" s="8" t="inlineStr"/>
@@ -7285,7 +7293,7 @@
       <c r="V86" s="6" t="inlineStr"/>
       <c r="W86" s="7" t="inlineStr">
         <is>
-          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
+          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
         </is>
       </c>
     </row>
@@ -7299,13 +7307,13 @@
         </is>
       </c>
       <c r="C87" s="9" t="n">
-        <v>1450</v>
+        <v>1665</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" s="7" t="inlineStr">
         <is>
@@ -7314,23 +7322,23 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>Woodbridge Road, Bristol, BS4</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I87" s="7" t="n">
-        <v>678</v>
+        <v>434</v>
       </c>
       <c r="J87" s="7" t="n"/>
       <c r="K87" s="7" t="n"/>
       <c r="L87" s="7" t="n"/>
       <c r="M87" s="7" t="n"/>
       <c r="N87" s="7" t="n">
-        <v>5700</v>
+        <v>13964</v>
       </c>
       <c r="O87" s="7" t="n">
         <v>0</v>
@@ -7338,12 +7346,12 @@
       <c r="P87" s="7" t="n"/>
       <c r="Q87" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R87" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S87" s="8" t="inlineStr"/>
@@ -7360,7 +7368,7 @@
       <c r="V87" s="6" t="inlineStr"/>
       <c r="W87" s="7" t="inlineStr">
         <is>
-          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
+          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
         </is>
       </c>
     </row>
@@ -7374,13 +7382,13 @@
         </is>
       </c>
       <c r="C88" s="9" t="n">
-        <v>2010</v>
+        <v>1400</v>
       </c>
       <c r="D88" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E88" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
@@ -7389,7 +7397,7 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>The Atrium, Redcliffe Street, BS1</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
@@ -7397,15 +7405,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I88" s="7" t="n">
-        <v>722</v>
-      </c>
+      <c r="I88" s="7" t="n"/>
       <c r="J88" s="7" t="n"/>
       <c r="K88" s="7" t="n"/>
       <c r="L88" s="7" t="n"/>
       <c r="M88" s="7" t="n"/>
       <c r="N88" s="7" t="n">
-        <v>13860</v>
+        <v>20292</v>
       </c>
       <c r="O88" s="7" t="n">
         <v>0</v>
@@ -7418,7 +7424,7 @@
       </c>
       <c r="R88" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S88" s="8" t="inlineStr"/>
@@ -7435,7 +7441,7 @@
       <c r="V88" s="6" t="inlineStr"/>
       <c r="W88" s="7" t="inlineStr">
         <is>
-          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
+          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
         </is>
       </c>
     </row>
@@ -7449,7 +7455,7 @@
         </is>
       </c>
       <c r="C89" s="9" t="n">
-        <v>1630</v>
+        <v>1460</v>
       </c>
       <c r="D89" s="7" t="n">
         <v>1</v>
@@ -7464,7 +7470,7 @@
       </c>
       <c r="G89" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
@@ -7473,14 +7479,14 @@
         </is>
       </c>
       <c r="I89" s="7" t="n">
-        <v>486</v>
+        <v>473</v>
       </c>
       <c r="J89" s="7" t="n"/>
       <c r="K89" s="7" t="n"/>
       <c r="L89" s="7" t="n"/>
       <c r="M89" s="7" t="n"/>
       <c r="N89" s="7" t="n">
-        <v>13860</v>
+        <v>21476</v>
       </c>
       <c r="O89" s="7" t="n">
         <v>0</v>
@@ -7488,12 +7494,12 @@
       <c r="P89" s="7" t="n"/>
       <c r="Q89" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R89" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S89" s="8" t="inlineStr"/>
@@ -7510,7 +7516,7 @@
       <c r="V89" s="6" t="inlineStr"/>
       <c r="W89" s="7" t="inlineStr">
         <is>
-          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
+          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
         </is>
       </c>
     </row>
@@ -7524,13 +7530,13 @@
         </is>
       </c>
       <c r="C90" s="9" t="n">
-        <v>1635</v>
+        <v>1990</v>
       </c>
       <c r="D90" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F90" s="7" t="inlineStr">
         <is>
@@ -7539,7 +7545,7 @@
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
@@ -7548,14 +7554,14 @@
         </is>
       </c>
       <c r="I90" s="7" t="n">
-        <v>560</v>
+        <v>682</v>
       </c>
       <c r="J90" s="7" t="n"/>
       <c r="K90" s="7" t="n"/>
       <c r="L90" s="7" t="n"/>
       <c r="M90" s="7" t="n"/>
       <c r="N90" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O90" s="7" t="n">
         <v>0</v>
@@ -7563,12 +7569,12 @@
       <c r="P90" s="7" t="n"/>
       <c r="Q90" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R90" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S90" s="8" t="inlineStr"/>
@@ -7585,7 +7591,7 @@
       <c r="V90" s="6" t="inlineStr"/>
       <c r="W90" s="7" t="inlineStr">
         <is>
-          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
+          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7605,7 @@
         </is>
       </c>
       <c r="C91" s="9" t="n">
-        <v>1665</v>
+        <v>1640</v>
       </c>
       <c r="D91" s="7" t="n">
         <v>1</v>
@@ -7614,7 +7620,7 @@
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
@@ -7623,14 +7629,14 @@
         </is>
       </c>
       <c r="I91" s="7" t="n">
-        <v>434</v>
+        <v>487</v>
       </c>
       <c r="J91" s="7" t="n"/>
       <c r="K91" s="7" t="n"/>
       <c r="L91" s="7" t="n"/>
       <c r="M91" s="7" t="n"/>
       <c r="N91" s="7" t="n">
-        <v>13964</v>
+        <v>13356</v>
       </c>
       <c r="O91" s="7" t="n">
         <v>0</v>
@@ -7638,12 +7644,12 @@
       <c r="P91" s="7" t="n"/>
       <c r="Q91" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R91" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S91" s="8" t="inlineStr"/>
@@ -7660,7 +7666,7 @@
       <c r="V91" s="6" t="inlineStr"/>
       <c r="W91" s="7" t="inlineStr">
         <is>
-          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
+          <t>ecc803f25866be367a83778bda0456688426a26e</t>
         </is>
       </c>
     </row>
@@ -7674,7 +7680,7 @@
         </is>
       </c>
       <c r="C92" s="9" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
       <c r="D92" s="7" t="n">
         <v>1</v>
@@ -7689,7 +7695,7 @@
       </c>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>The Atrium, Redcliffe Street, BS1</t>
+          <t>City Centre, Deanery Road, BS1 5AF</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr">
@@ -7697,13 +7703,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I92" s="7" t="n"/>
+      <c r="I92" s="7" t="n">
+        <v>570</v>
+      </c>
       <c r="J92" s="7" t="n"/>
       <c r="K92" s="7" t="n"/>
       <c r="L92" s="7" t="n"/>
       <c r="M92" s="7" t="n"/>
       <c r="N92" s="7" t="n">
-        <v>20292</v>
+        <v>19300</v>
       </c>
       <c r="O92" s="7" t="n">
         <v>0</v>
@@ -7711,12 +7719,12 @@
       <c r="P92" s="7" t="n"/>
       <c r="Q92" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R92" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S92" s="8" t="inlineStr"/>
@@ -7733,7 +7741,7 @@
       <c r="V92" s="6" t="inlineStr"/>
       <c r="W92" s="7" t="inlineStr">
         <is>
-          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
+          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
         </is>
       </c>
     </row>
@@ -7747,7 +7755,7 @@
         </is>
       </c>
       <c r="C93" s="9" t="n">
-        <v>1460</v>
+        <v>1995</v>
       </c>
       <c r="D93" s="7" t="n">
         <v>1</v>
@@ -7762,7 +7770,7 @@
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
@@ -7770,15 +7778,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I93" s="7" t="n">
-        <v>473</v>
-      </c>
+      <c r="I93" s="7" t="n"/>
       <c r="J93" s="7" t="n"/>
       <c r="K93" s="7" t="n"/>
       <c r="L93" s="7" t="n"/>
       <c r="M93" s="7" t="n"/>
       <c r="N93" s="7" t="n">
-        <v>21476</v>
+        <v>21196</v>
       </c>
       <c r="O93" s="7" t="n">
         <v>0</v>
@@ -7791,7 +7797,7 @@
       </c>
       <c r="R93" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S93" s="8" t="inlineStr"/>
@@ -7808,7 +7814,7 @@
       <c r="V93" s="6" t="inlineStr"/>
       <c r="W93" s="7" t="inlineStr">
         <is>
-          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
+          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
         </is>
       </c>
     </row>
@@ -7822,13 +7828,13 @@
         </is>
       </c>
       <c r="C94" s="9" t="n">
-        <v>1990</v>
+        <v>1395</v>
       </c>
       <c r="D94" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E94" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" s="7" t="inlineStr">
         <is>
@@ -7837,7 +7843,7 @@
       </c>
       <c r="G94" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
@@ -7845,15 +7851,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I94" s="7" t="n">
-        <v>682</v>
-      </c>
+      <c r="I94" s="7" t="n"/>
       <c r="J94" s="7" t="n"/>
       <c r="K94" s="7" t="n"/>
       <c r="L94" s="7" t="n"/>
       <c r="M94" s="7" t="n"/>
       <c r="N94" s="7" t="n">
-        <v>13964</v>
+        <v>20524</v>
       </c>
       <c r="O94" s="7" t="n">
         <v>0</v>
@@ -7861,12 +7865,12 @@
       <c r="P94" s="7" t="n"/>
       <c r="Q94" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R94" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S94" s="8" t="inlineStr"/>
@@ -7883,7 +7887,7 @@
       <c r="V94" s="6" t="inlineStr"/>
       <c r="W94" s="7" t="inlineStr">
         <is>
-          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
@@ -7897,13 +7901,13 @@
         </is>
       </c>
       <c r="C95" s="9" t="n">
-        <v>1640</v>
+        <v>2085</v>
       </c>
       <c r="D95" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E95" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
@@ -7912,7 +7916,7 @@
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
@@ -7921,14 +7925,14 @@
         </is>
       </c>
       <c r="I95" s="7" t="n">
-        <v>487</v>
+        <v>722</v>
       </c>
       <c r="J95" s="7" t="n"/>
       <c r="K95" s="7" t="n"/>
       <c r="L95" s="7" t="n"/>
       <c r="M95" s="7" t="n"/>
       <c r="N95" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O95" s="7" t="n">
         <v>0</v>
@@ -7936,12 +7940,12 @@
       <c r="P95" s="7" t="n"/>
       <c r="Q95" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R95" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S95" s="8" t="inlineStr"/>
@@ -7958,7 +7962,7 @@
       <c r="V95" s="6" t="inlineStr"/>
       <c r="W95" s="7" t="inlineStr">
         <is>
-          <t>ecc803f25866be367a83778bda0456688426a26e</t>
+          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
         </is>
       </c>
     </row>
@@ -7972,7 +7976,7 @@
         </is>
       </c>
       <c r="C96" s="9" t="n">
-        <v>1300</v>
+        <v>1485</v>
       </c>
       <c r="D96" s="7" t="n">
         <v>1</v>
@@ -7987,7 +7991,7 @@
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Deanery Road, BS1 5AF</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
@@ -7996,14 +8000,14 @@
         </is>
       </c>
       <c r="I96" s="7" t="n">
-        <v>570</v>
+        <v>470</v>
       </c>
       <c r="J96" s="7" t="n"/>
       <c r="K96" s="7" t="n"/>
       <c r="L96" s="7" t="n"/>
       <c r="M96" s="7" t="n"/>
       <c r="N96" s="7" t="n">
-        <v>19300</v>
+        <v>21476</v>
       </c>
       <c r="O96" s="7" t="n">
         <v>0</v>
@@ -8011,12 +8015,12 @@
       <c r="P96" s="7" t="n"/>
       <c r="Q96" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R96" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S96" s="8" t="inlineStr"/>
@@ -8033,7 +8037,7 @@
       <c r="V96" s="6" t="inlineStr"/>
       <c r="W96" s="7" t="inlineStr">
         <is>
-          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
+          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
         </is>
       </c>
     </row>
@@ -8047,7 +8051,7 @@
         </is>
       </c>
       <c r="C97" s="9" t="n">
-        <v>1995</v>
+        <v>1650</v>
       </c>
       <c r="D97" s="7" t="n">
         <v>1</v>
@@ -8062,7 +8066,7 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
@@ -8070,13 +8074,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I97" s="7" t="n"/>
+      <c r="I97" s="7" t="n">
+        <v>553</v>
+      </c>
       <c r="J97" s="7" t="n"/>
       <c r="K97" s="7" t="n"/>
       <c r="L97" s="7" t="n"/>
       <c r="M97" s="7" t="n"/>
       <c r="N97" s="7" t="n">
-        <v>21196</v>
+        <v>13356</v>
       </c>
       <c r="O97" s="7" t="n">
         <v>0</v>
@@ -8084,12 +8090,12 @@
       <c r="P97" s="7" t="n"/>
       <c r="Q97" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R97" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S97" s="8" t="inlineStr"/>
@@ -8106,7 +8112,7 @@
       <c r="V97" s="6" t="inlineStr"/>
       <c r="W97" s="7" t="inlineStr">
         <is>
-          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
+          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
         </is>
       </c>
     </row>
@@ -8120,13 +8126,13 @@
         </is>
       </c>
       <c r="C98" s="9" t="n">
-        <v>1395</v>
+        <v>1650</v>
       </c>
       <c r="D98" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E98" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
@@ -8135,7 +8141,7 @@
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
@@ -8149,7 +8155,7 @@
       <c r="L98" s="7" t="n"/>
       <c r="M98" s="7" t="n"/>
       <c r="N98" s="7" t="n">
-        <v>20524</v>
+        <v>20880</v>
       </c>
       <c r="O98" s="7" t="n">
         <v>0</v>
@@ -8157,7 +8163,7 @@
       <c r="P98" s="7" t="n"/>
       <c r="Q98" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R98" s="7" t="inlineStr">
@@ -8179,7 +8185,7 @@
       <c r="V98" s="6" t="inlineStr"/>
       <c r="W98" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
         </is>
       </c>
     </row>
@@ -8193,7 +8199,7 @@
         </is>
       </c>
       <c r="C99" s="9" t="n">
-        <v>2085</v>
+        <v>1900</v>
       </c>
       <c r="D99" s="7" t="n">
         <v>2</v>
@@ -8208,7 +8214,7 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Waverley House, BS1</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
@@ -8216,15 +8222,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I99" s="7" t="n">
-        <v>722</v>
-      </c>
+      <c r="I99" s="7" t="n"/>
       <c r="J99" s="7" t="n"/>
       <c r="K99" s="7" t="n"/>
       <c r="L99" s="7" t="n"/>
       <c r="M99" s="7" t="n"/>
       <c r="N99" s="7" t="n">
-        <v>13860</v>
+        <v>17956</v>
       </c>
       <c r="O99" s="7" t="n">
         <v>0</v>
@@ -8232,12 +8236,12 @@
       <c r="P99" s="7" t="n"/>
       <c r="Q99" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R99" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S99" s="8" t="inlineStr"/>
@@ -8254,7 +8258,7 @@
       <c r="V99" s="6" t="inlineStr"/>
       <c r="W99" s="7" t="inlineStr">
         <is>
-          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
+          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
         </is>
       </c>
     </row>
@@ -8268,14 +8272,12 @@
         </is>
       </c>
       <c r="C100" s="9" t="n">
-        <v>1485</v>
+        <v>1450</v>
       </c>
       <c r="D100" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E100" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E100" s="7" t="n"/>
       <c r="F100" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -8283,36 +8285,34 @@
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I100" s="7" t="n">
-        <v>470</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I100" s="7" t="n"/>
       <c r="J100" s="7" t="n"/>
       <c r="K100" s="7" t="n"/>
       <c r="L100" s="7" t="n"/>
       <c r="M100" s="7" t="n"/>
       <c r="N100" s="7" t="n">
-        <v>21476</v>
+        <v>19488</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P100" s="7" t="n"/>
       <c r="Q100" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R100" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S100" s="8" t="inlineStr"/>
@@ -8329,7 +8329,7 @@
       <c r="V100" s="6" t="inlineStr"/>
       <c r="W100" s="7" t="inlineStr">
         <is>
-          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
+          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8343,7 @@
         </is>
       </c>
       <c r="C101" s="9" t="n">
-        <v>1650</v>
+        <v>1500</v>
       </c>
       <c r="D101" s="7" t="n">
         <v>1</v>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
@@ -8366,15 +8366,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I101" s="7" t="n">
-        <v>553</v>
-      </c>
+      <c r="I101" s="7" t="n"/>
       <c r="J101" s="7" t="n"/>
       <c r="K101" s="7" t="n"/>
       <c r="L101" s="7" t="n"/>
       <c r="M101" s="7" t="n"/>
       <c r="N101" s="7" t="n">
-        <v>13356</v>
+        <v>20768</v>
       </c>
       <c r="O101" s="7" t="n">
         <v>0</v>
@@ -8382,12 +8380,12 @@
       <c r="P101" s="7" t="n"/>
       <c r="Q101" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R101" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S101" s="8" t="inlineStr"/>
@@ -8404,7 +8402,7 @@
       <c r="V101" s="6" t="inlineStr"/>
       <c r="W101" s="7" t="inlineStr">
         <is>
-          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
+          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
         </is>
       </c>
     </row>
@@ -8418,13 +8416,13 @@
         </is>
       </c>
       <c r="C102" s="9" t="n">
-        <v>1650</v>
+        <v>1450</v>
       </c>
       <c r="D102" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E102" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F102" s="7" t="inlineStr">
         <is>
@@ -8433,7 +8431,7 @@
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Welsh Back, Bristol</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr">
@@ -8447,7 +8445,7 @@
       <c r="L102" s="7" t="n"/>
       <c r="M102" s="7" t="n"/>
       <c r="N102" s="7" t="n">
-        <v>20880</v>
+        <v>13668</v>
       </c>
       <c r="O102" s="7" t="n">
         <v>0</v>
@@ -8455,12 +8453,12 @@
       <c r="P102" s="7" t="n"/>
       <c r="Q102" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R102" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Wildheart Residential Management Limited, Epsom</t>
         </is>
       </c>
       <c r="S102" s="8" t="inlineStr"/>
@@ -8477,7 +8475,7 @@
       <c r="V102" s="6" t="inlineStr"/>
       <c r="W102" s="7" t="inlineStr">
         <is>
-          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
+          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
         </is>
       </c>
     </row>
@@ -8491,36 +8489,38 @@
         </is>
       </c>
       <c r="C103" s="9" t="n">
-        <v>1900</v>
+        <v>2250</v>
       </c>
       <c r="D103" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E103" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>Waverley House, BS1</t>
+          <t>Newfoundland Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I103" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I103" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J103" s="7" t="n"/>
       <c r="K103" s="7" t="n"/>
       <c r="L103" s="7" t="n"/>
       <c r="M103" s="7" t="n"/>
       <c r="N103" s="7" t="n">
-        <v>17956</v>
+        <v>19800</v>
       </c>
       <c r="O103" s="7" t="n">
         <v>0</v>
@@ -8528,12 +8528,12 @@
       <c r="P103" s="7" t="n"/>
       <c r="Q103" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R103" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Lets Rent Bristol, Bristol</t>
         </is>
       </c>
       <c r="S103" s="8" t="inlineStr"/>
@@ -8550,7 +8550,7 @@
       <c r="V103" s="6" t="inlineStr"/>
       <c r="W103" s="7" t="inlineStr">
         <is>
-          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
+          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
         </is>
       </c>
     </row>
@@ -13006,83 +13006,10 @@
         </is>
       </c>
     </row>
-    <row r="164">
-      <c r="A164" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B164" s="8" t="inlineStr">
-        <is>
-          <t>Keyword match only (no API key configured for full scoring).</t>
-        </is>
-      </c>
-      <c r="C164" s="9" t="n">
-        <v>1250</v>
-      </c>
-      <c r="D164" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E164" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F164" s="7" t="inlineStr">
-        <is>
-          <t>flat</t>
-        </is>
-      </c>
-      <c r="G164" s="8" t="inlineStr">
-        <is>
-          <t>Southville, Bristol, BS3</t>
-        </is>
-      </c>
-      <c r="H164" s="7" t="inlineStr">
-        <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I164" s="7" t="n"/>
-      <c r="J164" s="7" t="n"/>
-      <c r="K164" s="7" t="n"/>
-      <c r="L164" s="7" t="n"/>
-      <c r="M164" s="7" t="n"/>
-      <c r="N164" s="7" t="n">
-        <v>11576</v>
-      </c>
-      <c r="O164" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P164" s="7" t="n"/>
-      <c r="Q164" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="R164" s="7" t="inlineStr">
-        <is>
-          <t>OpenRent, London</t>
-        </is>
-      </c>
-      <c r="S164" s="8" t="inlineStr"/>
-      <c r="T164" s="10" t="inlineStr">
-        <is>
-          <t>View listing</t>
-        </is>
-      </c>
-      <c r="U164" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="V164" s="6" t="inlineStr"/>
-      <c r="W164" s="7" t="inlineStr">
-        <is>
-          <t>805d107aec4cff74fe0c62f5dbc8a4b4cfbadeec</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W164"/>
+  <autoFilter ref="A1:W163"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -13249,7 +13176,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T161" r:id="rId160"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T162" r:id="rId161"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T163" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T164" r:id="rId163"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 108
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W155"/>
+  <dimension ref="A1:W156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1196,7 +1196,7 @@
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="n"/>
       <c r="N7" s="7" t="n">
-        <v>16644</v>
+        <v>16664</v>
       </c>
       <c r="O7" s="7" t="n">
         <v>0</v>
@@ -2290,7 +2290,7 @@
       <c r="L21" s="7" t="n"/>
       <c r="M21" s="7" t="n"/>
       <c r="N21" s="7" t="n">
-        <v>20780</v>
+        <v>13408</v>
       </c>
       <c r="O21" s="7" t="n">
         <v>0</v>
@@ -2527,7 +2527,7 @@
       <c r="L24" s="7" t="n"/>
       <c r="M24" s="7" t="n"/>
       <c r="N24" s="7" t="n">
-        <v>20780</v>
+        <v>13408</v>
       </c>
       <c r="O24" s="7" t="n">
         <v>0</v>
@@ -8528,7 +8528,7 @@
       <c r="L103" s="7" t="n"/>
       <c r="M103" s="7" t="n"/>
       <c r="N103" s="7" t="n">
-        <v>16644</v>
+        <v>16664</v>
       </c>
       <c r="O103" s="7" t="n">
         <v>0</v>
@@ -8572,13 +8572,13 @@
         </is>
       </c>
       <c r="C104" s="9" t="n">
-        <v>2500</v>
+        <v>1295</v>
       </c>
       <c r="D104" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E104" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F104" s="7" t="inlineStr">
         <is>
@@ -8587,21 +8587,23 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>Harbourside, Great Western House, BS1</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I104" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I104" s="7" t="n">
+        <v>474</v>
+      </c>
       <c r="J104" s="7" t="n"/>
       <c r="K104" s="7" t="n"/>
       <c r="L104" s="7" t="n"/>
       <c r="M104" s="7" t="n"/>
       <c r="N104" s="7" t="n">
-        <v>21360</v>
+        <v>14412</v>
       </c>
       <c r="O104" s="7" t="n">
         <v>0</v>
@@ -8609,12 +8611,12 @@
       <c r="P104" s="7" t="n"/>
       <c r="Q104" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R104" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S104" s="8" t="inlineStr"/>
@@ -8631,7 +8633,7 @@
       <c r="V104" s="6" t="inlineStr"/>
       <c r="W104" s="7" t="inlineStr">
         <is>
-          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
+          <t>466dad45b709c8ce2ab5e9d022bce4baabb5cecc</t>
         </is>
       </c>
     </row>
@@ -8645,13 +8647,13 @@
         </is>
       </c>
       <c r="C105" s="9" t="n">
-        <v>1650</v>
+        <v>2500</v>
       </c>
       <c r="D105" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E105" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
@@ -8660,7 +8662,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>Crown &amp; Anchor House, Bristol, BS2</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr">
@@ -8674,7 +8676,7 @@
       <c r="L105" s="7" t="n"/>
       <c r="M105" s="7" t="n"/>
       <c r="N105" s="7" t="n">
-        <v>20472</v>
+        <v>21360</v>
       </c>
       <c r="O105" s="7" t="n">
         <v>0</v>
@@ -8682,12 +8684,12 @@
       <c r="P105" s="7" t="n"/>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R105" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S105" s="8" t="inlineStr"/>
@@ -8704,7 +8706,7 @@
       <c r="V105" s="6" t="inlineStr"/>
       <c r="W105" s="7" t="inlineStr">
         <is>
-          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
+          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
         </is>
       </c>
     </row>
@@ -8718,13 +8720,13 @@
         </is>
       </c>
       <c r="C106" s="9" t="n">
-        <v>1450</v>
+        <v>1650</v>
       </c>
       <c r="D106" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E106" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
@@ -8733,23 +8735,21 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>Woodbridge Road, Bristol, BS4</t>
+          <t>Crown &amp; Anchor House, Bristol, BS2</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I106" s="7" t="n">
-        <v>678</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I106" s="7" t="n"/>
       <c r="J106" s="7" t="n"/>
       <c r="K106" s="7" t="n"/>
       <c r="L106" s="7" t="n"/>
       <c r="M106" s="7" t="n"/>
       <c r="N106" s="7" t="n">
-        <v>5700</v>
+        <v>20472</v>
       </c>
       <c r="O106" s="7" t="n">
         <v>0</v>
@@ -8757,12 +8757,12 @@
       <c r="P106" s="7" t="n"/>
       <c r="Q106" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R106" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S106" s="8" t="inlineStr"/>
@@ -8779,7 +8779,7 @@
       <c r="V106" s="6" t="inlineStr"/>
       <c r="W106" s="7" t="inlineStr">
         <is>
-          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
+          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
         </is>
       </c>
     </row>
@@ -8796,9 +8796,11 @@
         <v>1450</v>
       </c>
       <c r="D107" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E107" s="7" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="E107" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -8806,34 +8808,36 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Woodbridge Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I107" s="7" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I107" s="7" t="n">
+        <v>678</v>
+      </c>
       <c r="J107" s="7" t="n"/>
       <c r="K107" s="7" t="n"/>
       <c r="L107" s="7" t="n"/>
       <c r="M107" s="7" t="n"/>
       <c r="N107" s="7" t="n">
-        <v>19488</v>
+        <v>5700</v>
       </c>
       <c r="O107" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P107" s="7" t="n"/>
       <c r="Q107" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R107" s="7" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S107" s="8" t="inlineStr"/>
@@ -8850,7 +8854,7 @@
       <c r="V107" s="6" t="inlineStr"/>
       <c r="W107" s="7" t="inlineStr">
         <is>
-          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
+          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
         </is>
       </c>
     </row>
@@ -8864,14 +8868,12 @@
         </is>
       </c>
       <c r="C108" s="9" t="n">
-        <v>1500</v>
+        <v>1450</v>
       </c>
       <c r="D108" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E108" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E108" s="7" t="n"/>
       <c r="F108" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -8879,12 +8881,12 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I108" s="7" t="n"/>
@@ -8893,20 +8895,20 @@
       <c r="L108" s="7" t="n"/>
       <c r="M108" s="7" t="n"/>
       <c r="N108" s="7" t="n">
-        <v>20768</v>
+        <v>19488</v>
       </c>
       <c r="O108" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P108" s="7" t="n"/>
       <c r="Q108" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R108" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S108" s="8" t="inlineStr"/>
@@ -8923,7 +8925,7 @@
       <c r="V108" s="6" t="inlineStr"/>
       <c r="W108" s="7" t="inlineStr">
         <is>
-          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
+          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
         </is>
       </c>
     </row>
@@ -8937,38 +8939,36 @@
         </is>
       </c>
       <c r="C109" s="9" t="n">
-        <v>2250</v>
+        <v>1500</v>
       </c>
       <c r="D109" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E109" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>Newfoundland Road, Bristol, BS2</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H109" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I109" s="7" t="n">
-        <v>980</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I109" s="7" t="n"/>
       <c r="J109" s="7" t="n"/>
       <c r="K109" s="7" t="n"/>
       <c r="L109" s="7" t="n"/>
       <c r="M109" s="7" t="n"/>
       <c r="N109" s="7" t="n">
-        <v>19800</v>
+        <v>20768</v>
       </c>
       <c r="O109" s="7" t="n">
         <v>0</v>
@@ -8976,12 +8976,12 @@
       <c r="P109" s="7" t="n"/>
       <c r="Q109" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R109" s="7" t="inlineStr">
         <is>
-          <t>Lets Rent Bristol, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S109" s="8" t="inlineStr"/>
@@ -8998,7 +8998,7 @@
       <c r="V109" s="6" t="inlineStr"/>
       <c r="W109" s="7" t="inlineStr">
         <is>
-          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
+          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
         </is>
       </c>
     </row>
@@ -9012,36 +9012,38 @@
         </is>
       </c>
       <c r="C110" s="9" t="n">
-        <v>2000</v>
+        <v>2250</v>
       </c>
       <c r="D110" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E110" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F110" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>Protheroes House, Hobbs Lane, BS1</t>
+          <t>Newfoundland Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H110" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I110" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I110" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J110" s="7" t="n"/>
       <c r="K110" s="7" t="n"/>
       <c r="L110" s="7" t="n"/>
       <c r="M110" s="7" t="n"/>
       <c r="N110" s="7" t="n">
-        <v>13584</v>
+        <v>19800</v>
       </c>
       <c r="O110" s="7" t="n">
         <v>0</v>
@@ -9049,12 +9051,12 @@
       <c r="P110" s="7" t="n"/>
       <c r="Q110" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R110" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Lets Rent Bristol, Bristol</t>
         </is>
       </c>
       <c r="S110" s="8" t="inlineStr"/>
@@ -9071,7 +9073,7 @@
       <c r="V110" s="6" t="inlineStr"/>
       <c r="W110" s="7" t="inlineStr">
         <is>
-          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
+          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
         </is>
       </c>
     </row>
@@ -9085,27 +9087,27 @@
         </is>
       </c>
       <c r="C111" s="9" t="n">
-        <v>2400</v>
+        <v>2000</v>
       </c>
       <c r="D111" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E111" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>Balmain Street, Totterdown, Bristol, BS4</t>
+          <t>Protheroes House, Hobbs Lane, BS1</t>
         </is>
       </c>
       <c r="H111" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I111" s="7" t="n"/>
@@ -9114,7 +9116,7 @@
       <c r="L111" s="7" t="n"/>
       <c r="M111" s="7" t="n"/>
       <c r="N111" s="7" t="n">
-        <v>5524</v>
+        <v>13584</v>
       </c>
       <c r="O111" s="7" t="n">
         <v>0</v>
@@ -9122,12 +9124,12 @@
       <c r="P111" s="7" t="n"/>
       <c r="Q111" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R111" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S111" s="8" t="inlineStr"/>
@@ -9144,7 +9146,7 @@
       <c r="V111" s="6" t="inlineStr"/>
       <c r="W111" s="7" t="inlineStr">
         <is>
-          <t>dd411af39a083f886127138c0a969254da83858b</t>
+          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
         </is>
       </c>
     </row>
@@ -9158,51 +9160,49 @@
         </is>
       </c>
       <c r="C112" s="9" t="n">
-        <v>1665</v>
+        <v>2400</v>
       </c>
       <c r="D112" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E112" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F112" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Balmain Street, Totterdown, Bristol, BS4</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I112" s="7" t="n">
-        <v>578</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I112" s="7" t="n"/>
       <c r="J112" s="7" t="n"/>
       <c r="K112" s="7" t="n"/>
       <c r="L112" s="7" t="n"/>
       <c r="M112" s="7" t="n"/>
       <c r="N112" s="7" t="n">
-        <v>13356</v>
+        <v>5524</v>
       </c>
       <c r="O112" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P112" s="7" t="n"/>
       <c r="Q112" s="7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R112" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S112" s="8" t="inlineStr"/>
@@ -9219,7 +9219,7 @@
       <c r="V112" s="6" t="inlineStr"/>
       <c r="W112" s="7" t="inlineStr">
         <is>
-          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
+          <t>dd411af39a083f886127138c0a969254da83858b</t>
         </is>
       </c>
     </row>
@@ -9233,7 +9233,7 @@
         </is>
       </c>
       <c r="C113" s="9" t="n">
-        <v>1635</v>
+        <v>1665</v>
       </c>
       <c r="D113" s="7" t="n">
         <v>1</v>
@@ -9248,7 +9248,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H113" s="7" t="inlineStr">
@@ -9257,14 +9257,14 @@
         </is>
       </c>
       <c r="I113" s="7" t="n">
-        <v>485</v>
+        <v>578</v>
       </c>
       <c r="J113" s="7" t="n"/>
       <c r="K113" s="7" t="n"/>
       <c r="L113" s="7" t="n"/>
       <c r="M113" s="7" t="n"/>
       <c r="N113" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O113" s="7" t="n">
         <v>1</v>
@@ -9272,12 +9272,12 @@
       <c r="P113" s="7" t="n"/>
       <c r="Q113" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R113" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S113" s="8" t="inlineStr"/>
@@ -9294,7 +9294,7 @@
       <c r="V113" s="6" t="inlineStr"/>
       <c r="W113" s="7" t="inlineStr">
         <is>
-          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
+          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
         </is>
       </c>
     </row>
@@ -9308,7 +9308,7 @@
         </is>
       </c>
       <c r="C114" s="9" t="n">
-        <v>1615</v>
+        <v>1635</v>
       </c>
       <c r="D114" s="7" t="n">
         <v>1</v>
@@ -9332,7 +9332,7 @@
         </is>
       </c>
       <c r="I114" s="7" t="n">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="J114" s="7" t="n"/>
       <c r="K114" s="7" t="n"/>
@@ -9347,7 +9347,7 @@
       <c r="P114" s="7" t="n"/>
       <c r="Q114" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R114" s="7" t="inlineStr">
@@ -9369,7 +9369,7 @@
       <c r="V114" s="6" t="inlineStr"/>
       <c r="W114" s="7" t="inlineStr">
         <is>
-          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
+          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
         </is>
       </c>
     </row>
@@ -9383,7 +9383,7 @@
         </is>
       </c>
       <c r="C115" s="9" t="n">
-        <v>1640</v>
+        <v>1615</v>
       </c>
       <c r="D115" s="7" t="n">
         <v>1</v>
@@ -9398,7 +9398,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H115" s="7" t="inlineStr">
@@ -9407,14 +9407,14 @@
         </is>
       </c>
       <c r="I115" s="7" t="n">
-        <v>560</v>
+        <v>487</v>
       </c>
       <c r="J115" s="7" t="n"/>
       <c r="K115" s="7" t="n"/>
       <c r="L115" s="7" t="n"/>
       <c r="M115" s="7" t="n"/>
       <c r="N115" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O115" s="7" t="n">
         <v>1</v>
@@ -9422,12 +9422,12 @@
       <c r="P115" s="7" t="n"/>
       <c r="Q115" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R115" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S115" s="8" t="inlineStr"/>
@@ -9444,7 +9444,7 @@
       <c r="V115" s="6" t="inlineStr"/>
       <c r="W115" s="7" t="inlineStr">
         <is>
-          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
+          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
         </is>
       </c>
     </row>
@@ -9458,7 +9458,7 @@
         </is>
       </c>
       <c r="C116" s="9" t="n">
-        <v>1615</v>
+        <v>1640</v>
       </c>
       <c r="D116" s="7" t="n">
         <v>1</v>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H116" s="7" t="inlineStr">
@@ -9482,14 +9482,14 @@
         </is>
       </c>
       <c r="I116" s="7" t="n">
-        <v>484</v>
+        <v>560</v>
       </c>
       <c r="J116" s="7" t="n"/>
       <c r="K116" s="7" t="n"/>
       <c r="L116" s="7" t="n"/>
       <c r="M116" s="7" t="n"/>
       <c r="N116" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O116" s="7" t="n">
         <v>1</v>
@@ -9502,7 +9502,7 @@
       </c>
       <c r="R116" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S116" s="8" t="inlineStr"/>
@@ -9519,7 +9519,7 @@
       <c r="V116" s="6" t="inlineStr"/>
       <c r="W116" s="7" t="inlineStr">
         <is>
-          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
+          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
         </is>
       </c>
     </row>
@@ -9557,7 +9557,7 @@
         </is>
       </c>
       <c r="I117" s="7" t="n">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="J117" s="7" t="n"/>
       <c r="K117" s="7" t="n"/>
@@ -9567,12 +9567,12 @@
         <v>13860</v>
       </c>
       <c r="O117" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P117" s="7" t="n"/>
       <c r="Q117" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R117" s="7" t="inlineStr">
@@ -9594,7 +9594,7 @@
       <c r="V117" s="6" t="inlineStr"/>
       <c r="W117" s="7" t="inlineStr">
         <is>
-          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
+          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
         </is>
       </c>
     </row>
@@ -9608,7 +9608,7 @@
         </is>
       </c>
       <c r="C118" s="9" t="n">
-        <v>1645</v>
+        <v>1615</v>
       </c>
       <c r="D118" s="7" t="n">
         <v>1</v>
@@ -9623,7 +9623,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H118" s="7" t="inlineStr">
@@ -9632,14 +9632,14 @@
         </is>
       </c>
       <c r="I118" s="7" t="n">
-        <v>570</v>
+        <v>486</v>
       </c>
       <c r="J118" s="7" t="n"/>
       <c r="K118" s="7" t="n"/>
       <c r="L118" s="7" t="n"/>
       <c r="M118" s="7" t="n"/>
       <c r="N118" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O118" s="7" t="n">
         <v>0</v>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="R118" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S118" s="8" t="inlineStr"/>
@@ -9669,7 +9669,7 @@
       <c r="V118" s="6" t="inlineStr"/>
       <c r="W118" s="7" t="inlineStr">
         <is>
-          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
+          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
         </is>
       </c>
     </row>
@@ -9683,7 +9683,7 @@
         </is>
       </c>
       <c r="C119" s="9" t="n">
-        <v>1630</v>
+        <v>1645</v>
       </c>
       <c r="D119" s="7" t="n">
         <v>1</v>
@@ -9707,7 +9707,7 @@
         </is>
       </c>
       <c r="I119" s="7" t="n">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="J119" s="7" t="n"/>
       <c r="K119" s="7" t="n"/>
@@ -9722,7 +9722,7 @@
       <c r="P119" s="7" t="n"/>
       <c r="Q119" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R119" s="7" t="inlineStr">
@@ -9744,7 +9744,7 @@
       <c r="V119" s="6" t="inlineStr"/>
       <c r="W119" s="7" t="inlineStr">
         <is>
-          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
+          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
         </is>
       </c>
     </row>
@@ -9758,10 +9758,10 @@
         </is>
       </c>
       <c r="C120" s="9" t="n">
-        <v>1800</v>
+        <v>1630</v>
       </c>
       <c r="D120" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E120" s="7" t="n">
         <v>1</v>
@@ -9773,7 +9773,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H120" s="7" t="inlineStr">
@@ -9781,13 +9781,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I120" s="7" t="n"/>
+      <c r="I120" s="7" t="n">
+        <v>560</v>
+      </c>
       <c r="J120" s="7" t="n"/>
       <c r="K120" s="7" t="n"/>
       <c r="L120" s="7" t="n"/>
       <c r="M120" s="7" t="n"/>
       <c r="N120" s="7" t="n">
-        <v>21176</v>
+        <v>13356</v>
       </c>
       <c r="O120" s="7" t="n">
         <v>0</v>
@@ -9800,7 +9802,7 @@
       </c>
       <c r="R120" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S120" s="8" t="inlineStr"/>
@@ -9817,7 +9819,7 @@
       <c r="V120" s="6" t="inlineStr"/>
       <c r="W120" s="7" t="inlineStr">
         <is>
-          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
+          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
         </is>
       </c>
     </row>
@@ -9831,10 +9833,10 @@
         </is>
       </c>
       <c r="C121" s="9" t="n">
-        <v>1635</v>
+        <v>1800</v>
       </c>
       <c r="D121" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E121" s="7" t="n">
         <v>1</v>
@@ -9846,7 +9848,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H121" s="7" t="inlineStr">
@@ -9854,15 +9856,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I121" s="7" t="n">
-        <v>569</v>
-      </c>
+      <c r="I121" s="7" t="n"/>
       <c r="J121" s="7" t="n"/>
       <c r="K121" s="7" t="n"/>
       <c r="L121" s="7" t="n"/>
       <c r="M121" s="7" t="n"/>
       <c r="N121" s="7" t="n">
-        <v>13356</v>
+        <v>21176</v>
       </c>
       <c r="O121" s="7" t="n">
         <v>0</v>
@@ -9870,12 +9870,12 @@
       <c r="P121" s="7" t="n"/>
       <c r="Q121" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R121" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S121" s="8" t="inlineStr"/>
@@ -9892,7 +9892,7 @@
       <c r="V121" s="6" t="inlineStr"/>
       <c r="W121" s="7" t="inlineStr">
         <is>
-          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
+          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
         </is>
       </c>
     </row>
@@ -9906,10 +9906,10 @@
         </is>
       </c>
       <c r="C122" s="9" t="n">
-        <v>1925</v>
+        <v>1635</v>
       </c>
       <c r="D122" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E122" s="7" t="n">
         <v>1</v>
@@ -9921,7 +9921,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H122" s="7" t="inlineStr">
@@ -9930,14 +9930,14 @@
         </is>
       </c>
       <c r="I122" s="7" t="n">
-        <v>655</v>
+        <v>569</v>
       </c>
       <c r="J122" s="7" t="n"/>
       <c r="K122" s="7" t="n"/>
       <c r="L122" s="7" t="n"/>
       <c r="M122" s="7" t="n"/>
       <c r="N122" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O122" s="7" t="n">
         <v>0</v>
@@ -9945,12 +9945,12 @@
       <c r="P122" s="7" t="n"/>
       <c r="Q122" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R122" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S122" s="8" t="inlineStr"/>
@@ -9967,7 +9967,7 @@
       <c r="V122" s="6" t="inlineStr"/>
       <c r="W122" s="7" t="inlineStr">
         <is>
-          <t>892dd053ae3538c7c123f255e926bef984caf6de</t>
+          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
         </is>
       </c>
     </row>
@@ -9981,13 +9981,13 @@
         </is>
       </c>
       <c r="C123" s="9" t="n">
-        <v>1800</v>
+        <v>1925</v>
       </c>
       <c r="D123" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E123" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F123" s="7" t="inlineStr">
         <is>
@@ -9996,7 +9996,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>Park St, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H123" s="7" t="inlineStr">
@@ -10004,13 +10004,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I123" s="7" t="n"/>
+      <c r="I123" s="7" t="n">
+        <v>655</v>
+      </c>
       <c r="J123" s="7" t="n"/>
       <c r="K123" s="7" t="n"/>
       <c r="L123" s="7" t="n"/>
       <c r="M123" s="7" t="n"/>
       <c r="N123" s="7" t="n">
-        <v>20644</v>
+        <v>21476</v>
       </c>
       <c r="O123" s="7" t="n">
         <v>0</v>
@@ -10018,12 +10020,12 @@
       <c r="P123" s="7" t="n"/>
       <c r="Q123" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R123" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S123" s="8" t="inlineStr"/>
@@ -10040,7 +10042,7 @@
       <c r="V123" s="6" t="inlineStr"/>
       <c r="W123" s="7" t="inlineStr">
         <is>
-          <t>8e49447f07b7d2adcefccb79294af764ba54db50</t>
+          <t>892dd053ae3538c7c123f255e926bef984caf6de</t>
         </is>
       </c>
     </row>
@@ -10054,13 +10056,13 @@
         </is>
       </c>
       <c r="C124" s="9" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="D124" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E124" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F124" s="7" t="inlineStr">
         <is>
@@ -10069,7 +10071,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>Marsh House, Bristol, BS1</t>
+          <t>Park St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H124" s="7" t="inlineStr">
@@ -10083,7 +10085,7 @@
       <c r="L124" s="7" t="n"/>
       <c r="M124" s="7" t="n"/>
       <c r="N124" s="7" t="n">
-        <v>20952</v>
+        <v>20644</v>
       </c>
       <c r="O124" s="7" t="n">
         <v>0</v>
@@ -10091,12 +10093,12 @@
       <c r="P124" s="7" t="n"/>
       <c r="Q124" s="7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R124" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S124" s="8" t="inlineStr"/>
@@ -10113,7 +10115,7 @@
       <c r="V124" s="6" t="inlineStr"/>
       <c r="W124" s="7" t="inlineStr">
         <is>
-          <t>dc8b7c88d86188af3ee5262a5f1215944eb3e402</t>
+          <t>8e49447f07b7d2adcefccb79294af764ba54db50</t>
         </is>
       </c>
     </row>
@@ -10127,10 +10129,10 @@
         </is>
       </c>
       <c r="C125" s="9" t="n">
-        <v>1800</v>
+        <v>1650</v>
       </c>
       <c r="D125" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E125" s="7" t="n">
         <v>1</v>
@@ -10142,7 +10144,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Marsh House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H125" s="7" t="inlineStr">
@@ -10156,7 +10158,7 @@
       <c r="L125" s="7" t="n"/>
       <c r="M125" s="7" t="n"/>
       <c r="N125" s="7" t="n">
-        <v>20592</v>
+        <v>20952</v>
       </c>
       <c r="O125" s="7" t="n">
         <v>0</v>
@@ -10164,12 +10166,12 @@
       <c r="P125" s="7" t="n"/>
       <c r="Q125" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R125" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S125" s="8" t="inlineStr"/>
@@ -10186,7 +10188,7 @@
       <c r="V125" s="6" t="inlineStr"/>
       <c r="W125" s="7" t="inlineStr">
         <is>
-          <t>7aa830b20d3fe9e9350b37a53ede99615caa3290</t>
+          <t>dc8b7c88d86188af3ee5262a5f1215944eb3e402</t>
         </is>
       </c>
     </row>
@@ -10200,10 +10202,10 @@
         </is>
       </c>
       <c r="C126" s="9" t="n">
-        <v>1350</v>
+        <v>1800</v>
       </c>
       <c r="D126" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E126" s="7" t="n">
         <v>1</v>
@@ -10215,7 +10217,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H126" s="7" t="inlineStr">
@@ -10223,15 +10225,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I126" s="7" t="n">
-        <v>518</v>
-      </c>
+      <c r="I126" s="7" t="n"/>
       <c r="J126" s="7" t="n"/>
       <c r="K126" s="7" t="n"/>
       <c r="L126" s="7" t="n"/>
       <c r="M126" s="7" t="n"/>
       <c r="N126" s="7" t="n">
-        <v>16416</v>
+        <v>20592</v>
       </c>
       <c r="O126" s="7" t="n">
         <v>0</v>
@@ -10239,12 +10239,12 @@
       <c r="P126" s="7" t="n"/>
       <c r="Q126" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R126" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S126" s="8" t="inlineStr"/>
@@ -10261,7 +10261,7 @@
       <c r="V126" s="6" t="inlineStr"/>
       <c r="W126" s="7" t="inlineStr">
         <is>
-          <t>77b9e2d97ea9d3f764e1fbd2fdd0b5bf1d5b75b8</t>
+          <t>7aa830b20d3fe9e9350b37a53ede99615caa3290</t>
         </is>
       </c>
     </row>
@@ -10275,7 +10275,7 @@
         </is>
       </c>
       <c r="C127" s="9" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="D127" s="7" t="n">
         <v>1</v>
@@ -10290,7 +10290,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H127" s="7" t="inlineStr">
@@ -10298,13 +10298,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I127" s="7" t="n"/>
+      <c r="I127" s="7" t="n">
+        <v>518</v>
+      </c>
       <c r="J127" s="7" t="n"/>
       <c r="K127" s="7" t="n"/>
       <c r="L127" s="7" t="n"/>
       <c r="M127" s="7" t="n"/>
       <c r="N127" s="7" t="n">
-        <v>20524</v>
+        <v>16416</v>
       </c>
       <c r="O127" s="7" t="n">
         <v>0</v>
@@ -10317,7 +10319,7 @@
       </c>
       <c r="R127" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S127" s="8" t="inlineStr"/>
@@ -10334,7 +10336,7 @@
       <c r="V127" s="6" t="inlineStr"/>
       <c r="W127" s="7" t="inlineStr">
         <is>
-          <t>adbd7c1c798d9f667bce5c8c0d31831cec0ebf67</t>
+          <t>77b9e2d97ea9d3f764e1fbd2fdd0b5bf1d5b75b8</t>
         </is>
       </c>
     </row>
@@ -10348,10 +10350,10 @@
         </is>
       </c>
       <c r="C128" s="9" t="n">
-        <v>1500</v>
+        <v>1450</v>
       </c>
       <c r="D128" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E128" s="7" t="n">
         <v>1</v>
@@ -10363,12 +10365,12 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>The Quadrant, Bristol, BS2</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H128" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I128" s="7" t="n"/>
@@ -10377,7 +10379,7 @@
       <c r="L128" s="7" t="n"/>
       <c r="M128" s="7" t="n"/>
       <c r="N128" s="7" t="n">
-        <v>20056</v>
+        <v>20524</v>
       </c>
       <c r="O128" s="7" t="n">
         <v>0</v>
@@ -10385,12 +10387,12 @@
       <c r="P128" s="7" t="n"/>
       <c r="Q128" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R128" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S128" s="8" t="inlineStr"/>
@@ -10407,7 +10409,7 @@
       <c r="V128" s="6" t="inlineStr"/>
       <c r="W128" s="7" t="inlineStr">
         <is>
-          <t>c77814f9166c93a32f4a1ce46b46c87a68a6196a</t>
+          <t>adbd7c1c798d9f667bce5c8c0d31831cec0ebf67</t>
         </is>
       </c>
     </row>
@@ -10421,13 +10423,13 @@
         </is>
       </c>
       <c r="C129" s="9" t="n">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="D129" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E129" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
@@ -10436,12 +10438,12 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>The Quadrant, Bristol, BS2</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I129" s="7" t="n"/>
@@ -10450,20 +10452,20 @@
       <c r="L129" s="7" t="n"/>
       <c r="M129" s="7" t="n"/>
       <c r="N129" s="7" t="n">
-        <v>21020</v>
+        <v>20056</v>
       </c>
       <c r="O129" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P129" s="7" t="n"/>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R129" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S129" s="8" t="inlineStr"/>
@@ -10480,7 +10482,7 @@
       <c r="V129" s="6" t="inlineStr"/>
       <c r="W129" s="7" t="inlineStr">
         <is>
-          <t>9fe5cc28570329e8d733373bcf933c665273bc0e</t>
+          <t>c77814f9166c93a32f4a1ce46b46c87a68a6196a</t>
         </is>
       </c>
     </row>
@@ -10494,13 +10496,13 @@
         </is>
       </c>
       <c r="C130" s="9" t="n">
-        <v>1250</v>
+        <v>1800</v>
       </c>
       <c r="D130" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E130" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
@@ -10509,7 +10511,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Jessop Court, BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
@@ -10517,15 +10519,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I130" s="7" t="n">
-        <v>538</v>
-      </c>
+      <c r="I130" s="7" t="n"/>
       <c r="J130" s="7" t="n"/>
       <c r="K130" s="7" t="n"/>
       <c r="L130" s="7" t="n"/>
       <c r="M130" s="7" t="n"/>
       <c r="N130" s="7" t="n">
-        <v>20788</v>
+        <v>21020</v>
       </c>
       <c r="O130" s="7" t="n">
         <v>1</v>
@@ -10533,12 +10533,12 @@
       <c r="P130" s="7" t="n"/>
       <c r="Q130" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R130" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S130" s="8" t="inlineStr"/>
@@ -10555,7 +10555,7 @@
       <c r="V130" s="6" t="inlineStr"/>
       <c r="W130" s="7" t="inlineStr">
         <is>
-          <t>34093b6e05a2deb3da2e1a98a249e966d7af0cdf</t>
+          <t>9fe5cc28570329e8d733373bcf933c665273bc0e</t>
         </is>
       </c>
     </row>
@@ -10584,7 +10584,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>St. Stephens Street, Bristol, BS1</t>
+          <t>City Centre, Jessop Court, BS1</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr">
@@ -10592,13 +10592,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I131" s="7" t="n"/>
+      <c r="I131" s="7" t="n">
+        <v>538</v>
+      </c>
       <c r="J131" s="7" t="n"/>
       <c r="K131" s="7" t="n"/>
       <c r="L131" s="7" t="n"/>
       <c r="M131" s="7" t="n"/>
       <c r="N131" s="7" t="n">
-        <v>13940</v>
+        <v>20788</v>
       </c>
       <c r="O131" s="7" t="n">
         <v>1</v>
@@ -10606,12 +10608,12 @@
       <c r="P131" s="7" t="n"/>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S131" s="8" t="inlineStr"/>
@@ -10628,7 +10630,7 @@
       <c r="V131" s="6" t="inlineStr"/>
       <c r="W131" s="7" t="inlineStr">
         <is>
-          <t>705e73e870fdf398639d5c8b181c8e21b143f622</t>
+          <t>34093b6e05a2deb3da2e1a98a249e966d7af0cdf</t>
         </is>
       </c>
     </row>
@@ -10642,7 +10644,7 @@
         </is>
       </c>
       <c r="C132" s="9" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
       <c r="D132" s="7" t="n">
         <v>1</v>
@@ -10657,12 +10659,12 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>Cutting Room, Bristol, BS3</t>
+          <t>St. Stephens Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I132" s="7" t="n"/>
@@ -10671,7 +10673,7 @@
       <c r="L132" s="7" t="n"/>
       <c r="M132" s="7" t="n"/>
       <c r="N132" s="7" t="n">
-        <v>13836</v>
+        <v>13940</v>
       </c>
       <c r="O132" s="7" t="n">
         <v>1</v>
@@ -10679,12 +10681,12 @@
       <c r="P132" s="7" t="n"/>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Southville</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S132" s="8" t="inlineStr"/>
@@ -10701,7 +10703,7 @@
       <c r="V132" s="6" t="inlineStr"/>
       <c r="W132" s="7" t="inlineStr">
         <is>
-          <t>8bb5fbce4e6d80f79ecceb7d5bb4f35766fbb83c</t>
+          <t>705e73e870fdf398639d5c8b181c8e21b143f622</t>
         </is>
       </c>
     </row>
@@ -10715,7 +10717,7 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1650</v>
+        <v>1500</v>
       </c>
       <c r="D133" s="7" t="n">
         <v>1</v>
@@ -10730,36 +10732,34 @@
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Cutting Room, Bristol, BS3</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I133" s="7" t="n">
-        <v>486</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I133" s="7" t="n"/>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>13860</v>
+        <v>13836</v>
       </c>
       <c r="O133" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S133" s="8" t="inlineStr"/>
@@ -10776,7 +10776,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>e26a5dedfb7c4bcd1308250a8955318f00994505</t>
+          <t>8bb5fbce4e6d80f79ecceb7d5bb4f35766fbb83c</t>
         </is>
       </c>
     </row>
@@ -10790,13 +10790,13 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>2240</v>
+        <v>1650</v>
       </c>
       <c r="D134" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E134" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
@@ -10805,7 +10805,7 @@
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
@@ -10814,14 +10814,14 @@
         </is>
       </c>
       <c r="I134" s="7" t="n">
-        <v>884</v>
+        <v>486</v>
       </c>
       <c r="J134" s="7" t="n"/>
       <c r="K134" s="7" t="n"/>
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="7" t="n">
-        <v>13388</v>
+        <v>13860</v>
       </c>
       <c r="O134" s="7" t="n">
         <v>0</v>
@@ -10829,12 +10829,12 @@
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10851,7 +10851,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>0b2cd6178fe0f6128804b82d5b9e39ea5967f124</t>
+          <t>e26a5dedfb7c4bcd1308250a8955318f00994505</t>
         </is>
       </c>
     </row>
@@ -10865,13 +10865,13 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1650</v>
+        <v>2240</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
@@ -10889,14 +10889,14 @@
         </is>
       </c>
       <c r="I135" s="7" t="n">
-        <v>553</v>
+        <v>884</v>
       </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="7" t="n">
-        <v>13356</v>
+        <v>13388</v>
       </c>
       <c r="O135" s="7" t="n">
         <v>0</v>
@@ -10904,7 +10904,7 @@
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
@@ -10926,7 +10926,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>d6bb31b3e903e1ec64e3eea9a96c3b08bb9873e3</t>
+          <t>0b2cd6178fe0f6128804b82d5b9e39ea5967f124</t>
         </is>
       </c>
     </row>
@@ -10940,7 +10940,7 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>1640</v>
+        <v>1650</v>
       </c>
       <c r="D136" s="7" t="n">
         <v>1</v>
@@ -10955,7 +10955,7 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
@@ -10964,14 +10964,14 @@
         </is>
       </c>
       <c r="I136" s="7" t="n">
-        <v>485</v>
+        <v>553</v>
       </c>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -10984,7 +10984,7 @@
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11001,7 +11001,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>47301f8a472393cf4550a7380ee71363e6337581</t>
+          <t>d6bb31b3e903e1ec64e3eea9a96c3b08bb9873e3</t>
         </is>
       </c>
     </row>
@@ -11015,7 +11015,7 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1660</v>
+        <v>1640</v>
       </c>
       <c r="D137" s="7" t="n">
         <v>1</v>
@@ -11030,7 +11030,7 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
@@ -11039,14 +11039,14 @@
         </is>
       </c>
       <c r="I137" s="7" t="n">
-        <v>578</v>
+        <v>485</v>
       </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O137" s="7" t="n">
         <v>0</v>
@@ -11054,12 +11054,12 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S137" s="8" t="inlineStr"/>
@@ -11076,7 +11076,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>5f45fddd60a4f7306d53e1880e39147d0065c173</t>
+          <t>47301f8a472393cf4550a7380ee71363e6337581</t>
         </is>
       </c>
     </row>
@@ -11090,7 +11090,7 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1630</v>
+        <v>1660</v>
       </c>
       <c r="D138" s="7" t="n">
         <v>1</v>
@@ -11105,7 +11105,7 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
@@ -11114,14 +11114,14 @@
         </is>
       </c>
       <c r="I138" s="7" t="n">
-        <v>486</v>
+        <v>578</v>
       </c>
       <c r="J138" s="7" t="n"/>
       <c r="K138" s="7" t="n"/>
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11129,12 +11129,12 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11151,7 +11151,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>91d51985531a7953cdf1bb0173d032c892f5c019</t>
+          <t>5f45fddd60a4f7306d53e1880e39147d0065c173</t>
         </is>
       </c>
     </row>
@@ -11165,7 +11165,7 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>1585</v>
+        <v>1630</v>
       </c>
       <c r="D139" s="7" t="n">
         <v>1</v>
@@ -11180,7 +11180,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11189,14 +11189,14 @@
         </is>
       </c>
       <c r="I139" s="7" t="n">
-        <v>505</v>
+        <v>486</v>
       </c>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11204,12 +11204,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11226,7 +11226,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>4fc7c891593aa7586ebede2a12c2a9af8edbe973</t>
+          <t>91d51985531a7953cdf1bb0173d032c892f5c019</t>
         </is>
       </c>
     </row>
@@ -11240,7 +11240,7 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1890</v>
+        <v>1585</v>
       </c>
       <c r="D140" s="7" t="n">
         <v>1</v>
@@ -11255,7 +11255,7 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
@@ -11264,14 +11264,14 @@
         </is>
       </c>
       <c r="I140" s="7" t="n">
-        <v>538</v>
+        <v>505</v>
       </c>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11279,12 +11279,12 @@
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11301,7 +11301,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>f819b6d7cea8e4f9f3bc624d2737801ca68a6b49</t>
+          <t>4fc7c891593aa7586ebede2a12c2a9af8edbe973</t>
         </is>
       </c>
     </row>
@@ -11315,7 +11315,7 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1510</v>
+        <v>1890</v>
       </c>
       <c r="D141" s="7" t="n">
         <v>1</v>
@@ -11330,7 +11330,7 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
@@ -11339,14 +11339,14 @@
         </is>
       </c>
       <c r="I141" s="7" t="n">
-        <v>509</v>
+        <v>538</v>
       </c>
       <c r="J141" s="7" t="n"/>
       <c r="K141" s="7" t="n"/>
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11354,12 +11354,12 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11376,7 +11376,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>3ebe55674c01ebb6e152801ec69490ad7da0c8cc</t>
+          <t>f819b6d7cea8e4f9f3bc624d2737801ca68a6b49</t>
         </is>
       </c>
     </row>
@@ -11390,10 +11390,10 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>2100</v>
+        <v>1510</v>
       </c>
       <c r="D142" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E142" s="7" t="n">
         <v>1</v>
@@ -11405,21 +11405,23 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>Old Market Street, St Philips, Bristol, Bristol City, BS2</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I142" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I142" s="7" t="n">
+        <v>509</v>
+      </c>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>13716</v>
+        <v>21476</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11427,12 +11429,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Yours Link Limited, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11449,7 +11451,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>2328edfeefd3149329151e5048af6234618528dc</t>
+          <t>3ebe55674c01ebb6e152801ec69490ad7da0c8cc</t>
         </is>
       </c>
     </row>
@@ -11463,10 +11465,10 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1400</v>
+        <v>2100</v>
       </c>
       <c r="D143" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E143" s="7" t="n">
         <v>1</v>
@@ -11478,12 +11480,12 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol City Centre, BS1</t>
+          <t>Old Market Street, St Philips, Bristol, Bristol City, BS2</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I143" s="7" t="n"/>
@@ -11492,7 +11494,7 @@
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>13404</v>
+        <v>13716</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11500,12 +11502,12 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Yours Link Limited, London</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11522,7 +11524,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>80ae63ab944f6cd80f590015e53caffc4c3b1f4f</t>
+          <t>2328edfeefd3149329151e5048af6234618528dc</t>
         </is>
       </c>
     </row>
@@ -11536,7 +11538,7 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1350</v>
+        <v>1400</v>
       </c>
       <c r="D144" s="7" t="n">
         <v>1</v>
@@ -11551,7 +11553,7 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>Finzels Reach, Castle Wharf, BS1 6JU</t>
+          <t>Central Quay North, Bristol City Centre, BS1</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
@@ -11559,15 +11561,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I144" s="7" t="n">
-        <v>603</v>
-      </c>
+      <c r="I144" s="7" t="n"/>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>14052</v>
+        <v>13404</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11575,12 +11575,12 @@
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11597,7 +11597,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>f635c3d4727470f01fd1777da4ca6eea453c6655</t>
+          <t>80ae63ab944f6cd80f590015e53caffc4c3b1f4f</t>
         </is>
       </c>
     </row>
@@ -11611,7 +11611,7 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>1400</v>
+        <v>1350</v>
       </c>
       <c r="D145" s="7" t="n">
         <v>1</v>
@@ -11626,7 +11626,7 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Finzels Reach, Castle Wharf, BS1 6JU</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
@@ -11634,13 +11634,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I145" s="7" t="n"/>
+      <c r="I145" s="7" t="n">
+        <v>603</v>
+      </c>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>16580</v>
+        <v>14052</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11648,12 +11650,12 @@
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S145" s="8" t="inlineStr"/>
@@ -11670,7 +11672,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>680172a6c9a0d74ac3232df41c01ab789bdfd3a8</t>
+          <t>f635c3d4727470f01fd1777da4ca6eea453c6655</t>
         </is>
       </c>
     </row>
@@ -11684,7 +11686,7 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>1350</v>
+        <v>1400</v>
       </c>
       <c r="D146" s="7" t="n">
         <v>1</v>
@@ -11699,7 +11701,7 @@
       </c>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>Protheroes House, Hobbs Lane, City Cenrre, Bristol, BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
@@ -11713,7 +11715,7 @@
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>13584</v>
+        <v>16580</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>0</v>
@@ -11721,12 +11723,12 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Romans, Clifton</t>
         </is>
       </c>
       <c r="S146" s="8" t="inlineStr"/>
@@ -11743,7 +11745,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>b875a37866336756017edebdebb9268d8d435810</t>
+          <t>680172a6c9a0d74ac3232df41c01ab789bdfd3a8</t>
         </is>
       </c>
     </row>
@@ -11772,7 +11774,7 @@
       </c>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Deanery Road, BS1 5QH</t>
+          <t>Protheroes House, Hobbs Lane, City Cenrre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H147" s="7" t="inlineStr">
@@ -11780,15 +11782,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I147" s="7" t="n">
-        <v>549</v>
-      </c>
+      <c r="I147" s="7" t="n"/>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="7" t="n">
-        <v>11916</v>
+        <v>13584</v>
       </c>
       <c r="O147" s="7" t="n">
         <v>0</v>
@@ -11796,12 +11796,12 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S147" s="8" t="inlineStr"/>
@@ -11818,7 +11818,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>e0fe1f3069e7bd647d5729169c7f51a5fabb84f8</t>
+          <t>b875a37866336756017edebdebb9268d8d435810</t>
         </is>
       </c>
     </row>
@@ -11832,7 +11832,7 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>1500</v>
+        <v>1350</v>
       </c>
       <c r="D148" s="7" t="n">
         <v>1</v>
@@ -11847,7 +11847,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Flat 109, Invicta, Millennium Promenade, Bristol, Bristol, City of, BS1</t>
+          <t>City Centre, Deanery Road, BS1 5QH</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
@@ -11855,13 +11855,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I148" s="7" t="n"/>
+      <c r="I148" s="7" t="n">
+        <v>549</v>
+      </c>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>16168</v>
+        <v>11916</v>
       </c>
       <c r="O148" s="7" t="n">
         <v>0</v>
@@ -11869,12 +11871,12 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Bishopston</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11891,7 +11893,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>f987cb39e8da7d77742156cb9d1860ba1ec36a04</t>
+          <t>e0fe1f3069e7bd647d5729169c7f51a5fabb84f8</t>
         </is>
       </c>
     </row>
@@ -11920,12 +11922,12 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>Cutting Room, Bedminster</t>
+          <t>Flat 109, Invicta, Millennium Promenade, Bristol, Bristol, City of, BS1</t>
         </is>
       </c>
       <c r="H149" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I149" s="7" t="n"/>
@@ -11934,7 +11936,7 @@
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="7" t="n">
-        <v>13796</v>
+        <v>16168</v>
       </c>
       <c r="O149" s="7" t="n">
         <v>0</v>
@@ -11942,12 +11944,12 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
         <is>
-          <t>Taylors Lettings, Bedminster</t>
+          <t>CJ Hole, Bishopston</t>
         </is>
       </c>
       <c r="S149" s="8" t="inlineStr"/>
@@ -11964,7 +11966,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>9c1c90149ff9e9ef3f44e220729613570307258e</t>
+          <t>f987cb39e8da7d77742156cb9d1860ba1ec36a04</t>
         </is>
       </c>
     </row>
@@ -11978,10 +11980,10 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1999</v>
+        <v>1500</v>
       </c>
       <c r="D150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E150" s="7" t="n">
         <v>1</v>
@@ -11993,12 +11995,12 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Cutting Room, Bedminster</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I150" s="7" t="n"/>
@@ -12007,7 +12009,7 @@
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>20800</v>
+        <v>13796</v>
       </c>
       <c r="O150" s="7" t="n">
         <v>0</v>
@@ -12015,12 +12017,12 @@
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Taylors Lettings, Bedminster</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12037,7 +12039,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
+          <t>9c1c90149ff9e9ef3f44e220729613570307258e</t>
         </is>
       </c>
     </row>
@@ -12051,10 +12053,10 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1250</v>
+        <v>1999</v>
       </c>
       <c r="D151" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E151" s="7" t="n">
         <v>1</v>
@@ -12066,7 +12068,7 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Victoria Street, Bristol, BS1 6DR</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr">
@@ -12080,7 +12082,7 @@
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>13612</v>
+        <v>20800</v>
       </c>
       <c r="O151" s="7" t="n">
         <v>0</v>
@@ -12088,12 +12090,12 @@
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>Visum, Nationwide</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12110,7 +12112,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
+          <t>5cec67aa8ba885c4c8f85e47d3354d187da9d897</t>
         </is>
       </c>
     </row>
@@ -12124,13 +12126,13 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1995</v>
+        <v>1250</v>
       </c>
       <c r="D152" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E152" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
@@ -12139,7 +12141,7 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>Park St, Bristol, BS1</t>
+          <t>Victoria Street, Bristol, BS1 6DR</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
@@ -12153,7 +12155,7 @@
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>20420</v>
+        <v>13612</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12161,12 +12163,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Visum, Nationwide</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12183,7 +12185,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>67c94b7f29659c2b4ec3a6c47a160e66ad16c322</t>
+          <t>78fe8e0511ccc37f104368075238c845f57d7864</t>
         </is>
       </c>
     </row>
@@ -12197,7 +12199,7 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>2300</v>
+        <v>1995</v>
       </c>
       <c r="D153" s="7" t="n">
         <v>2</v>
@@ -12212,12 +12214,12 @@
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Park St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I153" s="7" t="n"/>
@@ -12226,7 +12228,7 @@
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>14172</v>
+        <v>20420</v>
       </c>
       <c r="O153" s="7" t="n">
         <v>0</v>
@@ -12234,12 +12236,12 @@
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12256,7 +12258,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>cef9e437d00bef794aeb191d11d2926b26b03190</t>
+          <t>67c94b7f29659c2b4ec3a6c47a160e66ad16c322</t>
         </is>
       </c>
     </row>
@@ -12270,13 +12272,13 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1350</v>
+        <v>2300</v>
       </c>
       <c r="D154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
@@ -12285,7 +12287,7 @@
       </c>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>Glass Wharf, Bristol</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr">
@@ -12299,7 +12301,7 @@
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="7" t="n">
-        <v>20972</v>
+        <v>14172</v>
       </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
@@ -12307,12 +12309,12 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S154" s="8" t="inlineStr"/>
@@ -12329,7 +12331,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>58386ab060e5ad520b5bcba6592f39f1e64abdfa</t>
+          <t>cef9e437d00bef794aeb191d11d2926b26b03190</t>
         </is>
       </c>
     </row>
@@ -12343,7 +12345,7 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>1200</v>
+        <v>1350</v>
       </c>
       <c r="D155" s="7" t="n">
         <v>1</v>
@@ -12358,12 +12360,12 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Knowle Road - Totterdown</t>
+          <t>Glass Wharf, Bristol</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I155" s="7" t="n"/>
@@ -12372,7 +12374,7 @@
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="7" t="n">
-        <v>4424</v>
+        <v>20972</v>
       </c>
       <c r="O155" s="7" t="n">
         <v>0</v>
@@ -12380,12 +12382,12 @@
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12402,14 +12404,87 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
+          <t>58386ab060e5ad520b5bcba6592f39f1e64abdfa</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C156" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D156" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E156" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F156" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G156" s="8" t="inlineStr">
+        <is>
+          <t>Knowle Road - Totterdown</t>
+        </is>
+      </c>
+      <c r="H156" s="7" t="inlineStr">
+        <is>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I156" s="7" t="n"/>
+      <c r="J156" s="7" t="n"/>
+      <c r="K156" s="7" t="n"/>
+      <c r="L156" s="7" t="n"/>
+      <c r="M156" s="7" t="n"/>
+      <c r="N156" s="7" t="n">
+        <v>4424</v>
+      </c>
+      <c r="O156" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P156" s="7" t="n"/>
+      <c r="Q156" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="R156" s="7" t="inlineStr">
+        <is>
+          <t>Ocean, Southville</t>
+        </is>
+      </c>
+      <c r="S156" s="8" t="inlineStr"/>
+      <c r="T156" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V156" s="6" t="inlineStr"/>
+      <c r="W156" s="7" t="inlineStr">
+        <is>
           <t>f21962eb5746e5a8e03039ab495b2574f154a799</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W155"/>
+  <autoFilter ref="A1:W156"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12568,6 +12643,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T153" r:id="rId152"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T154" r:id="rId153"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T156" r:id="rId155"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 116
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -1976,7 +1976,7 @@
       <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="n"/>
       <c r="N17" s="7" t="n">
-        <v>13408</v>
+        <v>20780</v>
       </c>
       <c r="O17" s="7" t="n">
         <v>0</v>
@@ -2213,7 +2213,7 @@
       <c r="L20" s="7" t="n"/>
       <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n">
-        <v>13408</v>
+        <v>20780</v>
       </c>
       <c r="O20" s="7" t="n">
         <v>0</v>
@@ -5772,7 +5772,7 @@
         </is>
       </c>
       <c r="C66" s="9" t="n">
-        <v>1900</v>
+        <v>1850</v>
       </c>
       <c r="D66" s="7" t="n">
         <v>2</v>
@@ -7208,7 +7208,7 @@
       <c r="L85" s="7" t="n"/>
       <c r="M85" s="7" t="n"/>
       <c r="N85" s="7" t="n">
-        <v>13840</v>
+        <v>21476</v>
       </c>
       <c r="O85" s="7" t="n">
         <v>0</v>
@@ -7654,7 +7654,7 @@
       <c r="L91" s="7" t="n"/>
       <c r="M91" s="7" t="n"/>
       <c r="N91" s="7" t="n">
-        <v>13840</v>
+        <v>21476</v>
       </c>
       <c r="O91" s="7" t="n">
         <v>0</v>
@@ -8694,7 +8694,7 @@
       <c r="L105" s="7" t="n"/>
       <c r="M105" s="7" t="n"/>
       <c r="N105" s="7" t="n">
-        <v>13840</v>
+        <v>21476</v>
       </c>
       <c r="O105" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
House search data from run 124
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$193</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W191"/>
+  <dimension ref="A1:W193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2442,7 +2442,7 @@
       <c r="L23" s="7" t="n"/>
       <c r="M23" s="7" t="n"/>
       <c r="N23" s="7" t="n">
-        <v>20780</v>
+        <v>13408</v>
       </c>
       <c r="O23" s="7" t="n">
         <v>1</v>
@@ -9483,7 +9483,7 @@
         <v>13860</v>
       </c>
       <c r="O115" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P115" s="7" t="n"/>
       <c r="Q115" s="7" t="inlineStr">
@@ -10789,13 +10789,13 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1200</v>
+        <v>2300</v>
       </c>
       <c r="D133" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E133" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
@@ -10804,7 +10804,7 @@
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
@@ -10813,14 +10813,14 @@
         </is>
       </c>
       <c r="I133" s="7" t="n">
-        <v>517</v>
+        <v>773</v>
       </c>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>21904</v>
+        <v>14172</v>
       </c>
       <c r="O133" s="7" t="n">
         <v>1</v>
@@ -10828,12 +10828,12 @@
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S133" s="8" t="inlineStr"/>
@@ -10850,7 +10850,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>e87a39f40860abe2278117f28f53ec7cbbd1d241</t>
+          <t>7594e7db3c52acddddafbbdb135025e4f15aa52c</t>
         </is>
       </c>
     </row>
@@ -10864,7 +10864,7 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>1630</v>
+        <v>1150</v>
       </c>
       <c r="D134" s="7" t="n">
         <v>1</v>
@@ -10879,36 +10879,34 @@
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I134" s="7" t="n">
-        <v>486</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I134" s="7" t="n"/>
       <c r="J134" s="7" t="n"/>
       <c r="K134" s="7" t="n"/>
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="7" t="n">
-        <v>13860</v>
+        <v>15376</v>
       </c>
       <c r="O134" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10925,7 +10923,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
+          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
         </is>
       </c>
     </row>
@@ -10939,7 +10937,7 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1640</v>
+        <v>1200</v>
       </c>
       <c r="D135" s="7" t="n">
         <v>1</v>
@@ -10954,36 +10952,36 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I135" s="7" t="n">
-        <v>487</v>
+        <v>517</v>
       </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="7" t="n">
-        <v>13356</v>
+        <v>21904</v>
       </c>
       <c r="O135" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S135" s="8" t="inlineStr"/>
@@ -11000,7 +10998,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>ecc803f25866be367a83778bda0456688426a26e</t>
+          <t>e87a39f40860abe2278117f28f53ec7cbbd1d241</t>
         </is>
       </c>
     </row>
@@ -11014,13 +11012,13 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>2085</v>
+        <v>1630</v>
       </c>
       <c r="D136" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E136" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
@@ -11038,7 +11036,7 @@
         </is>
       </c>
       <c r="I136" s="7" t="n">
-        <v>722</v>
+        <v>486</v>
       </c>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
@@ -11053,7 +11051,7 @@
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
@@ -11075,7 +11073,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
+          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
         </is>
       </c>
     </row>
@@ -11089,7 +11087,7 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1650</v>
+        <v>1640</v>
       </c>
       <c r="D137" s="7" t="n">
         <v>1</v>
@@ -11113,7 +11111,7 @@
         </is>
       </c>
       <c r="I137" s="7" t="n">
-        <v>553</v>
+        <v>487</v>
       </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
@@ -11128,7 +11126,7 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
@@ -11150,7 +11148,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
+          <t>ecc803f25866be367a83778bda0456688426a26e</t>
         </is>
       </c>
     </row>
@@ -11164,13 +11162,13 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1350</v>
+        <v>2085</v>
       </c>
       <c r="D138" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E138" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
@@ -11179,7 +11177,7 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
@@ -11188,14 +11186,14 @@
         </is>
       </c>
       <c r="I138" s="7" t="n">
-        <v>518</v>
+        <v>722</v>
       </c>
       <c r="J138" s="7" t="n"/>
       <c r="K138" s="7" t="n"/>
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>16664</v>
+        <v>13860</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11203,12 +11201,12 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11225,7 +11223,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>61cb6cbca03d4b33a5e567abbe422df6574deb7a</t>
+          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
         </is>
       </c>
     </row>
@@ -11239,10 +11237,10 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>1550</v>
+        <v>1650</v>
       </c>
       <c r="D139" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E139" s="7" t="n">
         <v>1</v>
@@ -11254,21 +11252,23 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Crown And Anchor House, Temple Quay, Temple Quay, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I139" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I139" s="7" t="n">
+        <v>553</v>
+      </c>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>20472</v>
+        <v>13356</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11276,12 +11276,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11298,7 +11298,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>e76245b9d5be47e78934469ea3c31d3d0433291c</t>
+          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
         </is>
       </c>
     </row>
@@ -11312,7 +11312,7 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1665</v>
+        <v>1350</v>
       </c>
       <c r="D140" s="7" t="n">
         <v>1</v>
@@ -11327,7 +11327,7 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
@@ -11336,14 +11336,14 @@
         </is>
       </c>
       <c r="I140" s="7" t="n">
-        <v>569</v>
+        <v>518</v>
       </c>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>13356</v>
+        <v>16664</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11351,12 +11351,12 @@
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11373,7 +11373,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>22588bce8839df85d69555bd640fcbb3902101ff</t>
+          <t>61cb6cbca03d4b33a5e567abbe422df6574deb7a</t>
         </is>
       </c>
     </row>
@@ -11387,7 +11387,7 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1850</v>
+        <v>1550</v>
       </c>
       <c r="D141" s="7" t="n">
         <v>2</v>
@@ -11397,17 +11397,17 @@
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Webb Street, Bristol, BS5</t>
+          <t>Crown And Anchor House, Temple Quay, Temple Quay, BS2</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I141" s="7" t="n"/>
@@ -11416,7 +11416,7 @@
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>19580</v>
+        <v>20472</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11424,12 +11424,12 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11446,7 +11446,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
+          <t>e76245b9d5be47e78934469ea3c31d3d0433291c</t>
         </is>
       </c>
     </row>
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>1200</v>
+        <v>1665</v>
       </c>
       <c r="D142" s="7" t="n">
         <v>1</v>
@@ -11475,21 +11475,23 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>Bushy Park, The Bank Bushy Park, BS4</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I142" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I142" s="7" t="n">
+        <v>569</v>
+      </c>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>7216</v>
+        <v>13356</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11497,12 +11499,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11519,7 +11521,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
+          <t>22588bce8839df85d69555bd640fcbb3902101ff</t>
         </is>
       </c>
     </row>
@@ -11533,27 +11535,27 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1750</v>
+        <v>1850</v>
       </c>
       <c r="D143" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E143" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Number One Bristol, Bristol</t>
+          <t>Webb Street, Bristol, BS5</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I143" s="7" t="n"/>
@@ -11562,7 +11564,7 @@
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>21808</v>
+        <v>19580</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11570,12 +11572,12 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>Zest, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11592,7 +11594,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>d2b416547517343eef3a43500d63f738ac4ae423</t>
+          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
         </is>
       </c>
     </row>
@@ -11606,7 +11608,7 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1295</v>
+        <v>1200</v>
       </c>
       <c r="D144" s="7" t="n">
         <v>1</v>
@@ -11621,23 +11623,21 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Great Western House, BS1</t>
+          <t>Bushy Park, The Bank Bushy Park, BS4</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I144" s="7" t="n">
-        <v>474</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I144" s="7" t="n"/>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>14412</v>
+        <v>7216</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11645,12 +11645,12 @@
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11667,7 +11667,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>466dad45b709c8ce2ab5e9d022bce4baabb5cecc</t>
+          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
         </is>
       </c>
     </row>
@@ -11681,13 +11681,13 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>1325</v>
+        <v>1750</v>
       </c>
       <c r="D145" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E145" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
@@ -11696,7 +11696,7 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>Broad Street, Bristol, BS1</t>
+          <t>Number One Bristol, Bristol</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
@@ -11710,7 +11710,7 @@
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>21788</v>
+        <v>21808</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11718,12 +11718,12 @@
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Zest, Bristol</t>
         </is>
       </c>
       <c r="S145" s="8" t="inlineStr"/>
@@ -11740,7 +11740,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
+          <t>d2b416547517343eef3a43500d63f738ac4ae423</t>
         </is>
       </c>
     </row>
@@ -11754,13 +11754,13 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>2200</v>
+        <v>1295</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E146" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
@@ -11769,7 +11769,7 @@
       </c>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
+          <t>Harbourside, Great Western House, BS1</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
@@ -11777,13 +11777,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I146" s="7" t="n"/>
+      <c r="I146" s="7" t="n">
+        <v>474</v>
+      </c>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>16788</v>
+        <v>14412</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>0</v>
@@ -11791,12 +11793,12 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S146" s="8" t="inlineStr"/>
@@ -11813,7 +11815,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
+          <t>466dad45b709c8ce2ab5e9d022bce4baabb5cecc</t>
         </is>
       </c>
     </row>
@@ -11827,7 +11829,7 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>1500</v>
+        <v>1325</v>
       </c>
       <c r="D147" s="7" t="n">
         <v>1</v>
@@ -11842,7 +11844,7 @@
       </c>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>Eclipse, Broad Weir, Bristol</t>
+          <t>Broad Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H147" s="7" t="inlineStr">
@@ -11856,7 +11858,7 @@
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="7" t="n">
-        <v>22164</v>
+        <v>21788</v>
       </c>
       <c r="O147" s="7" t="n">
         <v>0</v>
@@ -11864,12 +11866,12 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>Martin &amp; Co, Bath</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S147" s="8" t="inlineStr"/>
@@ -11886,7 +11888,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
+          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
         </is>
       </c>
     </row>
@@ -11900,13 +11902,13 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>1800</v>
+        <v>2200</v>
       </c>
       <c r="D148" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E148" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
@@ -11915,7 +11917,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Broad Weir, City Centre, Bristol, BS1</t>
+          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
@@ -11923,15 +11925,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I148" s="7" t="n">
-        <v>474</v>
-      </c>
+      <c r="I148" s="7" t="n"/>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>22080</v>
+        <v>16788</v>
       </c>
       <c r="O148" s="7" t="n">
         <v>0</v>
@@ -11939,12 +11939,12 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Clifton</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11961,7 +11961,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
+          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
         </is>
       </c>
     </row>
@@ -11975,7 +11975,7 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>1300</v>
+        <v>1500</v>
       </c>
       <c r="D149" s="7" t="n">
         <v>1</v>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Deanery Road, BS1 5AF</t>
+          <t>Eclipse, Broad Weir, Bristol</t>
         </is>
       </c>
       <c r="H149" s="7" t="inlineStr">
@@ -11998,15 +11998,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I149" s="7" t="n">
-        <v>570</v>
-      </c>
+      <c r="I149" s="7" t="n"/>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="7" t="n">
-        <v>19300</v>
+        <v>22164</v>
       </c>
       <c r="O149" s="7" t="n">
         <v>0</v>
@@ -12014,12 +12012,12 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Martin &amp; Co, Bath</t>
         </is>
       </c>
       <c r="S149" s="8" t="inlineStr"/>
@@ -12036,7 +12034,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
+          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
         </is>
       </c>
     </row>
@@ -12050,13 +12048,13 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="D150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
@@ -12065,21 +12063,23 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>Broad Weir, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I150" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I150" s="7" t="n">
+        <v>474</v>
+      </c>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>21360</v>
+        <v>22080</v>
       </c>
       <c r="O150" s="7" t="n">
         <v>0</v>
@@ -12087,12 +12087,12 @@
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12109,7 +12109,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
+          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
         </is>
       </c>
     </row>
@@ -12123,10 +12123,10 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1650</v>
+        <v>1300</v>
       </c>
       <c r="D151" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E151" s="7" t="n">
         <v>1</v>
@@ -12138,21 +12138,23 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Crown &amp; Anchor House, Bristol, BS2</t>
+          <t>City Centre, Deanery Road, BS1 5AF</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I151" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I151" s="7" t="n">
+        <v>570</v>
+      </c>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>20472</v>
+        <v>19300</v>
       </c>
       <c r="O151" s="7" t="n">
         <v>0</v>
@@ -12160,12 +12162,12 @@
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12182,7 +12184,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
+          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
         </is>
       </c>
     </row>
@@ -12196,10 +12198,10 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1450</v>
+        <v>2500</v>
       </c>
       <c r="D152" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E152" s="7" t="n">
         <v>2</v>
@@ -12211,23 +12213,21 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>Woodbridge Road, Bristol, BS4</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I152" s="7" t="n">
-        <v>678</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I152" s="7" t="n"/>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>5700</v>
+        <v>21360</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12235,12 +12235,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12257,7 +12257,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
+          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
         </is>
       </c>
     </row>
@@ -12271,12 +12271,14 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>1450</v>
+        <v>1650</v>
       </c>
       <c r="D153" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E153" s="7" t="n"/>
+      <c r="E153" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -12284,12 +12286,12 @@
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Crown &amp; Anchor House, Bristol, BS2</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I153" s="7" t="n"/>
@@ -12298,20 +12300,20 @@
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>19488</v>
+        <v>20472</v>
       </c>
       <c r="O153" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12328,7 +12330,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
+          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
         </is>
       </c>
     </row>
@@ -12342,13 +12344,13 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1500</v>
+        <v>1450</v>
       </c>
       <c r="D154" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
@@ -12357,21 +12359,23 @@
       </c>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Woodbridge Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I154" s="7" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I154" s="7" t="n">
+        <v>678</v>
+      </c>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="7" t="n">
-        <v>20768</v>
+        <v>5700</v>
       </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
@@ -12379,12 +12383,12 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S154" s="8" t="inlineStr"/>
@@ -12401,7 +12405,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
+          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
         </is>
       </c>
     </row>
@@ -12415,51 +12419,47 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>2250</v>
+        <v>1450</v>
       </c>
       <c r="D155" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E155" s="7" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E155" s="7" t="n"/>
       <c r="F155" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Newfoundland Road, Bristol, BS2</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I155" s="7" t="n">
-        <v>980</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I155" s="7" t="n"/>
       <c r="J155" s="7" t="n"/>
       <c r="K155" s="7" t="n"/>
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="7" t="n">
-        <v>19800</v>
+        <v>19488</v>
       </c>
       <c r="O155" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>Lets Rent Bristol, Bristol</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12476,7 +12476,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
+          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
         </is>
       </c>
     </row>
@@ -12490,13 +12490,13 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D156" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E156" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F156" s="7" t="inlineStr">
         <is>
@@ -12505,7 +12505,7 @@
       </c>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>Protheroes House, Hobbs Lane, BS1</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr">
@@ -12519,7 +12519,7 @@
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="7" t="n">
-        <v>13584</v>
+        <v>20768</v>
       </c>
       <c r="O156" s="7" t="n">
         <v>0</v>
@@ -12527,12 +12527,12 @@
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S156" s="8" t="inlineStr"/>
@@ -12549,7 +12549,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
+          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
         </is>
       </c>
     </row>
@@ -12563,13 +12563,13 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>2400</v>
+        <v>2250</v>
       </c>
       <c r="D157" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E157" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
@@ -12578,21 +12578,23 @@
       </c>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>Balmain Street, Totterdown, Bristol, BS4</t>
+          <t>Newfoundland Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H157" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I157" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I157" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="7" t="n">
-        <v>5524</v>
+        <v>19800</v>
       </c>
       <c r="O157" s="7" t="n">
         <v>0</v>
@@ -12600,12 +12602,12 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Lets Rent Bristol, Bristol</t>
         </is>
       </c>
       <c r="S157" s="8" t="inlineStr"/>
@@ -12622,7 +12624,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>dd411af39a083f886127138c0a969254da83858b</t>
+          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
         </is>
       </c>
     </row>
@@ -12636,13 +12638,13 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>1665</v>
+        <v>2000</v>
       </c>
       <c r="D158" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E158" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F158" s="7" t="inlineStr">
         <is>
@@ -12651,7 +12653,7 @@
       </c>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Protheroes House, Hobbs Lane, BS1</t>
         </is>
       </c>
       <c r="H158" s="7" t="inlineStr">
@@ -12659,28 +12661,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I158" s="7" t="n">
-        <v>578</v>
-      </c>
+      <c r="I158" s="7" t="n"/>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>13356</v>
+        <v>13584</v>
       </c>
       <c r="O158" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S158" s="8" t="inlineStr"/>
@@ -12697,7 +12697,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
+          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
         </is>
       </c>
     </row>
@@ -12711,51 +12711,49 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1635</v>
+        <v>2400</v>
       </c>
       <c r="D159" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E159" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F159" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Balmain Street, Totterdown, Bristol, BS4</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I159" s="7" t="n">
-        <v>485</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I159" s="7" t="n"/>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="7" t="n">
-        <v>13860</v>
+        <v>5524</v>
       </c>
       <c r="O159" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12772,7 +12770,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
+          <t>dd411af39a083f886127138c0a969254da83858b</t>
         </is>
       </c>
     </row>
@@ -12786,7 +12784,7 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>1615</v>
+        <v>1665</v>
       </c>
       <c r="D160" s="7" t="n">
         <v>1</v>
@@ -12801,7 +12799,7 @@
       </c>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H160" s="7" t="inlineStr">
@@ -12810,14 +12808,14 @@
         </is>
       </c>
       <c r="I160" s="7" t="n">
-        <v>487</v>
+        <v>578</v>
       </c>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
       <c r="N160" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O160" s="7" t="n">
         <v>1</v>
@@ -12825,12 +12823,12 @@
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S160" s="8" t="inlineStr"/>
@@ -12847,7 +12845,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
+          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
         </is>
       </c>
     </row>
@@ -12861,7 +12859,7 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>1640</v>
+        <v>1635</v>
       </c>
       <c r="D161" s="7" t="n">
         <v>1</v>
@@ -12876,7 +12874,7 @@
       </c>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H161" s="7" t="inlineStr">
@@ -12885,14 +12883,14 @@
         </is>
       </c>
       <c r="I161" s="7" t="n">
-        <v>560</v>
+        <v>485</v>
       </c>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
       <c r="N161" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O161" s="7" t="n">
         <v>1</v>
@@ -12900,12 +12898,12 @@
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S161" s="8" t="inlineStr"/>
@@ -12922,7 +12920,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
+          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
         </is>
       </c>
     </row>
@@ -12960,7 +12958,7 @@
         </is>
       </c>
       <c r="I162" s="7" t="n">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
@@ -12975,7 +12973,7 @@
       <c r="P162" s="7" t="n"/>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
@@ -12997,7 +12995,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
+          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
         </is>
       </c>
     </row>
@@ -13011,7 +13009,7 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1615</v>
+        <v>1640</v>
       </c>
       <c r="D163" s="7" t="n">
         <v>1</v>
@@ -13026,7 +13024,7 @@
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
@@ -13035,27 +13033,27 @@
         </is>
       </c>
       <c r="I163" s="7" t="n">
-        <v>486</v>
+        <v>560</v>
       </c>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O163" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13072,7 +13070,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
+          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
         </is>
       </c>
     </row>
@@ -13086,7 +13084,7 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>1645</v>
+        <v>1615</v>
       </c>
       <c r="D164" s="7" t="n">
         <v>1</v>
@@ -13101,7 +13099,7 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
@@ -13110,27 +13108,27 @@
         </is>
       </c>
       <c r="I164" s="7" t="n">
-        <v>570</v>
+        <v>484</v>
       </c>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O164" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13147,7 +13145,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
+          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
         </is>
       </c>
     </row>
@@ -13161,7 +13159,7 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1630</v>
+        <v>1615</v>
       </c>
       <c r="D165" s="7" t="n">
         <v>1</v>
@@ -13176,7 +13174,7 @@
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H165" s="7" t="inlineStr">
@@ -13185,14 +13183,14 @@
         </is>
       </c>
       <c r="I165" s="7" t="n">
-        <v>560</v>
+        <v>486</v>
       </c>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O165" s="7" t="n">
         <v>0</v>
@@ -13200,12 +13198,12 @@
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R165" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S165" s="8" t="inlineStr"/>
@@ -13222,7 +13220,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
+          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
         </is>
       </c>
     </row>
@@ -13236,10 +13234,10 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>1800</v>
+        <v>1645</v>
       </c>
       <c r="D166" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E166" s="7" t="n">
         <v>1</v>
@@ -13251,7 +13249,7 @@
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H166" s="7" t="inlineStr">
@@ -13259,13 +13257,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I166" s="7" t="n"/>
+      <c r="I166" s="7" t="n">
+        <v>570</v>
+      </c>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="7" t="n">
-        <v>21176</v>
+        <v>13356</v>
       </c>
       <c r="O166" s="7" t="n">
         <v>0</v>
@@ -13273,12 +13273,12 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
@@ -13295,7 +13295,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
+          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
         </is>
       </c>
     </row>
@@ -13309,7 +13309,7 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>1635</v>
+        <v>1630</v>
       </c>
       <c r="D167" s="7" t="n">
         <v>1</v>
@@ -13333,7 +13333,7 @@
         </is>
       </c>
       <c r="I167" s="7" t="n">
-        <v>569</v>
+        <v>560</v>
       </c>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
@@ -13348,7 +13348,7 @@
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
@@ -13370,7 +13370,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
+          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
         </is>
       </c>
     </row>
@@ -13384,7 +13384,7 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1925</v>
+        <v>1800</v>
       </c>
       <c r="D168" s="7" t="n">
         <v>2</v>
@@ -13399,7 +13399,7 @@
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
@@ -13407,15 +13407,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I168" s="7" t="n">
-        <v>655</v>
-      </c>
+      <c r="I168" s="7" t="n"/>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="7" t="n">
-        <v>21476</v>
+        <v>21176</v>
       </c>
       <c r="O168" s="7" t="n">
         <v>0</v>
@@ -13423,12 +13421,12 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13445,7 +13443,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>892dd053ae3538c7c123f255e926bef984caf6de</t>
+          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
         </is>
       </c>
     </row>
@@ -13459,13 +13457,13 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1800</v>
+        <v>1635</v>
       </c>
       <c r="D169" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E169" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
@@ -13474,7 +13472,7 @@
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Park St, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
@@ -13482,13 +13480,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I169" s="7" t="n"/>
+      <c r="I169" s="7" t="n">
+        <v>569</v>
+      </c>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>20644</v>
+        <v>13356</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13496,12 +13496,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13518,7 +13518,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>8e49447f07b7d2adcefccb79294af764ba54db50</t>
+          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
         </is>
       </c>
     </row>
@@ -13532,10 +13532,10 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>1650</v>
+        <v>1925</v>
       </c>
       <c r="D170" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E170" s="7" t="n">
         <v>1</v>
@@ -13547,7 +13547,7 @@
       </c>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t>Marsh House, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H170" s="7" t="inlineStr">
@@ -13555,13 +13555,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I170" s="7" t="n"/>
+      <c r="I170" s="7" t="n">
+        <v>655</v>
+      </c>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
       <c r="L170" s="7" t="n"/>
       <c r="M170" s="7" t="n"/>
       <c r="N170" s="7" t="n">
-        <v>20952</v>
+        <v>21476</v>
       </c>
       <c r="O170" s="7" t="n">
         <v>0</v>
@@ -13569,12 +13571,12 @@
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -13591,7 +13593,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>dc8b7c88d86188af3ee5262a5f1215944eb3e402</t>
+          <t>892dd053ae3538c7c123f255e926bef984caf6de</t>
         </is>
       </c>
     </row>
@@ -13611,7 +13613,7 @@
         <v>2</v>
       </c>
       <c r="E171" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F171" s="7" t="inlineStr">
         <is>
@@ -13620,7 +13622,7 @@
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Park St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H171" s="7" t="inlineStr">
@@ -13634,7 +13636,7 @@
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="7" t="n">
-        <v>20592</v>
+        <v>20644</v>
       </c>
       <c r="O171" s="7" t="n">
         <v>0</v>
@@ -13642,7 +13644,7 @@
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
@@ -13664,7 +13666,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>7aa830b20d3fe9e9350b37a53ede99615caa3290</t>
+          <t>8e49447f07b7d2adcefccb79294af764ba54db50</t>
         </is>
       </c>
     </row>
@@ -13678,7 +13680,7 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1350</v>
+        <v>1650</v>
       </c>
       <c r="D172" s="7" t="n">
         <v>1</v>
@@ -13693,7 +13695,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>Marsh House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H172" s="7" t="inlineStr">
@@ -13701,15 +13703,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I172" s="7" t="n">
-        <v>518</v>
-      </c>
+      <c r="I172" s="7" t="n"/>
       <c r="J172" s="7" t="n"/>
       <c r="K172" s="7" t="n"/>
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="7" t="n">
-        <v>16416</v>
+        <v>20952</v>
       </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
@@ -13717,12 +13717,12 @@
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -13739,7 +13739,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>77b9e2d97ea9d3f764e1fbd2fdd0b5bf1d5b75b8</t>
+          <t>dc8b7c88d86188af3ee5262a5f1215944eb3e402</t>
         </is>
       </c>
     </row>
@@ -13753,10 +13753,10 @@
         </is>
       </c>
       <c r="C173" s="9" t="n">
-        <v>1450</v>
+        <v>1800</v>
       </c>
       <c r="D173" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E173" s="7" t="n">
         <v>1</v>
@@ -13768,7 +13768,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
@@ -13782,7 +13782,7 @@
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>20524</v>
+        <v>20592</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13790,7 +13790,7 @@
       <c r="P173" s="7" t="n"/>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
@@ -13812,7 +13812,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>adbd7c1c798d9f667bce5c8c0d31831cec0ebf67</t>
+          <t>7aa830b20d3fe9e9350b37a53ede99615caa3290</t>
         </is>
       </c>
     </row>
@@ -13826,10 +13826,10 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1500</v>
+        <v>1350</v>
       </c>
       <c r="D174" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E174" s="7" t="n">
         <v>1</v>
@@ -13841,21 +13841,23 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>The Quadrant, Bristol, BS2</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I174" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I174" s="7" t="n">
+        <v>518</v>
+      </c>
       <c r="J174" s="7" t="n"/>
       <c r="K174" s="7" t="n"/>
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>20056</v>
+        <v>16416</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13863,12 +13865,12 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -13885,7 +13887,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>c77814f9166c93a32f4a1ce46b46c87a68a6196a</t>
+          <t>77b9e2d97ea9d3f764e1fbd2fdd0b5bf1d5b75b8</t>
         </is>
       </c>
     </row>
@@ -13899,13 +13901,13 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>1800</v>
+        <v>1450</v>
       </c>
       <c r="D175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
@@ -13914,7 +13916,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
@@ -13928,15 +13930,15 @@
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
       <c r="N175" s="7" t="n">
-        <v>21020</v>
+        <v>20524</v>
       </c>
       <c r="O175" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
@@ -13958,7 +13960,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>9fe5cc28570329e8d733373bcf933c665273bc0e</t>
+          <t>adbd7c1c798d9f667bce5c8c0d31831cec0ebf67</t>
         </is>
       </c>
     </row>
@@ -13972,10 +13974,10 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>1250</v>
+        <v>1500</v>
       </c>
       <c r="D176" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E176" s="7" t="n">
         <v>1</v>
@@ -13987,36 +13989,34 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Jessop Court, BS1</t>
+          <t>The Quadrant, Bristol, BS2</t>
         </is>
       </c>
       <c r="H176" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I176" s="7" t="n">
-        <v>538</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I176" s="7" t="n"/>
       <c r="J176" s="7" t="n"/>
       <c r="K176" s="7" t="n"/>
       <c r="L176" s="7" t="n"/>
       <c r="M176" s="7" t="n"/>
       <c r="N176" s="7" t="n">
-        <v>20788</v>
+        <v>20056</v>
       </c>
       <c r="O176" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -14033,7 +14033,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>34093b6e05a2deb3da2e1a98a249e966d7af0cdf</t>
+          <t>c77814f9166c93a32f4a1ce46b46c87a68a6196a</t>
         </is>
       </c>
     </row>
@@ -14047,13 +14047,13 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>1250</v>
+        <v>1800</v>
       </c>
       <c r="D177" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E177" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F177" s="7" t="inlineStr">
         <is>
@@ -14062,7 +14062,7 @@
       </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>St. Stephens Street, Bristol, BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H177" s="7" t="inlineStr">
@@ -14076,7 +14076,7 @@
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
       <c r="N177" s="7" t="n">
-        <v>13940</v>
+        <v>21020</v>
       </c>
       <c r="O177" s="7" t="n">
         <v>1</v>
@@ -14084,12 +14084,12 @@
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S177" s="8" t="inlineStr"/>
@@ -14106,7 +14106,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>705e73e870fdf398639d5c8b181c8e21b143f622</t>
+          <t>9fe5cc28570329e8d733373bcf933c665273bc0e</t>
         </is>
       </c>
     </row>
@@ -14120,7 +14120,7 @@
         </is>
       </c>
       <c r="C178" s="9" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
       <c r="D178" s="7" t="n">
         <v>1</v>
@@ -14135,21 +14135,23 @@
       </c>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t>Cutting Room, Bristol, BS3</t>
+          <t>City Centre, Jessop Court, BS1</t>
         </is>
       </c>
       <c r="H178" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I178" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I178" s="7" t="n">
+        <v>538</v>
+      </c>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
       <c r="L178" s="7" t="n"/>
       <c r="M178" s="7" t="n"/>
       <c r="N178" s="7" t="n">
-        <v>13836</v>
+        <v>20788</v>
       </c>
       <c r="O178" s="7" t="n">
         <v>1</v>
@@ -14157,12 +14159,12 @@
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Southville</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S178" s="8" t="inlineStr"/>
@@ -14179,7 +14181,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>8bb5fbce4e6d80f79ecceb7d5bb4f35766fbb83c</t>
+          <t>34093b6e05a2deb3da2e1a98a249e966d7af0cdf</t>
         </is>
       </c>
     </row>
@@ -14193,7 +14195,7 @@
         </is>
       </c>
       <c r="C179" s="9" t="n">
-        <v>1650</v>
+        <v>1250</v>
       </c>
       <c r="D179" s="7" t="n">
         <v>1</v>
@@ -14208,7 +14210,7 @@
       </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>St. Stephens Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H179" s="7" t="inlineStr">
@@ -14216,28 +14218,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I179" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I179" s="7" t="n"/>
       <c r="J179" s="7" t="n"/>
       <c r="K179" s="7" t="n"/>
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
       <c r="N179" s="7" t="n">
-        <v>13860</v>
+        <v>13940</v>
       </c>
       <c r="O179" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -14254,7 +14254,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>e26a5dedfb7c4bcd1308250a8955318f00994505</t>
+          <t>705e73e870fdf398639d5c8b181c8e21b143f622</t>
         </is>
       </c>
     </row>
@@ -14268,13 +14268,13 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>2240</v>
+        <v>1500</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E180" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F180" s="7" t="inlineStr">
         <is>
@@ -14283,36 +14283,34 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Cutting Room, Bristol, BS3</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I180" s="7" t="n">
-        <v>884</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I180" s="7" t="n"/>
       <c r="J180" s="7" t="n"/>
       <c r="K180" s="7" t="n"/>
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="7" t="n">
-        <v>13388</v>
+        <v>13836</v>
       </c>
       <c r="O180" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14329,7 +14327,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>0b2cd6178fe0f6128804b82d5b9e39ea5967f124</t>
+          <t>8bb5fbce4e6d80f79ecceb7d5bb4f35766fbb83c</t>
         </is>
       </c>
     </row>
@@ -14358,7 +14356,7 @@
       </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H181" s="7" t="inlineStr">
@@ -14367,14 +14365,14 @@
         </is>
       </c>
       <c r="I181" s="7" t="n">
-        <v>553</v>
+        <v>486</v>
       </c>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O181" s="7" t="n">
         <v>0</v>
@@ -14382,12 +14380,12 @@
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S181" s="8" t="inlineStr"/>
@@ -14404,7 +14402,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>d6bb31b3e903e1ec64e3eea9a96c3b08bb9873e3</t>
+          <t>e26a5dedfb7c4bcd1308250a8955318f00994505</t>
         </is>
       </c>
     </row>
@@ -14418,13 +14416,13 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>1640</v>
+        <v>2240</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
@@ -14433,7 +14431,7 @@
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
@@ -14442,14 +14440,14 @@
         </is>
       </c>
       <c r="I182" s="7" t="n">
-        <v>485</v>
+        <v>884</v>
       </c>
       <c r="J182" s="7" t="n"/>
       <c r="K182" s="7" t="n"/>
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>13860</v>
+        <v>13388</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14457,12 +14455,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14479,7 +14477,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>47301f8a472393cf4550a7380ee71363e6337581</t>
+          <t>0b2cd6178fe0f6128804b82d5b9e39ea5967f124</t>
         </is>
       </c>
     </row>
@@ -14493,7 +14491,7 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>1660</v>
+        <v>1650</v>
       </c>
       <c r="D183" s="7" t="n">
         <v>1</v>
@@ -14517,7 +14515,7 @@
         </is>
       </c>
       <c r="I183" s="7" t="n">
-        <v>578</v>
+        <v>553</v>
       </c>
       <c r="J183" s="7" t="n"/>
       <c r="K183" s="7" t="n"/>
@@ -14532,7 +14530,7 @@
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">
@@ -14554,7 +14552,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>5f45fddd60a4f7306d53e1880e39147d0065c173</t>
+          <t>d6bb31b3e903e1ec64e3eea9a96c3b08bb9873e3</t>
         </is>
       </c>
     </row>
@@ -14568,7 +14566,7 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>1630</v>
+        <v>1640</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>1</v>
@@ -14592,7 +14590,7 @@
         </is>
       </c>
       <c r="I184" s="7" t="n">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="J184" s="7" t="n"/>
       <c r="K184" s="7" t="n"/>
@@ -14607,7 +14605,7 @@
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
@@ -14629,7 +14627,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>91d51985531a7953cdf1bb0173d032c892f5c019</t>
+          <t>47301f8a472393cf4550a7380ee71363e6337581</t>
         </is>
       </c>
     </row>
@@ -14643,7 +14641,7 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>1585</v>
+        <v>1660</v>
       </c>
       <c r="D185" s="7" t="n">
         <v>1</v>
@@ -14658,7 +14656,7 @@
       </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
@@ -14667,14 +14665,14 @@
         </is>
       </c>
       <c r="I185" s="7" t="n">
-        <v>505</v>
+        <v>578</v>
       </c>
       <c r="J185" s="7" t="n"/>
       <c r="K185" s="7" t="n"/>
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="7" t="n">
-        <v>13964</v>
+        <v>13356</v>
       </c>
       <c r="O185" s="7" t="n">
         <v>0</v>
@@ -14682,12 +14680,12 @@
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S185" s="8" t="inlineStr"/>
@@ -14704,7 +14702,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>4fc7c891593aa7586ebede2a12c2a9af8edbe973</t>
+          <t>5f45fddd60a4f7306d53e1880e39147d0065c173</t>
         </is>
       </c>
     </row>
@@ -14718,7 +14716,7 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>1890</v>
+        <v>1630</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>1</v>
@@ -14733,7 +14731,7 @@
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
@@ -14742,14 +14740,14 @@
         </is>
       </c>
       <c r="I186" s="7" t="n">
-        <v>538</v>
+        <v>486</v>
       </c>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O186" s="7" t="n">
         <v>0</v>
@@ -14757,12 +14755,12 @@
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14779,7 +14777,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>f819b6d7cea8e4f9f3bc624d2737801ca68a6b49</t>
+          <t>91d51985531a7953cdf1bb0173d032c892f5c019</t>
         </is>
       </c>
     </row>
@@ -14793,7 +14791,7 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>1510</v>
+        <v>1585</v>
       </c>
       <c r="D187" s="7" t="n">
         <v>1</v>
@@ -14817,14 +14815,14 @@
         </is>
       </c>
       <c r="I187" s="7" t="n">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>21476</v>
+        <v>13964</v>
       </c>
       <c r="O187" s="7" t="n">
         <v>0</v>
@@ -14832,7 +14830,7 @@
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="R187" s="7" t="inlineStr">
@@ -14854,7 +14852,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>3ebe55674c01ebb6e152801ec69490ad7da0c8cc</t>
+          <t>4fc7c891593aa7586ebede2a12c2a9af8edbe973</t>
         </is>
       </c>
     </row>
@@ -14868,10 +14866,10 @@
         </is>
       </c>
       <c r="C188" s="9" t="n">
-        <v>2100</v>
+        <v>1890</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E188" s="7" t="n">
         <v>1</v>
@@ -14883,21 +14881,23 @@
       </c>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t>Old Market Street, St Philips, Bristol, Bristol City, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I188" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I188" s="7" t="n">
+        <v>538</v>
+      </c>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
       <c r="L188" s="7" t="n"/>
       <c r="M188" s="7" t="n"/>
       <c r="N188" s="7" t="n">
-        <v>13716</v>
+        <v>13356</v>
       </c>
       <c r="O188" s="7" t="n">
         <v>0</v>
@@ -14905,12 +14905,12 @@
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
         <is>
-          <t>Yours Link Limited, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S188" s="8" t="inlineStr"/>
@@ -14927,7 +14927,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>2328edfeefd3149329151e5048af6234618528dc</t>
+          <t>f819b6d7cea8e4f9f3bc624d2737801ca68a6b49</t>
         </is>
       </c>
     </row>
@@ -14941,7 +14941,7 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>1400</v>
+        <v>1510</v>
       </c>
       <c r="D189" s="7" t="n">
         <v>1</v>
@@ -14956,7 +14956,7 @@
       </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol City Centre, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
@@ -14964,13 +14964,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I189" s="7" t="n"/>
+      <c r="I189" s="7" t="n">
+        <v>509</v>
+      </c>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
       <c r="L189" s="7" t="n"/>
       <c r="M189" s="7" t="n"/>
       <c r="N189" s="7" t="n">
-        <v>13404</v>
+        <v>21476</v>
       </c>
       <c r="O189" s="7" t="n">
         <v>0</v>
@@ -14978,12 +14980,12 @@
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R189" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S189" s="8" t="inlineStr"/>
@@ -15000,7 +15002,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>80ae63ab944f6cd80f590015e53caffc4c3b1f4f</t>
+          <t>3ebe55674c01ebb6e152801ec69490ad7da0c8cc</t>
         </is>
       </c>
     </row>
@@ -15014,10 +15016,10 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>1350</v>
+        <v>2100</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E190" s="7" t="n">
         <v>1</v>
@@ -15029,23 +15031,21 @@
       </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>Finzels Reach, Castle Wharf, BS1 6JU</t>
+          <t>Old Market Street, St Philips, Bristol, Bristol City, BS2</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I190" s="7" t="n">
-        <v>603</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I190" s="7" t="n"/>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="7" t="n">
-        <v>14052</v>
+        <v>13716</v>
       </c>
       <c r="O190" s="7" t="n">
         <v>0</v>
@@ -15053,12 +15053,12 @@
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Yours Link Limited, London</t>
         </is>
       </c>
       <c r="S190" s="8" t="inlineStr"/>
@@ -15075,7 +15075,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>f635c3d4727470f01fd1777da4ca6eea453c6655</t>
+          <t>2328edfeefd3149329151e5048af6234618528dc</t>
         </is>
       </c>
     </row>
@@ -15104,7 +15104,7 @@
       </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Central Quay North, Bristol City Centre, BS1</t>
         </is>
       </c>
       <c r="H191" s="7" t="inlineStr">
@@ -15118,7 +15118,7 @@
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
       <c r="N191" s="7" t="n">
-        <v>16580</v>
+        <v>13404</v>
       </c>
       <c r="O191" s="7" t="n">
         <v>0</v>
@@ -15126,12 +15126,12 @@
       <c r="P191" s="7" t="n"/>
       <c r="Q191" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R191" s="7" t="inlineStr">
         <is>
-          <t>Romans, Clifton</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S191" s="8" t="inlineStr"/>
@@ -15148,14 +15148,162 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
+          <t>80ae63ab944f6cd80f590015e53caffc4c3b1f4f</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B192" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C192" s="9" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F192" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G192" s="8" t="inlineStr">
+        <is>
+          <t>Finzels Reach, Castle Wharf, BS1 6JU</t>
+        </is>
+      </c>
+      <c r="H192" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I192" s="7" t="n">
+        <v>603</v>
+      </c>
+      <c r="J192" s="7" t="n"/>
+      <c r="K192" s="7" t="n"/>
+      <c r="L192" s="7" t="n"/>
+      <c r="M192" s="7" t="n"/>
+      <c r="N192" s="7" t="n">
+        <v>14052</v>
+      </c>
+      <c r="O192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P192" s="7" t="n"/>
+      <c r="Q192" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="R192" s="7" t="inlineStr">
+        <is>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
+        </is>
+      </c>
+      <c r="S192" s="8" t="inlineStr"/>
+      <c r="T192" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V192" s="6" t="inlineStr"/>
+      <c r="W192" s="7" t="inlineStr">
+        <is>
+          <t>f635c3d4727470f01fd1777da4ca6eea453c6655</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B193" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C193" s="9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D193" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E193" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F193" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G193" s="8" t="inlineStr">
+        <is>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+        </is>
+      </c>
+      <c r="H193" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I193" s="7" t="n"/>
+      <c r="J193" s="7" t="n"/>
+      <c r="K193" s="7" t="n"/>
+      <c r="L193" s="7" t="n"/>
+      <c r="M193" s="7" t="n"/>
+      <c r="N193" s="7" t="n">
+        <v>16580</v>
+      </c>
+      <c r="O193" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P193" s="7" t="n"/>
+      <c r="Q193" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="R193" s="7" t="inlineStr">
+        <is>
+          <t>Romans, Clifton</t>
+        </is>
+      </c>
+      <c r="S193" s="8" t="inlineStr"/>
+      <c r="T193" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V193" s="6" t="inlineStr"/>
+      <c r="W193" s="7" t="inlineStr">
+        <is>
           <t>680172a6c9a0d74ac3232df41c01ab789bdfd3a8</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W191"/>
+  <autoFilter ref="A1:W193"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15350,6 +15498,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T189" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T190" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T193" r:id="rId192"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 132
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -963,7 +963,7 @@
       <c r="L4" s="7" t="n"/>
       <c r="M4" s="7" t="n"/>
       <c r="N4" s="7" t="n">
-        <v>16644</v>
+        <v>16664</v>
       </c>
       <c r="O4" s="7" t="n">
         <v>0</v>
@@ -2211,7 +2211,7 @@
       <c r="L20" s="7" t="n"/>
       <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n">
-        <v>20780</v>
+        <v>20924</v>
       </c>
       <c r="O20" s="7" t="n">
         <v>0</v>
@@ -2987,7 +2987,7 @@
       <c r="L30" s="7" t="n"/>
       <c r="M30" s="7" t="n"/>
       <c r="N30" s="7" t="n">
-        <v>20780</v>
+        <v>20924</v>
       </c>
       <c r="O30" s="7" t="n">
         <v>0</v>
@@ -7094,7 +7094,7 @@
       <c r="L83" s="7" t="n"/>
       <c r="M83" s="7" t="n"/>
       <c r="N83" s="7" t="n">
-        <v>21476</v>
+        <v>21740</v>
       </c>
       <c r="O83" s="7" t="n">
         <v>0</v>
@@ -7836,7 +7836,7 @@
       <c r="L93" s="7" t="n"/>
       <c r="M93" s="7" t="n"/>
       <c r="N93" s="7" t="n">
-        <v>21476</v>
+        <v>21740</v>
       </c>
       <c r="O93" s="7" t="n">
         <v>0</v>
@@ -8282,7 +8282,7 @@
       <c r="L99" s="7" t="n"/>
       <c r="M99" s="7" t="n"/>
       <c r="N99" s="7" t="n">
-        <v>16644</v>
+        <v>16664</v>
       </c>
       <c r="O99" s="7" t="n">
         <v>0</v>
@@ -8432,7 +8432,7 @@
       <c r="L101" s="7" t="n"/>
       <c r="M101" s="7" t="n"/>
       <c r="N101" s="7" t="n">
-        <v>21476</v>
+        <v>21740</v>
       </c>
       <c r="O101" s="7" t="n">
         <v>0</v>
@@ -8878,7 +8878,7 @@
       <c r="L107" s="7" t="n"/>
       <c r="M107" s="7" t="n"/>
       <c r="N107" s="7" t="n">
-        <v>21476</v>
+        <v>21740</v>
       </c>
       <c r="O107" s="7" t="n">
         <v>0</v>
@@ -9251,7 +9251,7 @@
       <c r="L112" s="7" t="n"/>
       <c r="M112" s="7" t="n"/>
       <c r="N112" s="7" t="n">
-        <v>21476</v>
+        <v>21740</v>
       </c>
       <c r="O112" s="7" t="n">
         <v>0</v>
@@ -9697,7 +9697,7 @@
       <c r="L118" s="7" t="n"/>
       <c r="M118" s="7" t="n"/>
       <c r="N118" s="7" t="n">
-        <v>21476</v>
+        <v>21740</v>
       </c>
       <c r="O118" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
House search data from run 138
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W198"/>
+  <dimension ref="A1:W199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>2695</v>
+        <v>2625</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>2</v>
@@ -3224,7 +3224,7 @@
       <c r="L33" s="7" t="n"/>
       <c r="M33" s="7" t="n"/>
       <c r="N33" s="7" t="n">
-        <v>11956</v>
+        <v>11632</v>
       </c>
       <c r="O33" s="7" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
       <c r="L34" s="7" t="n"/>
       <c r="M34" s="7" t="n"/>
       <c r="N34" s="7" t="n">
-        <v>11956</v>
+        <v>11632</v>
       </c>
       <c r="O34" s="7" t="n">
         <v>0</v>
@@ -10641,7 +10641,7 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>1395</v>
+        <v>1400</v>
       </c>
       <c r="D131" s="7" t="n">
         <v>1</v>
@@ -10656,7 +10656,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Taylors Bank, Bristol, BS1</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr">
@@ -10670,7 +10670,7 @@
       <c r="L131" s="7" t="n"/>
       <c r="M131" s="7" t="n"/>
       <c r="N131" s="7" t="n">
-        <v>20524</v>
+        <v>21996</v>
       </c>
       <c r="O131" s="7" t="n">
         <v>0</v>
@@ -10678,7 +10678,7 @@
       <c r="P131" s="7" t="n"/>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
@@ -10700,7 +10700,7 @@
       <c r="V131" s="6" t="inlineStr"/>
       <c r="W131" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>464a8221babcd58554ee30417192b0a25eacccb0</t>
         </is>
       </c>
     </row>
@@ -10714,7 +10714,7 @@
         </is>
       </c>
       <c r="C132" s="9" t="n">
-        <v>1200</v>
+        <v>1395</v>
       </c>
       <c r="D132" s="7" t="n">
         <v>1</v>
@@ -10724,28 +10724,26 @@
       </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2 0JN</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I132" s="7" t="n">
-        <v>452</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I132" s="7" t="n"/>
       <c r="J132" s="7" t="n"/>
       <c r="K132" s="7" t="n"/>
       <c r="L132" s="7" t="n"/>
       <c r="M132" s="7" t="n"/>
       <c r="N132" s="7" t="n">
-        <v>20472</v>
+        <v>20524</v>
       </c>
       <c r="O132" s="7" t="n">
         <v>0</v>
@@ -10753,12 +10751,12 @@
       <c r="P132" s="7" t="n"/>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S132" s="8" t="inlineStr"/>
@@ -10775,7 +10773,7 @@
       <c r="V132" s="6" t="inlineStr"/>
       <c r="W132" s="7" t="inlineStr">
         <is>
-          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
@@ -10789,7 +10787,7 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1450</v>
+        <v>1200</v>
       </c>
       <c r="D133" s="7" t="n">
         <v>1</v>
@@ -10799,26 +10797,28 @@
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Sweetman Place, Bristol, BS2 0JN</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I133" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I133" s="7" t="n">
+        <v>452</v>
+      </c>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>16664</v>
+        <v>20472</v>
       </c>
       <c r="O133" s="7" t="n">
         <v>0</v>
@@ -10826,12 +10826,12 @@
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S133" s="8" t="inlineStr"/>
@@ -10848,7 +10848,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
+          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
         </is>
       </c>
     </row>
@@ -10862,13 +10862,13 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>3200</v>
+        <v>1450</v>
       </c>
       <c r="D134" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E134" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
@@ -10877,7 +10877,7 @@
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
@@ -10899,12 +10899,12 @@
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>LettingaProperty.com, Nationwide - Lettings</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10921,7 +10921,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
+          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
         </is>
       </c>
     </row>
@@ -10935,13 +10935,13 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1600</v>
+        <v>3200</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
@@ -10950,7 +10950,7 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
@@ -10964,7 +10964,7 @@
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="7" t="n">
-        <v>21996</v>
+        <v>16664</v>
       </c>
       <c r="O135" s="7" t="n">
         <v>0</v>
@@ -10977,7 +10977,7 @@
       </c>
       <c r="R135" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>LettingaProperty.com, Nationwide - Lettings</t>
         </is>
       </c>
       <c r="S135" s="8" t="inlineStr"/>
@@ -10994,7 +10994,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
+          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
         </is>
       </c>
     </row>
@@ -11008,13 +11008,13 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>2400</v>
+        <v>1600</v>
       </c>
       <c r="D136" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E136" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
@@ -11023,7 +11023,7 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Colston Avenue, Bristol, BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
@@ -11037,7 +11037,7 @@
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>14108</v>
+        <v>21996</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -11045,12 +11045,12 @@
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11067,7 +11067,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
+          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
         </is>
       </c>
     </row>
@@ -11081,13 +11081,13 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1300</v>
+        <v>2400</v>
       </c>
       <c r="D137" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E137" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
@@ -11096,23 +11096,21 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>East Street, Bedminster, BS3</t>
+          <t>Colston Avenue, Bristol, BS1</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I137" s="7" t="n">
-        <v>560</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I137" s="7" t="n"/>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="7" t="n">
-        <v>14176</v>
+        <v>14108</v>
       </c>
       <c r="O137" s="7" t="n">
         <v>0</v>
@@ -11125,7 +11123,7 @@
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>Xeno Property, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S137" s="8" t="inlineStr"/>
@@ -11142,7 +11140,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
+          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
         </is>
       </c>
     </row>
@@ -11156,7 +11154,7 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1450</v>
+        <v>1300</v>
       </c>
       <c r="D138" s="7" t="n">
         <v>1</v>
@@ -11171,21 +11169,23 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol</t>
+          <t>East Street, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I138" s="7" t="n"/>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I138" s="7" t="n">
+        <v>560</v>
+      </c>
       <c r="J138" s="7" t="n"/>
       <c r="K138" s="7" t="n"/>
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>13668</v>
+        <v>14176</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11193,12 +11193,12 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>Wildheart Residential Management Limited, Epsom</t>
+          <t>Xeno Property, Bristol</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11215,7 +11215,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
+          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
         </is>
       </c>
     </row>
@@ -11229,7 +11229,7 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>1605</v>
+        <v>1450</v>
       </c>
       <c r="D139" s="7" t="n">
         <v>1</v>
@@ -11244,7 +11244,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Welsh Back, Bristol</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11252,15 +11252,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I139" s="7" t="n">
-        <v>487</v>
-      </c>
+      <c r="I139" s="7" t="n"/>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>13860</v>
+        <v>13668</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11268,12 +11266,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Wildheart Residential Management Limited, Epsom</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11290,7 +11288,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
+          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
         </is>
       </c>
     </row>
@@ -11304,13 +11302,13 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>2185</v>
+        <v>1605</v>
       </c>
       <c r="D140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
@@ -11328,7 +11326,7 @@
         </is>
       </c>
       <c r="I140" s="7" t="n">
-        <v>721</v>
+        <v>487</v>
       </c>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
@@ -11365,7 +11363,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
+          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
         </is>
       </c>
     </row>
@@ -11379,13 +11377,13 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1640</v>
+        <v>2185</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
@@ -11403,7 +11401,7 @@
         </is>
       </c>
       <c r="I141" s="7" t="n">
-        <v>484</v>
+        <v>721</v>
       </c>
       <c r="J141" s="7" t="n"/>
       <c r="K141" s="7" t="n"/>
@@ -11418,7 +11416,7 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
@@ -11440,7 +11438,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
+          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
         </is>
       </c>
     </row>
@@ -11454,13 +11452,13 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>2010</v>
+        <v>1640</v>
       </c>
       <c r="D142" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E142" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
@@ -11478,7 +11476,7 @@
         </is>
       </c>
       <c r="I142" s="7" t="n">
-        <v>722</v>
+        <v>484</v>
       </c>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
@@ -11493,7 +11491,7 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
@@ -11515,7 +11513,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
+          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
         </is>
       </c>
     </row>
@@ -11529,13 +11527,13 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1635</v>
+        <v>2010</v>
       </c>
       <c r="D143" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E143" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
@@ -11544,7 +11542,7 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
@@ -11553,14 +11551,14 @@
         </is>
       </c>
       <c r="I143" s="7" t="n">
-        <v>560</v>
+        <v>722</v>
       </c>
       <c r="J143" s="7" t="n"/>
       <c r="K143" s="7" t="n"/>
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11573,7 +11571,7 @@
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11590,7 +11588,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
+          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11602,7 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1665</v>
+        <v>1635</v>
       </c>
       <c r="D144" s="7" t="n">
         <v>1</v>
@@ -11619,7 +11617,7 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
@@ -11628,14 +11626,14 @@
         </is>
       </c>
       <c r="I144" s="7" t="n">
-        <v>434</v>
+        <v>560</v>
       </c>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>13964</v>
+        <v>13356</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11648,7 +11646,7 @@
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11665,7 +11663,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
+          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
         </is>
       </c>
     </row>
@@ -11679,13 +11677,13 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>1990</v>
+        <v>1665</v>
       </c>
       <c r="D145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
@@ -11703,7 +11701,7 @@
         </is>
       </c>
       <c r="I145" s="7" t="n">
-        <v>682</v>
+        <v>434</v>
       </c>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
@@ -11713,12 +11711,12 @@
         <v>13964</v>
       </c>
       <c r="O145" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
@@ -11740,7 +11738,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
+          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
         </is>
       </c>
     </row>
@@ -11754,13 +11752,13 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>1480</v>
+        <v>1990</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E146" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
@@ -11769,7 +11767,7 @@
       </c>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
@@ -11778,14 +11776,14 @@
         </is>
       </c>
       <c r="I146" s="7" t="n">
-        <v>417</v>
+        <v>682</v>
       </c>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>1</v>
@@ -11793,12 +11791,12 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S146" s="8" t="inlineStr"/>
@@ -11815,7 +11813,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
+          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
         </is>
       </c>
     </row>
@@ -11829,13 +11827,13 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>1750</v>
+        <v>1480</v>
       </c>
       <c r="D147" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E147" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F147" s="7" t="inlineStr">
         <is>
@@ -11844,7 +11842,7 @@
       </c>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H147" s="7" t="inlineStr">
@@ -11852,26 +11850,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I147" s="7" t="n"/>
+      <c r="I147" s="7" t="n">
+        <v>417</v>
+      </c>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="7" t="n">
-        <v>20828</v>
+        <v>13356</v>
       </c>
       <c r="O147" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S147" s="8" t="inlineStr"/>
@@ -11888,7 +11888,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
+          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
         </is>
       </c>
     </row>
@@ -11902,7 +11902,7 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>2080</v>
+        <v>1750</v>
       </c>
       <c r="D148" s="7" t="n">
         <v>2</v>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
@@ -11925,18 +11925,16 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I148" s="7" t="n">
-        <v>705</v>
-      </c>
+      <c r="I148" s="7" t="n"/>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>13356</v>
+        <v>20828</v>
       </c>
       <c r="O148" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
@@ -11946,7 +11944,7 @@
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11963,7 +11961,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
+          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
         </is>
       </c>
     </row>
@@ -11977,13 +11975,13 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>1680</v>
+        <v>2080</v>
       </c>
       <c r="D149" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E149" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F149" s="7" t="inlineStr">
         <is>
@@ -12001,7 +11999,7 @@
         </is>
       </c>
       <c r="I149" s="7" t="n">
-        <v>487</v>
+        <v>705</v>
       </c>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
@@ -12038,7 +12036,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
+          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
         </is>
       </c>
     </row>
@@ -12052,13 +12050,13 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1845</v>
+        <v>1680</v>
       </c>
       <c r="D150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
@@ -12067,7 +12065,7 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
@@ -12076,27 +12074,27 @@
         </is>
       </c>
       <c r="I150" s="7" t="n">
-        <v>641</v>
+        <v>487</v>
       </c>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O150" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12113,7 +12111,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
+          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
         </is>
       </c>
     </row>
@@ -12127,13 +12125,13 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1685</v>
+        <v>1845</v>
       </c>
       <c r="D151" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E151" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F151" s="7" t="inlineStr">
         <is>
@@ -12142,7 +12140,7 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr">
@@ -12151,17 +12149,17 @@
         </is>
       </c>
       <c r="I151" s="7" t="n">
-        <v>578</v>
+        <v>641</v>
       </c>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>13356</v>
+        <v>21476</v>
       </c>
       <c r="O151" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
@@ -12171,7 +12169,7 @@
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12188,7 +12186,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
+          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
         </is>
       </c>
     </row>
@@ -12202,7 +12200,7 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1765</v>
+        <v>1685</v>
       </c>
       <c r="D152" s="7" t="n">
         <v>1</v>
@@ -12226,7 +12224,7 @@
         </is>
       </c>
       <c r="I152" s="7" t="n">
-        <v>641</v>
+        <v>578</v>
       </c>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
@@ -12241,7 +12239,7 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
@@ -12263,7 +12261,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
+          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
         </is>
       </c>
     </row>
@@ -12277,13 +12275,13 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>2240</v>
+        <v>1765</v>
       </c>
       <c r="D153" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E153" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
@@ -12301,17 +12299,17 @@
         </is>
       </c>
       <c r="I153" s="7" t="n">
-        <v>884</v>
+        <v>641</v>
       </c>
       <c r="J153" s="7" t="n"/>
       <c r="K153" s="7" t="n"/>
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>13388</v>
+        <v>13356</v>
       </c>
       <c r="O153" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
@@ -12338,7 +12336,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
+          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
         </is>
       </c>
     </row>
@@ -12352,13 +12350,13 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1150</v>
+        <v>2240</v>
       </c>
       <c r="D154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
@@ -12367,7 +12365,7 @@
       </c>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>John Street, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr">
@@ -12376,25 +12374,27 @@
         </is>
       </c>
       <c r="I154" s="7" t="n">
-        <v>248</v>
+        <v>884</v>
       </c>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
-      <c r="N154" s="7" t="n"/>
+      <c r="N154" s="7" t="n">
+        <v>13388</v>
+      </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S154" s="8" t="inlineStr"/>
@@ -12411,7 +12411,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
+          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
         </is>
       </c>
     </row>
@@ -12425,49 +12425,49 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>3400</v>
+        <v>1150</v>
       </c>
       <c r="D155" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E155" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F155" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Barton Road, Bristol, BS2</t>
+          <t>John Street, BS1</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I155" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I155" s="7" t="n">
+        <v>248</v>
+      </c>
       <c r="J155" s="7" t="n"/>
       <c r="K155" s="7" t="n"/>
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
-      <c r="N155" s="7" t="n">
-        <v>19720</v>
-      </c>
+      <c r="N155" s="7" t="n"/>
       <c r="O155" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12484,7 +12484,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
+          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
         </is>
       </c>
     </row>
@@ -12498,27 +12498,27 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>1250</v>
+        <v>3400</v>
       </c>
       <c r="D156" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E156" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F156" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>St Peters Court, Bedminster</t>
+          <t>Barton Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I156" s="7" t="n"/>
@@ -12527,7 +12527,7 @@
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="7" t="n">
-        <v>15352</v>
+        <v>19720</v>
       </c>
       <c r="O156" s="7" t="n">
         <v>1</v>
@@ -12535,12 +12535,12 @@
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S156" s="8" t="inlineStr"/>
@@ -12557,7 +12557,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
+          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
         </is>
       </c>
     </row>
@@ -12571,13 +12571,13 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>2300</v>
+        <v>1250</v>
       </c>
       <c r="D157" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E157" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
@@ -12586,23 +12586,21 @@
       </c>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>St Peters Court, Bedminster</t>
         </is>
       </c>
       <c r="H157" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I157" s="7" t="n">
-        <v>773</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I157" s="7" t="n"/>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="7" t="n">
-        <v>14172</v>
+        <v>15352</v>
       </c>
       <c r="O157" s="7" t="n">
         <v>1</v>
@@ -12610,12 +12608,12 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol</t>
         </is>
       </c>
       <c r="S157" s="8" t="inlineStr"/>
@@ -12632,7 +12630,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>08411d7c5a6f10970306f10b45d00f0717234e1f</t>
+          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
         </is>
       </c>
     </row>
@@ -12646,13 +12644,13 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>1200</v>
+        <v>2300</v>
       </c>
       <c r="D158" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E158" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F158" s="7" t="inlineStr">
         <is>
@@ -12661,7 +12659,7 @@
       </c>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H158" s="7" t="inlineStr">
@@ -12670,14 +12668,14 @@
         </is>
       </c>
       <c r="I158" s="7" t="n">
-        <v>517</v>
+        <v>773</v>
       </c>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>21904</v>
+        <v>14172</v>
       </c>
       <c r="O158" s="7" t="n">
         <v>1</v>
@@ -12685,12 +12683,12 @@
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S158" s="8" t="inlineStr"/>
@@ -12707,7 +12705,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>e87a39f40860abe2278117f28f53ec7cbbd1d241</t>
+          <t>08411d7c5a6f10970306f10b45d00f0717234e1f</t>
         </is>
       </c>
     </row>
@@ -12721,7 +12719,7 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1630</v>
+        <v>1200</v>
       </c>
       <c r="D159" s="7" t="n">
         <v>1</v>
@@ -12736,36 +12734,36 @@
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I159" s="7" t="n">
-        <v>486</v>
+        <v>517</v>
       </c>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="7" t="n">
-        <v>13860</v>
+        <v>21904</v>
       </c>
       <c r="O159" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12782,7 +12780,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
+          <t>e87a39f40860abe2278117f28f53ec7cbbd1d241</t>
         </is>
       </c>
     </row>
@@ -12796,7 +12794,7 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>1640</v>
+        <v>1630</v>
       </c>
       <c r="D160" s="7" t="n">
         <v>1</v>
@@ -12811,7 +12809,7 @@
       </c>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H160" s="7" t="inlineStr">
@@ -12820,14 +12818,14 @@
         </is>
       </c>
       <c r="I160" s="7" t="n">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
       <c r="N160" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O160" s="7" t="n">
         <v>0</v>
@@ -12835,12 +12833,12 @@
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S160" s="8" t="inlineStr"/>
@@ -12857,7 +12855,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>ecc803f25866be367a83778bda0456688426a26e</t>
+          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
         </is>
       </c>
     </row>
@@ -12871,13 +12869,13 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>2085</v>
+        <v>1640</v>
       </c>
       <c r="D161" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E161" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F161" s="7" t="inlineStr">
         <is>
@@ -12886,7 +12884,7 @@
       </c>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H161" s="7" t="inlineStr">
@@ -12895,14 +12893,14 @@
         </is>
       </c>
       <c r="I161" s="7" t="n">
-        <v>722</v>
+        <v>487</v>
       </c>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
       <c r="N161" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O161" s="7" t="n">
         <v>0</v>
@@ -12910,12 +12908,12 @@
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S161" s="8" t="inlineStr"/>
@@ -12932,7 +12930,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
+          <t>ecc803f25866be367a83778bda0456688426a26e</t>
         </is>
       </c>
     </row>
@@ -12946,13 +12944,13 @@
         </is>
       </c>
       <c r="C162" s="9" t="n">
-        <v>1650</v>
+        <v>2085</v>
       </c>
       <c r="D162" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E162" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F162" s="7" t="inlineStr">
         <is>
@@ -12961,7 +12959,7 @@
       </c>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
@@ -12970,14 +12968,14 @@
         </is>
       </c>
       <c r="I162" s="7" t="n">
-        <v>553</v>
+        <v>722</v>
       </c>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
       <c r="N162" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O162" s="7" t="n">
         <v>0</v>
@@ -12990,7 +12988,7 @@
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S162" s="8" t="inlineStr"/>
@@ -13007,7 +13005,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
+          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
         </is>
       </c>
     </row>
@@ -13021,7 +13019,7 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1350</v>
+        <v>1650</v>
       </c>
       <c r="D163" s="7" t="n">
         <v>1</v>
@@ -13036,7 +13034,7 @@
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
@@ -13045,14 +13043,14 @@
         </is>
       </c>
       <c r="I163" s="7" t="n">
-        <v>518</v>
+        <v>553</v>
       </c>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="7" t="n">
-        <v>16664</v>
+        <v>13356</v>
       </c>
       <c r="O163" s="7" t="n">
         <v>0</v>
@@ -13060,12 +13058,12 @@
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13082,7 +13080,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>61cb6cbca03d4b33a5e567abbe422df6574deb7a</t>
+          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
         </is>
       </c>
     </row>
@@ -13096,10 +13094,10 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>1550</v>
+        <v>1350</v>
       </c>
       <c r="D164" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E164" s="7" t="n">
         <v>1</v>
@@ -13111,21 +13109,23 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Crown And Anchor House, Temple Quay, Temple Quay, BS2</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I164" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I164" s="7" t="n">
+        <v>518</v>
+      </c>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="7" t="n">
-        <v>20472</v>
+        <v>16664</v>
       </c>
       <c r="O164" s="7" t="n">
         <v>0</v>
@@ -13133,12 +13133,12 @@
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13155,7 +13155,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>e76245b9d5be47e78934469ea3c31d3d0433291c</t>
+          <t>61cb6cbca03d4b33a5e567abbe422df6574deb7a</t>
         </is>
       </c>
     </row>
@@ -13169,10 +13169,10 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1665</v>
+        <v>1550</v>
       </c>
       <c r="D165" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E165" s="7" t="n">
         <v>1</v>
@@ -13184,23 +13184,21 @@
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Crown And Anchor House, Temple Quay, Temple Quay, BS2</t>
         </is>
       </c>
       <c r="H165" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I165" s="7" t="n">
-        <v>569</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I165" s="7" t="n"/>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>13356</v>
+        <v>20472</v>
       </c>
       <c r="O165" s="7" t="n">
         <v>0</v>
@@ -13213,7 +13211,7 @@
       </c>
       <c r="R165" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S165" s="8" t="inlineStr"/>
@@ -13230,7 +13228,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>22588bce8839df85d69555bd640fcbb3902101ff</t>
+          <t>e76245b9d5be47e78934469ea3c31d3d0433291c</t>
         </is>
       </c>
     </row>
@@ -13244,36 +13242,38 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>1850</v>
+        <v>1665</v>
       </c>
       <c r="D166" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E166" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F166" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>Webb Street, Bristol, BS5</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H166" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I166" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I166" s="7" t="n">
+        <v>569</v>
+      </c>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="7" t="n">
-        <v>19580</v>
+        <v>13356</v>
       </c>
       <c r="O166" s="7" t="n">
         <v>0</v>
@@ -13281,12 +13281,12 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
@@ -13303,7 +13303,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
+          <t>22588bce8839df85d69555bd640fcbb3902101ff</t>
         </is>
       </c>
     </row>
@@ -13317,27 +13317,27 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>1200</v>
+        <v>1850</v>
       </c>
       <c r="D167" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E167" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F167" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>Bushy Park, The Bank Bushy Park, BS4</t>
+          <t>Webb Street, Bristol, BS5</t>
         </is>
       </c>
       <c r="H167" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I167" s="7" t="n"/>
@@ -13346,7 +13346,7 @@
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="7" t="n">
-        <v>7216</v>
+        <v>19580</v>
       </c>
       <c r="O167" s="7" t="n">
         <v>0</v>
@@ -13354,12 +13354,12 @@
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S167" s="8" t="inlineStr"/>
@@ -13376,7 +13376,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
+          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
         </is>
       </c>
     </row>
@@ -13390,13 +13390,13 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1750</v>
+        <v>1200</v>
       </c>
       <c r="D168" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E168" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F168" s="7" t="inlineStr">
         <is>
@@ -13405,12 +13405,12 @@
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Number One Bristol, Bristol</t>
+          <t>Bushy Park, The Bank Bushy Park, BS4</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I168" s="7" t="n"/>
@@ -13419,7 +13419,7 @@
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="7" t="n">
-        <v>21808</v>
+        <v>7216</v>
       </c>
       <c r="O168" s="7" t="n">
         <v>0</v>
@@ -13427,12 +13427,12 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Zest, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13449,7 +13449,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>d2b416547517343eef3a43500d63f738ac4ae423</t>
+          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
         </is>
       </c>
     </row>
@@ -13463,13 +13463,13 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1295</v>
+        <v>1750</v>
       </c>
       <c r="D169" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E169" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
@@ -13478,7 +13478,7 @@
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Great Western House, BS1</t>
+          <t>Number One Bristol, Bristol</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
@@ -13486,15 +13486,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I169" s="7" t="n">
-        <v>474</v>
-      </c>
+      <c r="I169" s="7" t="n"/>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>14412</v>
+        <v>21808</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13502,12 +13500,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Zest, Bristol</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13524,7 +13522,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>466dad45b709c8ce2ab5e9d022bce4baabb5cecc</t>
+          <t>d2b416547517343eef3a43500d63f738ac4ae423</t>
         </is>
       </c>
     </row>
@@ -13538,7 +13536,7 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>1325</v>
+        <v>1295</v>
       </c>
       <c r="D170" s="7" t="n">
         <v>1</v>
@@ -13553,7 +13551,7 @@
       </c>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t>Broad Street, Bristol, BS1</t>
+          <t>Harbourside, Great Western House, BS1</t>
         </is>
       </c>
       <c r="H170" s="7" t="inlineStr">
@@ -13561,13 +13559,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I170" s="7" t="n"/>
+      <c r="I170" s="7" t="n">
+        <v>474</v>
+      </c>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
       <c r="L170" s="7" t="n"/>
       <c r="M170" s="7" t="n"/>
       <c r="N170" s="7" t="n">
-        <v>21788</v>
+        <v>14412</v>
       </c>
       <c r="O170" s="7" t="n">
         <v>0</v>
@@ -13575,12 +13575,12 @@
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -13597,7 +13597,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
+          <t>466dad45b709c8ce2ab5e9d022bce4baabb5cecc</t>
         </is>
       </c>
     </row>
@@ -13611,13 +13611,13 @@
         </is>
       </c>
       <c r="C171" s="9" t="n">
-        <v>2200</v>
+        <v>1325</v>
       </c>
       <c r="D171" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E171" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F171" s="7" t="inlineStr">
         <is>
@@ -13626,7 +13626,7 @@
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
+          <t>Broad Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H171" s="7" t="inlineStr">
@@ -13640,7 +13640,7 @@
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="7" t="n">
-        <v>16788</v>
+        <v>21788</v>
       </c>
       <c r="O171" s="7" t="n">
         <v>0</v>
@@ -13648,12 +13648,12 @@
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -13670,7 +13670,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
+          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
         </is>
       </c>
     </row>
@@ -13684,13 +13684,13 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1500</v>
+        <v>2200</v>
       </c>
       <c r="D172" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E172" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F172" s="7" t="inlineStr">
         <is>
@@ -13699,7 +13699,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>Eclipse, Broad Weir, Bristol</t>
+          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H172" s="7" t="inlineStr">
@@ -13713,7 +13713,7 @@
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="7" t="n">
-        <v>22164</v>
+        <v>16788</v>
       </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
@@ -13721,12 +13721,12 @@
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
         <is>
-          <t>Martin &amp; Co, Bath</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -13743,7 +13743,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
+          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
         </is>
       </c>
     </row>
@@ -13757,7 +13757,7 @@
         </is>
       </c>
       <c r="C173" s="9" t="n">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="D173" s="7" t="n">
         <v>1</v>
@@ -13772,7 +13772,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Broad Weir, City Centre, Bristol, BS1</t>
+          <t>Eclipse, Broad Weir, Bristol</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
@@ -13780,15 +13780,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I173" s="7" t="n">
-        <v>474</v>
-      </c>
+      <c r="I173" s="7" t="n"/>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>22080</v>
+        <v>22164</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13796,12 +13794,12 @@
       <c r="P173" s="7" t="n"/>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Clifton</t>
+          <t>Martin &amp; Co, Bath</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -13818,7 +13816,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
+          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
         </is>
       </c>
     </row>
@@ -13832,7 +13830,7 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1300</v>
+        <v>1800</v>
       </c>
       <c r="D174" s="7" t="n">
         <v>1</v>
@@ -13847,7 +13845,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Deanery Road, BS1 5AF</t>
+          <t>Broad Weir, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
@@ -13856,14 +13854,14 @@
         </is>
       </c>
       <c r="I174" s="7" t="n">
-        <v>570</v>
+        <v>474</v>
       </c>
       <c r="J174" s="7" t="n"/>
       <c r="K174" s="7" t="n"/>
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>19300</v>
+        <v>22080</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13871,12 +13869,12 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -13893,7 +13891,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
+          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
         </is>
       </c>
     </row>
@@ -13907,13 +13905,13 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>2500</v>
+        <v>1300</v>
       </c>
       <c r="D175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
@@ -13922,21 +13920,23 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>City Centre, Deanery Road, BS1 5AF</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I175" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I175" s="7" t="n">
+        <v>570</v>
+      </c>
       <c r="J175" s="7" t="n"/>
       <c r="K175" s="7" t="n"/>
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
       <c r="N175" s="7" t="n">
-        <v>21360</v>
+        <v>19300</v>
       </c>
       <c r="O175" s="7" t="n">
         <v>0</v>
@@ -13944,12 +13944,12 @@
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -13966,7 +13966,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
+          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
         </is>
       </c>
     </row>
@@ -13980,13 +13980,13 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>1650</v>
+        <v>2500</v>
       </c>
       <c r="D176" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E176" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F176" s="7" t="inlineStr">
         <is>
@@ -13995,7 +13995,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>Crown &amp; Anchor House, Bristol, BS2</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H176" s="7" t="inlineStr">
@@ -14009,7 +14009,7 @@
       <c r="L176" s="7" t="n"/>
       <c r="M176" s="7" t="n"/>
       <c r="N176" s="7" t="n">
-        <v>20472</v>
+        <v>21360</v>
       </c>
       <c r="O176" s="7" t="n">
         <v>0</v>
@@ -14017,12 +14017,12 @@
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -14039,7 +14039,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
+          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
         </is>
       </c>
     </row>
@@ -14053,13 +14053,13 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>1450</v>
+        <v>1650</v>
       </c>
       <c r="D177" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E177" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F177" s="7" t="inlineStr">
         <is>
@@ -14068,23 +14068,21 @@
       </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>Woodbridge Road, Bristol, BS4</t>
+          <t>Crown &amp; Anchor House, Bristol, BS2</t>
         </is>
       </c>
       <c r="H177" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I177" s="7" t="n">
-        <v>678</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I177" s="7" t="n"/>
       <c r="J177" s="7" t="n"/>
       <c r="K177" s="7" t="n"/>
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
       <c r="N177" s="7" t="n">
-        <v>5700</v>
+        <v>20472</v>
       </c>
       <c r="O177" s="7" t="n">
         <v>0</v>
@@ -14092,12 +14090,12 @@
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S177" s="8" t="inlineStr"/>
@@ -14114,7 +14112,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
+          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
         </is>
       </c>
     </row>
@@ -14131,9 +14129,11 @@
         <v>1450</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E178" s="7" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="E178" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="F178" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -14141,34 +14141,36 @@
       </c>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Woodbridge Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H178" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I178" s="7" t="n"/>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I178" s="7" t="n">
+        <v>678</v>
+      </c>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
       <c r="L178" s="7" t="n"/>
       <c r="M178" s="7" t="n"/>
       <c r="N178" s="7" t="n">
-        <v>19488</v>
+        <v>5700</v>
       </c>
       <c r="O178" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S178" s="8" t="inlineStr"/>
@@ -14185,7 +14187,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
+          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
         </is>
       </c>
     </row>
@@ -14199,14 +14201,12 @@
         </is>
       </c>
       <c r="C179" s="9" t="n">
-        <v>1500</v>
+        <v>1450</v>
       </c>
       <c r="D179" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E179" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E179" s="7" t="n"/>
       <c r="F179" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -14214,12 +14214,12 @@
       </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H179" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I179" s="7" t="n"/>
@@ -14228,20 +14228,20 @@
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
       <c r="N179" s="7" t="n">
-        <v>20768</v>
+        <v>19488</v>
       </c>
       <c r="O179" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -14258,7 +14258,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
+          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
         </is>
       </c>
     </row>
@@ -14272,38 +14272,36 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>2250</v>
+        <v>1500</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E180" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F180" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Newfoundland Road, Bristol, BS2</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I180" s="7" t="n">
-        <v>980</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I180" s="7" t="n"/>
       <c r="J180" s="7" t="n"/>
       <c r="K180" s="7" t="n"/>
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="7" t="n">
-        <v>19800</v>
+        <v>20768</v>
       </c>
       <c r="O180" s="7" t="n">
         <v>0</v>
@@ -14311,12 +14309,12 @@
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>Lets Rent Bristol, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14333,7 +14331,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
+          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
         </is>
       </c>
     </row>
@@ -14347,36 +14345,38 @@
         </is>
       </c>
       <c r="C181" s="9" t="n">
-        <v>2000</v>
+        <v>2250</v>
       </c>
       <c r="D181" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E181" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F181" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>Protheroes House, Hobbs Lane, BS1</t>
+          <t>Newfoundland Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H181" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I181" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I181" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="7" t="n">
-        <v>13584</v>
+        <v>19800</v>
       </c>
       <c r="O181" s="7" t="n">
         <v>0</v>
@@ -14384,12 +14384,12 @@
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Lets Rent Bristol, Bristol</t>
         </is>
       </c>
       <c r="S181" s="8" t="inlineStr"/>
@@ -14406,7 +14406,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
+          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
         </is>
       </c>
     </row>
@@ -14420,27 +14420,27 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>2400</v>
+        <v>2000</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Balmain Street, Totterdown, Bristol, BS4</t>
+          <t>Protheroes House, Hobbs Lane, BS1</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I182" s="7" t="n"/>
@@ -14449,7 +14449,7 @@
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>5524</v>
+        <v>13584</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14457,12 +14457,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14479,7 +14479,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>dd411af39a083f886127138c0a969254da83858b</t>
+          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
         </is>
       </c>
     </row>
@@ -14493,51 +14493,49 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>1665</v>
+        <v>2400</v>
       </c>
       <c r="D183" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E183" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F183" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Balmain Street, Totterdown, Bristol, BS4</t>
         </is>
       </c>
       <c r="H183" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I183" s="7" t="n">
-        <v>578</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I183" s="7" t="n"/>
       <c r="J183" s="7" t="n"/>
       <c r="K183" s="7" t="n"/>
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="7" t="n">
-        <v>13356</v>
+        <v>5524</v>
       </c>
       <c r="O183" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S183" s="8" t="inlineStr"/>
@@ -14554,7 +14552,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
+          <t>dd411af39a083f886127138c0a969254da83858b</t>
         </is>
       </c>
     </row>
@@ -14568,7 +14566,7 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>1635</v>
+        <v>1665</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>1</v>
@@ -14583,7 +14581,7 @@
       </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H184" s="7" t="inlineStr">
@@ -14592,14 +14590,14 @@
         </is>
       </c>
       <c r="I184" s="7" t="n">
-        <v>485</v>
+        <v>578</v>
       </c>
       <c r="J184" s="7" t="n"/>
       <c r="K184" s="7" t="n"/>
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
       <c r="N184" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O184" s="7" t="n">
         <v>1</v>
@@ -14607,12 +14605,12 @@
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S184" s="8" t="inlineStr"/>
@@ -14629,7 +14627,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
+          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
         </is>
       </c>
     </row>
@@ -14643,7 +14641,7 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>1615</v>
+        <v>1635</v>
       </c>
       <c r="D185" s="7" t="n">
         <v>1</v>
@@ -14667,7 +14665,7 @@
         </is>
       </c>
       <c r="I185" s="7" t="n">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="J185" s="7" t="n"/>
       <c r="K185" s="7" t="n"/>
@@ -14682,7 +14680,7 @@
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R185" s="7" t="inlineStr">
@@ -14704,7 +14702,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
+          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
         </is>
       </c>
     </row>
@@ -14718,7 +14716,7 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>1640</v>
+        <v>1615</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>1</v>
@@ -14733,7 +14731,7 @@
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
@@ -14742,14 +14740,14 @@
         </is>
       </c>
       <c r="I186" s="7" t="n">
-        <v>560</v>
+        <v>487</v>
       </c>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O186" s="7" t="n">
         <v>1</v>
@@ -14757,12 +14755,12 @@
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14779,7 +14777,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
+          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
         </is>
       </c>
     </row>
@@ -14793,7 +14791,7 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>1615</v>
+        <v>1640</v>
       </c>
       <c r="D187" s="7" t="n">
         <v>1</v>
@@ -14808,7 +14806,7 @@
       </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
@@ -14817,14 +14815,14 @@
         </is>
       </c>
       <c r="I187" s="7" t="n">
-        <v>484</v>
+        <v>560</v>
       </c>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>13860</v>
+        <v>13356</v>
       </c>
       <c r="O187" s="7" t="n">
         <v>1</v>
@@ -14837,7 +14835,7 @@
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S187" s="8" t="inlineStr"/>
@@ -14854,7 +14852,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
+          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
         </is>
       </c>
     </row>
@@ -14892,7 +14890,7 @@
         </is>
       </c>
       <c r="I188" s="7" t="n">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
@@ -14902,12 +14900,12 @@
         <v>13860</v>
       </c>
       <c r="O188" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
@@ -14929,7 +14927,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
+          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
         </is>
       </c>
     </row>
@@ -14943,7 +14941,7 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>1645</v>
+        <v>1615</v>
       </c>
       <c r="D189" s="7" t="n">
         <v>1</v>
@@ -14958,7 +14956,7 @@
       </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
@@ -14967,14 +14965,14 @@
         </is>
       </c>
       <c r="I189" s="7" t="n">
-        <v>570</v>
+        <v>486</v>
       </c>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
       <c r="L189" s="7" t="n"/>
       <c r="M189" s="7" t="n"/>
       <c r="N189" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O189" s="7" t="n">
         <v>0</v>
@@ -14987,7 +14985,7 @@
       </c>
       <c r="R189" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S189" s="8" t="inlineStr"/>
@@ -15004,7 +15002,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
+          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
         </is>
       </c>
     </row>
@@ -15018,7 +15016,7 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>1630</v>
+        <v>1645</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1</v>
@@ -15042,7 +15040,7 @@
         </is>
       </c>
       <c r="I190" s="7" t="n">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
@@ -15057,7 +15055,7 @@
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
@@ -15079,7 +15077,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
+          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
         </is>
       </c>
     </row>
@@ -15093,10 +15091,10 @@
         </is>
       </c>
       <c r="C191" s="9" t="n">
-        <v>1800</v>
+        <v>1630</v>
       </c>
       <c r="D191" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E191" s="7" t="n">
         <v>1</v>
@@ -15108,7 +15106,7 @@
       </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H191" s="7" t="inlineStr">
@@ -15116,13 +15114,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I191" s="7" t="n"/>
+      <c r="I191" s="7" t="n">
+        <v>560</v>
+      </c>
       <c r="J191" s="7" t="n"/>
       <c r="K191" s="7" t="n"/>
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
       <c r="N191" s="7" t="n">
-        <v>21176</v>
+        <v>13356</v>
       </c>
       <c r="O191" s="7" t="n">
         <v>0</v>
@@ -15135,7 +15135,7 @@
       </c>
       <c r="R191" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S191" s="8" t="inlineStr"/>
@@ -15152,7 +15152,7 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
-          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
+          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
         </is>
       </c>
     </row>
@@ -15166,10 +15166,10 @@
         </is>
       </c>
       <c r="C192" s="9" t="n">
-        <v>1635</v>
+        <v>1800</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E192" s="7" t="n">
         <v>1</v>
@@ -15181,7 +15181,7 @@
       </c>
       <c r="G192" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Bristol City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H192" s="7" t="inlineStr">
@@ -15189,15 +15189,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I192" s="7" t="n">
-        <v>569</v>
-      </c>
+      <c r="I192" s="7" t="n"/>
       <c r="J192" s="7" t="n"/>
       <c r="K192" s="7" t="n"/>
       <c r="L192" s="7" t="n"/>
       <c r="M192" s="7" t="n"/>
       <c r="N192" s="7" t="n">
-        <v>13356</v>
+        <v>21176</v>
       </c>
       <c r="O192" s="7" t="n">
         <v>0</v>
@@ -15205,12 +15203,12 @@
       <c r="P192" s="7" t="n"/>
       <c r="Q192" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R192" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S192" s="8" t="inlineStr"/>
@@ -15227,7 +15225,7 @@
       <c r="V192" s="6" t="inlineStr"/>
       <c r="W192" s="7" t="inlineStr">
         <is>
-          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
+          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
         </is>
       </c>
     </row>
@@ -15241,10 +15239,10 @@
         </is>
       </c>
       <c r="C193" s="9" t="n">
-        <v>1925</v>
+        <v>1635</v>
       </c>
       <c r="D193" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E193" s="7" t="n">
         <v>1</v>
@@ -15256,7 +15254,7 @@
       </c>
       <c r="G193" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H193" s="7" t="inlineStr">
@@ -15265,14 +15263,14 @@
         </is>
       </c>
       <c r="I193" s="7" t="n">
-        <v>655</v>
+        <v>569</v>
       </c>
       <c r="J193" s="7" t="n"/>
       <c r="K193" s="7" t="n"/>
       <c r="L193" s="7" t="n"/>
       <c r="M193" s="7" t="n"/>
       <c r="N193" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O193" s="7" t="n">
         <v>0</v>
@@ -15280,12 +15278,12 @@
       <c r="P193" s="7" t="n"/>
       <c r="Q193" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R193" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S193" s="8" t="inlineStr"/>
@@ -15302,7 +15300,7 @@
       <c r="V193" s="6" t="inlineStr"/>
       <c r="W193" s="7" t="inlineStr">
         <is>
-          <t>892dd053ae3538c7c123f255e926bef984caf6de</t>
+          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
         </is>
       </c>
     </row>
@@ -15316,13 +15314,13 @@
         </is>
       </c>
       <c r="C194" s="9" t="n">
-        <v>1800</v>
+        <v>1925</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E194" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F194" s="7" t="inlineStr">
         <is>
@@ -15331,7 +15329,7 @@
       </c>
       <c r="G194" s="8" t="inlineStr">
         <is>
-          <t>Park St, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H194" s="7" t="inlineStr">
@@ -15339,13 +15337,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I194" s="7" t="n"/>
+      <c r="I194" s="7" t="n">
+        <v>655</v>
+      </c>
       <c r="J194" s="7" t="n"/>
       <c r="K194" s="7" t="n"/>
       <c r="L194" s="7" t="n"/>
       <c r="M194" s="7" t="n"/>
       <c r="N194" s="7" t="n">
-        <v>20644</v>
+        <v>21476</v>
       </c>
       <c r="O194" s="7" t="n">
         <v>0</v>
@@ -15353,12 +15353,12 @@
       <c r="P194" s="7" t="n"/>
       <c r="Q194" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R194" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S194" s="8" t="inlineStr"/>
@@ -15375,7 +15375,7 @@
       <c r="V194" s="6" t="inlineStr"/>
       <c r="W194" s="7" t="inlineStr">
         <is>
-          <t>8e49447f07b7d2adcefccb79294af764ba54db50</t>
+          <t>892dd053ae3538c7c123f255e926bef984caf6de</t>
         </is>
       </c>
     </row>
@@ -15389,13 +15389,13 @@
         </is>
       </c>
       <c r="C195" s="9" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="D195" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E195" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F195" s="7" t="inlineStr">
         <is>
@@ -15404,7 +15404,7 @@
       </c>
       <c r="G195" s="8" t="inlineStr">
         <is>
-          <t>Marsh House, Bristol, BS1</t>
+          <t>Park St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H195" s="7" t="inlineStr">
@@ -15418,7 +15418,7 @@
       <c r="L195" s="7" t="n"/>
       <c r="M195" s="7" t="n"/>
       <c r="N195" s="7" t="n">
-        <v>20952</v>
+        <v>20644</v>
       </c>
       <c r="O195" s="7" t="n">
         <v>0</v>
@@ -15426,12 +15426,12 @@
       <c r="P195" s="7" t="n"/>
       <c r="Q195" s="7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R195" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S195" s="8" t="inlineStr"/>
@@ -15448,7 +15448,7 @@
       <c r="V195" s="6" t="inlineStr"/>
       <c r="W195" s="7" t="inlineStr">
         <is>
-          <t>dc8b7c88d86188af3ee5262a5f1215944eb3e402</t>
+          <t>8e49447f07b7d2adcefccb79294af764ba54db50</t>
         </is>
       </c>
     </row>
@@ -15462,10 +15462,10 @@
         </is>
       </c>
       <c r="C196" s="9" t="n">
-        <v>1800</v>
+        <v>1650</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E196" s="7" t="n">
         <v>1</v>
@@ -15477,7 +15477,7 @@
       </c>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t>Swann House, Bristol, BS1</t>
+          <t>Marsh House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H196" s="7" t="inlineStr">
@@ -15491,7 +15491,7 @@
       <c r="L196" s="7" t="n"/>
       <c r="M196" s="7" t="n"/>
       <c r="N196" s="7" t="n">
-        <v>20592</v>
+        <v>20952</v>
       </c>
       <c r="O196" s="7" t="n">
         <v>0</v>
@@ -15499,12 +15499,12 @@
       <c r="P196" s="7" t="n"/>
       <c r="Q196" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R196" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S196" s="8" t="inlineStr"/>
@@ -15521,7 +15521,7 @@
       <c r="V196" s="6" t="inlineStr"/>
       <c r="W196" s="7" t="inlineStr">
         <is>
-          <t>7aa830b20d3fe9e9350b37a53ede99615caa3290</t>
+          <t>dc8b7c88d86188af3ee5262a5f1215944eb3e402</t>
         </is>
       </c>
     </row>
@@ -15535,10 +15535,10 @@
         </is>
       </c>
       <c r="C197" s="9" t="n">
-        <v>1350</v>
+        <v>1800</v>
       </c>
       <c r="D197" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E197" s="7" t="n">
         <v>1</v>
@@ -15550,7 +15550,7 @@
       </c>
       <c r="G197" s="8" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>Swann House, Bristol, BS1</t>
         </is>
       </c>
       <c r="H197" s="7" t="inlineStr">
@@ -15558,15 +15558,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I197" s="7" t="n">
-        <v>518</v>
-      </c>
+      <c r="I197" s="7" t="n"/>
       <c r="J197" s="7" t="n"/>
       <c r="K197" s="7" t="n"/>
       <c r="L197" s="7" t="n"/>
       <c r="M197" s="7" t="n"/>
       <c r="N197" s="7" t="n">
-        <v>16416</v>
+        <v>20592</v>
       </c>
       <c r="O197" s="7" t="n">
         <v>0</v>
@@ -15574,12 +15572,12 @@
       <c r="P197" s="7" t="n"/>
       <c r="Q197" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R197" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S197" s="8" t="inlineStr"/>
@@ -15596,7 +15594,7 @@
       <c r="V197" s="6" t="inlineStr"/>
       <c r="W197" s="7" t="inlineStr">
         <is>
-          <t>77b9e2d97ea9d3f764e1fbd2fdd0b5bf1d5b75b8</t>
+          <t>7aa830b20d3fe9e9350b37a53ede99615caa3290</t>
         </is>
       </c>
     </row>
@@ -15610,7 +15608,7 @@
         </is>
       </c>
       <c r="C198" s="9" t="n">
-        <v>1450</v>
+        <v>1350</v>
       </c>
       <c r="D198" s="7" t="n">
         <v>1</v>
@@ -15625,7 +15623,7 @@
       </c>
       <c r="G198" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H198" s="7" t="inlineStr">
@@ -15633,13 +15631,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I198" s="7" t="n"/>
+      <c r="I198" s="7" t="n">
+        <v>518</v>
+      </c>
       <c r="J198" s="7" t="n"/>
       <c r="K198" s="7" t="n"/>
       <c r="L198" s="7" t="n"/>
       <c r="M198" s="7" t="n"/>
       <c r="N198" s="7" t="n">
-        <v>20524</v>
+        <v>16416</v>
       </c>
       <c r="O198" s="7" t="n">
         <v>0</v>
@@ -15652,7 +15652,7 @@
       </c>
       <c r="R198" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S198" s="8" t="inlineStr"/>
@@ -15669,14 +15669,87 @@
       <c r="V198" s="6" t="inlineStr"/>
       <c r="W198" s="7" t="inlineStr">
         <is>
+          <t>77b9e2d97ea9d3f764e1fbd2fdd0b5bf1d5b75b8</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B199" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C199" s="9" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D199" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E199" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F199" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G199" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Court, Bristol, BS1</t>
+        </is>
+      </c>
+      <c r="H199" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I199" s="7" t="n"/>
+      <c r="J199" s="7" t="n"/>
+      <c r="K199" s="7" t="n"/>
+      <c r="L199" s="7" t="n"/>
+      <c r="M199" s="7" t="n"/>
+      <c r="N199" s="7" t="n">
+        <v>20524</v>
+      </c>
+      <c r="O199" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P199" s="7" t="n"/>
+      <c r="Q199" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="R199" s="7" t="inlineStr">
+        <is>
+          <t>OpenRent, London</t>
+        </is>
+      </c>
+      <c r="S199" s="8" t="inlineStr"/>
+      <c r="T199" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V199" s="6" t="inlineStr"/>
+      <c r="W199" s="7" t="inlineStr">
+        <is>
           <t>adbd7c1c798d9f667bce5c8c0d31831cec0ebf67</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W198"/>
+  <autoFilter ref="A1:W199"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15878,6 +15951,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T196" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T197" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T199" r:id="rId198"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 140
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W198"/>
+  <dimension ref="A1:W201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2523,7 +2523,7 @@
       <c r="L24" s="7" t="n"/>
       <c r="M24" s="7" t="n"/>
       <c r="N24" s="7" t="n">
-        <v>20924</v>
+        <v>20780</v>
       </c>
       <c r="O24" s="7" t="n">
         <v>0</v>
@@ -9238,7 +9238,7 @@
         </is>
       </c>
       <c r="C112" s="9" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="D112" s="7" t="n">
         <v>1</v>
@@ -10570,13 +10570,13 @@
         </is>
       </c>
       <c r="C130" s="9" t="n">
-        <v>1700</v>
+        <v>1985</v>
       </c>
       <c r="D130" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E130" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
@@ -10594,14 +10594,14 @@
         </is>
       </c>
       <c r="I130" s="7" t="n">
-        <v>646</v>
+        <v>771</v>
       </c>
       <c r="J130" s="7" t="n"/>
       <c r="K130" s="7" t="n"/>
       <c r="L130" s="7" t="n"/>
       <c r="M130" s="7" t="n"/>
       <c r="N130" s="7" t="n">
-        <v>20928</v>
+        <v>21740</v>
       </c>
       <c r="O130" s="7" t="n">
         <v>0</v>
@@ -10609,12 +10609,12 @@
       <c r="P130" s="7" t="n"/>
       <c r="Q130" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R130" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S130" s="8" t="inlineStr"/>
@@ -10631,7 +10631,7 @@
       <c r="V130" s="6" t="inlineStr"/>
       <c r="W130" s="7" t="inlineStr">
         <is>
-          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
+          <t>5414e121fde47f0b60451ddda4019d5d93133f4a</t>
         </is>
       </c>
     </row>
@@ -10645,13 +10645,13 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>2105</v>
+        <v>1650</v>
       </c>
       <c r="D131" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E131" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
@@ -10669,7 +10669,7 @@
         </is>
       </c>
       <c r="I131" s="7" t="n">
-        <v>745</v>
+        <v>484</v>
       </c>
       <c r="J131" s="7" t="n"/>
       <c r="K131" s="7" t="n"/>
@@ -10684,7 +10684,7 @@
       <c r="P131" s="7" t="n"/>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
@@ -10706,7 +10706,7 @@
       <c r="V131" s="6" t="inlineStr"/>
       <c r="W131" s="7" t="inlineStr">
         <is>
-          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
+          <t>a6340397b31ca11a123cb584f2f878317e73b7eb</t>
         </is>
       </c>
     </row>
@@ -10720,7 +10720,7 @@
         </is>
       </c>
       <c r="C132" s="9" t="n">
-        <v>1595</v>
+        <v>1630</v>
       </c>
       <c r="D132" s="7" t="n">
         <v>1</v>
@@ -10744,7 +10744,7 @@
         </is>
       </c>
       <c r="I132" s="7" t="n">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="J132" s="7" t="n"/>
       <c r="K132" s="7" t="n"/>
@@ -10759,7 +10759,7 @@
       <c r="P132" s="7" t="n"/>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
@@ -10781,7 +10781,7 @@
       <c r="V132" s="6" t="inlineStr"/>
       <c r="W132" s="7" t="inlineStr">
         <is>
-          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
+          <t>5cdc78c7612a522b9bc5bc24a2beb93eb2703b6b</t>
         </is>
       </c>
     </row>
@@ -10795,7 +10795,7 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1999</v>
+        <v>1700</v>
       </c>
       <c r="D133" s="7" t="n">
         <v>2</v>
@@ -10810,21 +10810,23 @@
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I133" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I133" s="7" t="n">
+        <v>646</v>
+      </c>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>21736</v>
+        <v>20928</v>
       </c>
       <c r="O133" s="7" t="n">
         <v>0</v>
@@ -10832,12 +10834,12 @@
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S133" s="8" t="inlineStr"/>
@@ -10854,7 +10856,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
+          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
         </is>
       </c>
     </row>
@@ -10868,13 +10870,13 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>1605</v>
+        <v>2105</v>
       </c>
       <c r="D134" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E134" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
@@ -10883,7 +10885,7 @@
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
@@ -10892,14 +10894,14 @@
         </is>
       </c>
       <c r="I134" s="7" t="n">
-        <v>487</v>
+        <v>745</v>
       </c>
       <c r="J134" s="7" t="n"/>
       <c r="K134" s="7" t="n"/>
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="7" t="n">
-        <v>21732</v>
+        <v>20984</v>
       </c>
       <c r="O134" s="7" t="n">
         <v>0</v>
@@ -10907,12 +10909,12 @@
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10929,7 +10931,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
+          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
         </is>
       </c>
     </row>
@@ -10943,7 +10945,7 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1390</v>
+        <v>1595</v>
       </c>
       <c r="D135" s="7" t="n">
         <v>1</v>
@@ -10958,7 +10960,7 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
@@ -10966,24 +10968,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I135" s="7" t="n"/>
+      <c r="I135" s="7" t="n">
+        <v>484</v>
+      </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
-      <c r="N135" s="7" t="n"/>
+      <c r="N135" s="7" t="n">
+        <v>21732</v>
+      </c>
       <c r="O135" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S135" s="8" t="inlineStr"/>
@@ -11000,7 +11006,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
         </is>
       </c>
     </row>
@@ -11014,10 +11020,10 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>1395</v>
+        <v>1999</v>
       </c>
       <c r="D136" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E136" s="7" t="n">
         <v>1</v>
@@ -11029,12 +11035,12 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I136" s="7" t="n"/>
@@ -11043,7 +11049,7 @@
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>20524</v>
+        <v>21736</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -11051,7 +11057,7 @@
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
@@ -11073,7 +11079,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
         </is>
       </c>
     </row>
@@ -11087,7 +11093,7 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1200</v>
+        <v>1605</v>
       </c>
       <c r="D137" s="7" t="n">
         <v>1</v>
@@ -11097,28 +11103,28 @@
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2 0JN</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I137" s="7" t="n">
-        <v>452</v>
+        <v>487</v>
       </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="7" t="n">
-        <v>20472</v>
+        <v>21732</v>
       </c>
       <c r="O137" s="7" t="n">
         <v>0</v>
@@ -11126,12 +11132,12 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S137" s="8" t="inlineStr"/>
@@ -11148,7 +11154,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
+          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
         </is>
       </c>
     </row>
@@ -11162,7 +11168,7 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1450</v>
+        <v>1390</v>
       </c>
       <c r="D138" s="7" t="n">
         <v>1</v>
@@ -11177,7 +11183,7 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
@@ -11190,21 +11196,19 @@
       <c r="K138" s="7" t="n"/>
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
-      <c r="N138" s="7" t="n">
-        <v>16664</v>
-      </c>
+      <c r="N138" s="7" t="n"/>
       <c r="O138" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11221,7 +11225,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
+          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
         </is>
       </c>
     </row>
@@ -11235,13 +11239,13 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>3200</v>
+        <v>1395</v>
       </c>
       <c r="D139" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E139" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
@@ -11250,7 +11254,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11264,7 +11268,7 @@
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>16664</v>
+        <v>20524</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11272,12 +11276,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>LettingaProperty.com, Nationwide - Lettings</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11294,7 +11298,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
@@ -11308,7 +11312,7 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="D140" s="7" t="n">
         <v>1</v>
@@ -11318,26 +11322,28 @@
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Sweetman Place, Bristol, BS2 0JN</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I140" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I140" s="7" t="n">
+        <v>452</v>
+      </c>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>21996</v>
+        <v>20472</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11345,12 +11351,12 @@
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11367,7 +11373,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
+          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
         </is>
       </c>
     </row>
@@ -11381,13 +11387,13 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>2400</v>
+        <v>1450</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E141" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
@@ -11396,7 +11402,7 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Colston Avenue, Bristol, BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
@@ -11410,7 +11416,7 @@
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>14108</v>
+        <v>16664</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11418,12 +11424,12 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11440,7 +11446,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
+          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
         </is>
       </c>
     </row>
@@ -11454,13 +11460,13 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>1300</v>
+        <v>3200</v>
       </c>
       <c r="D142" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E142" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
@@ -11469,23 +11475,21 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>East Street, Bedminster, BS3</t>
+          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I142" s="7" t="n">
-        <v>560</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I142" s="7" t="n"/>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>14176</v>
+        <v>16664</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11493,12 +11497,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Xeno Property, Bristol</t>
+          <t>LettingaProperty.com, Nationwide - Lettings</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11515,7 +11519,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
+          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
         </is>
       </c>
     </row>
@@ -11529,7 +11533,7 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1450</v>
+        <v>1600</v>
       </c>
       <c r="D143" s="7" t="n">
         <v>1</v>
@@ -11544,7 +11548,7 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
@@ -11558,7 +11562,7 @@
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>13668</v>
+        <v>21996</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11566,12 +11570,12 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>Wildheart Residential Management Limited, Epsom</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11588,7 +11592,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
+          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
         </is>
       </c>
     </row>
@@ -11602,13 +11606,13 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1605</v>
+        <v>2400</v>
       </c>
       <c r="D144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
@@ -11617,7 +11621,7 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Colston Avenue, Bristol, BS1</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
@@ -11625,15 +11629,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I144" s="7" t="n">
-        <v>487</v>
-      </c>
+      <c r="I144" s="7" t="n"/>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>13860</v>
+        <v>14108</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11641,12 +11643,12 @@
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11663,7 +11665,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
+          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
         </is>
       </c>
     </row>
@@ -11677,13 +11679,13 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>2185</v>
+        <v>1300</v>
       </c>
       <c r="D145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
@@ -11692,23 +11694,23 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>East Street, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I145" s="7" t="n">
-        <v>721</v>
+        <v>560</v>
       </c>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>13860</v>
+        <v>14176</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11716,12 +11718,12 @@
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Xeno Property, Bristol</t>
         </is>
       </c>
       <c r="S145" s="8" t="inlineStr"/>
@@ -11738,7 +11740,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
+          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
         </is>
       </c>
     </row>
@@ -11752,7 +11754,7 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>1640</v>
+        <v>1450</v>
       </c>
       <c r="D146" s="7" t="n">
         <v>1</v>
@@ -11767,7 +11769,7 @@
       </c>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Welsh Back, Bristol</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
@@ -11775,15 +11777,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I146" s="7" t="n">
-        <v>484</v>
-      </c>
+      <c r="I146" s="7" t="n"/>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>13860</v>
+        <v>13668</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>0</v>
@@ -11791,12 +11791,12 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Wildheart Residential Management Limited, Epsom</t>
         </is>
       </c>
       <c r="S146" s="8" t="inlineStr"/>
@@ -11813,7 +11813,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
+          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
         </is>
       </c>
     </row>
@@ -11827,13 +11827,13 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>2010</v>
+        <v>1605</v>
       </c>
       <c r="D147" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E147" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F147" s="7" t="inlineStr">
         <is>
@@ -11851,7 +11851,7 @@
         </is>
       </c>
       <c r="I147" s="7" t="n">
-        <v>722</v>
+        <v>487</v>
       </c>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
@@ -11866,7 +11866,7 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
@@ -11888,7 +11888,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
+          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
         </is>
       </c>
     </row>
@@ -11902,13 +11902,13 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>1635</v>
+        <v>2185</v>
       </c>
       <c r="D148" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E148" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
@@ -11926,14 +11926,14 @@
         </is>
       </c>
       <c r="I148" s="7" t="n">
-        <v>560</v>
+        <v>721</v>
       </c>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O148" s="7" t="n">
         <v>0</v>
@@ -11941,12 +11941,12 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11963,7 +11963,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
+          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
         </is>
       </c>
     </row>
@@ -11977,7 +11977,7 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>1665</v>
+        <v>1640</v>
       </c>
       <c r="D149" s="7" t="n">
         <v>1</v>
@@ -11992,7 +11992,7 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H149" s="7" t="inlineStr">
@@ -12001,14 +12001,14 @@
         </is>
       </c>
       <c r="I149" s="7" t="n">
-        <v>434</v>
+        <v>484</v>
       </c>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O149" s="7" t="n">
         <v>0</v>
@@ -12016,12 +12016,12 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S149" s="8" t="inlineStr"/>
@@ -12038,7 +12038,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
+          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
         </is>
       </c>
     </row>
@@ -12052,7 +12052,7 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1990</v>
+        <v>2010</v>
       </c>
       <c r="D150" s="7" t="n">
         <v>2</v>
@@ -12067,7 +12067,7 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
@@ -12076,27 +12076,27 @@
         </is>
       </c>
       <c r="I150" s="7" t="n">
-        <v>682</v>
+        <v>722</v>
       </c>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O150" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12113,7 +12113,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
+          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
         </is>
       </c>
     </row>
@@ -12127,7 +12127,7 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1480</v>
+        <v>1635</v>
       </c>
       <c r="D151" s="7" t="n">
         <v>1</v>
@@ -12151,7 +12151,7 @@
         </is>
       </c>
       <c r="I151" s="7" t="n">
-        <v>417</v>
+        <v>560</v>
       </c>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
@@ -12161,12 +12161,12 @@
         <v>13356</v>
       </c>
       <c r="O151" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R151" s="7" t="inlineStr">
@@ -12188,7 +12188,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
+          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
         </is>
       </c>
     </row>
@@ -12202,13 +12202,13 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1750</v>
+        <v>1665</v>
       </c>
       <c r="D152" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E152" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
@@ -12217,7 +12217,7 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
@@ -12225,13 +12225,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I152" s="7" t="n"/>
+      <c r="I152" s="7" t="n">
+        <v>434</v>
+      </c>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>20828</v>
+        <v>13964</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12239,12 +12241,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12261,7 +12263,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
+          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
         </is>
       </c>
     </row>
@@ -12275,7 +12277,7 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>2080</v>
+        <v>1990</v>
       </c>
       <c r="D153" s="7" t="n">
         <v>2</v>
@@ -12290,7 +12292,7 @@
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
@@ -12299,14 +12301,14 @@
         </is>
       </c>
       <c r="I153" s="7" t="n">
-        <v>705</v>
+        <v>682</v>
       </c>
       <c r="J153" s="7" t="n"/>
       <c r="K153" s="7" t="n"/>
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O153" s="7" t="n">
         <v>1</v>
@@ -12314,12 +12316,12 @@
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12336,7 +12338,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
+          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
         </is>
       </c>
     </row>
@@ -12350,7 +12352,7 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1680</v>
+        <v>1480</v>
       </c>
       <c r="D154" s="7" t="n">
         <v>1</v>
@@ -12374,7 +12376,7 @@
         </is>
       </c>
       <c r="I154" s="7" t="n">
-        <v>487</v>
+        <v>417</v>
       </c>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
@@ -12389,7 +12391,7 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
@@ -12411,7 +12413,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
+          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
         </is>
       </c>
     </row>
@@ -12425,7 +12427,7 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>1845</v>
+        <v>1750</v>
       </c>
       <c r="D155" s="7" t="n">
         <v>2</v>
@@ -12440,7 +12442,7 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
@@ -12448,15 +12450,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I155" s="7" t="n">
-        <v>641</v>
-      </c>
+      <c r="I155" s="7" t="n"/>
       <c r="J155" s="7" t="n"/>
       <c r="K155" s="7" t="n"/>
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="7" t="n">
-        <v>21476</v>
+        <v>20828</v>
       </c>
       <c r="O155" s="7" t="n">
         <v>0</v>
@@ -12464,12 +12464,12 @@
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12486,7 +12486,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
+          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
         </is>
       </c>
     </row>
@@ -12500,13 +12500,13 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>1685</v>
+        <v>2080</v>
       </c>
       <c r="D156" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E156" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F156" s="7" t="inlineStr">
         <is>
@@ -12524,7 +12524,7 @@
         </is>
       </c>
       <c r="I156" s="7" t="n">
-        <v>578</v>
+        <v>705</v>
       </c>
       <c r="J156" s="7" t="n"/>
       <c r="K156" s="7" t="n"/>
@@ -12539,7 +12539,7 @@
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
@@ -12561,7 +12561,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
+          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
         </is>
       </c>
     </row>
@@ -12575,7 +12575,7 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>1765</v>
+        <v>1680</v>
       </c>
       <c r="D157" s="7" t="n">
         <v>1</v>
@@ -12599,7 +12599,7 @@
         </is>
       </c>
       <c r="I157" s="7" t="n">
-        <v>641</v>
+        <v>487</v>
       </c>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
@@ -12614,7 +12614,7 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
@@ -12636,7 +12636,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
+          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
         </is>
       </c>
     </row>
@@ -12650,7 +12650,7 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>2240</v>
+        <v>1845</v>
       </c>
       <c r="D158" s="7" t="n">
         <v>2</v>
@@ -12665,7 +12665,7 @@
       </c>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H158" s="7" t="inlineStr">
@@ -12674,14 +12674,14 @@
         </is>
       </c>
       <c r="I158" s="7" t="n">
-        <v>884</v>
+        <v>641</v>
       </c>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>13388</v>
+        <v>21476</v>
       </c>
       <c r="O158" s="7" t="n">
         <v>0</v>
@@ -12689,12 +12689,12 @@
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S158" s="8" t="inlineStr"/>
@@ -12711,7 +12711,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
+          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
         </is>
       </c>
     </row>
@@ -12725,7 +12725,7 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1150</v>
+        <v>1685</v>
       </c>
       <c r="D159" s="7" t="n">
         <v>1</v>
@@ -12740,7 +12740,7 @@
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>John Street, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
@@ -12749,25 +12749,27 @@
         </is>
       </c>
       <c r="I159" s="7" t="n">
-        <v>248</v>
+        <v>578</v>
       </c>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
-      <c r="N159" s="7" t="n"/>
+      <c r="N159" s="7" t="n">
+        <v>13356</v>
+      </c>
       <c r="O159" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12784,7 +12786,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
+          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
         </is>
       </c>
     </row>
@@ -12798,36 +12800,38 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>3400</v>
+        <v>1765</v>
       </c>
       <c r="D160" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E160" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F160" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>Barton Road, Bristol, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H160" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I160" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I160" s="7" t="n">
+        <v>641</v>
+      </c>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
       <c r="N160" s="7" t="n">
-        <v>19720</v>
+        <v>13356</v>
       </c>
       <c r="O160" s="7" t="n">
         <v>1</v>
@@ -12835,12 +12839,12 @@
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S160" s="8" t="inlineStr"/>
@@ -12857,7 +12861,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
+          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
         </is>
       </c>
     </row>
@@ -12871,13 +12875,13 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>1250</v>
+        <v>2240</v>
       </c>
       <c r="D161" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E161" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F161" s="7" t="inlineStr">
         <is>
@@ -12886,34 +12890,36 @@
       </c>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>St Peters Court, Bedminster</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H161" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I161" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I161" s="7" t="n">
+        <v>884</v>
+      </c>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
       <c r="N161" s="7" t="n">
-        <v>15352</v>
+        <v>13388</v>
       </c>
       <c r="O161" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S161" s="8" t="inlineStr"/>
@@ -12930,7 +12936,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
+          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
         </is>
       </c>
     </row>
@@ -12944,13 +12950,13 @@
         </is>
       </c>
       <c r="C162" s="9" t="n">
-        <v>2300</v>
+        <v>1150</v>
       </c>
       <c r="D162" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E162" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F162" s="7" t="inlineStr">
         <is>
@@ -12959,36 +12965,34 @@
       </c>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>John Street, BS1</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I162" s="7" t="n">
-        <v>773</v>
+        <v>248</v>
       </c>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
-      <c r="N162" s="7" t="n">
-        <v>14172</v>
-      </c>
+      <c r="N162" s="7" t="n"/>
       <c r="O162" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P162" s="7" t="n"/>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S162" s="8" t="inlineStr"/>
@@ -13005,7 +13009,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>08411d7c5a6f10970306f10b45d00f0717234e1f</t>
+          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
         </is>
       </c>
     </row>
@@ -13019,22 +13023,22 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1200</v>
+        <v>3400</v>
       </c>
       <c r="D163" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E163" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F163" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
+          <t>Barton Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
@@ -13042,15 +13046,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I163" s="7" t="n">
-        <v>517</v>
-      </c>
+      <c r="I163" s="7" t="n"/>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="7" t="n">
-        <v>21904</v>
+        <v>19720</v>
       </c>
       <c r="O163" s="7" t="n">
         <v>1</v>
@@ -13058,12 +13060,12 @@
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13080,7 +13082,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>e87a39f40860abe2278117f28f53ec7cbbd1d241</t>
+          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
         </is>
       </c>
     </row>
@@ -13094,7 +13096,7 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>1630</v>
+        <v>1250</v>
       </c>
       <c r="D164" s="7" t="n">
         <v>1</v>
@@ -13109,36 +13111,34 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>St Peters Court, Bedminster</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I164" s="7" t="n">
-        <v>486</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I164" s="7" t="n"/>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="7" t="n">
-        <v>13860</v>
+        <v>15352</v>
       </c>
       <c r="O164" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13155,7 +13155,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
+          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
         </is>
       </c>
     </row>
@@ -13169,13 +13169,13 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1640</v>
+        <v>2300</v>
       </c>
       <c r="D165" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E165" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F165" s="7" t="inlineStr">
         <is>
@@ -13184,36 +13184,36 @@
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H165" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I165" s="7" t="n">
-        <v>487</v>
+        <v>773</v>
       </c>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>13356</v>
+        <v>14172</v>
       </c>
       <c r="O165" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R165" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S165" s="8" t="inlineStr"/>
@@ -13230,7 +13230,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>ecc803f25866be367a83778bda0456688426a26e</t>
+          <t>08411d7c5a6f10970306f10b45d00f0717234e1f</t>
         </is>
       </c>
     </row>
@@ -13244,13 +13244,13 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>2085</v>
+        <v>1200</v>
       </c>
       <c r="D166" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E166" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F166" s="7" t="inlineStr">
         <is>
@@ -13259,36 +13259,36 @@
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
         </is>
       </c>
       <c r="H166" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I166" s="7" t="n">
-        <v>722</v>
+        <v>517</v>
       </c>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="7" t="n">
-        <v>13860</v>
+        <v>21904</v>
       </c>
       <c r="O166" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
@@ -13305,7 +13305,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
+          <t>e87a39f40860abe2278117f28f53ec7cbbd1d241</t>
         </is>
       </c>
     </row>
@@ -13319,7 +13319,7 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>1650</v>
+        <v>1630</v>
       </c>
       <c r="D167" s="7" t="n">
         <v>1</v>
@@ -13334,7 +13334,7 @@
       </c>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H167" s="7" t="inlineStr">
@@ -13343,14 +13343,14 @@
         </is>
       </c>
       <c r="I167" s="7" t="n">
-        <v>553</v>
+        <v>486</v>
       </c>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O167" s="7" t="n">
         <v>0</v>
@@ -13358,12 +13358,12 @@
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S167" s="8" t="inlineStr"/>
@@ -13380,7 +13380,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
+          <t>df0c16effec13d09d19ae06478084aa14aedef28</t>
         </is>
       </c>
     </row>
@@ -13394,7 +13394,7 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1350</v>
+        <v>1640</v>
       </c>
       <c r="D168" s="7" t="n">
         <v>1</v>
@@ -13409,7 +13409,7 @@
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Wapping Wharf, Anchorage, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
@@ -13418,14 +13418,14 @@
         </is>
       </c>
       <c r="I168" s="7" t="n">
-        <v>518</v>
+        <v>487</v>
       </c>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="7" t="n">
-        <v>16664</v>
+        <v>13356</v>
       </c>
       <c r="O168" s="7" t="n">
         <v>0</v>
@@ -13433,12 +13433,12 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13455,7 +13455,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>61cb6cbca03d4b33a5e567abbe422df6574deb7a</t>
+          <t>ecc803f25866be367a83778bda0456688426a26e</t>
         </is>
       </c>
     </row>
@@ -13469,13 +13469,13 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1550</v>
+        <v>2085</v>
       </c>
       <c r="D169" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E169" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
@@ -13484,21 +13484,23 @@
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Crown And Anchor House, Temple Quay, Temple Quay, BS2</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I169" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I169" s="7" t="n">
+        <v>722</v>
+      </c>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>20472</v>
+        <v>13860</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13506,12 +13508,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13528,7 +13530,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>e76245b9d5be47e78934469ea3c31d3d0433291c</t>
+          <t>4e31a77443c6836b221dcaa241ec4e65b0f0f117</t>
         </is>
       </c>
     </row>
@@ -13542,7 +13544,7 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>1665</v>
+        <v>1650</v>
       </c>
       <c r="D170" s="7" t="n">
         <v>1</v>
@@ -13566,7 +13568,7 @@
         </is>
       </c>
       <c r="I170" s="7" t="n">
-        <v>569</v>
+        <v>553</v>
       </c>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
@@ -13581,7 +13583,7 @@
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
@@ -13603,7 +13605,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>22588bce8839df85d69555bd640fcbb3902101ff</t>
+          <t>38f5522a4668f50fa87475e0579a5151b4dbf30b</t>
         </is>
       </c>
     </row>
@@ -13617,36 +13619,38 @@
         </is>
       </c>
       <c r="C171" s="9" t="n">
-        <v>1850</v>
+        <v>1350</v>
       </c>
       <c r="D171" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E171" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F171" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>Webb Street, Bristol, BS5</t>
+          <t>Wapping Wharf, Anchorage, BS1</t>
         </is>
       </c>
       <c r="H171" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
-        </is>
-      </c>
-      <c r="I171" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I171" s="7" t="n">
+        <v>518</v>
+      </c>
       <c r="J171" s="7" t="n"/>
       <c r="K171" s="7" t="n"/>
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="7" t="n">
-        <v>19580</v>
+        <v>16664</v>
       </c>
       <c r="O171" s="7" t="n">
         <v>0</v>
@@ -13654,12 +13658,12 @@
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -13676,7 +13680,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
+          <t>61cb6cbca03d4b33a5e567abbe422df6574deb7a</t>
         </is>
       </c>
     </row>
@@ -13690,10 +13694,10 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1200</v>
+        <v>1550</v>
       </c>
       <c r="D172" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E172" s="7" t="n">
         <v>1</v>
@@ -13705,12 +13709,12 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>Bushy Park, The Bank Bushy Park, BS4</t>
+          <t>Crown And Anchor House, Temple Quay, Temple Quay, BS2</t>
         </is>
       </c>
       <c r="H172" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I172" s="7" t="n"/>
@@ -13719,7 +13723,7 @@
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="7" t="n">
-        <v>7216</v>
+        <v>20472</v>
       </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
@@ -13727,12 +13731,12 @@
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -13749,7 +13753,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
+          <t>e76245b9d5be47e78934469ea3c31d3d0433291c</t>
         </is>
       </c>
     </row>
@@ -13763,13 +13767,13 @@
         </is>
       </c>
       <c r="C173" s="9" t="n">
-        <v>1750</v>
+        <v>1665</v>
       </c>
       <c r="D173" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E173" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
@@ -13778,7 +13782,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Number One Bristol, Bristol</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
@@ -13786,13 +13790,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I173" s="7" t="n"/>
+      <c r="I173" s="7" t="n">
+        <v>569</v>
+      </c>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>21808</v>
+        <v>13356</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13805,7 +13811,7 @@
       </c>
       <c r="R173" s="7" t="inlineStr">
         <is>
-          <t>Zest, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -13822,7 +13828,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>d2b416547517343eef3a43500d63f738ac4ae423</t>
+          <t>22588bce8839df85d69555bd640fcbb3902101ff</t>
         </is>
       </c>
     </row>
@@ -13836,38 +13842,36 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1295</v>
+        <v>1850</v>
       </c>
       <c r="D174" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E174" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F174" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Great Western House, BS1</t>
+          <t>Webb Street, Bristol, BS5</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I174" s="7" t="n">
-        <v>474</v>
-      </c>
+          <t>BS5</t>
+        </is>
+      </c>
+      <c r="I174" s="7" t="n"/>
       <c r="J174" s="7" t="n"/>
       <c r="K174" s="7" t="n"/>
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>14412</v>
+        <v>19580</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13875,12 +13879,12 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -13897,7 +13901,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>466dad45b709c8ce2ab5e9d022bce4baabb5cecc</t>
+          <t>aef99c3165f6b6530e2b7bb4c35465760a386735</t>
         </is>
       </c>
     </row>
@@ -13911,7 +13915,7 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>1325</v>
+        <v>1200</v>
       </c>
       <c r="D175" s="7" t="n">
         <v>1</v>
@@ -13926,12 +13930,12 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Broad Street, Bristol, BS1</t>
+          <t>Bushy Park, The Bank Bushy Park, BS4</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I175" s="7" t="n"/>
@@ -13940,7 +13944,7 @@
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
       <c r="N175" s="7" t="n">
-        <v>21788</v>
+        <v>7216</v>
       </c>
       <c r="O175" s="7" t="n">
         <v>0</v>
@@ -13948,12 +13952,12 @@
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -13970,7 +13974,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
+          <t>66c0cb8192a0b0f430860f03a41c731d52b6e9aa</t>
         </is>
       </c>
     </row>
@@ -13984,7 +13988,7 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>2200</v>
+        <v>1750</v>
       </c>
       <c r="D176" s="7" t="n">
         <v>2</v>
@@ -13999,7 +14003,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
+          <t>Number One Bristol, Bristol</t>
         </is>
       </c>
       <c r="H176" s="7" t="inlineStr">
@@ -14013,7 +14017,7 @@
       <c r="L176" s="7" t="n"/>
       <c r="M176" s="7" t="n"/>
       <c r="N176" s="7" t="n">
-        <v>16788</v>
+        <v>21808</v>
       </c>
       <c r="O176" s="7" t="n">
         <v>0</v>
@@ -14021,12 +14025,12 @@
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Zest, Bristol</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -14043,7 +14047,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
+          <t>d2b416547517343eef3a43500d63f738ac4ae423</t>
         </is>
       </c>
     </row>
@@ -14057,7 +14061,7 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>1500</v>
+        <v>1295</v>
       </c>
       <c r="D177" s="7" t="n">
         <v>1</v>
@@ -14072,7 +14076,7 @@
       </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>Eclipse, Broad Weir, Bristol</t>
+          <t>Harbourside, Great Western House, BS1</t>
         </is>
       </c>
       <c r="H177" s="7" t="inlineStr">
@@ -14080,13 +14084,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I177" s="7" t="n"/>
+      <c r="I177" s="7" t="n">
+        <v>474</v>
+      </c>
       <c r="J177" s="7" t="n"/>
       <c r="K177" s="7" t="n"/>
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
       <c r="N177" s="7" t="n">
-        <v>22164</v>
+        <v>14412</v>
       </c>
       <c r="O177" s="7" t="n">
         <v>0</v>
@@ -14094,12 +14100,12 @@
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
         <is>
-          <t>Martin &amp; Co, Bath</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S177" s="8" t="inlineStr"/>
@@ -14116,7 +14122,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
+          <t>466dad45b709c8ce2ab5e9d022bce4baabb5cecc</t>
         </is>
       </c>
     </row>
@@ -14130,7 +14136,7 @@
         </is>
       </c>
       <c r="C178" s="9" t="n">
-        <v>1800</v>
+        <v>1325</v>
       </c>
       <c r="D178" s="7" t="n">
         <v>1</v>
@@ -14145,7 +14151,7 @@
       </c>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t>Broad Weir, City Centre, Bristol, BS1</t>
+          <t>Broad Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H178" s="7" t="inlineStr">
@@ -14153,15 +14159,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I178" s="7" t="n">
-        <v>474</v>
-      </c>
+      <c r="I178" s="7" t="n"/>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
       <c r="L178" s="7" t="n"/>
       <c r="M178" s="7" t="n"/>
       <c r="N178" s="7" t="n">
-        <v>22080</v>
+        <v>21788</v>
       </c>
       <c r="O178" s="7" t="n">
         <v>0</v>
@@ -14169,12 +14173,12 @@
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
         <is>
-          <t>CJ Hole, Clifton</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S178" s="8" t="inlineStr"/>
@@ -14191,7 +14195,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
+          <t>3761bbfac8c5ddd7f51121e3d8fabe2b13e98db4</t>
         </is>
       </c>
     </row>
@@ -14205,13 +14209,13 @@
         </is>
       </c>
       <c r="C179" s="9" t="n">
-        <v>1300</v>
+        <v>2200</v>
       </c>
       <c r="D179" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E179" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
@@ -14220,7 +14224,7 @@
       </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Deanery Road, BS1 5AF</t>
+          <t>The Crescent, Hannover Quay, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H179" s="7" t="inlineStr">
@@ -14228,15 +14232,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I179" s="7" t="n">
-        <v>570</v>
-      </c>
+      <c r="I179" s="7" t="n"/>
       <c r="J179" s="7" t="n"/>
       <c r="K179" s="7" t="n"/>
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
       <c r="N179" s="7" t="n">
-        <v>19300</v>
+        <v>16788</v>
       </c>
       <c r="O179" s="7" t="n">
         <v>0</v>
@@ -14244,12 +14246,12 @@
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Clifton</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -14266,7 +14268,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
+          <t>40cd3b6f189ef431d57aa8f6bcda5d67740edb54</t>
         </is>
       </c>
     </row>
@@ -14280,13 +14282,13 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E180" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F180" s="7" t="inlineStr">
         <is>
@@ -14295,12 +14297,12 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>Eclipse, Broad Weir, Bristol</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I180" s="7" t="n"/>
@@ -14309,7 +14311,7 @@
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="7" t="n">
-        <v>21360</v>
+        <v>22164</v>
       </c>
       <c r="O180" s="7" t="n">
         <v>0</v>
@@ -14317,12 +14319,12 @@
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>Martin &amp; Co, Bath</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14339,7 +14341,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
+          <t>7f548d57ee03a8e44411e6ddef298583dbcff454</t>
         </is>
       </c>
     </row>
@@ -14353,10 +14355,10 @@
         </is>
       </c>
       <c r="C181" s="9" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="D181" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E181" s="7" t="n">
         <v>1</v>
@@ -14368,21 +14370,23 @@
       </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>Crown &amp; Anchor House, Bristol, BS2</t>
+          <t>Broad Weir, City Centre, Bristol, BS1</t>
         </is>
       </c>
       <c r="H181" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I181" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I181" s="7" t="n">
+        <v>474</v>
+      </c>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="7" t="n">
-        <v>20472</v>
+        <v>22080</v>
       </c>
       <c r="O181" s="7" t="n">
         <v>0</v>
@@ -14390,12 +14394,12 @@
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>CJ Hole, Clifton</t>
         </is>
       </c>
       <c r="S181" s="8" t="inlineStr"/>
@@ -14412,7 +14416,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
+          <t>b1d0054a7e91f9c193f0edd9741c7de04d9f3ae5</t>
         </is>
       </c>
     </row>
@@ -14426,13 +14430,13 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>1450</v>
+        <v>1300</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E182" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
@@ -14441,23 +14445,23 @@
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Woodbridge Road, Bristol, BS4</t>
+          <t>City Centre, Deanery Road, BS1 5AF</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I182" s="7" t="n">
-        <v>678</v>
+        <v>570</v>
       </c>
       <c r="J182" s="7" t="n"/>
       <c r="K182" s="7" t="n"/>
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>5700</v>
+        <v>19300</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14465,12 +14469,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>The Bristol Residential Letting Co, Clifton</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14487,7 +14491,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
+          <t>e283466e90e9ed628744c068e51436d40c54df63</t>
         </is>
       </c>
     </row>
@@ -14501,12 +14505,14 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>1450</v>
+        <v>2500</v>
       </c>
       <c r="D183" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E183" s="7" t="n"/>
+      <c r="E183" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="F183" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -14514,12 +14520,12 @@
       </c>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t>Stapleton Road, Bristol, BS5</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H183" s="7" t="inlineStr">
         <is>
-          <t>BS5</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I183" s="7" t="n"/>
@@ -14528,20 +14534,20 @@
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="7" t="n">
-        <v>19488</v>
+        <v>21360</v>
       </c>
       <c r="O183" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">
         <is>
-          <t>Phoenix Property Company, Bristol</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S183" s="8" t="inlineStr"/>
@@ -14558,7 +14564,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
+          <t>e1df346a81811cc10b08914fa9dfdc676b041ab1</t>
         </is>
       </c>
     </row>
@@ -14572,10 +14578,10 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>1500</v>
+        <v>1650</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E184" s="7" t="n">
         <v>1</v>
@@ -14587,12 +14593,12 @@
       </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Crown &amp; Anchor House, Bristol, BS2</t>
         </is>
       </c>
       <c r="H184" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I184" s="7" t="n"/>
@@ -14601,7 +14607,7 @@
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
       <c r="N184" s="7" t="n">
-        <v>20768</v>
+        <v>20472</v>
       </c>
       <c r="O184" s="7" t="n">
         <v>0</v>
@@ -14609,12 +14615,12 @@
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S184" s="8" t="inlineStr"/>
@@ -14631,7 +14637,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
+          <t>3525b51aece5997254983946ed3fc64c7343c2cc</t>
         </is>
       </c>
     </row>
@@ -14645,7 +14651,7 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>2250</v>
+        <v>1450</v>
       </c>
       <c r="D185" s="7" t="n">
         <v>3</v>
@@ -14655,28 +14661,28 @@
       </c>
       <c r="F185" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>Newfoundland Road, Bristol, BS2</t>
+          <t>Woodbridge Road, Bristol, BS4</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I185" s="7" t="n">
-        <v>980</v>
+        <v>678</v>
       </c>
       <c r="J185" s="7" t="n"/>
       <c r="K185" s="7" t="n"/>
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="7" t="n">
-        <v>19800</v>
+        <v>5700</v>
       </c>
       <c r="O185" s="7" t="n">
         <v>0</v>
@@ -14684,12 +14690,12 @@
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
-          <t>Lets Rent Bristol, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S185" s="8" t="inlineStr"/>
@@ -14706,7 +14712,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
+          <t>2863956fd49205f9a06c7a0d686fde88889e07a2</t>
         </is>
       </c>
     </row>
@@ -14720,14 +14726,12 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>2000</v>
+        <v>1450</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E186" s="7" t="n">
-        <v>2</v>
-      </c>
+      <c r="E186" s="7" t="n"/>
       <c r="F186" s="7" t="inlineStr">
         <is>
           <t>flat</t>
@@ -14735,12 +14739,12 @@
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Protheroes House, Hobbs Lane, BS1</t>
+          <t>Stapleton Road, Bristol, BS5</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS5</t>
         </is>
       </c>
       <c r="I186" s="7" t="n"/>
@@ -14749,20 +14753,20 @@
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>13584</v>
+        <v>19488</v>
       </c>
       <c r="O186" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Phoenix Property Company, Bristol</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14779,7 +14783,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
+          <t>9696d556a9ab494e09c67abf76046ac09e9d61cc</t>
         </is>
       </c>
     </row>
@@ -14793,27 +14797,27 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>2400</v>
+        <v>1500</v>
       </c>
       <c r="D187" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E187" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F187" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>Balmain Street, Totterdown, Bristol, BS4</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I187" s="7" t="n"/>
@@ -14822,7 +14826,7 @@
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>5524</v>
+        <v>20768</v>
       </c>
       <c r="O187" s="7" t="n">
         <v>0</v>
@@ -14830,12 +14834,12 @@
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Henleaze</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S187" s="8" t="inlineStr"/>
@@ -14852,7 +14856,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>dd411af39a083f886127138c0a969254da83858b</t>
+          <t>7d11c2bfe6cdedc7cbec4b6e98068599a06dfcc8</t>
         </is>
       </c>
     </row>
@@ -14866,51 +14870,51 @@
         </is>
       </c>
       <c r="C188" s="9" t="n">
-        <v>1665</v>
+        <v>2250</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F188" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Newfoundland Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I188" s="7" t="n">
-        <v>578</v>
+        <v>980</v>
       </c>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
       <c r="L188" s="7" t="n"/>
       <c r="M188" s="7" t="n"/>
       <c r="N188" s="7" t="n">
-        <v>13356</v>
+        <v>19800</v>
       </c>
       <c r="O188" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Lets Rent Bristol, Bristol</t>
         </is>
       </c>
       <c r="S188" s="8" t="inlineStr"/>
@@ -14927,7 +14931,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
+          <t>64b0803e14c5bc0dc4823b988957a7c787f244e8</t>
         </is>
       </c>
     </row>
@@ -14941,13 +14945,13 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>1635</v>
+        <v>2000</v>
       </c>
       <c r="D189" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E189" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F189" s="7" t="inlineStr">
         <is>
@@ -14956,7 +14960,7 @@
       </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Protheroes House, Hobbs Lane, BS1</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
@@ -14964,28 +14968,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I189" s="7" t="n">
-        <v>485</v>
-      </c>
+      <c r="I189" s="7" t="n"/>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
       <c r="L189" s="7" t="n"/>
       <c r="M189" s="7" t="n"/>
       <c r="N189" s="7" t="n">
-        <v>13860</v>
+        <v>13584</v>
       </c>
       <c r="O189" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R189" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S189" s="8" t="inlineStr"/>
@@ -15002,7 +15004,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
+          <t>1f3cd55b7034f070e5f4ad05fa149569c375c4fe</t>
         </is>
       </c>
     </row>
@@ -15016,51 +15018,49 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>1615</v>
+        <v>2400</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E190" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F190" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Balmain Street, Totterdown, Bristol, BS4</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I190" s="7" t="n">
-        <v>487</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I190" s="7" t="n"/>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="7" t="n">
-        <v>13860</v>
+        <v>5524</v>
       </c>
       <c r="O190" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Letting Game, Henleaze</t>
         </is>
       </c>
       <c r="S190" s="8" t="inlineStr"/>
@@ -15077,7 +15077,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
+          <t>dd411af39a083f886127138c0a969254da83858b</t>
         </is>
       </c>
     </row>
@@ -15091,7 +15091,7 @@
         </is>
       </c>
       <c r="C191" s="9" t="n">
-        <v>1640</v>
+        <v>1665</v>
       </c>
       <c r="D191" s="7" t="n">
         <v>1</v>
@@ -15115,7 +15115,7 @@
         </is>
       </c>
       <c r="I191" s="7" t="n">
-        <v>560</v>
+        <v>578</v>
       </c>
       <c r="J191" s="7" t="n"/>
       <c r="K191" s="7" t="n"/>
@@ -15130,7 +15130,7 @@
       <c r="P191" s="7" t="n"/>
       <c r="Q191" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R191" s="7" t="inlineStr">
@@ -15152,7 +15152,7 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
-          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
+          <t>084a3845d376c7de92b6c65268745abc4ef7e8b7</t>
         </is>
       </c>
     </row>
@@ -15166,7 +15166,7 @@
         </is>
       </c>
       <c r="C192" s="9" t="n">
-        <v>1615</v>
+        <v>1635</v>
       </c>
       <c r="D192" s="7" t="n">
         <v>1</v>
@@ -15190,7 +15190,7 @@
         </is>
       </c>
       <c r="I192" s="7" t="n">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="J192" s="7" t="n"/>
       <c r="K192" s="7" t="n"/>
@@ -15205,7 +15205,7 @@
       <c r="P192" s="7" t="n"/>
       <c r="Q192" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="R192" s="7" t="inlineStr">
@@ -15227,7 +15227,7 @@
       <c r="V192" s="6" t="inlineStr"/>
       <c r="W192" s="7" t="inlineStr">
         <is>
-          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
+          <t>33dd09721d062d4d665bfbc7b969a57a7c1de111</t>
         </is>
       </c>
     </row>
@@ -15265,7 +15265,7 @@
         </is>
       </c>
       <c r="I193" s="7" t="n">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J193" s="7" t="n"/>
       <c r="K193" s="7" t="n"/>
@@ -15275,12 +15275,12 @@
         <v>13860</v>
       </c>
       <c r="O193" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P193" s="7" t="n"/>
       <c r="Q193" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="R193" s="7" t="inlineStr">
@@ -15302,7 +15302,7 @@
       <c r="V193" s="6" t="inlineStr"/>
       <c r="W193" s="7" t="inlineStr">
         <is>
-          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
+          <t>9cff0990c507752682af58c22f5de8882d7b889a</t>
         </is>
       </c>
     </row>
@@ -15316,7 +15316,7 @@
         </is>
       </c>
       <c r="C194" s="9" t="n">
-        <v>1645</v>
+        <v>1640</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>1</v>
@@ -15340,7 +15340,7 @@
         </is>
       </c>
       <c r="I194" s="7" t="n">
-        <v>570</v>
+        <v>560</v>
       </c>
       <c r="J194" s="7" t="n"/>
       <c r="K194" s="7" t="n"/>
@@ -15350,12 +15350,12 @@
         <v>13356</v>
       </c>
       <c r="O194" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P194" s="7" t="n"/>
       <c r="Q194" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R194" s="7" t="inlineStr">
@@ -15377,7 +15377,7 @@
       <c r="V194" s="6" t="inlineStr"/>
       <c r="W194" s="7" t="inlineStr">
         <is>
-          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
+          <t>1e301b26d1bde5018a5ab8c4c2c1fa60342ab1f3</t>
         </is>
       </c>
     </row>
@@ -15391,7 +15391,7 @@
         </is>
       </c>
       <c r="C195" s="9" t="n">
-        <v>1630</v>
+        <v>1615</v>
       </c>
       <c r="D195" s="7" t="n">
         <v>1</v>
@@ -15406,7 +15406,7 @@
       </c>
       <c r="G195" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H195" s="7" t="inlineStr">
@@ -15415,27 +15415,27 @@
         </is>
       </c>
       <c r="I195" s="7" t="n">
-        <v>560</v>
+        <v>484</v>
       </c>
       <c r="J195" s="7" t="n"/>
       <c r="K195" s="7" t="n"/>
       <c r="L195" s="7" t="n"/>
       <c r="M195" s="7" t="n"/>
       <c r="N195" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O195" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P195" s="7" t="n"/>
       <c r="Q195" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R195" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S195" s="8" t="inlineStr"/>
@@ -15452,7 +15452,7 @@
       <c r="V195" s="6" t="inlineStr"/>
       <c r="W195" s="7" t="inlineStr">
         <is>
-          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
+          <t>217c66fe158c3780988189a030b436c99b0b82b1</t>
         </is>
       </c>
     </row>
@@ -15466,10 +15466,10 @@
         </is>
       </c>
       <c r="C196" s="9" t="n">
-        <v>1800</v>
+        <v>1615</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E196" s="7" t="n">
         <v>1</v>
@@ -15481,7 +15481,7 @@
       </c>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t>Bristol City Centre, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H196" s="7" t="inlineStr">
@@ -15489,13 +15489,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I196" s="7" t="n"/>
+      <c r="I196" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J196" s="7" t="n"/>
       <c r="K196" s="7" t="n"/>
       <c r="L196" s="7" t="n"/>
       <c r="M196" s="7" t="n"/>
       <c r="N196" s="7" t="n">
-        <v>21176</v>
+        <v>13860</v>
       </c>
       <c r="O196" s="7" t="n">
         <v>0</v>
@@ -15503,12 +15505,12 @@
       <c r="P196" s="7" t="n"/>
       <c r="Q196" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R196" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S196" s="8" t="inlineStr"/>
@@ -15525,7 +15527,7 @@
       <c r="V196" s="6" t="inlineStr"/>
       <c r="W196" s="7" t="inlineStr">
         <is>
-          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
+          <t>77df388b70e403c223e0fee82cc61ec662a47021</t>
         </is>
       </c>
     </row>
@@ -15539,7 +15541,7 @@
         </is>
       </c>
       <c r="C197" s="9" t="n">
-        <v>1635</v>
+        <v>1645</v>
       </c>
       <c r="D197" s="7" t="n">
         <v>1</v>
@@ -15563,7 +15565,7 @@
         </is>
       </c>
       <c r="I197" s="7" t="n">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="J197" s="7" t="n"/>
       <c r="K197" s="7" t="n"/>
@@ -15578,7 +15580,7 @@
       <c r="P197" s="7" t="n"/>
       <c r="Q197" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R197" s="7" t="inlineStr">
@@ -15600,7 +15602,7 @@
       <c r="V197" s="6" t="inlineStr"/>
       <c r="W197" s="7" t="inlineStr">
         <is>
-          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
+          <t>64cdfd96982e10d0a1a9f1074ffa8ba326f9c9e3</t>
         </is>
       </c>
     </row>
@@ -15614,10 +15616,10 @@
         </is>
       </c>
       <c r="C198" s="9" t="n">
-        <v>1925</v>
+        <v>1630</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E198" s="7" t="n">
         <v>1</v>
@@ -15629,7 +15631,7 @@
       </c>
       <c r="G198" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H198" s="7" t="inlineStr">
@@ -15638,14 +15640,14 @@
         </is>
       </c>
       <c r="I198" s="7" t="n">
-        <v>655</v>
+        <v>560</v>
       </c>
       <c r="J198" s="7" t="n"/>
       <c r="K198" s="7" t="n"/>
       <c r="L198" s="7" t="n"/>
       <c r="M198" s="7" t="n"/>
       <c r="N198" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O198" s="7" t="n">
         <v>0</v>
@@ -15653,12 +15655,12 @@
       <c r="P198" s="7" t="n"/>
       <c r="Q198" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R198" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S198" s="8" t="inlineStr"/>
@@ -15675,14 +15677,237 @@
       <c r="V198" s="6" t="inlineStr"/>
       <c r="W198" s="7" t="inlineStr">
         <is>
+          <t>f357dafd25e2f2e0e4c787830c4c61abd66eeb7e</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B199" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C199" s="9" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D199" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E199" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F199" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G199" s="8" t="inlineStr">
+        <is>
+          <t>Bristol City Centre, Bristol, BS1</t>
+        </is>
+      </c>
+      <c r="H199" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I199" s="7" t="n"/>
+      <c r="J199" s="7" t="n"/>
+      <c r="K199" s="7" t="n"/>
+      <c r="L199" s="7" t="n"/>
+      <c r="M199" s="7" t="n"/>
+      <c r="N199" s="7" t="n">
+        <v>21176</v>
+      </c>
+      <c r="O199" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P199" s="7" t="n"/>
+      <c r="Q199" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R199" s="7" t="inlineStr">
+        <is>
+          <t>OpenRent, London</t>
+        </is>
+      </c>
+      <c r="S199" s="8" t="inlineStr"/>
+      <c r="T199" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V199" s="6" t="inlineStr"/>
+      <c r="W199" s="7" t="inlineStr">
+        <is>
+          <t>3107f5d36a119e97edd5608afb96e7cedee51bfd</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B200" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C200" s="9" t="n">
+        <v>1635</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E200" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F200" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G200" s="8" t="inlineStr">
+        <is>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
+        </is>
+      </c>
+      <c r="H200" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I200" s="7" t="n">
+        <v>569</v>
+      </c>
+      <c r="J200" s="7" t="n"/>
+      <c r="K200" s="7" t="n"/>
+      <c r="L200" s="7" t="n"/>
+      <c r="M200" s="7" t="n"/>
+      <c r="N200" s="7" t="n">
+        <v>13356</v>
+      </c>
+      <c r="O200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P200" s="7" t="n"/>
+      <c r="Q200" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="R200" s="7" t="inlineStr">
+        <is>
+          <t>Grainger, Glasshouse Square</t>
+        </is>
+      </c>
+      <c r="S200" s="8" t="inlineStr"/>
+      <c r="T200" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V200" s="6" t="inlineStr"/>
+      <c r="W200" s="7" t="inlineStr">
+        <is>
+          <t>8617d451df367d072eaa97809bbdbe30e56f4306</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B201" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C201" s="9" t="n">
+        <v>1925</v>
+      </c>
+      <c r="D201" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E201" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F201" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G201" s="8" t="inlineStr">
+        <is>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+        </is>
+      </c>
+      <c r="H201" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I201" s="7" t="n">
+        <v>655</v>
+      </c>
+      <c r="J201" s="7" t="n"/>
+      <c r="K201" s="7" t="n"/>
+      <c r="L201" s="7" t="n"/>
+      <c r="M201" s="7" t="n"/>
+      <c r="N201" s="7" t="n">
+        <v>21476</v>
+      </c>
+      <c r="O201" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P201" s="7" t="n"/>
+      <c r="Q201" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="R201" s="7" t="inlineStr">
+        <is>
+          <t>Grainger, Hawkins &amp; George</t>
+        </is>
+      </c>
+      <c r="S201" s="8" t="inlineStr"/>
+      <c r="T201" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V201" s="6" t="inlineStr"/>
+      <c r="W201" s="7" t="inlineStr">
+        <is>
           <t>892dd053ae3538c7c123f255e926bef984caf6de</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W198"/>
+  <autoFilter ref="A1:W201"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15884,6 +16109,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T196" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T197" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T201" r:id="rId200"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 144
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -2369,7 +2369,7 @@
       <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
       <c r="N22" s="7" t="n">
-        <v>20780</v>
+        <v>20924</v>
       </c>
       <c r="O22" s="7" t="n">
         <v>0</v>
@@ -8054,13 +8054,13 @@
         </is>
       </c>
       <c r="C96" s="9" t="n">
-        <v>1750</v>
+        <v>1630</v>
       </c>
       <c r="D96" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E96" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" s="7" t="inlineStr">
         <is>
@@ -8069,7 +8069,7 @@
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>Number One Bristol, Bristol</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
@@ -8077,26 +8077,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I96" s="7" t="n"/>
+      <c r="I96" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J96" s="7" t="n"/>
       <c r="K96" s="7" t="n"/>
       <c r="L96" s="7" t="n"/>
       <c r="M96" s="7" t="n"/>
       <c r="N96" s="7" t="n">
-        <v>21808</v>
+        <v>13860</v>
       </c>
       <c r="O96" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P96" s="7" t="n"/>
       <c r="Q96" s="7" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R96" s="7" t="inlineStr">
         <is>
-          <t>Zest, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S96" s="8" t="inlineStr"/>
@@ -8113,7 +8115,7 @@
       <c r="V96" s="6" t="inlineStr"/>
       <c r="W96" s="7" t="inlineStr">
         <is>
-          <t>e306cbd9ac7e7fba9b5cda62260edd6014c51521</t>
+          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
         </is>
       </c>
     </row>
@@ -8127,13 +8129,13 @@
         </is>
       </c>
       <c r="C97" s="9" t="n">
-        <v>1625</v>
+        <v>1750</v>
       </c>
       <c r="D97" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E97" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
@@ -8142,7 +8144,7 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Number One Bristol, Bristol</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
@@ -8150,15 +8152,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I97" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I97" s="7" t="n"/>
       <c r="J97" s="7" t="n"/>
       <c r="K97" s="7" t="n"/>
       <c r="L97" s="7" t="n"/>
       <c r="M97" s="7" t="n"/>
       <c r="N97" s="7" t="n">
-        <v>21732</v>
+        <v>21808</v>
       </c>
       <c r="O97" s="7" t="n">
         <v>0</v>
@@ -8166,12 +8166,12 @@
       <c r="P97" s="7" t="n"/>
       <c r="Q97" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="R97" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Zest, Bristol</t>
         </is>
       </c>
       <c r="S97" s="8" t="inlineStr"/>
@@ -8188,7 +8188,7 @@
       <c r="V97" s="6" t="inlineStr"/>
       <c r="W97" s="7" t="inlineStr">
         <is>
-          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
+          <t>e306cbd9ac7e7fba9b5cda62260edd6014c51521</t>
         </is>
       </c>
     </row>
@@ -8202,13 +8202,13 @@
         </is>
       </c>
       <c r="C98" s="9" t="n">
-        <v>1965</v>
+        <v>1625</v>
       </c>
       <c r="D98" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E98" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" s="7" t="inlineStr">
         <is>
@@ -8217,7 +8217,7 @@
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
@@ -8226,14 +8226,14 @@
         </is>
       </c>
       <c r="I98" s="7" t="n">
-        <v>771</v>
+        <v>486</v>
       </c>
       <c r="J98" s="7" t="n"/>
       <c r="K98" s="7" t="n"/>
       <c r="L98" s="7" t="n"/>
       <c r="M98" s="7" t="n"/>
       <c r="N98" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O98" s="7" t="n">
         <v>0</v>
@@ -8246,7 +8246,7 @@
       </c>
       <c r="R98" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S98" s="8" t="inlineStr"/>
@@ -8263,7 +8263,7 @@
       <c r="V98" s="6" t="inlineStr"/>
       <c r="W98" s="7" t="inlineStr">
         <is>
-          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
+          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
         </is>
       </c>
     </row>
@@ -8277,13 +8277,13 @@
         </is>
       </c>
       <c r="C99" s="9" t="n">
-        <v>1680</v>
+        <v>1965</v>
       </c>
       <c r="D99" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E99" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
@@ -8292,7 +8292,7 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
@@ -8300,13 +8300,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I99" s="7" t="n"/>
+      <c r="I99" s="7" t="n">
+        <v>771</v>
+      </c>
       <c r="J99" s="7" t="n"/>
       <c r="K99" s="7" t="n"/>
       <c r="L99" s="7" t="n"/>
       <c r="M99" s="7" t="n"/>
       <c r="N99" s="7" t="n">
-        <v>20628</v>
+        <v>21740</v>
       </c>
       <c r="O99" s="7" t="n">
         <v>0</v>
@@ -8314,12 +8316,12 @@
       <c r="P99" s="7" t="n"/>
       <c r="Q99" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R99" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S99" s="8" t="inlineStr"/>
@@ -8336,7 +8338,7 @@
       <c r="V99" s="6" t="inlineStr"/>
       <c r="W99" s="7" t="inlineStr">
         <is>
-          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
+          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
         </is>
       </c>
     </row>
@@ -8350,7 +8352,7 @@
         </is>
       </c>
       <c r="C100" s="9" t="n">
-        <v>2200</v>
+        <v>1680</v>
       </c>
       <c r="D100" s="7" t="n">
         <v>2</v>
@@ -8365,23 +8367,21 @@
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I100" s="7" t="n">
-        <v>661</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I100" s="7" t="n"/>
       <c r="J100" s="7" t="n"/>
       <c r="K100" s="7" t="n"/>
       <c r="L100" s="7" t="n"/>
       <c r="M100" s="7" t="n"/>
       <c r="N100" s="7" t="n">
-        <v>22072</v>
+        <v>20628</v>
       </c>
       <c r="O100" s="7" t="n">
         <v>0</v>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="R100" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S100" s="8" t="inlineStr"/>
@@ -8411,7 +8411,7 @@
       <c r="V100" s="6" t="inlineStr"/>
       <c r="W100" s="7" t="inlineStr">
         <is>
-          <t>01a611ff329a1ff4055c7129250ed2b8a30a5874</t>
+          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
         </is>
       </c>
     </row>
@@ -8425,10 +8425,10 @@
         </is>
       </c>
       <c r="C101" s="9" t="n">
-        <v>1450</v>
+        <v>2200</v>
       </c>
       <c r="D101" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E101" s="7" t="n">
         <v>1</v>
@@ -8440,21 +8440,23 @@
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>St. Thomas Street, Bristol, BS1</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I101" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I101" s="7" t="n">
+        <v>661</v>
+      </c>
       <c r="J101" s="7" t="n"/>
       <c r="K101" s="7" t="n"/>
       <c r="L101" s="7" t="n"/>
       <c r="M101" s="7" t="n"/>
       <c r="N101" s="7" t="n">
-        <v>20324</v>
+        <v>22072</v>
       </c>
       <c r="O101" s="7" t="n">
         <v>0</v>
@@ -8467,7 +8469,7 @@
       </c>
       <c r="R101" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S101" s="8" t="inlineStr"/>
@@ -8484,7 +8486,7 @@
       <c r="V101" s="6" t="inlineStr"/>
       <c r="W101" s="7" t="inlineStr">
         <is>
-          <t>fc36e9d85221c7614fe48d0b05792976367fd6f9</t>
+          <t>01a611ff329a1ff4055c7129250ed2b8a30a5874</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8500,7 @@
         </is>
       </c>
       <c r="C102" s="9" t="n">
-        <v>1625</v>
+        <v>1450</v>
       </c>
       <c r="D102" s="7" t="n">
         <v>1</v>
@@ -8513,7 +8515,7 @@
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>St. Thomas Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr">
@@ -8521,15 +8523,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I102" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I102" s="7" t="n"/>
       <c r="J102" s="7" t="n"/>
       <c r="K102" s="7" t="n"/>
       <c r="L102" s="7" t="n"/>
       <c r="M102" s="7" t="n"/>
       <c r="N102" s="7" t="n">
-        <v>21732</v>
+        <v>20324</v>
       </c>
       <c r="O102" s="7" t="n">
         <v>0</v>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="R102" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S102" s="8" t="inlineStr"/>
@@ -8559,7 +8559,7 @@
       <c r="V102" s="6" t="inlineStr"/>
       <c r="W102" s="7" t="inlineStr">
         <is>
-          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
+          <t>fc36e9d85221c7614fe48d0b05792976367fd6f9</t>
         </is>
       </c>
     </row>
@@ -8573,13 +8573,13 @@
         </is>
       </c>
       <c r="C103" s="9" t="n">
-        <v>1940</v>
+        <v>1625</v>
       </c>
       <c r="D103" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E103" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
@@ -8588,7 +8588,7 @@
       </c>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr">
@@ -8597,14 +8597,14 @@
         </is>
       </c>
       <c r="I103" s="7" t="n">
-        <v>607</v>
+        <v>486</v>
       </c>
       <c r="J103" s="7" t="n"/>
       <c r="K103" s="7" t="n"/>
       <c r="L103" s="7" t="n"/>
       <c r="M103" s="7" t="n"/>
       <c r="N103" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O103" s="7" t="n">
         <v>0</v>
@@ -8617,7 +8617,7 @@
       </c>
       <c r="R103" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S103" s="8" t="inlineStr"/>
@@ -8634,7 +8634,7 @@
       <c r="V103" s="6" t="inlineStr"/>
       <c r="W103" s="7" t="inlineStr">
         <is>
-          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
+          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
         </is>
       </c>
     </row>
@@ -8648,13 +8648,13 @@
         </is>
       </c>
       <c r="C104" s="9" t="n">
-        <v>1465</v>
+        <v>1940</v>
       </c>
       <c r="D104" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E104" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F104" s="7" t="inlineStr">
         <is>
@@ -8672,14 +8672,14 @@
         </is>
       </c>
       <c r="I104" s="7" t="n">
-        <v>505</v>
+        <v>607</v>
       </c>
       <c r="J104" s="7" t="n"/>
       <c r="K104" s="7" t="n"/>
       <c r="L104" s="7" t="n"/>
       <c r="M104" s="7" t="n"/>
       <c r="N104" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O104" s="7" t="n">
         <v>0</v>
@@ -8709,7 +8709,7 @@
       <c r="V104" s="6" t="inlineStr"/>
       <c r="W104" s="7" t="inlineStr">
         <is>
-          <t>e86143466441bbbf802706245b19ef679ec29055</t>
+          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
         </is>
       </c>
     </row>
@@ -8723,13 +8723,13 @@
         </is>
       </c>
       <c r="C105" s="9" t="n">
-        <v>2300</v>
+        <v>1465</v>
       </c>
       <c r="D105" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E105" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
@@ -8738,23 +8738,23 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I105" s="7" t="n">
-        <v>773</v>
+        <v>505</v>
       </c>
       <c r="J105" s="7" t="n"/>
       <c r="K105" s="7" t="n"/>
       <c r="L105" s="7" t="n"/>
       <c r="M105" s="7" t="n"/>
       <c r="N105" s="7" t="n">
-        <v>22072</v>
+        <v>21816</v>
       </c>
       <c r="O105" s="7" t="n">
         <v>0</v>
@@ -8762,12 +8762,12 @@
       <c r="P105" s="7" t="n"/>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R105" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S105" s="8" t="inlineStr"/>
@@ -8784,7 +8784,7 @@
       <c r="V105" s="6" t="inlineStr"/>
       <c r="W105" s="7" t="inlineStr">
         <is>
-          <t>7594e7db3c52acddddafbbdb135025e4f15aa52c</t>
+          <t>e86143466441bbbf802706245b19ef679ec29055</t>
         </is>
       </c>
     </row>
@@ -8798,13 +8798,13 @@
         </is>
       </c>
       <c r="C106" s="9" t="n">
-        <v>1150</v>
+        <v>2300</v>
       </c>
       <c r="D106" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E106" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
@@ -8813,21 +8813,23 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I106" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I106" s="7" t="n">
+        <v>773</v>
+      </c>
       <c r="J106" s="7" t="n"/>
       <c r="K106" s="7" t="n"/>
       <c r="L106" s="7" t="n"/>
       <c r="M106" s="7" t="n"/>
       <c r="N106" s="7" t="n">
-        <v>15376</v>
+        <v>22072</v>
       </c>
       <c r="O106" s="7" t="n">
         <v>0</v>
@@ -8840,7 +8842,7 @@
       </c>
       <c r="R106" s="7" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S106" s="8" t="inlineStr"/>
@@ -8857,7 +8859,7 @@
       <c r="V106" s="6" t="inlineStr"/>
       <c r="W106" s="7" t="inlineStr">
         <is>
-          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
+          <t>7594e7db3c52acddddafbbdb135025e4f15aa52c</t>
         </is>
       </c>
     </row>
@@ -8871,7 +8873,7 @@
         </is>
       </c>
       <c r="C107" s="9" t="n">
-        <v>1560</v>
+        <v>1150</v>
       </c>
       <c r="D107" s="7" t="n">
         <v>1</v>
@@ -8886,23 +8888,21 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H107" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I107" s="7" t="n">
-        <v>472</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I107" s="7" t="n"/>
       <c r="J107" s="7" t="n"/>
       <c r="K107" s="7" t="n"/>
       <c r="L107" s="7" t="n"/>
       <c r="M107" s="7" t="n"/>
       <c r="N107" s="7" t="n">
-        <v>20984</v>
+        <v>15376</v>
       </c>
       <c r="O107" s="7" t="n">
         <v>0</v>
@@ -8910,12 +8910,12 @@
       <c r="P107" s="7" t="n"/>
       <c r="Q107" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R107" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S107" s="8" t="inlineStr"/>
@@ -8932,7 +8932,7 @@
       <c r="V107" s="6" t="inlineStr"/>
       <c r="W107" s="7" t="inlineStr">
         <is>
-          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
+          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
         </is>
       </c>
     </row>
@@ -8946,13 +8946,13 @@
         </is>
       </c>
       <c r="C108" s="9" t="n">
-        <v>1970</v>
+        <v>1560</v>
       </c>
       <c r="D108" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E108" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F108" s="7" t="inlineStr">
         <is>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr">
@@ -8970,14 +8970,14 @@
         </is>
       </c>
       <c r="I108" s="7" t="n">
-        <v>750</v>
+        <v>472</v>
       </c>
       <c r="J108" s="7" t="n"/>
       <c r="K108" s="7" t="n"/>
       <c r="L108" s="7" t="n"/>
       <c r="M108" s="7" t="n"/>
       <c r="N108" s="7" t="n">
-        <v>21740</v>
+        <v>20984</v>
       </c>
       <c r="O108" s="7" t="n">
         <v>0</v>
@@ -8990,7 +8990,7 @@
       </c>
       <c r="R108" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S108" s="8" t="inlineStr"/>
@@ -9007,7 +9007,7 @@
       <c r="V108" s="6" t="inlineStr"/>
       <c r="W108" s="7" t="inlineStr">
         <is>
-          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
+          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
         </is>
       </c>
     </row>
@@ -9021,13 +9021,13 @@
         </is>
       </c>
       <c r="C109" s="9" t="n">
-        <v>1575</v>
+        <v>1970</v>
       </c>
       <c r="D109" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E109" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
@@ -9045,14 +9045,14 @@
         </is>
       </c>
       <c r="I109" s="7" t="n">
-        <v>430</v>
+        <v>750</v>
       </c>
       <c r="J109" s="7" t="n"/>
       <c r="K109" s="7" t="n"/>
       <c r="L109" s="7" t="n"/>
       <c r="M109" s="7" t="n"/>
       <c r="N109" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O109" s="7" t="n">
         <v>0</v>
@@ -9082,7 +9082,7 @@
       <c r="V109" s="6" t="inlineStr"/>
       <c r="W109" s="7" t="inlineStr">
         <is>
-          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
+          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
         </is>
       </c>
     </row>
@@ -9096,7 +9096,7 @@
         </is>
       </c>
       <c r="C110" s="9" t="n">
-        <v>1200</v>
+        <v>1575</v>
       </c>
       <c r="D110" s="7" t="n">
         <v>1</v>
@@ -9111,7 +9111,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Marsh House, BS1 4AQ</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H110" s="7" t="inlineStr">
@@ -9120,14 +9120,14 @@
         </is>
       </c>
       <c r="I110" s="7" t="n">
-        <v>462</v>
+        <v>430</v>
       </c>
       <c r="J110" s="7" t="n"/>
       <c r="K110" s="7" t="n"/>
       <c r="L110" s="7" t="n"/>
       <c r="M110" s="7" t="n"/>
       <c r="N110" s="7" t="n">
-        <v>20788</v>
+        <v>21816</v>
       </c>
       <c r="O110" s="7" t="n">
         <v>0</v>
@@ -9135,12 +9135,12 @@
       <c r="P110" s="7" t="n"/>
       <c r="Q110" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R110" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S110" s="8" t="inlineStr"/>
@@ -9157,7 +9157,7 @@
       <c r="V110" s="6" t="inlineStr"/>
       <c r="W110" s="7" t="inlineStr">
         <is>
-          <t>088c41fb8491fdd927ed6eb071c9ddf0192a4834</t>
+          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
         </is>
       </c>
     </row>
@@ -9171,7 +9171,7 @@
         </is>
       </c>
       <c r="C111" s="9" t="n">
-        <v>1550</v>
+        <v>1200</v>
       </c>
       <c r="D111" s="7" t="n">
         <v>1</v>
@@ -9186,7 +9186,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>City Centre, Marsh House, BS1 4AQ</t>
         </is>
       </c>
       <c r="H111" s="7" t="inlineStr">
@@ -9194,13 +9194,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I111" s="7" t="n"/>
+      <c r="I111" s="7" t="n">
+        <v>462</v>
+      </c>
       <c r="J111" s="7" t="n"/>
       <c r="K111" s="7" t="n"/>
       <c r="L111" s="7" t="n"/>
       <c r="M111" s="7" t="n"/>
       <c r="N111" s="7" t="n">
-        <v>21996</v>
+        <v>20788</v>
       </c>
       <c r="O111" s="7" t="n">
         <v>0</v>
@@ -9213,7 +9215,7 @@
       </c>
       <c r="R111" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S111" s="8" t="inlineStr"/>
@@ -9230,7 +9232,7 @@
       <c r="V111" s="6" t="inlineStr"/>
       <c r="W111" s="7" t="inlineStr">
         <is>
-          <t>9479f4ce03277dc57d4cd9fbd5a0c90eadc237db</t>
+          <t>088c41fb8491fdd927ed6eb071c9ddf0192a4834</t>
         </is>
       </c>
     </row>
@@ -9244,7 +9246,7 @@
         </is>
       </c>
       <c r="C112" s="9" t="n">
-        <v>1150</v>
+        <v>1550</v>
       </c>
       <c r="D112" s="7" t="n">
         <v>1</v>
@@ -9259,12 +9261,12 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>St. Philips, Bristol, BS2</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I112" s="7" t="n"/>
@@ -9273,7 +9275,7 @@
       <c r="L112" s="7" t="n"/>
       <c r="M112" s="7" t="n"/>
       <c r="N112" s="7" t="n">
-        <v>20784</v>
+        <v>21996</v>
       </c>
       <c r="O112" s="7" t="n">
         <v>0</v>
@@ -9286,7 +9288,7 @@
       </c>
       <c r="R112" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S112" s="8" t="inlineStr"/>
@@ -9303,7 +9305,7 @@
       <c r="V112" s="6" t="inlineStr"/>
       <c r="W112" s="7" t="inlineStr">
         <is>
-          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
+          <t>9479f4ce03277dc57d4cd9fbd5a0c90eadc237db</t>
         </is>
       </c>
     </row>
@@ -9317,7 +9319,7 @@
         </is>
       </c>
       <c r="C113" s="9" t="n">
-        <v>1660</v>
+        <v>1150</v>
       </c>
       <c r="D113" s="7" t="n">
         <v>1</v>
@@ -9332,23 +9334,21 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>St. Philips, Bristol, BS2</t>
         </is>
       </c>
       <c r="H113" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I113" s="7" t="n">
-        <v>558</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I113" s="7" t="n"/>
       <c r="J113" s="7" t="n"/>
       <c r="K113" s="7" t="n"/>
       <c r="L113" s="7" t="n"/>
       <c r="M113" s="7" t="n"/>
       <c r="N113" s="7" t="n">
-        <v>20984</v>
+        <v>20784</v>
       </c>
       <c r="O113" s="7" t="n">
         <v>0</v>
@@ -9361,7 +9361,7 @@
       </c>
       <c r="R113" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S113" s="8" t="inlineStr"/>
@@ -9378,7 +9378,7 @@
       <c r="V113" s="6" t="inlineStr"/>
       <c r="W113" s="7" t="inlineStr">
         <is>
-          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
+          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
         </is>
       </c>
     </row>
@@ -9392,13 +9392,13 @@
         </is>
       </c>
       <c r="C114" s="9" t="n">
-        <v>1860</v>
+        <v>1660</v>
       </c>
       <c r="D114" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E114" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F114" s="7" t="inlineStr">
         <is>
@@ -9407,7 +9407,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H114" s="7" t="inlineStr">
@@ -9416,14 +9416,14 @@
         </is>
       </c>
       <c r="I114" s="7" t="n">
-        <v>647</v>
+        <v>558</v>
       </c>
       <c r="J114" s="7" t="n"/>
       <c r="K114" s="7" t="n"/>
       <c r="L114" s="7" t="n"/>
       <c r="M114" s="7" t="n"/>
       <c r="N114" s="7" t="n">
-        <v>21740</v>
+        <v>20984</v>
       </c>
       <c r="O114" s="7" t="n">
         <v>0</v>
@@ -9436,7 +9436,7 @@
       </c>
       <c r="R114" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S114" s="8" t="inlineStr"/>
@@ -9453,7 +9453,7 @@
       <c r="V114" s="6" t="inlineStr"/>
       <c r="W114" s="7" t="inlineStr">
         <is>
-          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
+          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
         </is>
       </c>
     </row>
@@ -9467,13 +9467,13 @@
         </is>
       </c>
       <c r="C115" s="9" t="n">
-        <v>1600</v>
+        <v>1860</v>
       </c>
       <c r="D115" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E115" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
@@ -9491,14 +9491,14 @@
         </is>
       </c>
       <c r="I115" s="7" t="n">
-        <v>549</v>
+        <v>647</v>
       </c>
       <c r="J115" s="7" t="n"/>
       <c r="K115" s="7" t="n"/>
       <c r="L115" s="7" t="n"/>
       <c r="M115" s="7" t="n"/>
       <c r="N115" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O115" s="7" t="n">
         <v>0</v>
@@ -9528,7 +9528,7 @@
       <c r="V115" s="6" t="inlineStr"/>
       <c r="W115" s="7" t="inlineStr">
         <is>
-          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
+          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
         </is>
       </c>
     </row>
@@ -9542,10 +9542,10 @@
         </is>
       </c>
       <c r="C116" s="9" t="n">
-        <v>3000</v>
+        <v>1600</v>
       </c>
       <c r="D116" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E116" s="7" t="n">
         <v>1</v>
@@ -9557,21 +9557,23 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>North St, Bristol, BS3</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H116" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I116" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I116" s="7" t="n">
+        <v>549</v>
+      </c>
       <c r="J116" s="7" t="n"/>
       <c r="K116" s="7" t="n"/>
       <c r="L116" s="7" t="n"/>
       <c r="M116" s="7" t="n"/>
       <c r="N116" s="7" t="n">
-        <v>11928</v>
+        <v>21816</v>
       </c>
       <c r="O116" s="7" t="n">
         <v>0</v>
@@ -9579,12 +9581,12 @@
       <c r="P116" s="7" t="n"/>
       <c r="Q116" s="7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R116" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S116" s="8" t="inlineStr"/>
@@ -9601,7 +9603,7 @@
       <c r="V116" s="6" t="inlineStr"/>
       <c r="W116" s="7" t="inlineStr">
         <is>
-          <t>e38490ffec644261cb89a11e3d645356430839fe</t>
+          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
         </is>
       </c>
     </row>
@@ -9615,10 +9617,10 @@
         </is>
       </c>
       <c r="C117" s="9" t="n">
-        <v>1550</v>
+        <v>3000</v>
       </c>
       <c r="D117" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E117" s="7" t="n">
         <v>1</v>
@@ -9630,12 +9632,12 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>North St, Bristol, BS3</t>
         </is>
       </c>
       <c r="H117" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I117" s="7" t="n"/>
@@ -9644,7 +9646,7 @@
       <c r="L117" s="7" t="n"/>
       <c r="M117" s="7" t="n"/>
       <c r="N117" s="7" t="n">
-        <v>21100</v>
+        <v>11928</v>
       </c>
       <c r="O117" s="7" t="n">
         <v>0</v>
@@ -9652,12 +9654,12 @@
       <c r="P117" s="7" t="n"/>
       <c r="Q117" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R117" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S117" s="8" t="inlineStr"/>
@@ -9674,7 +9676,7 @@
       <c r="V117" s="6" t="inlineStr"/>
       <c r="W117" s="7" t="inlineStr">
         <is>
-          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
+          <t>e38490ffec644261cb89a11e3d645356430839fe</t>
         </is>
       </c>
     </row>
@@ -9688,13 +9690,13 @@
         </is>
       </c>
       <c r="C118" s="9" t="n">
-        <v>1750</v>
+        <v>1550</v>
       </c>
       <c r="D118" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E118" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F118" s="7" t="inlineStr">
         <is>
@@ -9703,7 +9705,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H118" s="7" t="inlineStr">
@@ -9711,15 +9713,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I118" s="7" t="n">
-        <v>849</v>
-      </c>
+      <c r="I118" s="7" t="n"/>
       <c r="J118" s="7" t="n"/>
       <c r="K118" s="7" t="n"/>
       <c r="L118" s="7" t="n"/>
       <c r="M118" s="7" t="n"/>
       <c r="N118" s="7" t="n">
-        <v>21028</v>
+        <v>21100</v>
       </c>
       <c r="O118" s="7" t="n">
         <v>0</v>
@@ -9732,7 +9732,7 @@
       </c>
       <c r="R118" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S118" s="8" t="inlineStr"/>
@@ -9749,7 +9749,7 @@
       <c r="V118" s="6" t="inlineStr"/>
       <c r="W118" s="7" t="inlineStr">
         <is>
-          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
+          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
         </is>
       </c>
     </row>
@@ -9763,13 +9763,13 @@
         </is>
       </c>
       <c r="C119" s="9" t="n">
-        <v>1300</v>
+        <v>1750</v>
       </c>
       <c r="D119" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E119" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F119" s="7" t="inlineStr">
         <is>
@@ -9778,7 +9778,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The Milliners, BS1 6WU</t>
+          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H119" s="7" t="inlineStr">
@@ -9787,14 +9787,14 @@
         </is>
       </c>
       <c r="I119" s="7" t="n">
-        <v>463</v>
+        <v>849</v>
       </c>
       <c r="J119" s="7" t="n"/>
       <c r="K119" s="7" t="n"/>
       <c r="L119" s="7" t="n"/>
       <c r="M119" s="7" t="n"/>
       <c r="N119" s="7" t="n">
-        <v>21440</v>
+        <v>21028</v>
       </c>
       <c r="O119" s="7" t="n">
         <v>0</v>
@@ -9807,7 +9807,7 @@
       </c>
       <c r="R119" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S119" s="8" t="inlineStr"/>
@@ -9824,7 +9824,7 @@
       <c r="V119" s="6" t="inlineStr"/>
       <c r="W119" s="7" t="inlineStr">
         <is>
-          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
+          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
         </is>
       </c>
     </row>
@@ -9838,13 +9838,13 @@
         </is>
       </c>
       <c r="C120" s="9" t="n">
-        <v>1900</v>
+        <v>1300</v>
       </c>
       <c r="D120" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E120" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F120" s="7" t="inlineStr">
         <is>
@@ -9853,7 +9853,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>City Centre, The Milliners, BS1 6WU</t>
         </is>
       </c>
       <c r="H120" s="7" t="inlineStr">
@@ -9862,14 +9862,14 @@
         </is>
       </c>
       <c r="I120" s="7" t="n">
-        <v>624</v>
+        <v>463</v>
       </c>
       <c r="J120" s="7" t="n"/>
       <c r="K120" s="7" t="n"/>
       <c r="L120" s="7" t="n"/>
       <c r="M120" s="7" t="n"/>
       <c r="N120" s="7" t="n">
-        <v>21740</v>
+        <v>21440</v>
       </c>
       <c r="O120" s="7" t="n">
         <v>0</v>
@@ -9882,7 +9882,7 @@
       </c>
       <c r="R120" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S120" s="8" t="inlineStr"/>
@@ -9899,7 +9899,7 @@
       <c r="V120" s="6" t="inlineStr"/>
       <c r="W120" s="7" t="inlineStr">
         <is>
-          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
+          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
         </is>
       </c>
     </row>
@@ -9913,13 +9913,13 @@
         </is>
       </c>
       <c r="C121" s="9" t="n">
-        <v>1685</v>
+        <v>1900</v>
       </c>
       <c r="D121" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E121" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F121" s="7" t="inlineStr">
         <is>
@@ -9928,7 +9928,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H121" s="7" t="inlineStr">
@@ -9937,14 +9937,14 @@
         </is>
       </c>
       <c r="I121" s="7" t="n">
-        <v>545</v>
+        <v>624</v>
       </c>
       <c r="J121" s="7" t="n"/>
       <c r="K121" s="7" t="n"/>
       <c r="L121" s="7" t="n"/>
       <c r="M121" s="7" t="n"/>
       <c r="N121" s="7" t="n">
-        <v>21024</v>
+        <v>21740</v>
       </c>
       <c r="O121" s="7" t="n">
         <v>0</v>
@@ -9957,7 +9957,7 @@
       </c>
       <c r="R121" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S121" s="8" t="inlineStr"/>
@@ -9974,7 +9974,7 @@
       <c r="V121" s="6" t="inlineStr"/>
       <c r="W121" s="7" t="inlineStr">
         <is>
-          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
+          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
         </is>
       </c>
     </row>
@@ -9988,7 +9988,7 @@
         </is>
       </c>
       <c r="C122" s="9" t="n">
-        <v>1500</v>
+        <v>1685</v>
       </c>
       <c r="D122" s="7" t="n">
         <v>1</v>
@@ -10003,21 +10003,23 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>Talavera Close, Bristol</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H122" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I122" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I122" s="7" t="n">
+        <v>545</v>
+      </c>
       <c r="J122" s="7" t="n"/>
       <c r="K122" s="7" t="n"/>
       <c r="L122" s="7" t="n"/>
       <c r="M122" s="7" t="n"/>
       <c r="N122" s="7" t="n">
-        <v>20276</v>
+        <v>21024</v>
       </c>
       <c r="O122" s="7" t="n">
         <v>0</v>
@@ -10025,12 +10027,12 @@
       <c r="P122" s="7" t="n"/>
       <c r="Q122" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R122" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S122" s="8" t="inlineStr"/>
@@ -10047,7 +10049,7 @@
       <c r="V122" s="6" t="inlineStr"/>
       <c r="W122" s="7" t="inlineStr">
         <is>
-          <t>411497eb8a2cc8699388af5157111972fa69b353</t>
+          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
         </is>
       </c>
     </row>
@@ -10061,13 +10063,13 @@
         </is>
       </c>
       <c r="C123" s="9" t="n">
-        <v>1550</v>
+        <v>1500</v>
       </c>
       <c r="D123" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E123" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F123" s="7" t="inlineStr">
         <is>
@@ -10076,7 +10078,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>Portland Heights - St. Pauls</t>
+          <t>Talavera Close, Bristol</t>
         </is>
       </c>
       <c r="H123" s="7" t="inlineStr">
@@ -10090,7 +10092,7 @@
       <c r="L123" s="7" t="n"/>
       <c r="M123" s="7" t="n"/>
       <c r="N123" s="7" t="n">
-        <v>21420</v>
+        <v>20276</v>
       </c>
       <c r="O123" s="7" t="n">
         <v>0</v>
@@ -10103,7 +10105,7 @@
       </c>
       <c r="R123" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Bishopston</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S123" s="8" t="inlineStr"/>
@@ -10120,7 +10122,7 @@
       <c r="V123" s="6" t="inlineStr"/>
       <c r="W123" s="7" t="inlineStr">
         <is>
-          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
+          <t>411497eb8a2cc8699388af5157111972fa69b353</t>
         </is>
       </c>
     </row>
@@ -10134,13 +10136,13 @@
         </is>
       </c>
       <c r="C124" s="9" t="n">
-        <v>1400</v>
+        <v>1550</v>
       </c>
       <c r="D124" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E124" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F124" s="7" t="inlineStr">
         <is>
@@ -10149,12 +10151,12 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>Taylors Bank, Bristol, BS1</t>
+          <t>Portland Heights - St. Pauls</t>
         </is>
       </c>
       <c r="H124" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I124" s="7" t="n"/>
@@ -10163,7 +10165,7 @@
       <c r="L124" s="7" t="n"/>
       <c r="M124" s="7" t="n"/>
       <c r="N124" s="7" t="n">
-        <v>21996</v>
+        <v>21420</v>
       </c>
       <c r="O124" s="7" t="n">
         <v>0</v>
@@ -10176,7 +10178,7 @@
       </c>
       <c r="R124" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Ocean, Bishopston</t>
         </is>
       </c>
       <c r="S124" s="8" t="inlineStr"/>
@@ -10193,7 +10195,7 @@
       <c r="V124" s="6" t="inlineStr"/>
       <c r="W124" s="7" t="inlineStr">
         <is>
-          <t>464a8221babcd58554ee30417192b0a25eacccb0</t>
+          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
         </is>
       </c>
     </row>
@@ -10207,7 +10209,7 @@
         </is>
       </c>
       <c r="C125" s="9" t="n">
-        <v>1350</v>
+        <v>1400</v>
       </c>
       <c r="D125" s="7" t="n">
         <v>1</v>
@@ -10222,7 +10224,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>Gas Ferry Road, Bristol, BS1</t>
+          <t>Taylors Bank, Bristol, BS1</t>
         </is>
       </c>
       <c r="H125" s="7" t="inlineStr">
@@ -10236,7 +10238,7 @@
       <c r="L125" s="7" t="n"/>
       <c r="M125" s="7" t="n"/>
       <c r="N125" s="7" t="n">
-        <v>15168</v>
+        <v>21996</v>
       </c>
       <c r="O125" s="7" t="n">
         <v>0</v>
@@ -10244,12 +10246,12 @@
       <c r="P125" s="7" t="n"/>
       <c r="Q125" s="7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R125" s="7" t="inlineStr">
         <is>
-          <t>Northwood, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S125" s="8" t="inlineStr"/>
@@ -10266,7 +10268,7 @@
       <c r="V125" s="6" t="inlineStr"/>
       <c r="W125" s="7" t="inlineStr">
         <is>
-          <t>b042a4b755dd663949f094bd579797d2c011a710</t>
+          <t>464a8221babcd58554ee30417192b0a25eacccb0</t>
         </is>
       </c>
     </row>
@@ -10280,7 +10282,7 @@
         </is>
       </c>
       <c r="C126" s="9" t="n">
-        <v>1150</v>
+        <v>1350</v>
       </c>
       <c r="D126" s="7" t="n">
         <v>1</v>
@@ -10295,23 +10297,21 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>Century Place, St. Paul Street, BS2 8AN</t>
+          <t>Gas Ferry Road, Bristol, BS1</t>
         </is>
       </c>
       <c r="H126" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I126" s="7" t="n">
-        <v>344</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I126" s="7" t="n"/>
       <c r="J126" s="7" t="n"/>
       <c r="K126" s="7" t="n"/>
       <c r="L126" s="7" t="n"/>
       <c r="M126" s="7" t="n"/>
       <c r="N126" s="7" t="n">
-        <v>21792</v>
+        <v>15168</v>
       </c>
       <c r="O126" s="7" t="n">
         <v>0</v>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="R126" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Northwood, Bristol</t>
         </is>
       </c>
       <c r="S126" s="8" t="inlineStr"/>
@@ -10341,7 +10341,7 @@
       <c r="V126" s="6" t="inlineStr"/>
       <c r="W126" s="7" t="inlineStr">
         <is>
-          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
+          <t>b042a4b755dd663949f094bd579797d2c011a710</t>
         </is>
       </c>
     </row>
@@ -10355,7 +10355,7 @@
         </is>
       </c>
       <c r="C127" s="9" t="n">
-        <v>1100</v>
+        <v>1150</v>
       </c>
       <c r="D127" s="7" t="n">
         <v>1</v>
@@ -10370,21 +10370,23 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>Bath Road - Arnos Vale</t>
+          <t>Century Place, St. Paul Street, BS2 8AN</t>
         </is>
       </c>
       <c r="H127" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I127" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I127" s="7" t="n">
+        <v>344</v>
+      </c>
       <c r="J127" s="7" t="n"/>
       <c r="K127" s="7" t="n"/>
       <c r="L127" s="7" t="n"/>
       <c r="M127" s="7" t="n"/>
       <c r="N127" s="7" t="n">
-        <v>6248</v>
+        <v>21792</v>
       </c>
       <c r="O127" s="7" t="n">
         <v>0</v>
@@ -10397,7 +10399,7 @@
       </c>
       <c r="R127" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S127" s="8" t="inlineStr"/>
@@ -10414,7 +10416,7 @@
       <c r="V127" s="6" t="inlineStr"/>
       <c r="W127" s="7" t="inlineStr">
         <is>
-          <t>e63386a22f0ffb4baee6b24143f47a42221ce776</t>
+          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
         </is>
       </c>
     </row>
@@ -10428,13 +10430,13 @@
         </is>
       </c>
       <c r="C128" s="9" t="n">
-        <v>1985</v>
+        <v>1100</v>
       </c>
       <c r="D128" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E128" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
@@ -10443,23 +10445,21 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Bath Road - Arnos Vale</t>
         </is>
       </c>
       <c r="H128" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I128" s="7" t="n">
-        <v>771</v>
-      </c>
+          <t>BS4</t>
+        </is>
+      </c>
+      <c r="I128" s="7" t="n"/>
       <c r="J128" s="7" t="n"/>
       <c r="K128" s="7" t="n"/>
       <c r="L128" s="7" t="n"/>
       <c r="M128" s="7" t="n"/>
       <c r="N128" s="7" t="n">
-        <v>21740</v>
+        <v>6248</v>
       </c>
       <c r="O128" s="7" t="n">
         <v>0</v>
@@ -10472,7 +10472,7 @@
       </c>
       <c r="R128" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S128" s="8" t="inlineStr"/>
@@ -10489,7 +10489,7 @@
       <c r="V128" s="6" t="inlineStr"/>
       <c r="W128" s="7" t="inlineStr">
         <is>
-          <t>5414e121fde47f0b60451ddda4019d5d93133f4a</t>
+          <t>e63386a22f0ffb4baee6b24143f47a42221ce776</t>
         </is>
       </c>
     </row>
@@ -10503,13 +10503,13 @@
         </is>
       </c>
       <c r="C129" s="9" t="n">
-        <v>1650</v>
+        <v>1985</v>
       </c>
       <c r="D129" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E129" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
@@ -10518,7 +10518,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
@@ -10527,14 +10527,14 @@
         </is>
       </c>
       <c r="I129" s="7" t="n">
-        <v>484</v>
+        <v>771</v>
       </c>
       <c r="J129" s="7" t="n"/>
       <c r="K129" s="7" t="n"/>
       <c r="L129" s="7" t="n"/>
       <c r="M129" s="7" t="n"/>
       <c r="N129" s="7" t="n">
-        <v>20984</v>
+        <v>21740</v>
       </c>
       <c r="O129" s="7" t="n">
         <v>0</v>
@@ -10547,7 +10547,7 @@
       </c>
       <c r="R129" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S129" s="8" t="inlineStr"/>
@@ -10564,7 +10564,7 @@
       <c r="V129" s="6" t="inlineStr"/>
       <c r="W129" s="7" t="inlineStr">
         <is>
-          <t>a6340397b31ca11a123cb584f2f878317e73b7eb</t>
+          <t>5414e121fde47f0b60451ddda4019d5d93133f4a</t>
         </is>
       </c>
     </row>
@@ -10578,7 +10578,7 @@
         </is>
       </c>
       <c r="C130" s="9" t="n">
-        <v>1630</v>
+        <v>1650</v>
       </c>
       <c r="D130" s="7" t="n">
         <v>1</v>
@@ -10593,7 +10593,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
@@ -10602,14 +10602,14 @@
         </is>
       </c>
       <c r="I130" s="7" t="n">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="J130" s="7" t="n"/>
       <c r="K130" s="7" t="n"/>
       <c r="L130" s="7" t="n"/>
       <c r="M130" s="7" t="n"/>
       <c r="N130" s="7" t="n">
-        <v>21732</v>
+        <v>20984</v>
       </c>
       <c r="O130" s="7" t="n">
         <v>0</v>
@@ -10622,7 +10622,7 @@
       </c>
       <c r="R130" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S130" s="8" t="inlineStr"/>
@@ -10639,7 +10639,7 @@
       <c r="V130" s="6" t="inlineStr"/>
       <c r="W130" s="7" t="inlineStr">
         <is>
-          <t>5cdc78c7612a522b9bc5bc24a2beb93eb2703b6b</t>
+          <t>a6340397b31ca11a123cb584f2f878317e73b7eb</t>
         </is>
       </c>
     </row>
@@ -10653,13 +10653,13 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>1800</v>
+        <v>1630</v>
       </c>
       <c r="D131" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E131" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
@@ -10668,7 +10668,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr">
@@ -10677,14 +10677,14 @@
         </is>
       </c>
       <c r="I131" s="7" t="n">
-        <v>980</v>
+        <v>485</v>
       </c>
       <c r="J131" s="7" t="n"/>
       <c r="K131" s="7" t="n"/>
       <c r="L131" s="7" t="n"/>
       <c r="M131" s="7" t="n"/>
       <c r="N131" s="7" t="n">
-        <v>20788</v>
+        <v>21732</v>
       </c>
       <c r="O131" s="7" t="n">
         <v>0</v>
@@ -10692,12 +10692,12 @@
       <c r="P131" s="7" t="n"/>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S131" s="8" t="inlineStr"/>
@@ -10714,7 +10714,7 @@
       <c r="V131" s="6" t="inlineStr"/>
       <c r="W131" s="7" t="inlineStr">
         <is>
-          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
+          <t>5cdc78c7612a522b9bc5bc24a2beb93eb2703b6b</t>
         </is>
       </c>
     </row>
@@ -10728,13 +10728,13 @@
         </is>
       </c>
       <c r="C132" s="9" t="n">
-        <v>1530</v>
+        <v>1800</v>
       </c>
       <c r="D132" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E132" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
@@ -10743,7 +10743,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr">
@@ -10752,14 +10752,14 @@
         </is>
       </c>
       <c r="I132" s="7" t="n">
-        <v>548</v>
+        <v>980</v>
       </c>
       <c r="J132" s="7" t="n"/>
       <c r="K132" s="7" t="n"/>
       <c r="L132" s="7" t="n"/>
       <c r="M132" s="7" t="n"/>
       <c r="N132" s="7" t="n">
-        <v>21740</v>
+        <v>20788</v>
       </c>
       <c r="O132" s="7" t="n">
         <v>0</v>
@@ -10772,7 +10772,7 @@
       </c>
       <c r="R132" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S132" s="8" t="inlineStr"/>
@@ -10789,7 +10789,7 @@
       <c r="V132" s="6" t="inlineStr"/>
       <c r="W132" s="7" t="inlineStr">
         <is>
-          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
+          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
         </is>
       </c>
     </row>
@@ -10803,36 +10803,38 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1700</v>
+        <v>1530</v>
       </c>
       <c r="D133" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E133" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>Dunkerry Road - Windmill Hill</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I133" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I133" s="7" t="n">
+        <v>548</v>
+      </c>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>8448</v>
+        <v>21740</v>
       </c>
       <c r="O133" s="7" t="n">
         <v>0</v>
@@ -10845,7 +10847,7 @@
       </c>
       <c r="R133" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S133" s="8" t="inlineStr"/>
@@ -10862,7 +10864,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
+          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
         </is>
       </c>
     </row>
@@ -10876,7 +10878,7 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>2130</v>
+        <v>1700</v>
       </c>
       <c r="D134" s="7" t="n">
         <v>2</v>
@@ -10886,28 +10888,26 @@
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Dunkerry Road - Windmill Hill</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I134" s="7" t="n">
-        <v>722</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I134" s="7" t="n"/>
       <c r="J134" s="7" t="n"/>
       <c r="K134" s="7" t="n"/>
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="7" t="n">
-        <v>21732</v>
+        <v>8448</v>
       </c>
       <c r="O134" s="7" t="n">
         <v>0</v>
@@ -10920,7 +10920,7 @@
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10937,7 +10937,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>f944c2b1bd69d2127577103ede3bdfcf33660e58</t>
+          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
         </is>
       </c>
     </row>
@@ -10951,13 +10951,13 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1635</v>
+        <v>2130</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
@@ -10975,7 +10975,7 @@
         </is>
       </c>
       <c r="I135" s="7" t="n">
-        <v>485</v>
+        <v>722</v>
       </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
@@ -11012,7 +11012,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>8e8e3a11bee7fef2f0d043aedc4bea860a81529e</t>
+          <t>f944c2b1bd69d2127577103ede3bdfcf33660e58</t>
         </is>
       </c>
     </row>
@@ -11026,13 +11026,13 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>2220</v>
+        <v>1635</v>
       </c>
       <c r="D136" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E136" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
@@ -11041,7 +11041,7 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
@@ -11050,14 +11050,14 @@
         </is>
       </c>
       <c r="I136" s="7" t="n">
-        <v>741</v>
+        <v>485</v>
       </c>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>20984</v>
+        <v>21732</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -11070,7 +11070,7 @@
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11087,7 +11087,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>eca904199b9ed7abf3fd1cb00b8cf56a578e0dd2</t>
+          <t>8e8e3a11bee7fef2f0d043aedc4bea860a81529e</t>
         </is>
       </c>
     </row>
@@ -11101,13 +11101,13 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1670</v>
+        <v>2220</v>
       </c>
       <c r="D137" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E137" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
@@ -11125,7 +11125,7 @@
         </is>
       </c>
       <c r="I137" s="7" t="n">
-        <v>561</v>
+        <v>741</v>
       </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
@@ -11162,7 +11162,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>e748012a511f5d5760d06bd53b8097e8c89a07c0</t>
+          <t>eca904199b9ed7abf3fd1cb00b8cf56a578e0dd2</t>
         </is>
       </c>
     </row>
@@ -11176,13 +11176,13 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>2472</v>
+        <v>1670</v>
       </c>
       <c r="D138" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E138" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
@@ -11191,21 +11191,23 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Paintworks 6.1.1, Arnos Vale, Bristol</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I138" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I138" s="7" t="n">
+        <v>561</v>
+      </c>
       <c r="J138" s="7" t="n"/>
       <c r="K138" s="7" t="n"/>
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>5276</v>
+        <v>20984</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11218,7 +11220,7 @@
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>Rengen Lettings, Rengen Lettings</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11235,7 +11237,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>e6120f9fa85e2c63863f50a3ceba968ee90b3fc1</t>
+          <t>e748012a511f5d5760d06bd53b8097e8c89a07c0</t>
         </is>
       </c>
     </row>
@@ -11249,13 +11251,13 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>1390</v>
+        <v>2472</v>
       </c>
       <c r="D139" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E139" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
@@ -11264,12 +11266,12 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Paintworks 6.1.1, Arnos Vale, Bristol</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I139" s="7" t="n"/>
@@ -11277,7 +11279,9 @@
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
-      <c r="N139" s="7" t="n"/>
+      <c r="N139" s="7" t="n">
+        <v>5276</v>
+      </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
       </c>
@@ -11289,7 +11293,7 @@
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Rengen Lettings, Rengen Lettings</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11306,7 +11310,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
+          <t>e6120f9fa85e2c63863f50a3ceba968ee90b3fc1</t>
         </is>
       </c>
     </row>
@@ -11320,7 +11324,7 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1630</v>
+        <v>1390</v>
       </c>
       <c r="D140" s="7" t="n">
         <v>1</v>
@@ -11335,7 +11339,7 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
@@ -11343,28 +11347,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I140" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I140" s="7" t="n"/>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
-      <c r="N140" s="7" t="n">
-        <v>13860</v>
-      </c>
+      <c r="N140" s="7" t="n"/>
       <c r="O140" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11381,7 +11381,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
+          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House search data from run 146
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -3070,7 +3070,7 @@
       <c r="L31" s="7" t="n"/>
       <c r="M31" s="7" t="n"/>
       <c r="N31" s="7" t="n">
-        <v>11956</v>
+        <v>11632</v>
       </c>
       <c r="O31" s="7" t="n">
         <v>0</v>
@@ -3149,7 +3149,7 @@
       <c r="L32" s="7" t="n"/>
       <c r="M32" s="7" t="n"/>
       <c r="N32" s="7" t="n">
-        <v>11956</v>
+        <v>11632</v>
       </c>
       <c r="O32" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
House search data from run 160
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -2908,7 +2908,7 @@
       <c r="L29" s="7" t="n"/>
       <c r="M29" s="7" t="n"/>
       <c r="N29" s="7" t="n">
-        <v>21140</v>
+        <v>21264</v>
       </c>
       <c r="O29" s="7" t="n">
         <v>0</v>
@@ -9944,7 +9944,7 @@
       <c r="L121" s="7" t="n"/>
       <c r="M121" s="7" t="n"/>
       <c r="N121" s="7" t="n">
-        <v>16644</v>
+        <v>16664</v>
       </c>
       <c r="O121" s="7" t="n">
         <v>0</v>
@@ -10168,7 +10168,9 @@
       <c r="K124" s="7" t="n"/>
       <c r="L124" s="7" t="n"/>
       <c r="M124" s="7" t="n"/>
-      <c r="N124" s="7" t="n"/>
+      <c r="N124" s="7" t="n">
+        <v>21816</v>
+      </c>
       <c r="O124" s="7" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
House search data from run 164
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$204</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W199"/>
+  <dimension ref="A1:W204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>2000</v>
+        <v>1900</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>2</v>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>1300</v>
+        <v>1250</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>1</v>
@@ -9243,7 +9243,7 @@
       <c r="L112" s="7" t="n"/>
       <c r="M112" s="7" t="n"/>
       <c r="N112" s="7" t="n">
-        <v>16644</v>
+        <v>16664</v>
       </c>
       <c r="O112" s="7" t="n">
         <v>0</v>
@@ -9913,7 +9913,9 @@
       <c r="K121" s="7" t="n"/>
       <c r="L121" s="7" t="n"/>
       <c r="M121" s="7" t="n"/>
-      <c r="N121" s="7" t="n"/>
+      <c r="N121" s="7" t="n">
+        <v>20984</v>
+      </c>
       <c r="O121" s="7" t="n">
         <v>0</v>
       </c>
@@ -10475,13 +10477,13 @@
         </is>
       </c>
       <c r="C129" s="9" t="n">
-        <v>1600</v>
+        <v>2000</v>
       </c>
       <c r="D129" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E129" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
@@ -10490,12 +10492,12 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Portland Square F5, Apartment 5, City Centre, Bristol, BS2</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="I129" s="7" t="n"/>
@@ -10504,7 +10506,7 @@
       <c r="L129" s="7" t="n"/>
       <c r="M129" s="7" t="n"/>
       <c r="N129" s="7" t="n">
-        <v>20880</v>
+        <v>21840</v>
       </c>
       <c r="O129" s="7" t="n">
         <v>0</v>
@@ -10512,12 +10514,12 @@
       <c r="P129" s="7" t="n"/>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="R129" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S129" s="8" t="inlineStr"/>
@@ -10534,7 +10536,7 @@
       <c r="V129" s="6" t="inlineStr"/>
       <c r="W129" s="7" t="inlineStr">
         <is>
-          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
+          <t>abb5b090eb0d82e77672a39bb0facaa221a2c372</t>
         </is>
       </c>
     </row>
@@ -10548,13 +10550,13 @@
         </is>
       </c>
       <c r="C130" s="9" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="D130" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E130" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
@@ -10563,7 +10565,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Central Quay North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
@@ -10571,15 +10573,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I130" s="7" t="n">
-        <v>980</v>
-      </c>
+      <c r="I130" s="7" t="n"/>
       <c r="J130" s="7" t="n"/>
       <c r="K130" s="7" t="n"/>
       <c r="L130" s="7" t="n"/>
       <c r="M130" s="7" t="n"/>
       <c r="N130" s="7" t="n">
-        <v>21316</v>
+        <v>21100</v>
       </c>
       <c r="O130" s="7" t="n">
         <v>0</v>
@@ -10587,12 +10587,12 @@
       <c r="P130" s="7" t="n"/>
       <c r="Q130" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="R130" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S130" s="8" t="inlineStr"/>
@@ -10609,7 +10609,7 @@
       <c r="V130" s="6" t="inlineStr"/>
       <c r="W130" s="7" t="inlineStr">
         <is>
-          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
+          <t>946fbed419874f744b194aa1db09758bba46a7b8</t>
         </is>
       </c>
     </row>
@@ -10623,13 +10623,13 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>1995</v>
+        <v>2195</v>
       </c>
       <c r="D131" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E131" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
@@ -10638,7 +10638,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr">
@@ -10646,13 +10646,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I131" s="7" t="n"/>
+      <c r="I131" s="7" t="n">
+        <v>721</v>
+      </c>
       <c r="J131" s="7" t="n"/>
       <c r="K131" s="7" t="n"/>
       <c r="L131" s="7" t="n"/>
       <c r="M131" s="7" t="n"/>
       <c r="N131" s="7" t="n">
-        <v>21196</v>
+        <v>21732</v>
       </c>
       <c r="O131" s="7" t="n">
         <v>0</v>
@@ -10660,12 +10662,12 @@
       <c r="P131" s="7" t="n"/>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S131" s="8" t="inlineStr"/>
@@ -10682,7 +10684,7 @@
       <c r="V131" s="6" t="inlineStr"/>
       <c r="W131" s="7" t="inlineStr">
         <is>
-          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
+          <t>e7698846f0eb069392a121a58c1ce6d5329ed671</t>
         </is>
       </c>
     </row>
@@ -10696,13 +10698,13 @@
         </is>
       </c>
       <c r="C132" s="9" t="n">
-        <v>1750</v>
+        <v>1630</v>
       </c>
       <c r="D132" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E132" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
@@ -10711,7 +10713,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr">
@@ -10720,14 +10722,14 @@
         </is>
       </c>
       <c r="I132" s="7" t="n">
-        <v>849</v>
+        <v>480</v>
       </c>
       <c r="J132" s="7" t="n"/>
       <c r="K132" s="7" t="n"/>
       <c r="L132" s="7" t="n"/>
       <c r="M132" s="7" t="n"/>
       <c r="N132" s="7" t="n">
-        <v>21028</v>
+        <v>20984</v>
       </c>
       <c r="O132" s="7" t="n">
         <v>0</v>
@@ -10735,12 +10737,12 @@
       <c r="P132" s="7" t="n"/>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S132" s="8" t="inlineStr"/>
@@ -10757,7 +10759,7 @@
       <c r="V132" s="6" t="inlineStr"/>
       <c r="W132" s="7" t="inlineStr">
         <is>
-          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
+          <t>91a2f48a2e8c56a8be1e48fed1754ebc75163300</t>
         </is>
       </c>
     </row>
@@ -10771,13 +10773,13 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1550</v>
+        <v>1615</v>
       </c>
       <c r="D133" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E133" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
@@ -10786,21 +10788,23 @@
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>Portland Heights - St. Pauls</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I133" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I133" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>21420</v>
+        <v>21732</v>
       </c>
       <c r="O133" s="7" t="n">
         <v>0</v>
@@ -10808,12 +10812,12 @@
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Bishopston</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S133" s="8" t="inlineStr"/>
@@ -10830,7 +10834,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
+          <t>ee489ac0e36680c518a8b49a2cbf5f32b02e30a3</t>
         </is>
       </c>
     </row>
@@ -10844,13 +10848,13 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>1400</v>
+        <v>1600</v>
       </c>
       <c r="D134" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E134" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
@@ -10859,7 +10863,7 @@
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>The Atrium, Redcliffe Street, BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
@@ -10873,7 +10877,7 @@
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="7" t="n">
-        <v>20292</v>
+        <v>20880</v>
       </c>
       <c r="O134" s="7" t="n">
         <v>0</v>
@@ -10881,12 +10885,12 @@
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10903,7 +10907,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
+          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
         </is>
       </c>
     </row>
@@ -10917,13 +10921,13 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1150</v>
+        <v>1800</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E135" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
@@ -10932,21 +10936,23 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I135" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I135" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="7" t="n">
-        <v>15376</v>
+        <v>21316</v>
       </c>
       <c r="O135" s="7" t="n">
         <v>0</v>
@@ -10954,12 +10960,12 @@
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S135" s="8" t="inlineStr"/>
@@ -10976,7 +10982,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
+          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
         </is>
       </c>
     </row>
@@ -10990,7 +10996,7 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>1300</v>
+        <v>1995</v>
       </c>
       <c r="D136" s="7" t="n">
         <v>1</v>
@@ -11005,7 +11011,7 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The Milliners, BS1 6WU</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
@@ -11013,15 +11019,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I136" s="7" t="n">
-        <v>463</v>
-      </c>
+      <c r="I136" s="7" t="n"/>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>21440</v>
+        <v>21196</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -11029,12 +11033,12 @@
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11051,7 +11055,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
+          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
         </is>
       </c>
     </row>
@@ -11065,13 +11069,13 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1150</v>
+        <v>1750</v>
       </c>
       <c r="D137" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E137" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
@@ -11080,23 +11084,23 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Century Place, St. Paul Street, BS2 8AN</t>
+          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I137" s="7" t="n">
-        <v>344</v>
+        <v>849</v>
       </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="7" t="n">
-        <v>21792</v>
+        <v>21028</v>
       </c>
       <c r="O137" s="7" t="n">
         <v>0</v>
@@ -11104,12 +11108,12 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S137" s="8" t="inlineStr"/>
@@ -11126,7 +11130,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
+          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
         </is>
       </c>
     </row>
@@ -11140,7 +11144,7 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1800</v>
+        <v>1550</v>
       </c>
       <c r="D138" s="7" t="n">
         <v>2</v>
@@ -11155,12 +11159,12 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Waverley House, BS1</t>
+          <t>Portland Heights - St. Pauls</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I138" s="7" t="n"/>
@@ -11169,7 +11173,7 @@
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>17956</v>
+        <v>21420</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11177,12 +11181,12 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Ocean, Bishopston</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11199,7 +11203,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
+          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
         </is>
       </c>
     </row>
@@ -11213,13 +11217,13 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>2170</v>
+        <v>1400</v>
       </c>
       <c r="D139" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E139" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
@@ -11228,7 +11232,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>The Atrium, Redcliffe Street, BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11236,15 +11240,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I139" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I139" s="7" t="n"/>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>21732</v>
+        <v>20292</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11252,12 +11254,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11274,7 +11276,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
+          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
         </is>
       </c>
     </row>
@@ -11288,13 +11290,13 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1965</v>
+        <v>1150</v>
       </c>
       <c r="D140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
@@ -11303,23 +11305,21 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I140" s="7" t="n">
-        <v>771</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I140" s="7" t="n"/>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>21740</v>
+        <v>15376</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11327,12 +11327,12 @@
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11349,7 +11349,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
+          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
         </is>
       </c>
     </row>
@@ -11363,10 +11363,10 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1680</v>
+        <v>1300</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E141" s="7" t="n">
         <v>1</v>
@@ -11378,7 +11378,7 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>City Centre, The Milliners, BS1 6WU</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
@@ -11386,13 +11386,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I141" s="7" t="n"/>
+      <c r="I141" s="7" t="n">
+        <v>463</v>
+      </c>
       <c r="J141" s="7" t="n"/>
       <c r="K141" s="7" t="n"/>
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>20628</v>
+        <v>21440</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11400,12 +11402,12 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11422,7 +11424,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
+          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
         </is>
       </c>
     </row>
@@ -11436,7 +11438,7 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>1625</v>
+        <v>1150</v>
       </c>
       <c r="D142" s="7" t="n">
         <v>1</v>
@@ -11451,23 +11453,23 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Century Place, St. Paul Street, BS2 8AN</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I142" s="7" t="n">
-        <v>486</v>
+        <v>344</v>
       </c>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>21732</v>
+        <v>21792</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11475,12 +11477,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11497,7 +11499,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
+          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
         </is>
       </c>
     </row>
@@ -11511,7 +11513,7 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1940</v>
+        <v>1800</v>
       </c>
       <c r="D143" s="7" t="n">
         <v>2</v>
@@ -11526,7 +11528,7 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Waverley House, BS1</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
@@ -11534,15 +11536,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I143" s="7" t="n">
-        <v>607</v>
-      </c>
+      <c r="I143" s="7" t="n"/>
       <c r="J143" s="7" t="n"/>
       <c r="K143" s="7" t="n"/>
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>21740</v>
+        <v>17956</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11550,12 +11550,12 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11572,7 +11572,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
+          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
         </is>
       </c>
     </row>
@@ -11586,13 +11586,13 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1465</v>
+        <v>2170</v>
       </c>
       <c r="D144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
@@ -11601,7 +11601,7 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
@@ -11610,14 +11610,14 @@
         </is>
       </c>
       <c r="I144" s="7" t="n">
-        <v>505</v>
+        <v>721</v>
       </c>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>21816</v>
+        <v>21732</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11625,12 +11625,12 @@
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11647,7 +11647,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>e86143466441bbbf802706245b19ef679ec29055</t>
+          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
         </is>
       </c>
     </row>
@@ -11661,7 +11661,7 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>2300</v>
+        <v>1965</v>
       </c>
       <c r="D145" s="7" t="n">
         <v>2</v>
@@ -11676,23 +11676,23 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I145" s="7" t="n">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>22072</v>
+        <v>21740</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11700,12 +11700,12 @@
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S145" s="8" t="inlineStr"/>
@@ -11722,7 +11722,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>7594e7db3c52acddddafbbdb135025e4f15aa52c</t>
+          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
         </is>
       </c>
     </row>
@@ -11736,10 +11736,10 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>1150</v>
+        <v>1680</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E146" s="7" t="n">
         <v>1</v>
@@ -11751,12 +11751,12 @@
       </c>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>St. Philips, Bristol, BS2</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I146" s="7" t="n"/>
@@ -11765,7 +11765,7 @@
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>20784</v>
+        <v>20628</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>0</v>
@@ -11773,7 +11773,7 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
@@ -11795,7 +11795,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
+          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
         </is>
       </c>
     </row>
@@ -11809,7 +11809,7 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>1685</v>
+        <v>1625</v>
       </c>
       <c r="D147" s="7" t="n">
         <v>1</v>
@@ -11824,7 +11824,7 @@
       </c>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H147" s="7" t="inlineStr">
@@ -11833,14 +11833,14 @@
         </is>
       </c>
       <c r="I147" s="7" t="n">
-        <v>545</v>
+        <v>486</v>
       </c>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="7" t="n">
-        <v>21024</v>
+        <v>21732</v>
       </c>
       <c r="O147" s="7" t="n">
         <v>0</v>
@@ -11848,12 +11848,12 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S147" s="8" t="inlineStr"/>
@@ -11870,7 +11870,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
+          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
         </is>
       </c>
     </row>
@@ -11884,7 +11884,7 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>1700</v>
+        <v>1940</v>
       </c>
       <c r="D148" s="7" t="n">
         <v>2</v>
@@ -11894,26 +11894,28 @@
       </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Dunkerry Road - Windmill Hill</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I148" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I148" s="7" t="n">
+        <v>607</v>
+      </c>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>8448</v>
+        <v>21740</v>
       </c>
       <c r="O148" s="7" t="n">
         <v>0</v>
@@ -11921,12 +11923,12 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11943,7 +11945,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
+          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
         </is>
       </c>
     </row>
@@ -11957,7 +11959,7 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>1460</v>
+        <v>1465</v>
       </c>
       <c r="D149" s="7" t="n">
         <v>1</v>
@@ -11981,14 +11983,14 @@
         </is>
       </c>
       <c r="I149" s="7" t="n">
-        <v>473</v>
+        <v>505</v>
       </c>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="7" t="n">
-        <v>13840</v>
+        <v>21816</v>
       </c>
       <c r="O149" s="7" t="n">
         <v>0</v>
@@ -11996,7 +11998,7 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
@@ -12018,7 +12020,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
+          <t>e86143466441bbbf802706245b19ef679ec29055</t>
         </is>
       </c>
     </row>
@@ -12032,13 +12034,13 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1630</v>
+        <v>2300</v>
       </c>
       <c r="D150" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E150" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
@@ -12047,36 +12049,36 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Castle Park View, Castle Street, Bristol</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I150" s="7" t="n">
-        <v>486</v>
+        <v>773</v>
       </c>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>13860</v>
+        <v>22072</v>
       </c>
       <c r="O150" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Savills Lettings, CPV</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12093,7 +12095,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
+          <t>7594e7db3c52acddddafbbdb135025e4f15aa52c</t>
         </is>
       </c>
     </row>
@@ -12107,7 +12109,7 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1625</v>
+        <v>1150</v>
       </c>
       <c r="D151" s="7" t="n">
         <v>1</v>
@@ -12122,23 +12124,21 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>St. Philips, Bristol, BS2</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I151" s="7" t="n">
-        <v>486</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I151" s="7" t="n"/>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>21732</v>
+        <v>20784</v>
       </c>
       <c r="O151" s="7" t="n">
         <v>0</v>
@@ -12146,12 +12146,12 @@
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12168,7 +12168,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
+          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
         </is>
       </c>
     </row>
@@ -12182,13 +12182,13 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1650</v>
+        <v>1685</v>
       </c>
       <c r="D152" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E152" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
@@ -12197,7 +12197,7 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Harris Lofts, BS1 4BB</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
@@ -12206,14 +12206,14 @@
         </is>
       </c>
       <c r="I152" s="7" t="n">
-        <v>667</v>
+        <v>545</v>
       </c>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>20088</v>
+        <v>21024</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12221,12 +12221,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12243,7 +12243,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
+          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
         </is>
       </c>
     </row>
@@ -12257,27 +12257,27 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>1650</v>
+        <v>1700</v>
       </c>
       <c r="D153" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E153" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Central Quey North, Broad Quay, BS1</t>
+          <t>Dunkerry Road - Windmill Hill</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I153" s="7" t="n"/>
@@ -12286,7 +12286,7 @@
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>20768</v>
+        <v>8448</v>
       </c>
       <c r="O153" s="7" t="n">
         <v>0</v>
@@ -12294,12 +12294,12 @@
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12316,7 +12316,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
+          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
         </is>
       </c>
     </row>
@@ -12330,7 +12330,7 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1550</v>
+        <v>1460</v>
       </c>
       <c r="D154" s="7" t="n">
         <v>1</v>
@@ -12345,7 +12345,7 @@
       </c>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr">
@@ -12353,13 +12353,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I154" s="7" t="n"/>
+      <c r="I154" s="7" t="n">
+        <v>473</v>
+      </c>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="7" t="n">
-        <v>21100</v>
+        <v>13840</v>
       </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
@@ -12367,12 +12369,12 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S154" s="8" t="inlineStr"/>
@@ -12389,7 +12391,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
+          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
         </is>
       </c>
     </row>
@@ -12403,7 +12405,7 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>1390</v>
+        <v>1630</v>
       </c>
       <c r="D155" s="7" t="n">
         <v>1</v>
@@ -12418,7 +12420,7 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
@@ -12426,24 +12428,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I155" s="7" t="n"/>
+      <c r="I155" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J155" s="7" t="n"/>
       <c r="K155" s="7" t="n"/>
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
-      <c r="N155" s="7" t="n"/>
+      <c r="N155" s="7" t="n">
+        <v>13860</v>
+      </c>
       <c r="O155" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12460,7 +12466,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
+          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
         </is>
       </c>
     </row>
@@ -12474,7 +12480,7 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>1485</v>
+        <v>1625</v>
       </c>
       <c r="D156" s="7" t="n">
         <v>1</v>
@@ -12489,7 +12495,7 @@
       </c>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr">
@@ -12498,14 +12504,14 @@
         </is>
       </c>
       <c r="I156" s="7" t="n">
-        <v>470</v>
+        <v>486</v>
       </c>
       <c r="J156" s="7" t="n"/>
       <c r="K156" s="7" t="n"/>
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O156" s="7" t="n">
         <v>0</v>
@@ -12513,12 +12519,12 @@
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S156" s="8" t="inlineStr"/>
@@ -12535,7 +12541,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
+          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
         </is>
       </c>
     </row>
@@ -12549,13 +12555,13 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>1635</v>
+        <v>1650</v>
       </c>
       <c r="D157" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E157" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
@@ -12564,7 +12570,7 @@
       </c>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Harbourside, Harris Lofts, BS1 4BB</t>
         </is>
       </c>
       <c r="H157" s="7" t="inlineStr">
@@ -12573,14 +12579,14 @@
         </is>
       </c>
       <c r="I157" s="7" t="n">
-        <v>486</v>
+        <v>667</v>
       </c>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="7" t="n">
-        <v>21732</v>
+        <v>20088</v>
       </c>
       <c r="O157" s="7" t="n">
         <v>0</v>
@@ -12588,12 +12594,12 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S157" s="8" t="inlineStr"/>
@@ -12610,7 +12616,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
+          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
         </is>
       </c>
     </row>
@@ -12624,13 +12630,13 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>2060</v>
+        <v>1650</v>
       </c>
       <c r="D158" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E158" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F158" s="7" t="inlineStr">
         <is>
@@ -12639,7 +12645,7 @@
       </c>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Central Quey North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H158" s="7" t="inlineStr">
@@ -12647,15 +12653,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I158" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I158" s="7" t="n"/>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>21732</v>
+        <v>20768</v>
       </c>
       <c r="O158" s="7" t="n">
         <v>0</v>
@@ -12663,12 +12667,12 @@
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S158" s="8" t="inlineStr"/>
@@ -12685,7 +12689,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
+          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
         </is>
       </c>
     </row>
@@ -12699,7 +12703,7 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1545</v>
+        <v>1550</v>
       </c>
       <c r="D159" s="7" t="n">
         <v>1</v>
@@ -12714,7 +12718,7 @@
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
@@ -12722,15 +12726,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I159" s="7" t="n">
-        <v>548</v>
-      </c>
+      <c r="I159" s="7" t="n"/>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="7" t="n">
-        <v>21740</v>
+        <v>21100</v>
       </c>
       <c r="O159" s="7" t="n">
         <v>0</v>
@@ -12738,12 +12740,12 @@
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12760,7 +12762,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
+          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
         </is>
       </c>
     </row>
@@ -12774,7 +12776,7 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>1640</v>
+        <v>1390</v>
       </c>
       <c r="D160" s="7" t="n">
         <v>1</v>
@@ -12789,7 +12791,7 @@
       </c>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H160" s="7" t="inlineStr">
@@ -12797,28 +12799,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I160" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I160" s="7" t="n"/>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
-      <c r="N160" s="7" t="n">
-        <v>21732</v>
-      </c>
+      <c r="N160" s="7" t="n"/>
       <c r="O160" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S160" s="8" t="inlineStr"/>
@@ -12835,7 +12833,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
+          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
         </is>
       </c>
     </row>
@@ -12849,10 +12847,10 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>2115</v>
+        <v>1485</v>
       </c>
       <c r="D161" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E161" s="7" t="n">
         <v>1</v>
@@ -12864,7 +12862,7 @@
       </c>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H161" s="7" t="inlineStr">
@@ -12873,14 +12871,14 @@
         </is>
       </c>
       <c r="I161" s="7" t="n">
-        <v>722</v>
+        <v>470</v>
       </c>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
       <c r="N161" s="7" t="n">
-        <v>21732</v>
+        <v>21740</v>
       </c>
       <c r="O161" s="7" t="n">
         <v>0</v>
@@ -12888,12 +12886,12 @@
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S161" s="8" t="inlineStr"/>
@@ -12910,7 +12908,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
+          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
         </is>
       </c>
     </row>
@@ -12924,13 +12922,13 @@
         </is>
       </c>
       <c r="C162" s="9" t="n">
-        <v>1970</v>
+        <v>1635</v>
       </c>
       <c r="D162" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E162" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F162" s="7" t="inlineStr">
         <is>
@@ -12939,7 +12937,7 @@
       </c>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
@@ -12948,14 +12946,14 @@
         </is>
       </c>
       <c r="I162" s="7" t="n">
-        <v>750</v>
+        <v>486</v>
       </c>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
       <c r="N162" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O162" s="7" t="n">
         <v>0</v>
@@ -12963,12 +12961,12 @@
       <c r="P162" s="7" t="n"/>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S162" s="8" t="inlineStr"/>
@@ -12985,7 +12983,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
+          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
         </is>
       </c>
     </row>
@@ -12999,13 +12997,13 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1575</v>
+        <v>2060</v>
       </c>
       <c r="D163" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E163" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F163" s="7" t="inlineStr">
         <is>
@@ -13014,7 +13012,7 @@
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
@@ -13023,14 +13021,14 @@
         </is>
       </c>
       <c r="I163" s="7" t="n">
-        <v>430</v>
+        <v>721</v>
       </c>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="7" t="n">
-        <v>21816</v>
+        <v>21732</v>
       </c>
       <c r="O163" s="7" t="n">
         <v>0</v>
@@ -13038,12 +13036,12 @@
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13060,7 +13058,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
+          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
         </is>
       </c>
     </row>
@@ -13074,7 +13072,7 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>1350</v>
+        <v>1545</v>
       </c>
       <c r="D164" s="7" t="n">
         <v>1</v>
@@ -13089,7 +13087,7 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Invicta, Millenium Promenade, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
@@ -13097,13 +13095,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I164" s="7" t="n"/>
+      <c r="I164" s="7" t="n">
+        <v>548</v>
+      </c>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="7" t="n">
-        <v>17344</v>
+        <v>21740</v>
       </c>
       <c r="O164" s="7" t="n">
         <v>0</v>
@@ -13111,12 +13111,12 @@
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13133,7 +13133,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
+          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
         </is>
       </c>
     </row>
@@ -13147,7 +13147,7 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1600</v>
+        <v>1640</v>
       </c>
       <c r="D165" s="7" t="n">
         <v>1</v>
@@ -13162,7 +13162,7 @@
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H165" s="7" t="inlineStr">
@@ -13170,13 +13170,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I165" s="7" t="n"/>
+      <c r="I165" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>13404</v>
+        <v>21732</v>
       </c>
       <c r="O165" s="7" t="n">
         <v>0</v>
@@ -13184,12 +13186,12 @@
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R165" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S165" s="8" t="inlineStr"/>
@@ -13206,7 +13208,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
+          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
         </is>
       </c>
     </row>
@@ -13220,7 +13222,7 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>1700</v>
+        <v>2115</v>
       </c>
       <c r="D166" s="7" t="n">
         <v>2</v>
@@ -13235,7 +13237,7 @@
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H166" s="7" t="inlineStr">
@@ -13244,14 +13246,14 @@
         </is>
       </c>
       <c r="I166" s="7" t="n">
-        <v>646</v>
+        <v>722</v>
       </c>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="7" t="n">
-        <v>20928</v>
+        <v>21732</v>
       </c>
       <c r="O166" s="7" t="n">
         <v>0</v>
@@ -13259,12 +13261,12 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
@@ -13281,7 +13283,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
+          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
         </is>
       </c>
     </row>
@@ -13295,7 +13297,7 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>2105</v>
+        <v>1970</v>
       </c>
       <c r="D167" s="7" t="n">
         <v>2</v>
@@ -13310,7 +13312,7 @@
       </c>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H167" s="7" t="inlineStr">
@@ -13319,14 +13321,14 @@
         </is>
       </c>
       <c r="I167" s="7" t="n">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="7" t="n">
-        <v>20984</v>
+        <v>21740</v>
       </c>
       <c r="O167" s="7" t="n">
         <v>0</v>
@@ -13334,12 +13336,12 @@
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S167" s="8" t="inlineStr"/>
@@ -13356,7 +13358,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
+          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
         </is>
       </c>
     </row>
@@ -13370,7 +13372,7 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1595</v>
+        <v>1575</v>
       </c>
       <c r="D168" s="7" t="n">
         <v>1</v>
@@ -13385,7 +13387,7 @@
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
@@ -13394,14 +13396,14 @@
         </is>
       </c>
       <c r="I168" s="7" t="n">
-        <v>484</v>
+        <v>430</v>
       </c>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="7" t="n">
-        <v>21732</v>
+        <v>21816</v>
       </c>
       <c r="O168" s="7" t="n">
         <v>0</v>
@@ -13409,12 +13411,12 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13431,7 +13433,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
+          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
         </is>
       </c>
     </row>
@@ -13445,10 +13447,10 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1999</v>
+        <v>1350</v>
       </c>
       <c r="D169" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E169" s="7" t="n">
         <v>1</v>
@@ -13460,12 +13462,12 @@
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Invicta, Millenium Promenade, BS1</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I169" s="7" t="n"/>
@@ -13474,7 +13476,7 @@
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>21736</v>
+        <v>17344</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13482,12 +13484,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13504,7 +13506,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
+          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
         </is>
       </c>
     </row>
@@ -13518,7 +13520,7 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>1605</v>
+        <v>1600</v>
       </c>
       <c r="D170" s="7" t="n">
         <v>1</v>
@@ -13533,7 +13535,7 @@
       </c>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Central Quay North, Bristol, BS1</t>
         </is>
       </c>
       <c r="H170" s="7" t="inlineStr">
@@ -13541,15 +13543,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I170" s="7" t="n">
-        <v>487</v>
-      </c>
+      <c r="I170" s="7" t="n"/>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
       <c r="L170" s="7" t="n"/>
       <c r="M170" s="7" t="n"/>
       <c r="N170" s="7" t="n">
-        <v>21732</v>
+        <v>13404</v>
       </c>
       <c r="O170" s="7" t="n">
         <v>0</v>
@@ -13557,12 +13557,12 @@
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -13579,7 +13579,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
+          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
         </is>
       </c>
     </row>
@@ -13593,10 +13593,10 @@
         </is>
       </c>
       <c r="C171" s="9" t="n">
-        <v>1390</v>
+        <v>1700</v>
       </c>
       <c r="D171" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E171" s="7" t="n">
         <v>1</v>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
         </is>
       </c>
       <c r="H171" s="7" t="inlineStr">
@@ -13616,24 +13616,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I171" s="7" t="n"/>
+      <c r="I171" s="7" t="n">
+        <v>646</v>
+      </c>
       <c r="J171" s="7" t="n"/>
       <c r="K171" s="7" t="n"/>
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
-      <c r="N171" s="7" t="n"/>
+      <c r="N171" s="7" t="n">
+        <v>20928</v>
+      </c>
       <c r="O171" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -13650,7 +13654,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
         </is>
       </c>
     </row>
@@ -13664,13 +13668,13 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1395</v>
+        <v>2105</v>
       </c>
       <c r="D172" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E172" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F172" s="7" t="inlineStr">
         <is>
@@ -13679,7 +13683,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H172" s="7" t="inlineStr">
@@ -13687,13 +13691,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I172" s="7" t="n"/>
+      <c r="I172" s="7" t="n">
+        <v>745</v>
+      </c>
       <c r="J172" s="7" t="n"/>
       <c r="K172" s="7" t="n"/>
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="7" t="n">
-        <v>20524</v>
+        <v>20984</v>
       </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
@@ -13701,12 +13707,12 @@
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -13723,7 +13729,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
         </is>
       </c>
     </row>
@@ -13737,7 +13743,7 @@
         </is>
       </c>
       <c r="C173" s="9" t="n">
-        <v>1200</v>
+        <v>1595</v>
       </c>
       <c r="D173" s="7" t="n">
         <v>1</v>
@@ -13747,28 +13753,28 @@
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2 0JN</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I173" s="7" t="n">
-        <v>452</v>
+        <v>484</v>
       </c>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>20472</v>
+        <v>21732</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13776,12 +13782,12 @@
       <c r="P173" s="7" t="n"/>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -13798,7 +13804,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
+          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
         </is>
       </c>
     </row>
@@ -13812,10 +13818,10 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1450</v>
+        <v>1999</v>
       </c>
       <c r="D174" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E174" s="7" t="n">
         <v>1</v>
@@ -13827,12 +13833,12 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I174" s="7" t="n"/>
@@ -13841,7 +13847,7 @@
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>16664</v>
+        <v>21736</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13849,12 +13855,12 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -13871,7 +13877,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
+          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
         </is>
       </c>
     </row>
@@ -13885,13 +13891,13 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>3200</v>
+        <v>1605</v>
       </c>
       <c r="D175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
@@ -13900,7 +13906,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
@@ -13908,13 +13914,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I175" s="7" t="n"/>
+      <c r="I175" s="7" t="n">
+        <v>487</v>
+      </c>
       <c r="J175" s="7" t="n"/>
       <c r="K175" s="7" t="n"/>
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
       <c r="N175" s="7" t="n">
-        <v>16664</v>
+        <v>21732</v>
       </c>
       <c r="O175" s="7" t="n">
         <v>0</v>
@@ -13922,12 +13930,12 @@
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
         <is>
-          <t>LettingaProperty.com, Nationwide - Lettings</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -13944,7 +13952,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
+          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
         </is>
       </c>
     </row>
@@ -13958,7 +13966,7 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>1600</v>
+        <v>1390</v>
       </c>
       <c r="D176" s="7" t="n">
         <v>1</v>
@@ -13973,7 +13981,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H176" s="7" t="inlineStr">
@@ -13986,21 +13994,19 @@
       <c r="K176" s="7" t="n"/>
       <c r="L176" s="7" t="n"/>
       <c r="M176" s="7" t="n"/>
-      <c r="N176" s="7" t="n">
-        <v>21996</v>
-      </c>
+      <c r="N176" s="7" t="n"/>
       <c r="O176" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -14017,7 +14023,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
+          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
         </is>
       </c>
     </row>
@@ -14031,13 +14037,13 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>2400</v>
+        <v>1395</v>
       </c>
       <c r="D177" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E177" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F177" s="7" t="inlineStr">
         <is>
@@ -14046,7 +14052,7 @@
       </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>Colston Avenue, Bristol, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H177" s="7" t="inlineStr">
@@ -14060,7 +14066,7 @@
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
       <c r="N177" s="7" t="n">
-        <v>14108</v>
+        <v>20524</v>
       </c>
       <c r="O177" s="7" t="n">
         <v>0</v>
@@ -14068,7 +14074,7 @@
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
@@ -14090,7 +14096,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
@@ -14104,7 +14110,7 @@
         </is>
       </c>
       <c r="C178" s="9" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="D178" s="7" t="n">
         <v>1</v>
@@ -14114,28 +14120,28 @@
       </c>
       <c r="F178" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t>East Street, Bedminster, BS3</t>
+          <t>Sweetman Place, Bristol, BS2 0JN</t>
         </is>
       </c>
       <c r="H178" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I178" s="7" t="n">
-        <v>560</v>
+        <v>452</v>
       </c>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
       <c r="L178" s="7" t="n"/>
       <c r="M178" s="7" t="n"/>
       <c r="N178" s="7" t="n">
-        <v>14176</v>
+        <v>20472</v>
       </c>
       <c r="O178" s="7" t="n">
         <v>0</v>
@@ -14143,12 +14149,12 @@
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
         <is>
-          <t>Xeno Property, Bristol</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S178" s="8" t="inlineStr"/>
@@ -14165,7 +14171,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
+          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
         </is>
       </c>
     </row>
@@ -14194,7 +14200,7 @@
       </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
         </is>
       </c>
       <c r="H179" s="7" t="inlineStr">
@@ -14208,7 +14214,7 @@
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
       <c r="N179" s="7" t="n">
-        <v>13668</v>
+        <v>16664</v>
       </c>
       <c r="O179" s="7" t="n">
         <v>0</v>
@@ -14216,12 +14222,12 @@
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
         <is>
-          <t>Wildheart Residential Management Limited, Epsom</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -14238,7 +14244,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
+          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
         </is>
       </c>
     </row>
@@ -14252,13 +14258,13 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>1605</v>
+        <v>3200</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E180" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F180" s="7" t="inlineStr">
         <is>
@@ -14267,7 +14273,7 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
@@ -14275,15 +14281,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I180" s="7" t="n">
-        <v>487</v>
-      </c>
+      <c r="I180" s="7" t="n"/>
       <c r="J180" s="7" t="n"/>
       <c r="K180" s="7" t="n"/>
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="7" t="n">
-        <v>13860</v>
+        <v>16664</v>
       </c>
       <c r="O180" s="7" t="n">
         <v>0</v>
@@ -14291,12 +14295,12 @@
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>LettingaProperty.com, Nationwide - Lettings</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14313,7 +14317,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
+          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
         </is>
       </c>
     </row>
@@ -14327,13 +14331,13 @@
         </is>
       </c>
       <c r="C181" s="9" t="n">
-        <v>2185</v>
+        <v>1600</v>
       </c>
       <c r="D181" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E181" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F181" s="7" t="inlineStr">
         <is>
@@ -14342,7 +14346,7 @@
       </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H181" s="7" t="inlineStr">
@@ -14350,15 +14354,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I181" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I181" s="7" t="n"/>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="7" t="n">
-        <v>13860</v>
+        <v>21996</v>
       </c>
       <c r="O181" s="7" t="n">
         <v>0</v>
@@ -14366,12 +14368,12 @@
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S181" s="8" t="inlineStr"/>
@@ -14388,7 +14390,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
+          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
         </is>
       </c>
     </row>
@@ -14402,13 +14404,13 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>1640</v>
+        <v>2400</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
@@ -14417,7 +14419,7 @@
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Colston Avenue, Bristol, BS1</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
@@ -14425,15 +14427,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I182" s="7" t="n">
-        <v>484</v>
-      </c>
+      <c r="I182" s="7" t="n"/>
       <c r="J182" s="7" t="n"/>
       <c r="K182" s="7" t="n"/>
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>13860</v>
+        <v>14108</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14441,12 +14441,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14463,7 +14463,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
+          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
         </is>
       </c>
     </row>
@@ -14477,13 +14477,13 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>2010</v>
+        <v>1300</v>
       </c>
       <c r="D183" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E183" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F183" s="7" t="inlineStr">
         <is>
@@ -14492,23 +14492,23 @@
       </c>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>East Street, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H183" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I183" s="7" t="n">
-        <v>722</v>
+        <v>560</v>
       </c>
       <c r="J183" s="7" t="n"/>
       <c r="K183" s="7" t="n"/>
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="7" t="n">
-        <v>13860</v>
+        <v>14176</v>
       </c>
       <c r="O183" s="7" t="n">
         <v>0</v>
@@ -14516,12 +14516,12 @@
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Xeno Property, Bristol</t>
         </is>
       </c>
       <c r="S183" s="8" t="inlineStr"/>
@@ -14538,7 +14538,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
+          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
         </is>
       </c>
     </row>
@@ -14552,7 +14552,7 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>1635</v>
+        <v>1450</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>1</v>
@@ -14567,7 +14567,7 @@
       </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Welsh Back, Bristol</t>
         </is>
       </c>
       <c r="H184" s="7" t="inlineStr">
@@ -14575,15 +14575,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I184" s="7" t="n">
-        <v>560</v>
-      </c>
+      <c r="I184" s="7" t="n"/>
       <c r="J184" s="7" t="n"/>
       <c r="K184" s="7" t="n"/>
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
       <c r="N184" s="7" t="n">
-        <v>13356</v>
+        <v>13668</v>
       </c>
       <c r="O184" s="7" t="n">
         <v>0</v>
@@ -14591,12 +14589,12 @@
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Wildheart Residential Management Limited, Epsom</t>
         </is>
       </c>
       <c r="S184" s="8" t="inlineStr"/>
@@ -14613,7 +14611,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
+          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
         </is>
       </c>
     </row>
@@ -14627,7 +14625,7 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>1665</v>
+        <v>1605</v>
       </c>
       <c r="D185" s="7" t="n">
         <v>1</v>
@@ -14642,7 +14640,7 @@
       </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
@@ -14651,14 +14649,14 @@
         </is>
       </c>
       <c r="I185" s="7" t="n">
-        <v>434</v>
+        <v>487</v>
       </c>
       <c r="J185" s="7" t="n"/>
       <c r="K185" s="7" t="n"/>
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O185" s="7" t="n">
         <v>0</v>
@@ -14666,12 +14664,12 @@
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S185" s="8" t="inlineStr"/>
@@ -14688,7 +14686,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
+          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
         </is>
       </c>
     </row>
@@ -14702,7 +14700,7 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>1990</v>
+        <v>2185</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>2</v>
@@ -14717,7 +14715,7 @@
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
@@ -14726,27 +14724,27 @@
         </is>
       </c>
       <c r="I186" s="7" t="n">
-        <v>682</v>
+        <v>721</v>
       </c>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O186" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14763,7 +14761,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
+          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
         </is>
       </c>
     </row>
@@ -14777,7 +14775,7 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>1480</v>
+        <v>1640</v>
       </c>
       <c r="D187" s="7" t="n">
         <v>1</v>
@@ -14792,7 +14790,7 @@
       </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
@@ -14801,27 +14799,27 @@
         </is>
       </c>
       <c r="I187" s="7" t="n">
-        <v>417</v>
+        <v>484</v>
       </c>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O187" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S187" s="8" t="inlineStr"/>
@@ -14838,7 +14836,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
+          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
         </is>
       </c>
     </row>
@@ -14852,7 +14850,7 @@
         </is>
       </c>
       <c r="C188" s="9" t="n">
-        <v>1750</v>
+        <v>2010</v>
       </c>
       <c r="D188" s="7" t="n">
         <v>2</v>
@@ -14867,7 +14865,7 @@
       </c>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
@@ -14875,13 +14873,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I188" s="7" t="n"/>
+      <c r="I188" s="7" t="n">
+        <v>722</v>
+      </c>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
       <c r="L188" s="7" t="n"/>
       <c r="M188" s="7" t="n"/>
       <c r="N188" s="7" t="n">
-        <v>20828</v>
+        <v>13860</v>
       </c>
       <c r="O188" s="7" t="n">
         <v>0</v>
@@ -14889,12 +14889,12 @@
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S188" s="8" t="inlineStr"/>
@@ -14911,7 +14911,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
+          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
         </is>
       </c>
     </row>
@@ -14925,13 +14925,13 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>2080</v>
+        <v>1635</v>
       </c>
       <c r="D189" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E189" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F189" s="7" t="inlineStr">
         <is>
@@ -14949,7 +14949,7 @@
         </is>
       </c>
       <c r="I189" s="7" t="n">
-        <v>705</v>
+        <v>560</v>
       </c>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
@@ -14959,12 +14959,12 @@
         <v>13356</v>
       </c>
       <c r="O189" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R189" s="7" t="inlineStr">
@@ -14986,7 +14986,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
+          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
         </is>
       </c>
     </row>
@@ -15000,7 +15000,7 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>1680</v>
+        <v>1665</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1</v>
@@ -15015,7 +15015,7 @@
       </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
@@ -15024,27 +15024,27 @@
         </is>
       </c>
       <c r="I190" s="7" t="n">
-        <v>487</v>
+        <v>434</v>
       </c>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O190" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S190" s="8" t="inlineStr"/>
@@ -15061,7 +15061,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
+          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
         </is>
       </c>
     </row>
@@ -15075,7 +15075,7 @@
         </is>
       </c>
       <c r="C191" s="9" t="n">
-        <v>1845</v>
+        <v>1990</v>
       </c>
       <c r="D191" s="7" t="n">
         <v>2</v>
@@ -15099,22 +15099,22 @@
         </is>
       </c>
       <c r="I191" s="7" t="n">
-        <v>641</v>
+        <v>682</v>
       </c>
       <c r="J191" s="7" t="n"/>
       <c r="K191" s="7" t="n"/>
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
       <c r="N191" s="7" t="n">
-        <v>21476</v>
+        <v>13964</v>
       </c>
       <c r="O191" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P191" s="7" t="n"/>
       <c r="Q191" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R191" s="7" t="inlineStr">
@@ -15136,7 +15136,7 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
-          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
+          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
         </is>
       </c>
     </row>
@@ -15150,7 +15150,7 @@
         </is>
       </c>
       <c r="C192" s="9" t="n">
-        <v>1685</v>
+        <v>1480</v>
       </c>
       <c r="D192" s="7" t="n">
         <v>1</v>
@@ -15174,7 +15174,7 @@
         </is>
       </c>
       <c r="I192" s="7" t="n">
-        <v>578</v>
+        <v>417</v>
       </c>
       <c r="J192" s="7" t="n"/>
       <c r="K192" s="7" t="n"/>
@@ -15189,7 +15189,7 @@
       <c r="P192" s="7" t="n"/>
       <c r="Q192" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R192" s="7" t="inlineStr">
@@ -15211,7 +15211,7 @@
       <c r="V192" s="6" t="inlineStr"/>
       <c r="W192" s="7" t="inlineStr">
         <is>
-          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
+          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
         </is>
       </c>
     </row>
@@ -15225,13 +15225,13 @@
         </is>
       </c>
       <c r="C193" s="9" t="n">
-        <v>1765</v>
+        <v>1750</v>
       </c>
       <c r="D193" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E193" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F193" s="7" t="inlineStr">
         <is>
@@ -15240,7 +15240,7 @@
       </c>
       <c r="G193" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H193" s="7" t="inlineStr">
@@ -15248,28 +15248,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I193" s="7" t="n">
-        <v>641</v>
-      </c>
+      <c r="I193" s="7" t="n"/>
       <c r="J193" s="7" t="n"/>
       <c r="K193" s="7" t="n"/>
       <c r="L193" s="7" t="n"/>
       <c r="M193" s="7" t="n"/>
       <c r="N193" s="7" t="n">
-        <v>13356</v>
+        <v>20828</v>
       </c>
       <c r="O193" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P193" s="7" t="n"/>
       <c r="Q193" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R193" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S193" s="8" t="inlineStr"/>
@@ -15286,7 +15284,7 @@
       <c r="V193" s="6" t="inlineStr"/>
       <c r="W193" s="7" t="inlineStr">
         <is>
-          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
+          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
         </is>
       </c>
     </row>
@@ -15300,7 +15298,7 @@
         </is>
       </c>
       <c r="C194" s="9" t="n">
-        <v>2240</v>
+        <v>2080</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>2</v>
@@ -15324,22 +15322,22 @@
         </is>
       </c>
       <c r="I194" s="7" t="n">
-        <v>884</v>
+        <v>705</v>
       </c>
       <c r="J194" s="7" t="n"/>
       <c r="K194" s="7" t="n"/>
       <c r="L194" s="7" t="n"/>
       <c r="M194" s="7" t="n"/>
       <c r="N194" s="7" t="n">
-        <v>13388</v>
+        <v>13356</v>
       </c>
       <c r="O194" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P194" s="7" t="n"/>
       <c r="Q194" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R194" s="7" t="inlineStr">
@@ -15361,7 +15359,7 @@
       <c r="V194" s="6" t="inlineStr"/>
       <c r="W194" s="7" t="inlineStr">
         <is>
-          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
+          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
         </is>
       </c>
     </row>
@@ -15375,7 +15373,7 @@
         </is>
       </c>
       <c r="C195" s="9" t="n">
-        <v>1150</v>
+        <v>1680</v>
       </c>
       <c r="D195" s="7" t="n">
         <v>1</v>
@@ -15390,7 +15388,7 @@
       </c>
       <c r="G195" s="8" t="inlineStr">
         <is>
-          <t>John Street, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H195" s="7" t="inlineStr">
@@ -15399,25 +15397,27 @@
         </is>
       </c>
       <c r="I195" s="7" t="n">
-        <v>248</v>
+        <v>487</v>
       </c>
       <c r="J195" s="7" t="n"/>
       <c r="K195" s="7" t="n"/>
       <c r="L195" s="7" t="n"/>
       <c r="M195" s="7" t="n"/>
-      <c r="N195" s="7" t="n"/>
+      <c r="N195" s="7" t="n">
+        <v>13356</v>
+      </c>
       <c r="O195" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P195" s="7" t="n"/>
       <c r="Q195" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R195" s="7" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S195" s="8" t="inlineStr"/>
@@ -15434,7 +15434,7 @@
       <c r="V195" s="6" t="inlineStr"/>
       <c r="W195" s="7" t="inlineStr">
         <is>
-          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
+          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
         </is>
       </c>
     </row>
@@ -15448,49 +15448,51 @@
         </is>
       </c>
       <c r="C196" s="9" t="n">
-        <v>3400</v>
+        <v>1845</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E196" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F196" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t>Barton Road, Bristol, BS2</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H196" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I196" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I196" s="7" t="n">
+        <v>641</v>
+      </c>
       <c r="J196" s="7" t="n"/>
       <c r="K196" s="7" t="n"/>
       <c r="L196" s="7" t="n"/>
       <c r="M196" s="7" t="n"/>
       <c r="N196" s="7" t="n">
-        <v>19720</v>
+        <v>21476</v>
       </c>
       <c r="O196" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P196" s="7" t="n"/>
       <c r="Q196" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R196" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S196" s="8" t="inlineStr"/>
@@ -15507,7 +15509,7 @@
       <c r="V196" s="6" t="inlineStr"/>
       <c r="W196" s="7" t="inlineStr">
         <is>
-          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
+          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
         </is>
       </c>
     </row>
@@ -15521,7 +15523,7 @@
         </is>
       </c>
       <c r="C197" s="9" t="n">
-        <v>1250</v>
+        <v>1685</v>
       </c>
       <c r="D197" s="7" t="n">
         <v>1</v>
@@ -15536,21 +15538,23 @@
       </c>
       <c r="G197" s="8" t="inlineStr">
         <is>
-          <t>St Peters Court, Bedminster</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H197" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I197" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I197" s="7" t="n">
+        <v>578</v>
+      </c>
       <c r="J197" s="7" t="n"/>
       <c r="K197" s="7" t="n"/>
       <c r="L197" s="7" t="n"/>
       <c r="M197" s="7" t="n"/>
       <c r="N197" s="7" t="n">
-        <v>15352</v>
+        <v>13356</v>
       </c>
       <c r="O197" s="7" t="n">
         <v>1</v>
@@ -15563,7 +15567,7 @@
       </c>
       <c r="R197" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S197" s="8" t="inlineStr"/>
@@ -15580,7 +15584,7 @@
       <c r="V197" s="6" t="inlineStr"/>
       <c r="W197" s="7" t="inlineStr">
         <is>
-          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
+          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
         </is>
       </c>
     </row>
@@ -15594,13 +15598,13 @@
         </is>
       </c>
       <c r="C198" s="9" t="n">
-        <v>2300</v>
+        <v>1765</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E198" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F198" s="7" t="inlineStr">
         <is>
@@ -15609,23 +15613,23 @@
       </c>
       <c r="G198" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H198" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I198" s="7" t="n">
-        <v>773</v>
+        <v>641</v>
       </c>
       <c r="J198" s="7" t="n"/>
       <c r="K198" s="7" t="n"/>
       <c r="L198" s="7" t="n"/>
       <c r="M198" s="7" t="n"/>
       <c r="N198" s="7" t="n">
-        <v>14172</v>
+        <v>13356</v>
       </c>
       <c r="O198" s="7" t="n">
         <v>1</v>
@@ -15638,7 +15642,7 @@
       </c>
       <c r="R198" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S198" s="8" t="inlineStr"/>
@@ -15655,7 +15659,7 @@
       <c r="V198" s="6" t="inlineStr"/>
       <c r="W198" s="7" t="inlineStr">
         <is>
-          <t>08411d7c5a6f10970306f10b45d00f0717234e1f</t>
+          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
         </is>
       </c>
     </row>
@@ -15669,13 +15673,13 @@
         </is>
       </c>
       <c r="C199" s="9" t="n">
-        <v>1200</v>
+        <v>2240</v>
       </c>
       <c r="D199" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E199" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F199" s="7" t="inlineStr">
         <is>
@@ -15684,36 +15688,36 @@
       </c>
       <c r="G199" s="8" t="inlineStr">
         <is>
-          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H199" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I199" s="7" t="n">
-        <v>517</v>
+        <v>884</v>
       </c>
       <c r="J199" s="7" t="n"/>
       <c r="K199" s="7" t="n"/>
       <c r="L199" s="7" t="n"/>
       <c r="M199" s="7" t="n"/>
       <c r="N199" s="7" t="n">
-        <v>21904</v>
+        <v>13388</v>
       </c>
       <c r="O199" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P199" s="7" t="n"/>
       <c r="Q199" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R199" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S199" s="8" t="inlineStr"/>
@@ -15730,14 +15734,383 @@
       <c r="V199" s="6" t="inlineStr"/>
       <c r="W199" s="7" t="inlineStr">
         <is>
+          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B200" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C200" s="9" t="n">
+        <v>1150</v>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E200" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F200" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G200" s="8" t="inlineStr">
+        <is>
+          <t>John Street, BS1</t>
+        </is>
+      </c>
+      <c r="H200" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I200" s="7" t="n">
+        <v>248</v>
+      </c>
+      <c r="J200" s="7" t="n"/>
+      <c r="K200" s="7" t="n"/>
+      <c r="L200" s="7" t="n"/>
+      <c r="M200" s="7" t="n"/>
+      <c r="N200" s="7" t="n"/>
+      <c r="O200" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P200" s="7" t="n"/>
+      <c r="Q200" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="R200" s="7" t="inlineStr">
+        <is>
+          <t>Bristol Property Centre, Bristol</t>
+        </is>
+      </c>
+      <c r="S200" s="8" t="inlineStr"/>
+      <c r="T200" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V200" s="6" t="inlineStr"/>
+      <c r="W200" s="7" t="inlineStr">
+        <is>
+          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B201" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C201" s="9" t="n">
+        <v>3400</v>
+      </c>
+      <c r="D201" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E201" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F201" s="7" t="inlineStr">
+        <is>
+          <t>terraced</t>
+        </is>
+      </c>
+      <c r="G201" s="8" t="inlineStr">
+        <is>
+          <t>Barton Road, Bristol, BS2</t>
+        </is>
+      </c>
+      <c r="H201" s="7" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I201" s="7" t="n"/>
+      <c r="J201" s="7" t="n"/>
+      <c r="K201" s="7" t="n"/>
+      <c r="L201" s="7" t="n"/>
+      <c r="M201" s="7" t="n"/>
+      <c r="N201" s="7" t="n">
+        <v>19720</v>
+      </c>
+      <c r="O201" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P201" s="7" t="n"/>
+      <c r="Q201" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="R201" s="7" t="inlineStr">
+        <is>
+          <t>OpenRent, London</t>
+        </is>
+      </c>
+      <c r="S201" s="8" t="inlineStr"/>
+      <c r="T201" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V201" s="6" t="inlineStr"/>
+      <c r="W201" s="7" t="inlineStr">
+        <is>
+          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B202" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C202" s="9" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E202" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F202" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G202" s="8" t="inlineStr">
+        <is>
+          <t>St Peters Court, Bedminster</t>
+        </is>
+      </c>
+      <c r="H202" s="7" t="inlineStr">
+        <is>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I202" s="7" t="n"/>
+      <c r="J202" s="7" t="n"/>
+      <c r="K202" s="7" t="n"/>
+      <c r="L202" s="7" t="n"/>
+      <c r="M202" s="7" t="n"/>
+      <c r="N202" s="7" t="n">
+        <v>15352</v>
+      </c>
+      <c r="O202" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P202" s="7" t="n"/>
+      <c r="Q202" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R202" s="7" t="inlineStr">
+        <is>
+          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+        </is>
+      </c>
+      <c r="S202" s="8" t="inlineStr"/>
+      <c r="T202" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V202" s="6" t="inlineStr"/>
+      <c r="W202" s="7" t="inlineStr">
+        <is>
+          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B203" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C203" s="9" t="n">
+        <v>2300</v>
+      </c>
+      <c r="D203" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E203" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F203" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G203" s="8" t="inlineStr">
+        <is>
+          <t>Castle Park View, Castle Street, Bristol</t>
+        </is>
+      </c>
+      <c r="H203" s="7" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I203" s="7" t="n">
+        <v>773</v>
+      </c>
+      <c r="J203" s="7" t="n"/>
+      <c r="K203" s="7" t="n"/>
+      <c r="L203" s="7" t="n"/>
+      <c r="M203" s="7" t="n"/>
+      <c r="N203" s="7" t="n">
+        <v>14172</v>
+      </c>
+      <c r="O203" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P203" s="7" t="n"/>
+      <c r="Q203" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="R203" s="7" t="inlineStr">
+        <is>
+          <t>Savills Lettings, CPV</t>
+        </is>
+      </c>
+      <c r="S203" s="8" t="inlineStr"/>
+      <c r="T203" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V203" s="6" t="inlineStr"/>
+      <c r="W203" s="7" t="inlineStr">
+        <is>
+          <t>08411d7c5a6f10970306f10b45d00f0717234e1f</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B204" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C204" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E204" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F204" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G204" s="8" t="inlineStr">
+        <is>
+          <t>City Centre, Kings Quarter Apartments, BS2 8HP</t>
+        </is>
+      </c>
+      <c r="H204" s="7" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I204" s="7" t="n">
+        <v>517</v>
+      </c>
+      <c r="J204" s="7" t="n"/>
+      <c r="K204" s="7" t="n"/>
+      <c r="L204" s="7" t="n"/>
+      <c r="M204" s="7" t="n"/>
+      <c r="N204" s="7" t="n">
+        <v>21904</v>
+      </c>
+      <c r="O204" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P204" s="7" t="n"/>
+      <c r="Q204" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="R204" s="7" t="inlineStr">
+        <is>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
+        </is>
+      </c>
+      <c r="S204" s="8" t="inlineStr"/>
+      <c r="T204" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V204" s="6" t="inlineStr"/>
+      <c r="W204" s="7" t="inlineStr">
+        <is>
           <t>e87a39f40860abe2278117f28f53ec7cbbd1d241</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W199"/>
+  <autoFilter ref="A1:W204"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15940,6 +16313,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T197" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T198" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T204" r:id="rId203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 166
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$206</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204 U205 U206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W204"/>
+  <dimension ref="A1:W206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>2000</v>
+        <v>1950</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>2</v>
@@ -3063,7 +3063,9 @@
       <c r="K31" s="7" t="n"/>
       <c r="L31" s="7" t="n"/>
       <c r="M31" s="7" t="n"/>
-      <c r="N31" s="7" t="n"/>
+      <c r="N31" s="7" t="n">
+        <v>21800</v>
+      </c>
       <c r="O31" s="7" t="n">
         <v>0</v>
       </c>
@@ -8633,7 +8635,7 @@
       <c r="L104" s="7" t="n"/>
       <c r="M104" s="7" t="n"/>
       <c r="N104" s="7" t="n">
-        <v>16664</v>
+        <v>17004</v>
       </c>
       <c r="O104" s="7" t="n">
         <v>0</v>
@@ -10307,7 +10309,7 @@
         </is>
       </c>
       <c r="C127" s="9" t="n">
-        <v>1600</v>
+        <v>1400</v>
       </c>
       <c r="D127" s="7" t="n">
         <v>1</v>
@@ -10322,12 +10324,12 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Redcross Village, Bristol, BS2</t>
         </is>
       </c>
       <c r="H127" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I127" s="7" t="n"/>
@@ -10336,7 +10338,7 @@
       <c r="L127" s="7" t="n"/>
       <c r="M127" s="7" t="n"/>
       <c r="N127" s="7" t="n">
-        <v>21996</v>
+        <v>21520</v>
       </c>
       <c r="O127" s="7" t="n">
         <v>0</v>
@@ -10344,12 +10346,12 @@
       <c r="P127" s="7" t="n"/>
       <c r="Q127" s="7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="R127" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Letting Game, Redland</t>
         </is>
       </c>
       <c r="S127" s="8" t="inlineStr"/>
@@ -10366,7 +10368,7 @@
       <c r="V127" s="6" t="inlineStr"/>
       <c r="W127" s="7" t="inlineStr">
         <is>
-          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
+          <t>811a7931cecb689888c03706aa5821a875281cb2</t>
         </is>
       </c>
     </row>
@@ -10380,7 +10382,7 @@
         </is>
       </c>
       <c r="C128" s="9" t="n">
-        <v>1560</v>
+        <v>1395</v>
       </c>
       <c r="D128" s="7" t="n">
         <v>1</v>
@@ -10395,7 +10397,7 @@
       </c>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Central Quay North, City Centre, Bristol</t>
         </is>
       </c>
       <c r="H128" s="7" t="inlineStr">
@@ -10403,15 +10405,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I128" s="7" t="n">
-        <v>472</v>
-      </c>
+      <c r="I128" s="7" t="n"/>
       <c r="J128" s="7" t="n"/>
       <c r="K128" s="7" t="n"/>
       <c r="L128" s="7" t="n"/>
       <c r="M128" s="7" t="n"/>
       <c r="N128" s="7" t="n">
-        <v>20984</v>
+        <v>21004</v>
       </c>
       <c r="O128" s="7" t="n">
         <v>0</v>
@@ -10419,12 +10419,12 @@
       <c r="P128" s="7" t="n"/>
       <c r="Q128" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="R128" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Gough Quarters, Clifton</t>
         </is>
       </c>
       <c r="S128" s="8" t="inlineStr"/>
@@ -10441,7 +10441,7 @@
       <c r="V128" s="6" t="inlineStr"/>
       <c r="W128" s="7" t="inlineStr">
         <is>
-          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
+          <t>f4f41204a9c7fec462f2e6b14f6e303762fd8e88</t>
         </is>
       </c>
     </row>
@@ -10455,7 +10455,7 @@
         </is>
       </c>
       <c r="C129" s="9" t="n">
-        <v>1660</v>
+        <v>1600</v>
       </c>
       <c r="D129" s="7" t="n">
         <v>1</v>
@@ -10470,7 +10470,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
@@ -10478,15 +10478,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I129" s="7" t="n">
-        <v>558</v>
-      </c>
+      <c r="I129" s="7" t="n"/>
       <c r="J129" s="7" t="n"/>
       <c r="K129" s="7" t="n"/>
       <c r="L129" s="7" t="n"/>
       <c r="M129" s="7" t="n"/>
       <c r="N129" s="7" t="n">
-        <v>20984</v>
+        <v>21996</v>
       </c>
       <c r="O129" s="7" t="n">
         <v>0</v>
@@ -10494,12 +10492,12 @@
       <c r="P129" s="7" t="n"/>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R129" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S129" s="8" t="inlineStr"/>
@@ -10516,7 +10514,7 @@
       <c r="V129" s="6" t="inlineStr"/>
       <c r="W129" s="7" t="inlineStr">
         <is>
-          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
+          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
         </is>
       </c>
     </row>
@@ -10530,13 +10528,13 @@
         </is>
       </c>
       <c r="C130" s="9" t="n">
-        <v>1860</v>
+        <v>1560</v>
       </c>
       <c r="D130" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E130" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
@@ -10545,7 +10543,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
@@ -10554,14 +10552,14 @@
         </is>
       </c>
       <c r="I130" s="7" t="n">
-        <v>647</v>
+        <v>472</v>
       </c>
       <c r="J130" s="7" t="n"/>
       <c r="K130" s="7" t="n"/>
       <c r="L130" s="7" t="n"/>
       <c r="M130" s="7" t="n"/>
       <c r="N130" s="7" t="n">
-        <v>21740</v>
+        <v>20984</v>
       </c>
       <c r="O130" s="7" t="n">
         <v>0</v>
@@ -10569,12 +10567,12 @@
       <c r="P130" s="7" t="n"/>
       <c r="Q130" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R130" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S130" s="8" t="inlineStr"/>
@@ -10591,7 +10589,7 @@
       <c r="V130" s="6" t="inlineStr"/>
       <c r="W130" s="7" t="inlineStr">
         <is>
-          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
+          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
         </is>
       </c>
     </row>
@@ -10605,7 +10603,7 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>1600</v>
+        <v>1660</v>
       </c>
       <c r="D131" s="7" t="n">
         <v>1</v>
@@ -10620,7 +10618,7 @@
       </c>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H131" s="7" t="inlineStr">
@@ -10629,14 +10627,14 @@
         </is>
       </c>
       <c r="I131" s="7" t="n">
-        <v>549</v>
+        <v>558</v>
       </c>
       <c r="J131" s="7" t="n"/>
       <c r="K131" s="7" t="n"/>
       <c r="L131" s="7" t="n"/>
       <c r="M131" s="7" t="n"/>
       <c r="N131" s="7" t="n">
-        <v>21816</v>
+        <v>20984</v>
       </c>
       <c r="O131" s="7" t="n">
         <v>0</v>
@@ -10649,7 +10647,7 @@
       </c>
       <c r="R131" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S131" s="8" t="inlineStr"/>
@@ -10666,7 +10664,7 @@
       <c r="V131" s="6" t="inlineStr"/>
       <c r="W131" s="7" t="inlineStr">
         <is>
-          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
+          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
         </is>
       </c>
     </row>
@@ -10680,7 +10678,7 @@
         </is>
       </c>
       <c r="C132" s="9" t="n">
-        <v>1900</v>
+        <v>1860</v>
       </c>
       <c r="D132" s="7" t="n">
         <v>2</v>
@@ -10704,7 +10702,7 @@
         </is>
       </c>
       <c r="I132" s="7" t="n">
-        <v>624</v>
+        <v>647</v>
       </c>
       <c r="J132" s="7" t="n"/>
       <c r="K132" s="7" t="n"/>
@@ -10719,7 +10717,7 @@
       <c r="P132" s="7" t="n"/>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
@@ -10741,7 +10739,7 @@
       <c r="V132" s="6" t="inlineStr"/>
       <c r="W132" s="7" t="inlineStr">
         <is>
-          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
+          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
         </is>
       </c>
     </row>
@@ -10755,7 +10753,7 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1530</v>
+        <v>1600</v>
       </c>
       <c r="D133" s="7" t="n">
         <v>1</v>
@@ -10779,14 +10777,14 @@
         </is>
       </c>
       <c r="I133" s="7" t="n">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>21740</v>
+        <v>21816</v>
       </c>
       <c r="O133" s="7" t="n">
         <v>0</v>
@@ -10794,7 +10792,7 @@
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
@@ -10816,7 +10814,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
+          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
         </is>
       </c>
     </row>
@@ -10830,7 +10828,7 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>2110</v>
+        <v>1900</v>
       </c>
       <c r="D134" s="7" t="n">
         <v>2</v>
@@ -10869,7 +10867,7 @@
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
@@ -10891,7 +10889,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
+          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10927,7 @@
         </is>
       </c>
       <c r="I135" s="7" t="n">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
@@ -10944,7 +10942,7 @@
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
@@ -10966,7 +10964,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
+          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
         </is>
       </c>
     </row>
@@ -10980,7 +10978,7 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>1600</v>
+        <v>2110</v>
       </c>
       <c r="D136" s="7" t="n">
         <v>2</v>
@@ -10995,7 +10993,7 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
@@ -11003,13 +11001,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I136" s="7" t="n"/>
+      <c r="I136" s="7" t="n">
+        <v>624</v>
+      </c>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>20880</v>
+        <v>21740</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -11017,12 +11017,12 @@
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11039,7 +11039,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
+          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
         </is>
       </c>
     </row>
@@ -11053,13 +11053,13 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1800</v>
+        <v>1530</v>
       </c>
       <c r="D137" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E137" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
@@ -11068,7 +11068,7 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
@@ -11077,14 +11077,14 @@
         </is>
       </c>
       <c r="I137" s="7" t="n">
-        <v>980</v>
+        <v>544</v>
       </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="7" t="n">
-        <v>21316</v>
+        <v>21740</v>
       </c>
       <c r="O137" s="7" t="n">
         <v>0</v>
@@ -11092,12 +11092,12 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S137" s="8" t="inlineStr"/>
@@ -11114,7 +11114,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
+          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
         </is>
       </c>
     </row>
@@ -11128,13 +11128,13 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1995</v>
+        <v>1600</v>
       </c>
       <c r="D138" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E138" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
@@ -11143,7 +11143,7 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
@@ -11157,7 +11157,7 @@
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>21196</v>
+        <v>20880</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11165,7 +11165,7 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
@@ -11187,7 +11187,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
+          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
         </is>
       </c>
     </row>
@@ -11201,7 +11201,7 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>1750</v>
+        <v>1800</v>
       </c>
       <c r="D139" s="7" t="n">
         <v>2</v>
@@ -11216,7 +11216,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11225,14 +11225,14 @@
         </is>
       </c>
       <c r="I139" s="7" t="n">
-        <v>849</v>
+        <v>980</v>
       </c>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>21028</v>
+        <v>21316</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11240,12 +11240,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11262,7 +11262,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
+          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
         </is>
       </c>
     </row>
@@ -11276,13 +11276,13 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1550</v>
+        <v>1995</v>
       </c>
       <c r="D140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
@@ -11291,12 +11291,12 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Portland Heights - St. Pauls</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I140" s="7" t="n"/>
@@ -11305,7 +11305,7 @@
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>21420</v>
+        <v>21196</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11313,12 +11313,12 @@
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Bishopston</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11335,7 +11335,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
+          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
         </is>
       </c>
     </row>
@@ -11349,13 +11349,13 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1400</v>
+        <v>1750</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
@@ -11364,7 +11364,7 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>The Atrium, Redcliffe Street, BS1</t>
+          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
@@ -11372,13 +11372,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I141" s="7" t="n"/>
+      <c r="I141" s="7" t="n">
+        <v>849</v>
+      </c>
       <c r="J141" s="7" t="n"/>
       <c r="K141" s="7" t="n"/>
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>20292</v>
+        <v>21028</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11386,12 +11388,12 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11408,7 +11410,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
+          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
         </is>
       </c>
     </row>
@@ -11422,13 +11424,13 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>1150</v>
+        <v>1550</v>
       </c>
       <c r="D142" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E142" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
@@ -11437,12 +11439,12 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
+          <t>Portland Heights - St. Pauls</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I142" s="7" t="n"/>
@@ -11451,7 +11453,7 @@
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>15376</v>
+        <v>21420</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11459,12 +11461,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Ocean, Bishopston</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11481,7 +11483,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
+          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
         </is>
       </c>
     </row>
@@ -11495,7 +11497,7 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="D143" s="7" t="n">
         <v>1</v>
@@ -11510,7 +11512,7 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The Milliners, BS1 6WU</t>
+          <t>The Atrium, Redcliffe Street, BS1</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
@@ -11518,15 +11520,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I143" s="7" t="n">
-        <v>463</v>
-      </c>
+      <c r="I143" s="7" t="n"/>
       <c r="J143" s="7" t="n"/>
       <c r="K143" s="7" t="n"/>
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>21440</v>
+        <v>20292</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11534,12 +11534,12 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11556,7 +11556,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
+          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
         </is>
       </c>
     </row>
@@ -11585,23 +11585,21 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>Century Place, St. Paul Street, BS2 8AN</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I144" s="7" t="n">
-        <v>344</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I144" s="7" t="n"/>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>21792</v>
+        <v>15376</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11609,12 +11607,12 @@
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11631,7 +11629,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
+          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
         </is>
       </c>
     </row>
@@ -11645,13 +11643,13 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>1800</v>
+        <v>1300</v>
       </c>
       <c r="D145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
@@ -11660,7 +11658,7 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>Waverley House, BS1</t>
+          <t>City Centre, The Milliners, BS1 6WU</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
@@ -11668,13 +11666,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I145" s="7" t="n"/>
+      <c r="I145" s="7" t="n">
+        <v>463</v>
+      </c>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>17956</v>
+        <v>21440</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11682,12 +11682,12 @@
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S145" s="8" t="inlineStr"/>
@@ -11704,7 +11704,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
+          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
         </is>
       </c>
     </row>
@@ -11718,13 +11718,13 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>2170</v>
+        <v>1150</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E146" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
@@ -11733,23 +11733,23 @@
       </c>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Century Place, St. Paul Street, BS2 8AN</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I146" s="7" t="n">
-        <v>721</v>
+        <v>344</v>
       </c>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>21732</v>
+        <v>21792</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>0</v>
@@ -11757,12 +11757,12 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S146" s="8" t="inlineStr"/>
@@ -11779,7 +11779,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
+          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
         </is>
       </c>
     </row>
@@ -11793,7 +11793,7 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>1965</v>
+        <v>1800</v>
       </c>
       <c r="D147" s="7" t="n">
         <v>2</v>
@@ -11808,7 +11808,7 @@
       </c>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Waverley House, BS1</t>
         </is>
       </c>
       <c r="H147" s="7" t="inlineStr">
@@ -11816,15 +11816,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I147" s="7" t="n">
-        <v>771</v>
-      </c>
+      <c r="I147" s="7" t="n"/>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="7" t="n">
-        <v>21740</v>
+        <v>17956</v>
       </c>
       <c r="O147" s="7" t="n">
         <v>0</v>
@@ -11832,12 +11830,12 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S147" s="8" t="inlineStr"/>
@@ -11854,7 +11852,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
+          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
         </is>
       </c>
     </row>
@@ -11868,13 +11866,13 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>1680</v>
+        <v>2170</v>
       </c>
       <c r="D148" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E148" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
@@ -11883,7 +11881,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
@@ -11891,13 +11889,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I148" s="7" t="n"/>
+      <c r="I148" s="7" t="n">
+        <v>721</v>
+      </c>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>20628</v>
+        <v>21732</v>
       </c>
       <c r="O148" s="7" t="n">
         <v>0</v>
@@ -11905,12 +11905,12 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11927,7 +11927,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
+          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
         </is>
       </c>
     </row>
@@ -11941,13 +11941,13 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>1625</v>
+        <v>1965</v>
       </c>
       <c r="D149" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E149" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F149" s="7" t="inlineStr">
         <is>
@@ -11956,7 +11956,7 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H149" s="7" t="inlineStr">
@@ -11965,14 +11965,14 @@
         </is>
       </c>
       <c r="I149" s="7" t="n">
-        <v>486</v>
+        <v>771</v>
       </c>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="7" t="n">
-        <v>21732</v>
+        <v>21740</v>
       </c>
       <c r="O149" s="7" t="n">
         <v>0</v>
@@ -11980,12 +11980,12 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S149" s="8" t="inlineStr"/>
@@ -12002,7 +12002,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
+          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
         </is>
       </c>
     </row>
@@ -12016,13 +12016,13 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1940</v>
+        <v>1680</v>
       </c>
       <c r="D150" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
@@ -12031,7 +12031,7 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
@@ -12039,15 +12039,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I150" s="7" t="n">
-        <v>607</v>
-      </c>
+      <c r="I150" s="7" t="n"/>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>21740</v>
+        <v>20628</v>
       </c>
       <c r="O150" s="7" t="n">
         <v>0</v>
@@ -12060,7 +12058,7 @@
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12077,7 +12075,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
+          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
         </is>
       </c>
     </row>
@@ -12091,7 +12089,7 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1465</v>
+        <v>1625</v>
       </c>
       <c r="D151" s="7" t="n">
         <v>1</v>
@@ -12106,7 +12104,7 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr">
@@ -12115,14 +12113,14 @@
         </is>
       </c>
       <c r="I151" s="7" t="n">
-        <v>505</v>
+        <v>486</v>
       </c>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>21816</v>
+        <v>21732</v>
       </c>
       <c r="O151" s="7" t="n">
         <v>0</v>
@@ -12135,7 +12133,7 @@
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12152,7 +12150,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>e86143466441bbbf802706245b19ef679ec29055</t>
+          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
         </is>
       </c>
     </row>
@@ -12166,13 +12164,13 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1150</v>
+        <v>1940</v>
       </c>
       <c r="D152" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E152" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
@@ -12181,21 +12179,23 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>St. Philips, Bristol, BS2</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I152" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I152" s="7" t="n">
+        <v>607</v>
+      </c>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>20784</v>
+        <v>21740</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12203,12 +12203,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12225,7 +12225,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
+          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
         </is>
       </c>
     </row>
@@ -12239,7 +12239,7 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>1685</v>
+        <v>1465</v>
       </c>
       <c r="D153" s="7" t="n">
         <v>1</v>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
@@ -12263,14 +12263,14 @@
         </is>
       </c>
       <c r="I153" s="7" t="n">
-        <v>545</v>
+        <v>505</v>
       </c>
       <c r="J153" s="7" t="n"/>
       <c r="K153" s="7" t="n"/>
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>21024</v>
+        <v>21816</v>
       </c>
       <c r="O153" s="7" t="n">
         <v>0</v>
@@ -12278,12 +12278,12 @@
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12300,7 +12300,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
+          <t>e86143466441bbbf802706245b19ef679ec29055</t>
         </is>
       </c>
     </row>
@@ -12314,27 +12314,27 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1700</v>
+        <v>1150</v>
       </c>
       <c r="D154" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E154" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>Dunkerry Road - Windmill Hill</t>
+          <t>St. Philips, Bristol, BS2</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I154" s="7" t="n"/>
@@ -12343,7 +12343,7 @@
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="7" t="n">
-        <v>8448</v>
+        <v>20784</v>
       </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
@@ -12351,12 +12351,12 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S154" s="8" t="inlineStr"/>
@@ -12373,7 +12373,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
+          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
         </is>
       </c>
     </row>
@@ -12387,7 +12387,7 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>1460</v>
+        <v>1685</v>
       </c>
       <c r="D155" s="7" t="n">
         <v>1</v>
@@ -12402,7 +12402,7 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
@@ -12411,14 +12411,14 @@
         </is>
       </c>
       <c r="I155" s="7" t="n">
-        <v>473</v>
+        <v>545</v>
       </c>
       <c r="J155" s="7" t="n"/>
       <c r="K155" s="7" t="n"/>
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="7" t="n">
-        <v>13840</v>
+        <v>21024</v>
       </c>
       <c r="O155" s="7" t="n">
         <v>0</v>
@@ -12426,12 +12426,12 @@
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12448,7 +12448,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
+          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
         </is>
       </c>
     </row>
@@ -12462,51 +12462,49 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>1630</v>
+        <v>1700</v>
       </c>
       <c r="D156" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E156" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F156" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Dunkerry Road - Windmill Hill</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I156" s="7" t="n">
-        <v>486</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I156" s="7" t="n"/>
       <c r="J156" s="7" t="n"/>
       <c r="K156" s="7" t="n"/>
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="7" t="n">
-        <v>13860</v>
+        <v>8448</v>
       </c>
       <c r="O156" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S156" s="8" t="inlineStr"/>
@@ -12523,7 +12521,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
+          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
         </is>
       </c>
     </row>
@@ -12537,7 +12535,7 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>1625</v>
+        <v>1460</v>
       </c>
       <c r="D157" s="7" t="n">
         <v>1</v>
@@ -12552,7 +12550,7 @@
       </c>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H157" s="7" t="inlineStr">
@@ -12561,14 +12559,14 @@
         </is>
       </c>
       <c r="I157" s="7" t="n">
-        <v>486</v>
+        <v>473</v>
       </c>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="7" t="n">
-        <v>21732</v>
+        <v>13840</v>
       </c>
       <c r="O157" s="7" t="n">
         <v>0</v>
@@ -12576,12 +12574,12 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S157" s="8" t="inlineStr"/>
@@ -12598,7 +12596,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
+          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
         </is>
       </c>
     </row>
@@ -12612,13 +12610,13 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>1650</v>
+        <v>1630</v>
       </c>
       <c r="D158" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E158" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F158" s="7" t="inlineStr">
         <is>
@@ -12627,7 +12625,7 @@
       </c>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Harris Lofts, BS1 4BB</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H158" s="7" t="inlineStr">
@@ -12636,27 +12634,27 @@
         </is>
       </c>
       <c r="I158" s="7" t="n">
-        <v>667</v>
+        <v>486</v>
       </c>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>20088</v>
+        <v>13860</v>
       </c>
       <c r="O158" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S158" s="8" t="inlineStr"/>
@@ -12673,7 +12671,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
+          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
         </is>
       </c>
     </row>
@@ -12687,7 +12685,7 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1650</v>
+        <v>1625</v>
       </c>
       <c r="D159" s="7" t="n">
         <v>1</v>
@@ -12702,7 +12700,7 @@
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>Central Quey North, Broad Quay, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
@@ -12710,13 +12708,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I159" s="7" t="n"/>
+      <c r="I159" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="7" t="n">
-        <v>20768</v>
+        <v>21732</v>
       </c>
       <c r="O159" s="7" t="n">
         <v>0</v>
@@ -12724,12 +12724,12 @@
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12746,7 +12746,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
+          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
         </is>
       </c>
     </row>
@@ -12760,13 +12760,13 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>1550</v>
+        <v>1650</v>
       </c>
       <c r="D160" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E160" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F160" s="7" t="inlineStr">
         <is>
@@ -12775,7 +12775,7 @@
       </c>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Harbourside, Harris Lofts, BS1 4BB</t>
         </is>
       </c>
       <c r="H160" s="7" t="inlineStr">
@@ -12783,13 +12783,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I160" s="7" t="n"/>
+      <c r="I160" s="7" t="n">
+        <v>667</v>
+      </c>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
       <c r="N160" s="7" t="n">
-        <v>21100</v>
+        <v>20088</v>
       </c>
       <c r="O160" s="7" t="n">
         <v>0</v>
@@ -12797,12 +12799,12 @@
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S160" s="8" t="inlineStr"/>
@@ -12819,7 +12821,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
+          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
         </is>
       </c>
     </row>
@@ -12833,7 +12835,7 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>1390</v>
+        <v>1650</v>
       </c>
       <c r="D161" s="7" t="n">
         <v>1</v>
@@ -12848,7 +12850,7 @@
       </c>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Central Quey North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H161" s="7" t="inlineStr">
@@ -12861,19 +12863,21 @@
       <c r="K161" s="7" t="n"/>
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
-      <c r="N161" s="7" t="n"/>
+      <c r="N161" s="7" t="n">
+        <v>20768</v>
+      </c>
       <c r="O161" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S161" s="8" t="inlineStr"/>
@@ -12890,7 +12894,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
+          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
         </is>
       </c>
     </row>
@@ -12904,7 +12908,7 @@
         </is>
       </c>
       <c r="C162" s="9" t="n">
-        <v>1485</v>
+        <v>1550</v>
       </c>
       <c r="D162" s="7" t="n">
         <v>1</v>
@@ -12919,7 +12923,7 @@
       </c>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
@@ -12927,15 +12931,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I162" s="7" t="n">
-        <v>470</v>
-      </c>
+      <c r="I162" s="7" t="n"/>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
       <c r="N162" s="7" t="n">
-        <v>21740</v>
+        <v>21100</v>
       </c>
       <c r="O162" s="7" t="n">
         <v>0</v>
@@ -12943,12 +12945,12 @@
       <c r="P162" s="7" t="n"/>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S162" s="8" t="inlineStr"/>
@@ -12965,7 +12967,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
+          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
         </is>
       </c>
     </row>
@@ -12979,7 +12981,7 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1635</v>
+        <v>1390</v>
       </c>
       <c r="D163" s="7" t="n">
         <v>1</v>
@@ -12994,7 +12996,7 @@
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
@@ -13002,28 +13004,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I163" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I163" s="7" t="n"/>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
-      <c r="N163" s="7" t="n">
-        <v>21732</v>
-      </c>
+      <c r="N163" s="7" t="n"/>
       <c r="O163" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13040,7 +13038,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
+          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
         </is>
       </c>
     </row>
@@ -13054,13 +13052,13 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>2060</v>
+        <v>1485</v>
       </c>
       <c r="D164" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E164" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F164" s="7" t="inlineStr">
         <is>
@@ -13069,7 +13067,7 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
@@ -13078,14 +13076,14 @@
         </is>
       </c>
       <c r="I164" s="7" t="n">
-        <v>721</v>
+        <v>470</v>
       </c>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="7" t="n">
-        <v>21732</v>
+        <v>21740</v>
       </c>
       <c r="O164" s="7" t="n">
         <v>0</v>
@@ -13093,12 +13091,12 @@
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13115,7 +13113,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
+          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
         </is>
       </c>
     </row>
@@ -13129,7 +13127,7 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1545</v>
+        <v>1635</v>
       </c>
       <c r="D165" s="7" t="n">
         <v>1</v>
@@ -13144,7 +13142,7 @@
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H165" s="7" t="inlineStr">
@@ -13153,14 +13151,14 @@
         </is>
       </c>
       <c r="I165" s="7" t="n">
-        <v>548</v>
+        <v>486</v>
       </c>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O165" s="7" t="n">
         <v>0</v>
@@ -13168,12 +13166,12 @@
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R165" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S165" s="8" t="inlineStr"/>
@@ -13190,7 +13188,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
+          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
         </is>
       </c>
     </row>
@@ -13204,13 +13202,13 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>1640</v>
+        <v>2060</v>
       </c>
       <c r="D166" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E166" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F166" s="7" t="inlineStr">
         <is>
@@ -13228,7 +13226,7 @@
         </is>
       </c>
       <c r="I166" s="7" t="n">
-        <v>486</v>
+        <v>721</v>
       </c>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
@@ -13243,7 +13241,7 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
@@ -13265,7 +13263,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
+          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
         </is>
       </c>
     </row>
@@ -13279,10 +13277,10 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>2115</v>
+        <v>1545</v>
       </c>
       <c r="D167" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E167" s="7" t="n">
         <v>1</v>
@@ -13294,7 +13292,7 @@
       </c>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H167" s="7" t="inlineStr">
@@ -13303,14 +13301,14 @@
         </is>
       </c>
       <c r="I167" s="7" t="n">
-        <v>722</v>
+        <v>548</v>
       </c>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="7" t="n">
-        <v>21732</v>
+        <v>21740</v>
       </c>
       <c r="O167" s="7" t="n">
         <v>0</v>
@@ -13323,7 +13321,7 @@
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S167" s="8" t="inlineStr"/>
@@ -13340,7 +13338,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
+          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
         </is>
       </c>
     </row>
@@ -13354,13 +13352,13 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1970</v>
+        <v>1640</v>
       </c>
       <c r="D168" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E168" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F168" s="7" t="inlineStr">
         <is>
@@ -13369,7 +13367,7 @@
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
@@ -13378,14 +13376,14 @@
         </is>
       </c>
       <c r="I168" s="7" t="n">
-        <v>750</v>
+        <v>486</v>
       </c>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O168" s="7" t="n">
         <v>0</v>
@@ -13393,12 +13391,12 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13415,7 +13413,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
+          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
         </is>
       </c>
     </row>
@@ -13429,10 +13427,10 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1575</v>
+        <v>2115</v>
       </c>
       <c r="D169" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E169" s="7" t="n">
         <v>1</v>
@@ -13444,7 +13442,7 @@
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
@@ -13453,14 +13451,14 @@
         </is>
       </c>
       <c r="I169" s="7" t="n">
-        <v>430</v>
+        <v>722</v>
       </c>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>21816</v>
+        <v>21732</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13468,12 +13466,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13490,7 +13488,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
+          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
         </is>
       </c>
     </row>
@@ -13504,13 +13502,13 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>1350</v>
+        <v>1970</v>
       </c>
       <c r="D170" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E170" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F170" s="7" t="inlineStr">
         <is>
@@ -13519,7 +13517,7 @@
       </c>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t>Invicta, Millenium Promenade, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H170" s="7" t="inlineStr">
@@ -13527,13 +13525,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I170" s="7" t="n"/>
+      <c r="I170" s="7" t="n">
+        <v>750</v>
+      </c>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
       <c r="L170" s="7" t="n"/>
       <c r="M170" s="7" t="n"/>
       <c r="N170" s="7" t="n">
-        <v>17344</v>
+        <v>21740</v>
       </c>
       <c r="O170" s="7" t="n">
         <v>0</v>
@@ -13541,12 +13541,12 @@
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -13563,7 +13563,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
+          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
         </is>
       </c>
     </row>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="C171" s="9" t="n">
-        <v>1600</v>
+        <v>1575</v>
       </c>
       <c r="D171" s="7" t="n">
         <v>1</v>
@@ -13592,7 +13592,7 @@
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H171" s="7" t="inlineStr">
@@ -13600,13 +13600,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I171" s="7" t="n"/>
+      <c r="I171" s="7" t="n">
+        <v>430</v>
+      </c>
       <c r="J171" s="7" t="n"/>
       <c r="K171" s="7" t="n"/>
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="7" t="n">
-        <v>13404</v>
+        <v>21816</v>
       </c>
       <c r="O171" s="7" t="n">
         <v>0</v>
@@ -13614,12 +13616,12 @@
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -13636,7 +13638,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
+          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
         </is>
       </c>
     </row>
@@ -13650,10 +13652,10 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1700</v>
+        <v>1350</v>
       </c>
       <c r="D172" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E172" s="7" t="n">
         <v>1</v>
@@ -13665,7 +13667,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
+          <t>Invicta, Millenium Promenade, BS1</t>
         </is>
       </c>
       <c r="H172" s="7" t="inlineStr">
@@ -13673,15 +13675,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I172" s="7" t="n">
-        <v>646</v>
-      </c>
+      <c r="I172" s="7" t="n"/>
       <c r="J172" s="7" t="n"/>
       <c r="K172" s="7" t="n"/>
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="7" t="n">
-        <v>20928</v>
+        <v>17344</v>
       </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
@@ -13689,12 +13689,12 @@
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -13711,7 +13711,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
+          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
         </is>
       </c>
     </row>
@@ -13725,13 +13725,13 @@
         </is>
       </c>
       <c r="C173" s="9" t="n">
-        <v>2105</v>
+        <v>1600</v>
       </c>
       <c r="D173" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E173" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
@@ -13740,7 +13740,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Central Quay North, Bristol, BS1</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
@@ -13748,15 +13748,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I173" s="7" t="n">
-        <v>745</v>
-      </c>
+      <c r="I173" s="7" t="n"/>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>20984</v>
+        <v>13404</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13764,12 +13762,12 @@
       <c r="P173" s="7" t="n"/>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -13786,7 +13784,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
+          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
         </is>
       </c>
     </row>
@@ -13800,10 +13798,10 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1595</v>
+        <v>1700</v>
       </c>
       <c r="D174" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E174" s="7" t="n">
         <v>1</v>
@@ -13815,7 +13813,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
@@ -13824,14 +13822,14 @@
         </is>
       </c>
       <c r="I174" s="7" t="n">
-        <v>484</v>
+        <v>646</v>
       </c>
       <c r="J174" s="7" t="n"/>
       <c r="K174" s="7" t="n"/>
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>21732</v>
+        <v>20928</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13839,12 +13837,12 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -13861,7 +13859,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
+          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
         </is>
       </c>
     </row>
@@ -13875,13 +13873,13 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>1999</v>
+        <v>2105</v>
       </c>
       <c r="D175" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E175" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
@@ -13890,21 +13888,23 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I175" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I175" s="7" t="n">
+        <v>745</v>
+      </c>
       <c r="J175" s="7" t="n"/>
       <c r="K175" s="7" t="n"/>
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
       <c r="N175" s="7" t="n">
-        <v>21736</v>
+        <v>20984</v>
       </c>
       <c r="O175" s="7" t="n">
         <v>0</v>
@@ -13912,12 +13912,12 @@
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -13934,7 +13934,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
+          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
         </is>
       </c>
     </row>
@@ -13948,7 +13948,7 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>1605</v>
+        <v>1595</v>
       </c>
       <c r="D176" s="7" t="n">
         <v>1</v>
@@ -13972,7 +13972,7 @@
         </is>
       </c>
       <c r="I176" s="7" t="n">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="J176" s="7" t="n"/>
       <c r="K176" s="7" t="n"/>
@@ -13987,7 +13987,7 @@
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
@@ -14009,7 +14009,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
+          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
         </is>
       </c>
     </row>
@@ -14023,10 +14023,10 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>1390</v>
+        <v>1999</v>
       </c>
       <c r="D177" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E177" s="7" t="n">
         <v>1</v>
@@ -14038,12 +14038,12 @@
       </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H177" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I177" s="7" t="n"/>
@@ -14051,14 +14051,16 @@
       <c r="K177" s="7" t="n"/>
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
-      <c r="N177" s="7" t="n"/>
+      <c r="N177" s="7" t="n">
+        <v>21736</v>
+      </c>
       <c r="O177" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
@@ -14080,7 +14082,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
         </is>
       </c>
     </row>
@@ -14094,7 +14096,7 @@
         </is>
       </c>
       <c r="C178" s="9" t="n">
-        <v>1395</v>
+        <v>1605</v>
       </c>
       <c r="D178" s="7" t="n">
         <v>1</v>
@@ -14109,7 +14111,7 @@
       </c>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H178" s="7" t="inlineStr">
@@ -14117,13 +14119,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I178" s="7" t="n"/>
+      <c r="I178" s="7" t="n">
+        <v>487</v>
+      </c>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
       <c r="L178" s="7" t="n"/>
       <c r="M178" s="7" t="n"/>
       <c r="N178" s="7" t="n">
-        <v>20524</v>
+        <v>21732</v>
       </c>
       <c r="O178" s="7" t="n">
         <v>0</v>
@@ -14131,12 +14135,12 @@
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S178" s="8" t="inlineStr"/>
@@ -14153,7 +14157,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
         </is>
       </c>
     </row>
@@ -14167,7 +14171,7 @@
         </is>
       </c>
       <c r="C179" s="9" t="n">
-        <v>1200</v>
+        <v>1390</v>
       </c>
       <c r="D179" s="7" t="n">
         <v>1</v>
@@ -14177,41 +14181,37 @@
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2 0JN</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H179" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I179" s="7" t="n">
-        <v>452</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I179" s="7" t="n"/>
       <c r="J179" s="7" t="n"/>
       <c r="K179" s="7" t="n"/>
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
-      <c r="N179" s="7" t="n">
-        <v>20472</v>
-      </c>
+      <c r="N179" s="7" t="n"/>
       <c r="O179" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -14228,7 +14228,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
+          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
         </is>
       </c>
     </row>
@@ -14242,7 +14242,7 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>1450</v>
+        <v>1395</v>
       </c>
       <c r="D180" s="7" t="n">
         <v>1</v>
@@ -14257,7 +14257,7 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
@@ -14271,7 +14271,7 @@
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="7" t="n">
-        <v>16664</v>
+        <v>20524</v>
       </c>
       <c r="O180" s="7" t="n">
         <v>0</v>
@@ -14279,12 +14279,12 @@
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14301,7 +14301,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
@@ -14315,36 +14315,38 @@
         </is>
       </c>
       <c r="C181" s="9" t="n">
-        <v>3200</v>
+        <v>1200</v>
       </c>
       <c r="D181" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E181" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F181" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
+          <t>Sweetman Place, Bristol, BS2 0JN</t>
         </is>
       </c>
       <c r="H181" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I181" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I181" s="7" t="n">
+        <v>452</v>
+      </c>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="7" t="n">
-        <v>16664</v>
+        <v>20472</v>
       </c>
       <c r="O181" s="7" t="n">
         <v>0</v>
@@ -14352,12 +14354,12 @@
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>LettingaProperty.com, Nationwide - Lettings</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S181" s="8" t="inlineStr"/>
@@ -14374,7 +14376,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
+          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
         </is>
       </c>
     </row>
@@ -14388,7 +14390,7 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>1600</v>
+        <v>1450</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>1</v>
@@ -14403,7 +14405,7 @@
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
@@ -14417,7 +14419,7 @@
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>21996</v>
+        <v>16664</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14425,12 +14427,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14447,7 +14449,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
+          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
         </is>
       </c>
     </row>
@@ -14461,7 +14463,7 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>2400</v>
+        <v>3200</v>
       </c>
       <c r="D183" s="7" t="n">
         <v>2</v>
@@ -14476,7 +14478,7 @@
       </c>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t>Colston Avenue, Bristol, BS1</t>
+          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
         </is>
       </c>
       <c r="H183" s="7" t="inlineStr">
@@ -14490,7 +14492,7 @@
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="7" t="n">
-        <v>14108</v>
+        <v>16664</v>
       </c>
       <c r="O183" s="7" t="n">
         <v>0</v>
@@ -14498,12 +14500,12 @@
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>LettingaProperty.com, Nationwide - Lettings</t>
         </is>
       </c>
       <c r="S183" s="8" t="inlineStr"/>
@@ -14520,7 +14522,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
+          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
         </is>
       </c>
     </row>
@@ -14534,7 +14536,7 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>1300</v>
+        <v>1600</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>1</v>
@@ -14549,23 +14551,21 @@
       </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>East Street, Bedminster, BS3</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H184" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I184" s="7" t="n">
-        <v>560</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I184" s="7" t="n"/>
       <c r="J184" s="7" t="n"/>
       <c r="K184" s="7" t="n"/>
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
       <c r="N184" s="7" t="n">
-        <v>14176</v>
+        <v>21996</v>
       </c>
       <c r="O184" s="7" t="n">
         <v>0</v>
@@ -14573,12 +14573,12 @@
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
         <is>
-          <t>Xeno Property, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S184" s="8" t="inlineStr"/>
@@ -14595,7 +14595,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
+          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
         </is>
       </c>
     </row>
@@ -14609,13 +14609,13 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>1450</v>
+        <v>2400</v>
       </c>
       <c r="D185" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E185" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F185" s="7" t="inlineStr">
         <is>
@@ -14624,7 +14624,7 @@
       </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol</t>
+          <t>Colston Avenue, Bristol, BS1</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
@@ -14638,7 +14638,7 @@
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="7" t="n">
-        <v>13668</v>
+        <v>14108</v>
       </c>
       <c r="O185" s="7" t="n">
         <v>0</v>
@@ -14646,12 +14646,12 @@
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
-          <t>Wildheart Residential Management Limited, Epsom</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S185" s="8" t="inlineStr"/>
@@ -14668,7 +14668,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
+          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
         </is>
       </c>
     </row>
@@ -14682,7 +14682,7 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>1605</v>
+        <v>1300</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>1</v>
@@ -14697,23 +14697,23 @@
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>East Street, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I186" s="7" t="n">
-        <v>487</v>
+        <v>560</v>
       </c>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>13860</v>
+        <v>14176</v>
       </c>
       <c r="O186" s="7" t="n">
         <v>0</v>
@@ -14721,12 +14721,12 @@
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Xeno Property, Bristol</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14743,7 +14743,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
+          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
         </is>
       </c>
     </row>
@@ -14757,13 +14757,13 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>2185</v>
+        <v>1450</v>
       </c>
       <c r="D187" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E187" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F187" s="7" t="inlineStr">
         <is>
@@ -14772,7 +14772,7 @@
       </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Welsh Back, Bristol</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
@@ -14780,15 +14780,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I187" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I187" s="7" t="n"/>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>13860</v>
+        <v>13668</v>
       </c>
       <c r="O187" s="7" t="n">
         <v>0</v>
@@ -14796,12 +14794,12 @@
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Wildheart Residential Management Limited, Epsom</t>
         </is>
       </c>
       <c r="S187" s="8" t="inlineStr"/>
@@ -14818,7 +14816,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
+          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
         </is>
       </c>
     </row>
@@ -14832,7 +14830,7 @@
         </is>
       </c>
       <c r="C188" s="9" t="n">
-        <v>1640</v>
+        <v>1605</v>
       </c>
       <c r="D188" s="7" t="n">
         <v>1</v>
@@ -14856,7 +14854,7 @@
         </is>
       </c>
       <c r="I188" s="7" t="n">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
@@ -14871,7 +14869,7 @@
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
@@ -14893,7 +14891,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
+          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
         </is>
       </c>
     </row>
@@ -14907,7 +14905,7 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>2010</v>
+        <v>2185</v>
       </c>
       <c r="D189" s="7" t="n">
         <v>2</v>
@@ -14931,7 +14929,7 @@
         </is>
       </c>
       <c r="I189" s="7" t="n">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
@@ -14946,7 +14944,7 @@
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R189" s="7" t="inlineStr">
@@ -14968,7 +14966,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
+          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
         </is>
       </c>
     </row>
@@ -14982,7 +14980,7 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>1635</v>
+        <v>1640</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1</v>
@@ -14997,7 +14995,7 @@
       </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
@@ -15006,14 +15004,14 @@
         </is>
       </c>
       <c r="I190" s="7" t="n">
-        <v>560</v>
+        <v>484</v>
       </c>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O190" s="7" t="n">
         <v>0</v>
@@ -15021,12 +15019,12 @@
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S190" s="8" t="inlineStr"/>
@@ -15043,7 +15041,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
+          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
         </is>
       </c>
     </row>
@@ -15057,13 +15055,13 @@
         </is>
       </c>
       <c r="C191" s="9" t="n">
-        <v>1665</v>
+        <v>2010</v>
       </c>
       <c r="D191" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E191" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F191" s="7" t="inlineStr">
         <is>
@@ -15072,7 +15070,7 @@
       </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H191" s="7" t="inlineStr">
@@ -15081,14 +15079,14 @@
         </is>
       </c>
       <c r="I191" s="7" t="n">
-        <v>434</v>
+        <v>722</v>
       </c>
       <c r="J191" s="7" t="n"/>
       <c r="K191" s="7" t="n"/>
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
       <c r="N191" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O191" s="7" t="n">
         <v>0</v>
@@ -15101,7 +15099,7 @@
       </c>
       <c r="R191" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S191" s="8" t="inlineStr"/>
@@ -15118,7 +15116,7 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
-          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
+          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
         </is>
       </c>
     </row>
@@ -15132,13 +15130,13 @@
         </is>
       </c>
       <c r="C192" s="9" t="n">
-        <v>1990</v>
+        <v>1635</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E192" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F192" s="7" t="inlineStr">
         <is>
@@ -15147,7 +15145,7 @@
       </c>
       <c r="G192" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H192" s="7" t="inlineStr">
@@ -15156,27 +15154,27 @@
         </is>
       </c>
       <c r="I192" s="7" t="n">
-        <v>682</v>
+        <v>560</v>
       </c>
       <c r="J192" s="7" t="n"/>
       <c r="K192" s="7" t="n"/>
       <c r="L192" s="7" t="n"/>
       <c r="M192" s="7" t="n"/>
       <c r="N192" s="7" t="n">
-        <v>13964</v>
+        <v>13356</v>
       </c>
       <c r="O192" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P192" s="7" t="n"/>
       <c r="Q192" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R192" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S192" s="8" t="inlineStr"/>
@@ -15193,7 +15191,7 @@
       <c r="V192" s="6" t="inlineStr"/>
       <c r="W192" s="7" t="inlineStr">
         <is>
-          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
+          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
         </is>
       </c>
     </row>
@@ -15207,7 +15205,7 @@
         </is>
       </c>
       <c r="C193" s="9" t="n">
-        <v>1480</v>
+        <v>1665</v>
       </c>
       <c r="D193" s="7" t="n">
         <v>1</v>
@@ -15222,7 +15220,7 @@
       </c>
       <c r="G193" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H193" s="7" t="inlineStr">
@@ -15231,27 +15229,27 @@
         </is>
       </c>
       <c r="I193" s="7" t="n">
-        <v>417</v>
+        <v>434</v>
       </c>
       <c r="J193" s="7" t="n"/>
       <c r="K193" s="7" t="n"/>
       <c r="L193" s="7" t="n"/>
       <c r="M193" s="7" t="n"/>
       <c r="N193" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O193" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P193" s="7" t="n"/>
       <c r="Q193" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R193" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S193" s="8" t="inlineStr"/>
@@ -15268,7 +15266,7 @@
       <c r="V193" s="6" t="inlineStr"/>
       <c r="W193" s="7" t="inlineStr">
         <is>
-          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
+          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
         </is>
       </c>
     </row>
@@ -15282,7 +15280,7 @@
         </is>
       </c>
       <c r="C194" s="9" t="n">
-        <v>1750</v>
+        <v>1990</v>
       </c>
       <c r="D194" s="7" t="n">
         <v>2</v>
@@ -15297,7 +15295,7 @@
       </c>
       <c r="G194" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H194" s="7" t="inlineStr">
@@ -15305,26 +15303,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I194" s="7" t="n"/>
+      <c r="I194" s="7" t="n">
+        <v>682</v>
+      </c>
       <c r="J194" s="7" t="n"/>
       <c r="K194" s="7" t="n"/>
       <c r="L194" s="7" t="n"/>
       <c r="M194" s="7" t="n"/>
       <c r="N194" s="7" t="n">
-        <v>20828</v>
+        <v>13964</v>
       </c>
       <c r="O194" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P194" s="7" t="n"/>
       <c r="Q194" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R194" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S194" s="8" t="inlineStr"/>
@@ -15341,7 +15341,7 @@
       <c r="V194" s="6" t="inlineStr"/>
       <c r="W194" s="7" t="inlineStr">
         <is>
-          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
+          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
         </is>
       </c>
     </row>
@@ -15355,13 +15355,13 @@
         </is>
       </c>
       <c r="C195" s="9" t="n">
-        <v>2080</v>
+        <v>1480</v>
       </c>
       <c r="D195" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E195" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F195" s="7" t="inlineStr">
         <is>
@@ -15379,7 +15379,7 @@
         </is>
       </c>
       <c r="I195" s="7" t="n">
-        <v>705</v>
+        <v>417</v>
       </c>
       <c r="J195" s="7" t="n"/>
       <c r="K195" s="7" t="n"/>
@@ -15394,7 +15394,7 @@
       <c r="P195" s="7" t="n"/>
       <c r="Q195" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R195" s="7" t="inlineStr">
@@ -15416,7 +15416,7 @@
       <c r="V195" s="6" t="inlineStr"/>
       <c r="W195" s="7" t="inlineStr">
         <is>
-          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
+          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
         </is>
       </c>
     </row>
@@ -15430,13 +15430,13 @@
         </is>
       </c>
       <c r="C196" s="9" t="n">
-        <v>1680</v>
+        <v>1750</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E196" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F196" s="7" t="inlineStr">
         <is>
@@ -15445,7 +15445,7 @@
       </c>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H196" s="7" t="inlineStr">
@@ -15453,18 +15453,16 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I196" s="7" t="n">
-        <v>487</v>
-      </c>
+      <c r="I196" s="7" t="n"/>
       <c r="J196" s="7" t="n"/>
       <c r="K196" s="7" t="n"/>
       <c r="L196" s="7" t="n"/>
       <c r="M196" s="7" t="n"/>
       <c r="N196" s="7" t="n">
-        <v>13356</v>
+        <v>20828</v>
       </c>
       <c r="O196" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P196" s="7" t="n"/>
       <c r="Q196" s="7" t="inlineStr">
@@ -15474,7 +15472,7 @@
       </c>
       <c r="R196" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S196" s="8" t="inlineStr"/>
@@ -15491,7 +15489,7 @@
       <c r="V196" s="6" t="inlineStr"/>
       <c r="W196" s="7" t="inlineStr">
         <is>
-          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
+          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
         </is>
       </c>
     </row>
@@ -15505,7 +15503,7 @@
         </is>
       </c>
       <c r="C197" s="9" t="n">
-        <v>1845</v>
+        <v>2080</v>
       </c>
       <c r="D197" s="7" t="n">
         <v>2</v>
@@ -15520,7 +15518,7 @@
       </c>
       <c r="G197" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H197" s="7" t="inlineStr">
@@ -15529,27 +15527,27 @@
         </is>
       </c>
       <c r="I197" s="7" t="n">
-        <v>641</v>
+        <v>705</v>
       </c>
       <c r="J197" s="7" t="n"/>
       <c r="K197" s="7" t="n"/>
       <c r="L197" s="7" t="n"/>
       <c r="M197" s="7" t="n"/>
       <c r="N197" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O197" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P197" s="7" t="n"/>
       <c r="Q197" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R197" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S197" s="8" t="inlineStr"/>
@@ -15566,7 +15564,7 @@
       <c r="V197" s="6" t="inlineStr"/>
       <c r="W197" s="7" t="inlineStr">
         <is>
-          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
+          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
         </is>
       </c>
     </row>
@@ -15580,7 +15578,7 @@
         </is>
       </c>
       <c r="C198" s="9" t="n">
-        <v>1685</v>
+        <v>1680</v>
       </c>
       <c r="D198" s="7" t="n">
         <v>1</v>
@@ -15604,7 +15602,7 @@
         </is>
       </c>
       <c r="I198" s="7" t="n">
-        <v>578</v>
+        <v>487</v>
       </c>
       <c r="J198" s="7" t="n"/>
       <c r="K198" s="7" t="n"/>
@@ -15619,7 +15617,7 @@
       <c r="P198" s="7" t="n"/>
       <c r="Q198" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R198" s="7" t="inlineStr">
@@ -15641,7 +15639,7 @@
       <c r="V198" s="6" t="inlineStr"/>
       <c r="W198" s="7" t="inlineStr">
         <is>
-          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
+          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
         </is>
       </c>
     </row>
@@ -15655,13 +15653,13 @@
         </is>
       </c>
       <c r="C199" s="9" t="n">
-        <v>1765</v>
+        <v>1845</v>
       </c>
       <c r="D199" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E199" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F199" s="7" t="inlineStr">
         <is>
@@ -15670,7 +15668,7 @@
       </c>
       <c r="G199" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H199" s="7" t="inlineStr">
@@ -15686,20 +15684,20 @@
       <c r="L199" s="7" t="n"/>
       <c r="M199" s="7" t="n"/>
       <c r="N199" s="7" t="n">
-        <v>13356</v>
+        <v>21476</v>
       </c>
       <c r="O199" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P199" s="7" t="n"/>
       <c r="Q199" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R199" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S199" s="8" t="inlineStr"/>
@@ -15716,7 +15714,7 @@
       <c r="V199" s="6" t="inlineStr"/>
       <c r="W199" s="7" t="inlineStr">
         <is>
-          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
+          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
         </is>
       </c>
     </row>
@@ -15730,13 +15728,13 @@
         </is>
       </c>
       <c r="C200" s="9" t="n">
-        <v>2240</v>
+        <v>1685</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E200" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F200" s="7" t="inlineStr">
         <is>
@@ -15754,22 +15752,22 @@
         </is>
       </c>
       <c r="I200" s="7" t="n">
-        <v>884</v>
+        <v>578</v>
       </c>
       <c r="J200" s="7" t="n"/>
       <c r="K200" s="7" t="n"/>
       <c r="L200" s="7" t="n"/>
       <c r="M200" s="7" t="n"/>
       <c r="N200" s="7" t="n">
-        <v>13388</v>
+        <v>13356</v>
       </c>
       <c r="O200" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P200" s="7" t="n"/>
       <c r="Q200" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R200" s="7" t="inlineStr">
@@ -15791,7 +15789,7 @@
       <c r="V200" s="6" t="inlineStr"/>
       <c r="W200" s="7" t="inlineStr">
         <is>
-          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
+          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
         </is>
       </c>
     </row>
@@ -15805,7 +15803,7 @@
         </is>
       </c>
       <c r="C201" s="9" t="n">
-        <v>1150</v>
+        <v>1765</v>
       </c>
       <c r="D201" s="7" t="n">
         <v>1</v>
@@ -15820,7 +15818,7 @@
       </c>
       <c r="G201" s="8" t="inlineStr">
         <is>
-          <t>John Street, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H201" s="7" t="inlineStr">
@@ -15829,25 +15827,27 @@
         </is>
       </c>
       <c r="I201" s="7" t="n">
-        <v>248</v>
+        <v>641</v>
       </c>
       <c r="J201" s="7" t="n"/>
       <c r="K201" s="7" t="n"/>
       <c r="L201" s="7" t="n"/>
       <c r="M201" s="7" t="n"/>
-      <c r="N201" s="7" t="n"/>
+      <c r="N201" s="7" t="n">
+        <v>13356</v>
+      </c>
       <c r="O201" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P201" s="7" t="n"/>
       <c r="Q201" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R201" s="7" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S201" s="8" t="inlineStr"/>
@@ -15864,7 +15864,7 @@
       <c r="V201" s="6" t="inlineStr"/>
       <c r="W201" s="7" t="inlineStr">
         <is>
-          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
+          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
         </is>
       </c>
     </row>
@@ -15878,49 +15878,51 @@
         </is>
       </c>
       <c r="C202" s="9" t="n">
-        <v>3400</v>
+        <v>2240</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E202" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F202" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G202" s="8" t="inlineStr">
         <is>
-          <t>Barton Road, Bristol, BS2</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H202" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I202" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I202" s="7" t="n">
+        <v>884</v>
+      </c>
       <c r="J202" s="7" t="n"/>
       <c r="K202" s="7" t="n"/>
       <c r="L202" s="7" t="n"/>
       <c r="M202" s="7" t="n"/>
       <c r="N202" s="7" t="n">
-        <v>19720</v>
+        <v>13388</v>
       </c>
       <c r="O202" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P202" s="7" t="n"/>
       <c r="Q202" s="7" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R202" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S202" s="8" t="inlineStr"/>
@@ -15937,7 +15939,7 @@
       <c r="V202" s="6" t="inlineStr"/>
       <c r="W202" s="7" t="inlineStr">
         <is>
-          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
+          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
         </is>
       </c>
     </row>
@@ -15951,7 +15953,7 @@
         </is>
       </c>
       <c r="C203" s="9" t="n">
-        <v>1250</v>
+        <v>1150</v>
       </c>
       <c r="D203" s="7" t="n">
         <v>1</v>
@@ -15966,34 +15968,34 @@
       </c>
       <c r="G203" s="8" t="inlineStr">
         <is>
-          <t>St Peters Court, Bedminster</t>
+          <t>John Street, BS1</t>
         </is>
       </c>
       <c r="H203" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I203" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I203" s="7" t="n">
+        <v>248</v>
+      </c>
       <c r="J203" s="7" t="n"/>
       <c r="K203" s="7" t="n"/>
       <c r="L203" s="7" t="n"/>
       <c r="M203" s="7" t="n"/>
-      <c r="N203" s="7" t="n">
-        <v>15352</v>
-      </c>
+      <c r="N203" s="7" t="n"/>
       <c r="O203" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P203" s="7" t="n"/>
       <c r="Q203" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R203" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+          <t>Bristol Property Centre, Bristol</t>
         </is>
       </c>
       <c r="S203" s="8" t="inlineStr"/>
@@ -16010,7 +16012,7 @@
       <c r="V203" s="6" t="inlineStr"/>
       <c r="W203" s="7" t="inlineStr">
         <is>
-          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
+          <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
         </is>
       </c>
     </row>
@@ -16024,22 +16026,22 @@
         </is>
       </c>
       <c r="C204" s="9" t="n">
-        <v>2300</v>
+        <v>3400</v>
       </c>
       <c r="D204" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E204" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F204" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G204" s="8" t="inlineStr">
         <is>
-          <t>Castle Park View, Castle Street, Bristol</t>
+          <t>Barton Road, Bristol, BS2</t>
         </is>
       </c>
       <c r="H204" s="7" t="inlineStr">
@@ -16047,15 +16049,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I204" s="7" t="n">
-        <v>773</v>
-      </c>
+      <c r="I204" s="7" t="n"/>
       <c r="J204" s="7" t="n"/>
       <c r="K204" s="7" t="n"/>
       <c r="L204" s="7" t="n"/>
       <c r="M204" s="7" t="n"/>
       <c r="N204" s="7" t="n">
-        <v>14172</v>
+        <v>19720</v>
       </c>
       <c r="O204" s="7" t="n">
         <v>1</v>
@@ -16063,12 +16063,12 @@
       <c r="P204" s="7" t="n"/>
       <c r="Q204" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="R204" s="7" t="inlineStr">
         <is>
-          <t>Savills Lettings, CPV</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S204" s="8" t="inlineStr"/>
@@ -16085,14 +16085,162 @@
       <c r="V204" s="6" t="inlineStr"/>
       <c r="W204" s="7" t="inlineStr">
         <is>
+          <t>a7f1932ce6ceff65a30f30ddc8f2aa5dea7428d0</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B205" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C205" s="9" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D205" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F205" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G205" s="8" t="inlineStr">
+        <is>
+          <t>St Peters Court, Bedminster</t>
+        </is>
+      </c>
+      <c r="H205" s="7" t="inlineStr">
+        <is>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I205" s="7" t="n"/>
+      <c r="J205" s="7" t="n"/>
+      <c r="K205" s="7" t="n"/>
+      <c r="L205" s="7" t="n"/>
+      <c r="M205" s="7" t="n"/>
+      <c r="N205" s="7" t="n">
+        <v>15352</v>
+      </c>
+      <c r="O205" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P205" s="7" t="n"/>
+      <c r="Q205" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R205" s="7" t="inlineStr">
+        <is>
+          <t>Chappell &amp; Matthews Lettings, Bristol</t>
+        </is>
+      </c>
+      <c r="S205" s="8" t="inlineStr"/>
+      <c r="T205" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V205" s="6" t="inlineStr"/>
+      <c r="W205" s="7" t="inlineStr">
+        <is>
+          <t>363ef947fcba1d439f031fcf679245a49cb8426e</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B206" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C206" s="9" t="n">
+        <v>2300</v>
+      </c>
+      <c r="D206" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E206" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F206" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G206" s="8" t="inlineStr">
+        <is>
+          <t>Castle Park View, Castle Street, Bristol</t>
+        </is>
+      </c>
+      <c r="H206" s="7" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I206" s="7" t="n">
+        <v>773</v>
+      </c>
+      <c r="J206" s="7" t="n"/>
+      <c r="K206" s="7" t="n"/>
+      <c r="L206" s="7" t="n"/>
+      <c r="M206" s="7" t="n"/>
+      <c r="N206" s="7" t="n">
+        <v>14172</v>
+      </c>
+      <c r="O206" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P206" s="7" t="n"/>
+      <c r="Q206" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="R206" s="7" t="inlineStr">
+        <is>
+          <t>Savills Lettings, CPV</t>
+        </is>
+      </c>
+      <c r="S206" s="8" t="inlineStr"/>
+      <c r="T206" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V206" s="6" t="inlineStr"/>
+      <c r="W206" s="7" t="inlineStr">
+        <is>
           <t>08411d7c5a6f10970306f10b45d00f0717234e1f</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W204"/>
+  <autoFilter ref="A1:W206"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204 U205 U206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16300,6 +16448,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T202" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T203" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T206" r:id="rId205"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 168
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$208</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204 U205 U206 U207 U208" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W204"/>
+  <dimension ref="A1:W208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2486,7 +2486,7 @@
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1495</v>
+        <v>1475</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>1</v>
@@ -10309,7 +10309,7 @@
         </is>
       </c>
       <c r="C127" s="9" t="n">
-        <v>1395</v>
+        <v>1350</v>
       </c>
       <c r="D127" s="7" t="n">
         <v>1</v>
@@ -10455,13 +10455,13 @@
         </is>
       </c>
       <c r="C129" s="9" t="n">
-        <v>2400</v>
+        <v>1999</v>
       </c>
       <c r="D129" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E129" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
@@ -10470,7 +10470,7 @@
       </c>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H129" s="7" t="inlineStr">
@@ -10484,7 +10484,7 @@
       <c r="L129" s="7" t="n"/>
       <c r="M129" s="7" t="n"/>
       <c r="N129" s="7" t="n">
-        <v>21360</v>
+        <v>21736</v>
       </c>
       <c r="O129" s="7" t="n">
         <v>0</v>
@@ -10492,12 +10492,12 @@
       <c r="P129" s="7" t="n"/>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="R129" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S129" s="8" t="inlineStr"/>
@@ -10514,7 +10514,7 @@
       <c r="V129" s="6" t="inlineStr"/>
       <c r="W129" s="7" t="inlineStr">
         <is>
-          <t>0b6e19cc97b73c7e581c5f306902c64d0c59b226</t>
+          <t>b188bd57bbbf81aacefb9ead81e003950d9dbb44</t>
         </is>
       </c>
     </row>
@@ -10528,7 +10528,7 @@
         </is>
       </c>
       <c r="C130" s="9" t="n">
-        <v>1600</v>
+        <v>1620</v>
       </c>
       <c r="D130" s="7" t="n">
         <v>1</v>
@@ -10543,7 +10543,7 @@
       </c>
       <c r="G130" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
@@ -10551,13 +10551,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I130" s="7" t="n"/>
+      <c r="I130" s="7" t="n">
+        <v>450</v>
+      </c>
       <c r="J130" s="7" t="n"/>
       <c r="K130" s="7" t="n"/>
       <c r="L130" s="7" t="n"/>
       <c r="M130" s="7" t="n"/>
       <c r="N130" s="7" t="n">
-        <v>21996</v>
+        <v>20984</v>
       </c>
       <c r="O130" s="7" t="n">
         <v>0</v>
@@ -10565,12 +10567,12 @@
       <c r="P130" s="7" t="n"/>
       <c r="Q130" s="7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="R130" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S130" s="8" t="inlineStr"/>
@@ -10587,7 +10589,7 @@
       <c r="V130" s="6" t="inlineStr"/>
       <c r="W130" s="7" t="inlineStr">
         <is>
-          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
+          <t>fe6e3df8f6718d87db10b02c67c678dfb5383040</t>
         </is>
       </c>
     </row>
@@ -10601,13 +10603,13 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>1560</v>
+        <v>2180</v>
       </c>
       <c r="D131" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E131" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
@@ -10625,7 +10627,7 @@
         </is>
       </c>
       <c r="I131" s="7" t="n">
-        <v>472</v>
+        <v>784</v>
       </c>
       <c r="J131" s="7" t="n"/>
       <c r="K131" s="7" t="n"/>
@@ -10640,7 +10642,7 @@
       <c r="P131" s="7" t="n"/>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
@@ -10662,7 +10664,7 @@
       <c r="V131" s="6" t="inlineStr"/>
       <c r="W131" s="7" t="inlineStr">
         <is>
-          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
+          <t>dc2f5e68d4c3bff21b0cc1f55886f21f2cd84107</t>
         </is>
       </c>
     </row>
@@ -10676,7 +10678,7 @@
         </is>
       </c>
       <c r="C132" s="9" t="n">
-        <v>1660</v>
+        <v>1640</v>
       </c>
       <c r="D132" s="7" t="n">
         <v>1</v>
@@ -10691,7 +10693,7 @@
       </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H132" s="7" t="inlineStr">
@@ -10700,14 +10702,14 @@
         </is>
       </c>
       <c r="I132" s="7" t="n">
-        <v>558</v>
+        <v>484</v>
       </c>
       <c r="J132" s="7" t="n"/>
       <c r="K132" s="7" t="n"/>
       <c r="L132" s="7" t="n"/>
       <c r="M132" s="7" t="n"/>
       <c r="N132" s="7" t="n">
-        <v>20984</v>
+        <v>21732</v>
       </c>
       <c r="O132" s="7" t="n">
         <v>0</v>
@@ -10715,12 +10717,12 @@
       <c r="P132" s="7" t="n"/>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S132" s="8" t="inlineStr"/>
@@ -10737,7 +10739,7 @@
       <c r="V132" s="6" t="inlineStr"/>
       <c r="W132" s="7" t="inlineStr">
         <is>
-          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
+          <t>9d0e8dd4112619a2af73a9e7521afe06378d948b</t>
         </is>
       </c>
     </row>
@@ -10751,7 +10753,7 @@
         </is>
       </c>
       <c r="C133" s="9" t="n">
-        <v>1860</v>
+        <v>2400</v>
       </c>
       <c r="D133" s="7" t="n">
         <v>2</v>
@@ -10766,23 +10768,21 @@
       </c>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I133" s="7" t="n">
-        <v>647</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I133" s="7" t="n"/>
       <c r="J133" s="7" t="n"/>
       <c r="K133" s="7" t="n"/>
       <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="n"/>
       <c r="N133" s="7" t="n">
-        <v>21740</v>
+        <v>21360</v>
       </c>
       <c r="O133" s="7" t="n">
         <v>0</v>
@@ -10790,12 +10790,12 @@
       <c r="P133" s="7" t="n"/>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S133" s="8" t="inlineStr"/>
@@ -10812,7 +10812,7 @@
       <c r="V133" s="6" t="inlineStr"/>
       <c r="W133" s="7" t="inlineStr">
         <is>
-          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
+          <t>0b6e19cc97b73c7e581c5f306902c64d0c59b226</t>
         </is>
       </c>
     </row>
@@ -10841,7 +10841,7 @@
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
@@ -10849,15 +10849,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I134" s="7" t="n">
-        <v>549</v>
-      </c>
+      <c r="I134" s="7" t="n"/>
       <c r="J134" s="7" t="n"/>
       <c r="K134" s="7" t="n"/>
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="7" t="n">
-        <v>21816</v>
+        <v>21996</v>
       </c>
       <c r="O134" s="7" t="n">
         <v>0</v>
@@ -10865,12 +10863,12 @@
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10887,7 +10885,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
+          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
         </is>
       </c>
     </row>
@@ -10901,13 +10899,13 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1900</v>
+        <v>1560</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E135" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
@@ -10916,7 +10914,7 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
@@ -10925,14 +10923,14 @@
         </is>
       </c>
       <c r="I135" s="7" t="n">
-        <v>624</v>
+        <v>472</v>
       </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="7" t="n">
-        <v>21740</v>
+        <v>20984</v>
       </c>
       <c r="O135" s="7" t="n">
         <v>0</v>
@@ -10940,12 +10938,12 @@
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S135" s="8" t="inlineStr"/>
@@ -10962,7 +10960,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
+          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
         </is>
       </c>
     </row>
@@ -10976,7 +10974,7 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>1530</v>
+        <v>1660</v>
       </c>
       <c r="D136" s="7" t="n">
         <v>1</v>
@@ -10991,7 +10989,7 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
@@ -11000,14 +10998,14 @@
         </is>
       </c>
       <c r="I136" s="7" t="n">
-        <v>548</v>
+        <v>558</v>
       </c>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>21740</v>
+        <v>20984</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -11015,12 +11013,12 @@
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11037,7 +11035,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
+          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
         </is>
       </c>
     </row>
@@ -11051,7 +11049,7 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>2110</v>
+        <v>1860</v>
       </c>
       <c r="D137" s="7" t="n">
         <v>2</v>
@@ -11075,7 +11073,7 @@
         </is>
       </c>
       <c r="I137" s="7" t="n">
-        <v>624</v>
+        <v>647</v>
       </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
@@ -11090,7 +11088,7 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
@@ -11112,7 +11110,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
+          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
         </is>
       </c>
     </row>
@@ -11126,7 +11124,7 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1530</v>
+        <v>1600</v>
       </c>
       <c r="D138" s="7" t="n">
         <v>1</v>
@@ -11150,14 +11148,14 @@
         </is>
       </c>
       <c r="I138" s="7" t="n">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="J138" s="7" t="n"/>
       <c r="K138" s="7" t="n"/>
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>21740</v>
+        <v>21816</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11165,7 +11163,7 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
@@ -11187,7 +11185,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
+          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
         </is>
       </c>
     </row>
@@ -11201,7 +11199,7 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>1600</v>
+        <v>1900</v>
       </c>
       <c r="D139" s="7" t="n">
         <v>2</v>
@@ -11216,7 +11214,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11224,13 +11222,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I139" s="7" t="n"/>
+      <c r="I139" s="7" t="n">
+        <v>624</v>
+      </c>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>20880</v>
+        <v>21740</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11238,12 +11238,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11260,7 +11260,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
+          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
         </is>
       </c>
     </row>
@@ -11274,13 +11274,13 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1800</v>
+        <v>1530</v>
       </c>
       <c r="D140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
@@ -11289,7 +11289,7 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
@@ -11298,14 +11298,14 @@
         </is>
       </c>
       <c r="I140" s="7" t="n">
-        <v>980</v>
+        <v>548</v>
       </c>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>21316</v>
+        <v>21740</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11318,7 +11318,7 @@
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11335,7 +11335,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
+          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
         </is>
       </c>
     </row>
@@ -11349,13 +11349,13 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1995</v>
+        <v>2110</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
@@ -11364,7 +11364,7 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
@@ -11372,13 +11372,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I141" s="7" t="n"/>
+      <c r="I141" s="7" t="n">
+        <v>624</v>
+      </c>
       <c r="J141" s="7" t="n"/>
       <c r="K141" s="7" t="n"/>
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>21196</v>
+        <v>21740</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11386,12 +11388,12 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11408,7 +11410,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
+          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
         </is>
       </c>
     </row>
@@ -11422,13 +11424,13 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>1750</v>
+        <v>1530</v>
       </c>
       <c r="D142" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E142" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
@@ -11437,7 +11439,7 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
@@ -11446,14 +11448,14 @@
         </is>
       </c>
       <c r="I142" s="7" t="n">
-        <v>849</v>
+        <v>544</v>
       </c>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>21028</v>
+        <v>21740</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11461,12 +11463,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11483,7 +11485,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
+          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
         </is>
       </c>
     </row>
@@ -11497,7 +11499,7 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1550</v>
+        <v>1600</v>
       </c>
       <c r="D143" s="7" t="n">
         <v>2</v>
@@ -11512,12 +11514,12 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Portland Heights - St. Pauls</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I143" s="7" t="n"/>
@@ -11526,7 +11528,7 @@
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>21420</v>
+        <v>20880</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11534,12 +11536,12 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Bishopston</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11556,7 +11558,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
+          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
         </is>
       </c>
     </row>
@@ -11570,13 +11572,13 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1400</v>
+        <v>1800</v>
       </c>
       <c r="D144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
@@ -11585,7 +11587,7 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>The Atrium, Redcliffe Street, BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
@@ -11593,13 +11595,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I144" s="7" t="n"/>
+      <c r="I144" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>20292</v>
+        <v>21316</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11607,12 +11611,12 @@
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11629,7 +11633,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
+          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11647,7 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>1150</v>
+        <v>1995</v>
       </c>
       <c r="D145" s="7" t="n">
         <v>1</v>
@@ -11658,12 +11662,12 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H145" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I145" s="7" t="n"/>
@@ -11672,7 +11676,7 @@
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>15376</v>
+        <v>21196</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11680,12 +11684,12 @@
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S145" s="8" t="inlineStr"/>
@@ -11702,7 +11706,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
+          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
         </is>
       </c>
     </row>
@@ -11716,13 +11720,13 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>1300</v>
+        <v>1750</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E146" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
@@ -11731,7 +11735,7 @@
       </c>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The Milliners, BS1 6WU</t>
+          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H146" s="7" t="inlineStr">
@@ -11740,14 +11744,14 @@
         </is>
       </c>
       <c r="I146" s="7" t="n">
-        <v>463</v>
+        <v>849</v>
       </c>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>21440</v>
+        <v>21028</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>0</v>
@@ -11760,7 +11764,7 @@
       </c>
       <c r="R146" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S146" s="8" t="inlineStr"/>
@@ -11777,7 +11781,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
+          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
         </is>
       </c>
     </row>
@@ -11791,13 +11795,13 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>1150</v>
+        <v>1550</v>
       </c>
       <c r="D147" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E147" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F147" s="7" t="inlineStr">
         <is>
@@ -11806,7 +11810,7 @@
       </c>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>Century Place, St. Paul Street, BS2 8AN</t>
+          <t>Portland Heights - St. Pauls</t>
         </is>
       </c>
       <c r="H147" s="7" t="inlineStr">
@@ -11814,15 +11818,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I147" s="7" t="n">
-        <v>344</v>
-      </c>
+      <c r="I147" s="7" t="n"/>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="7" t="n">
-        <v>21792</v>
+        <v>21420</v>
       </c>
       <c r="O147" s="7" t="n">
         <v>0</v>
@@ -11830,12 +11832,12 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Ocean, Bishopston</t>
         </is>
       </c>
       <c r="S147" s="8" t="inlineStr"/>
@@ -11852,7 +11854,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
+          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
         </is>
       </c>
     </row>
@@ -11866,13 +11868,13 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>1800</v>
+        <v>1400</v>
       </c>
       <c r="D148" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E148" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
@@ -11881,7 +11883,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Waverley House, BS1</t>
+          <t>The Atrium, Redcliffe Street, BS1</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
@@ -11895,7 +11897,7 @@
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>17956</v>
+        <v>20292</v>
       </c>
       <c r="O148" s="7" t="n">
         <v>0</v>
@@ -11903,12 +11905,12 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11925,7 +11927,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
+          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
         </is>
       </c>
     </row>
@@ -11939,13 +11941,13 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>2170</v>
+        <v>1150</v>
       </c>
       <c r="D149" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E149" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F149" s="7" t="inlineStr">
         <is>
@@ -11954,23 +11956,21 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H149" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I149" s="7" t="n">
-        <v>721</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I149" s="7" t="n"/>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="7" t="n">
-        <v>21732</v>
+        <v>15376</v>
       </c>
       <c r="O149" s="7" t="n">
         <v>0</v>
@@ -11978,12 +11978,12 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S149" s="8" t="inlineStr"/>
@@ -12000,7 +12000,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
+          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
         </is>
       </c>
     </row>
@@ -12014,13 +12014,13 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1965</v>
+        <v>1300</v>
       </c>
       <c r="D150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>City Centre, The Milliners, BS1 6WU</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
@@ -12038,14 +12038,14 @@
         </is>
       </c>
       <c r="I150" s="7" t="n">
-        <v>771</v>
+        <v>463</v>
       </c>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>21740</v>
+        <v>21440</v>
       </c>
       <c r="O150" s="7" t="n">
         <v>0</v>
@@ -12053,12 +12053,12 @@
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12075,7 +12075,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
+          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
         </is>
       </c>
     </row>
@@ -12089,10 +12089,10 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1680</v>
+        <v>1150</v>
       </c>
       <c r="D151" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E151" s="7" t="n">
         <v>1</v>
@@ -12104,21 +12104,23 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Century Place, St. Paul Street, BS2 8AN</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I151" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I151" s="7" t="n">
+        <v>344</v>
+      </c>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>20628</v>
+        <v>21792</v>
       </c>
       <c r="O151" s="7" t="n">
         <v>0</v>
@@ -12126,12 +12128,12 @@
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12148,7 +12150,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
+          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
         </is>
       </c>
     </row>
@@ -12162,13 +12164,13 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1625</v>
+        <v>1800</v>
       </c>
       <c r="D152" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E152" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
@@ -12177,7 +12179,7 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Waverley House, BS1</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
@@ -12185,15 +12187,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I152" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I152" s="7" t="n"/>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>21732</v>
+        <v>17956</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12201,12 +12201,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12223,7 +12223,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
+          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
         </is>
       </c>
     </row>
@@ -12237,7 +12237,7 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>1940</v>
+        <v>2170</v>
       </c>
       <c r="D153" s="7" t="n">
         <v>2</v>
@@ -12252,7 +12252,7 @@
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
@@ -12261,14 +12261,14 @@
         </is>
       </c>
       <c r="I153" s="7" t="n">
-        <v>607</v>
+        <v>721</v>
       </c>
       <c r="J153" s="7" t="n"/>
       <c r="K153" s="7" t="n"/>
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O153" s="7" t="n">
         <v>0</v>
@@ -12276,12 +12276,12 @@
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12298,7 +12298,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
+          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
         </is>
       </c>
     </row>
@@ -12312,13 +12312,13 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1465</v>
+        <v>1965</v>
       </c>
       <c r="D154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
@@ -12336,14 +12336,14 @@
         </is>
       </c>
       <c r="I154" s="7" t="n">
-        <v>505</v>
+        <v>771</v>
       </c>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
@@ -12351,7 +12351,7 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
@@ -12373,7 +12373,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>e86143466441bbbf802706245b19ef679ec29055</t>
+          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
         </is>
       </c>
     </row>
@@ -12387,10 +12387,10 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>1150</v>
+        <v>1680</v>
       </c>
       <c r="D155" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E155" s="7" t="n">
         <v>1</v>
@@ -12402,12 +12402,12 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>St. Philips, Bristol, BS2</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I155" s="7" t="n"/>
@@ -12416,7 +12416,7 @@
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="7" t="n">
-        <v>20784</v>
+        <v>20628</v>
       </c>
       <c r="O155" s="7" t="n">
         <v>0</v>
@@ -12424,7 +12424,7 @@
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
@@ -12446,7 +12446,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
+          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
         </is>
       </c>
     </row>
@@ -12460,7 +12460,7 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>1685</v>
+        <v>1625</v>
       </c>
       <c r="D156" s="7" t="n">
         <v>1</v>
@@ -12475,7 +12475,7 @@
       </c>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr">
@@ -12484,14 +12484,14 @@
         </is>
       </c>
       <c r="I156" s="7" t="n">
-        <v>545</v>
+        <v>486</v>
       </c>
       <c r="J156" s="7" t="n"/>
       <c r="K156" s="7" t="n"/>
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="7" t="n">
-        <v>21024</v>
+        <v>21732</v>
       </c>
       <c r="O156" s="7" t="n">
         <v>0</v>
@@ -12499,12 +12499,12 @@
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S156" s="8" t="inlineStr"/>
@@ -12521,7 +12521,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
+          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
         </is>
       </c>
     </row>
@@ -12535,7 +12535,7 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>1700</v>
+        <v>1940</v>
       </c>
       <c r="D157" s="7" t="n">
         <v>2</v>
@@ -12545,26 +12545,28 @@
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>Dunkerry Road - Windmill Hill</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H157" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I157" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I157" s="7" t="n">
+        <v>607</v>
+      </c>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="7" t="n">
-        <v>8448</v>
+        <v>21740</v>
       </c>
       <c r="O157" s="7" t="n">
         <v>0</v>
@@ -12572,12 +12574,12 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S157" s="8" t="inlineStr"/>
@@ -12594,7 +12596,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
+          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
         </is>
       </c>
     </row>
@@ -12608,7 +12610,7 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>1460</v>
+        <v>1465</v>
       </c>
       <c r="D158" s="7" t="n">
         <v>1</v>
@@ -12632,14 +12634,14 @@
         </is>
       </c>
       <c r="I158" s="7" t="n">
-        <v>473</v>
+        <v>505</v>
       </c>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>13840</v>
+        <v>21816</v>
       </c>
       <c r="O158" s="7" t="n">
         <v>0</v>
@@ -12647,7 +12649,7 @@
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
@@ -12669,7 +12671,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
+          <t>e86143466441bbbf802706245b19ef679ec29055</t>
         </is>
       </c>
     </row>
@@ -12683,7 +12685,7 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1630</v>
+        <v>1150</v>
       </c>
       <c r="D159" s="7" t="n">
         <v>1</v>
@@ -12698,36 +12700,34 @@
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>St. Philips, Bristol, BS2</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I159" s="7" t="n">
-        <v>486</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I159" s="7" t="n"/>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="7" t="n">
-        <v>13860</v>
+        <v>20784</v>
       </c>
       <c r="O159" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12744,7 +12744,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
+          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
         </is>
       </c>
     </row>
@@ -12758,7 +12758,7 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>1625</v>
+        <v>1685</v>
       </c>
       <c r="D160" s="7" t="n">
         <v>1</v>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H160" s="7" t="inlineStr">
@@ -12782,14 +12782,14 @@
         </is>
       </c>
       <c r="I160" s="7" t="n">
-        <v>486</v>
+        <v>545</v>
       </c>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
       <c r="N160" s="7" t="n">
-        <v>21732</v>
+        <v>21024</v>
       </c>
       <c r="O160" s="7" t="n">
         <v>0</v>
@@ -12797,12 +12797,12 @@
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S160" s="8" t="inlineStr"/>
@@ -12819,7 +12819,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
+          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
         </is>
       </c>
     </row>
@@ -12833,7 +12833,7 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>1650</v>
+        <v>1700</v>
       </c>
       <c r="D161" s="7" t="n">
         <v>2</v>
@@ -12843,28 +12843,26 @@
       </c>
       <c r="F161" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Harris Lofts, BS1 4BB</t>
+          <t>Dunkerry Road - Windmill Hill</t>
         </is>
       </c>
       <c r="H161" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I161" s="7" t="n">
-        <v>667</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I161" s="7" t="n"/>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
       <c r="N161" s="7" t="n">
-        <v>20088</v>
+        <v>8448</v>
       </c>
       <c r="O161" s="7" t="n">
         <v>0</v>
@@ -12872,12 +12870,12 @@
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S161" s="8" t="inlineStr"/>
@@ -12894,7 +12892,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
+          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
         </is>
       </c>
     </row>
@@ -12908,7 +12906,7 @@
         </is>
       </c>
       <c r="C162" s="9" t="n">
-        <v>1650</v>
+        <v>1460</v>
       </c>
       <c r="D162" s="7" t="n">
         <v>1</v>
@@ -12923,7 +12921,7 @@
       </c>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>Central Quey North, Broad Quay, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
@@ -12931,13 +12929,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I162" s="7" t="n"/>
+      <c r="I162" s="7" t="n">
+        <v>473</v>
+      </c>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
       <c r="N162" s="7" t="n">
-        <v>20768</v>
+        <v>13840</v>
       </c>
       <c r="O162" s="7" t="n">
         <v>0</v>
@@ -12945,12 +12945,12 @@
       <c r="P162" s="7" t="n"/>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S162" s="8" t="inlineStr"/>
@@ -12967,7 +12967,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
+          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
         </is>
       </c>
     </row>
@@ -12981,7 +12981,7 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1550</v>
+        <v>1630</v>
       </c>
       <c r="D163" s="7" t="n">
         <v>1</v>
@@ -12996,7 +12996,7 @@
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
@@ -13004,26 +13004,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I163" s="7" t="n"/>
+      <c r="I163" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="7" t="n">
-        <v>21100</v>
+        <v>13860</v>
       </c>
       <c r="O163" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13040,7 +13042,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
+          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
         </is>
       </c>
     </row>
@@ -13054,7 +13056,7 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>1390</v>
+        <v>1625</v>
       </c>
       <c r="D164" s="7" t="n">
         <v>1</v>
@@ -13069,7 +13071,7 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
@@ -13077,24 +13079,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I164" s="7" t="n"/>
+      <c r="I164" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
-      <c r="N164" s="7" t="n"/>
+      <c r="N164" s="7" t="n">
+        <v>21732</v>
+      </c>
       <c r="O164" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13111,7 +13117,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
+          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
         </is>
       </c>
     </row>
@@ -13125,13 +13131,13 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1485</v>
+        <v>1650</v>
       </c>
       <c r="D165" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E165" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F165" s="7" t="inlineStr">
         <is>
@@ -13140,7 +13146,7 @@
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Harbourside, Harris Lofts, BS1 4BB</t>
         </is>
       </c>
       <c r="H165" s="7" t="inlineStr">
@@ -13149,14 +13155,14 @@
         </is>
       </c>
       <c r="I165" s="7" t="n">
-        <v>470</v>
+        <v>667</v>
       </c>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>21740</v>
+        <v>20088</v>
       </c>
       <c r="O165" s="7" t="n">
         <v>0</v>
@@ -13164,12 +13170,12 @@
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R165" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S165" s="8" t="inlineStr"/>
@@ -13186,7 +13192,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
+          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
         </is>
       </c>
     </row>
@@ -13200,7 +13206,7 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>1635</v>
+        <v>1650</v>
       </c>
       <c r="D166" s="7" t="n">
         <v>1</v>
@@ -13215,7 +13221,7 @@
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Central Quey North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H166" s="7" t="inlineStr">
@@ -13223,15 +13229,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I166" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I166" s="7" t="n"/>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="7" t="n">
-        <v>21732</v>
+        <v>20768</v>
       </c>
       <c r="O166" s="7" t="n">
         <v>0</v>
@@ -13239,12 +13243,12 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
@@ -13261,7 +13265,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
+          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
         </is>
       </c>
     </row>
@@ -13275,13 +13279,13 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>2060</v>
+        <v>1550</v>
       </c>
       <c r="D167" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E167" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F167" s="7" t="inlineStr">
         <is>
@@ -13290,7 +13294,7 @@
       </c>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H167" s="7" t="inlineStr">
@@ -13298,15 +13302,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I167" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I167" s="7" t="n"/>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="7" t="n">
-        <v>21732</v>
+        <v>21100</v>
       </c>
       <c r="O167" s="7" t="n">
         <v>0</v>
@@ -13314,12 +13316,12 @@
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S167" s="8" t="inlineStr"/>
@@ -13336,7 +13338,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
+          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
         </is>
       </c>
     </row>
@@ -13350,7 +13352,7 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1545</v>
+        <v>1390</v>
       </c>
       <c r="D168" s="7" t="n">
         <v>1</v>
@@ -13365,7 +13367,7 @@
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
@@ -13373,28 +13375,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I168" s="7" t="n">
-        <v>548</v>
-      </c>
+      <c r="I168" s="7" t="n"/>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
-      <c r="N168" s="7" t="n">
-        <v>21740</v>
-      </c>
+      <c r="N168" s="7" t="n"/>
       <c r="O168" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13411,7 +13409,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
+          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
         </is>
       </c>
     </row>
@@ -13425,7 +13423,7 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1640</v>
+        <v>1485</v>
       </c>
       <c r="D169" s="7" t="n">
         <v>1</v>
@@ -13440,7 +13438,7 @@
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
@@ -13449,14 +13447,14 @@
         </is>
       </c>
       <c r="I169" s="7" t="n">
-        <v>486</v>
+        <v>470</v>
       </c>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>21732</v>
+        <v>21740</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13464,12 +13462,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13486,7 +13484,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
+          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
         </is>
       </c>
     </row>
@@ -13500,10 +13498,10 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>2115</v>
+        <v>1635</v>
       </c>
       <c r="D170" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E170" s="7" t="n">
         <v>1</v>
@@ -13524,7 +13522,7 @@
         </is>
       </c>
       <c r="I170" s="7" t="n">
-        <v>722</v>
+        <v>486</v>
       </c>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
@@ -13539,7 +13537,7 @@
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
@@ -13561,7 +13559,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
+          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
         </is>
       </c>
     </row>
@@ -13575,7 +13573,7 @@
         </is>
       </c>
       <c r="C171" s="9" t="n">
-        <v>1970</v>
+        <v>2060</v>
       </c>
       <c r="D171" s="7" t="n">
         <v>2</v>
@@ -13590,7 +13588,7 @@
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H171" s="7" t="inlineStr">
@@ -13599,14 +13597,14 @@
         </is>
       </c>
       <c r="I171" s="7" t="n">
-        <v>750</v>
+        <v>721</v>
       </c>
       <c r="J171" s="7" t="n"/>
       <c r="K171" s="7" t="n"/>
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O171" s="7" t="n">
         <v>0</v>
@@ -13614,12 +13612,12 @@
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -13636,7 +13634,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
+          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
         </is>
       </c>
     </row>
@@ -13650,7 +13648,7 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1575</v>
+        <v>1545</v>
       </c>
       <c r="D172" s="7" t="n">
         <v>1</v>
@@ -13674,14 +13672,14 @@
         </is>
       </c>
       <c r="I172" s="7" t="n">
-        <v>430</v>
+        <v>548</v>
       </c>
       <c r="J172" s="7" t="n"/>
       <c r="K172" s="7" t="n"/>
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
@@ -13689,7 +13687,7 @@
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
@@ -13711,7 +13709,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
+          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
         </is>
       </c>
     </row>
@@ -13725,7 +13723,7 @@
         </is>
       </c>
       <c r="C173" s="9" t="n">
-        <v>1350</v>
+        <v>1640</v>
       </c>
       <c r="D173" s="7" t="n">
         <v>1</v>
@@ -13740,7 +13738,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Invicta, Millenium Promenade, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
@@ -13748,13 +13746,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I173" s="7" t="n"/>
+      <c r="I173" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>17344</v>
+        <v>21732</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13762,12 +13762,12 @@
       <c r="P173" s="7" t="n"/>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -13784,7 +13784,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
+          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
         </is>
       </c>
     </row>
@@ -13798,10 +13798,10 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1600</v>
+        <v>2115</v>
       </c>
       <c r="D174" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E174" s="7" t="n">
         <v>1</v>
@@ -13813,7 +13813,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
@@ -13821,13 +13821,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I174" s="7" t="n"/>
+      <c r="I174" s="7" t="n">
+        <v>722</v>
+      </c>
       <c r="J174" s="7" t="n"/>
       <c r="K174" s="7" t="n"/>
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>13404</v>
+        <v>21732</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13835,12 +13837,12 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -13857,7 +13859,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
+          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
         </is>
       </c>
     </row>
@@ -13871,13 +13873,13 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>1700</v>
+        <v>1970</v>
       </c>
       <c r="D175" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E175" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
@@ -13886,7 +13888,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
@@ -13895,14 +13897,14 @@
         </is>
       </c>
       <c r="I175" s="7" t="n">
-        <v>646</v>
+        <v>750</v>
       </c>
       <c r="J175" s="7" t="n"/>
       <c r="K175" s="7" t="n"/>
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
       <c r="N175" s="7" t="n">
-        <v>20928</v>
+        <v>21740</v>
       </c>
       <c r="O175" s="7" t="n">
         <v>0</v>
@@ -13910,12 +13912,12 @@
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -13932,7 +13934,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
+          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
         </is>
       </c>
     </row>
@@ -13946,13 +13948,13 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>2105</v>
+        <v>1575</v>
       </c>
       <c r="D176" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E176" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F176" s="7" t="inlineStr">
         <is>
@@ -13961,7 +13963,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H176" s="7" t="inlineStr">
@@ -13970,14 +13972,14 @@
         </is>
       </c>
       <c r="I176" s="7" t="n">
-        <v>745</v>
+        <v>430</v>
       </c>
       <c r="J176" s="7" t="n"/>
       <c r="K176" s="7" t="n"/>
       <c r="L176" s="7" t="n"/>
       <c r="M176" s="7" t="n"/>
       <c r="N176" s="7" t="n">
-        <v>20984</v>
+        <v>21816</v>
       </c>
       <c r="O176" s="7" t="n">
         <v>0</v>
@@ -13985,12 +13987,12 @@
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -14007,7 +14009,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
+          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
         </is>
       </c>
     </row>
@@ -14021,7 +14023,7 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>1595</v>
+        <v>1350</v>
       </c>
       <c r="D177" s="7" t="n">
         <v>1</v>
@@ -14036,7 +14038,7 @@
       </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Invicta, Millenium Promenade, BS1</t>
         </is>
       </c>
       <c r="H177" s="7" t="inlineStr">
@@ -14044,15 +14046,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I177" s="7" t="n">
-        <v>484</v>
-      </c>
+      <c r="I177" s="7" t="n"/>
       <c r="J177" s="7" t="n"/>
       <c r="K177" s="7" t="n"/>
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
       <c r="N177" s="7" t="n">
-        <v>21732</v>
+        <v>17344</v>
       </c>
       <c r="O177" s="7" t="n">
         <v>0</v>
@@ -14060,12 +14060,12 @@
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S177" s="8" t="inlineStr"/>
@@ -14082,7 +14082,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
+          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
         </is>
       </c>
     </row>
@@ -14096,10 +14096,10 @@
         </is>
       </c>
       <c r="C178" s="9" t="n">
-        <v>1999</v>
+        <v>1600</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E178" s="7" t="n">
         <v>1</v>
@@ -14111,12 +14111,12 @@
       </c>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Central Quay North, Bristol, BS1</t>
         </is>
       </c>
       <c r="H178" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I178" s="7" t="n"/>
@@ -14125,7 +14125,7 @@
       <c r="L178" s="7" t="n"/>
       <c r="M178" s="7" t="n"/>
       <c r="N178" s="7" t="n">
-        <v>21736</v>
+        <v>13404</v>
       </c>
       <c r="O178" s="7" t="n">
         <v>0</v>
@@ -14133,12 +14133,12 @@
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S178" s="8" t="inlineStr"/>
@@ -14155,7 +14155,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
+          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
         </is>
       </c>
     </row>
@@ -14169,10 +14169,10 @@
         </is>
       </c>
       <c r="C179" s="9" t="n">
-        <v>1605</v>
+        <v>1700</v>
       </c>
       <c r="D179" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E179" s="7" t="n">
         <v>1</v>
@@ -14184,7 +14184,7 @@
       </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
         </is>
       </c>
       <c r="H179" s="7" t="inlineStr">
@@ -14193,14 +14193,14 @@
         </is>
       </c>
       <c r="I179" s="7" t="n">
-        <v>487</v>
+        <v>646</v>
       </c>
       <c r="J179" s="7" t="n"/>
       <c r="K179" s="7" t="n"/>
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
       <c r="N179" s="7" t="n">
-        <v>21732</v>
+        <v>20928</v>
       </c>
       <c r="O179" s="7" t="n">
         <v>0</v>
@@ -14208,12 +14208,12 @@
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -14230,7 +14230,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
+          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
         </is>
       </c>
     </row>
@@ -14244,13 +14244,13 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>1390</v>
+        <v>2105</v>
       </c>
       <c r="D180" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E180" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F180" s="7" t="inlineStr">
         <is>
@@ -14259,7 +14259,7 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
@@ -14267,24 +14267,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I180" s="7" t="n"/>
+      <c r="I180" s="7" t="n">
+        <v>745</v>
+      </c>
       <c r="J180" s="7" t="n"/>
       <c r="K180" s="7" t="n"/>
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
-      <c r="N180" s="7" t="n"/>
+      <c r="N180" s="7" t="n">
+        <v>20984</v>
+      </c>
       <c r="O180" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14301,7 +14305,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
         </is>
       </c>
     </row>
@@ -14315,7 +14319,7 @@
         </is>
       </c>
       <c r="C181" s="9" t="n">
-        <v>1395</v>
+        <v>1595</v>
       </c>
       <c r="D181" s="7" t="n">
         <v>1</v>
@@ -14330,7 +14334,7 @@
       </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H181" s="7" t="inlineStr">
@@ -14338,13 +14342,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I181" s="7" t="n"/>
+      <c r="I181" s="7" t="n">
+        <v>484</v>
+      </c>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="7" t="n">
-        <v>20524</v>
+        <v>21732</v>
       </c>
       <c r="O181" s="7" t="n">
         <v>0</v>
@@ -14352,12 +14358,12 @@
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S181" s="8" t="inlineStr"/>
@@ -14374,7 +14380,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
         </is>
       </c>
     </row>
@@ -14388,22 +14394,22 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>1200</v>
+        <v>1999</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2 0JN</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
@@ -14411,15 +14417,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I182" s="7" t="n">
-        <v>452</v>
-      </c>
+      <c r="I182" s="7" t="n"/>
       <c r="J182" s="7" t="n"/>
       <c r="K182" s="7" t="n"/>
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>20472</v>
+        <v>21736</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14427,12 +14431,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14449,7 +14453,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
+          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
         </is>
       </c>
     </row>
@@ -14463,7 +14467,7 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>1450</v>
+        <v>1605</v>
       </c>
       <c r="D183" s="7" t="n">
         <v>1</v>
@@ -14478,7 +14482,7 @@
       </c>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H183" s="7" t="inlineStr">
@@ -14486,13 +14490,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I183" s="7" t="n"/>
+      <c r="I183" s="7" t="n">
+        <v>487</v>
+      </c>
       <c r="J183" s="7" t="n"/>
       <c r="K183" s="7" t="n"/>
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="7" t="n">
-        <v>16664</v>
+        <v>21732</v>
       </c>
       <c r="O183" s="7" t="n">
         <v>0</v>
@@ -14500,12 +14506,12 @@
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S183" s="8" t="inlineStr"/>
@@ -14522,7 +14528,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
+          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
         </is>
       </c>
     </row>
@@ -14536,13 +14542,13 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>3200</v>
+        <v>1390</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E184" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F184" s="7" t="inlineStr">
         <is>
@@ -14551,7 +14557,7 @@
       </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H184" s="7" t="inlineStr">
@@ -14564,21 +14570,19 @@
       <c r="K184" s="7" t="n"/>
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
-      <c r="N184" s="7" t="n">
-        <v>16664</v>
-      </c>
+      <c r="N184" s="7" t="n"/>
       <c r="O184" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
         <is>
-          <t>LettingaProperty.com, Nationwide - Lettings</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S184" s="8" t="inlineStr"/>
@@ -14595,7 +14599,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
+          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
         </is>
       </c>
     </row>
@@ -14609,7 +14613,7 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>1600</v>
+        <v>1395</v>
       </c>
       <c r="D185" s="7" t="n">
         <v>1</v>
@@ -14624,7 +14628,7 @@
       </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
@@ -14638,7 +14642,7 @@
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="7" t="n">
-        <v>21996</v>
+        <v>20524</v>
       </c>
       <c r="O185" s="7" t="n">
         <v>0</v>
@@ -14646,12 +14650,12 @@
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S185" s="8" t="inlineStr"/>
@@ -14668,7 +14672,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
@@ -14682,36 +14686,38 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>2400</v>
+        <v>1200</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E186" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F186" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Colston Avenue, Bristol, BS1</t>
+          <t>Sweetman Place, Bristol, BS2 0JN</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I186" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I186" s="7" t="n">
+        <v>452</v>
+      </c>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>14108</v>
+        <v>20472</v>
       </c>
       <c r="O186" s="7" t="n">
         <v>0</v>
@@ -14719,12 +14725,12 @@
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14741,7 +14747,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
+          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
         </is>
       </c>
     </row>
@@ -14755,7 +14761,7 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>1300</v>
+        <v>1450</v>
       </c>
       <c r="D187" s="7" t="n">
         <v>1</v>
@@ -14770,23 +14776,21 @@
       </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>East Street, Bedminster, BS3</t>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I187" s="7" t="n">
-        <v>560</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I187" s="7" t="n"/>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>14176</v>
+        <v>16664</v>
       </c>
       <c r="O187" s="7" t="n">
         <v>0</v>
@@ -14794,12 +14798,12 @@
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>Xeno Property, Bristol</t>
+          <t>Howard, Bristol</t>
         </is>
       </c>
       <c r="S187" s="8" t="inlineStr"/>
@@ -14816,7 +14820,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
+          <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
         </is>
       </c>
     </row>
@@ -14830,13 +14834,13 @@
         </is>
       </c>
       <c r="C188" s="9" t="n">
-        <v>1450</v>
+        <v>3200</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F188" s="7" t="inlineStr">
         <is>
@@ -14845,7 +14849,7 @@
       </c>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Bristol</t>
+          <t>Anchorage Gaol, Ferry Steps, Somerset, BS1 6UZ</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
@@ -14859,7 +14863,7 @@
       <c r="L188" s="7" t="n"/>
       <c r="M188" s="7" t="n"/>
       <c r="N188" s="7" t="n">
-        <v>13668</v>
+        <v>16664</v>
       </c>
       <c r="O188" s="7" t="n">
         <v>0</v>
@@ -14867,12 +14871,12 @@
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
         <is>
-          <t>Wildheart Residential Management Limited, Epsom</t>
+          <t>LettingaProperty.com, Nationwide - Lettings</t>
         </is>
       </c>
       <c r="S188" s="8" t="inlineStr"/>
@@ -14889,7 +14893,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
+          <t>9a307d01d086bef2d9dd18f68e1c22a5cd3d5454</t>
         </is>
       </c>
     </row>
@@ -14903,7 +14907,7 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>1605</v>
+        <v>1600</v>
       </c>
       <c r="D189" s="7" t="n">
         <v>1</v>
@@ -14918,7 +14922,7 @@
       </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
@@ -14926,15 +14930,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I189" s="7" t="n">
-        <v>487</v>
-      </c>
+      <c r="I189" s="7" t="n"/>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
       <c r="L189" s="7" t="n"/>
       <c r="M189" s="7" t="n"/>
       <c r="N189" s="7" t="n">
-        <v>13860</v>
+        <v>21996</v>
       </c>
       <c r="O189" s="7" t="n">
         <v>0</v>
@@ -14942,12 +14944,12 @@
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="R189" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S189" s="8" t="inlineStr"/>
@@ -14964,7 +14966,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
+          <t>f276e39e96cb4a8864e19e1c94fa5736432f0af2</t>
         </is>
       </c>
     </row>
@@ -14978,7 +14980,7 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>2185</v>
+        <v>2400</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>2</v>
@@ -14993,7 +14995,7 @@
       </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Colston Avenue, Bristol, BS1</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
@@ -15001,15 +15003,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I190" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I190" s="7" t="n"/>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="7" t="n">
-        <v>13860</v>
+        <v>14108</v>
       </c>
       <c r="O190" s="7" t="n">
         <v>0</v>
@@ -15017,12 +15017,12 @@
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S190" s="8" t="inlineStr"/>
@@ -15039,7 +15039,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
+          <t>df7ab3768c5fab7a5f1c604eb51a3d3dc914128b</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
         </is>
       </c>
       <c r="C191" s="9" t="n">
-        <v>1640</v>
+        <v>1300</v>
       </c>
       <c r="D191" s="7" t="n">
         <v>1</v>
@@ -15068,23 +15068,23 @@
       </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>East Street, Bedminster, BS3</t>
         </is>
       </c>
       <c r="H191" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I191" s="7" t="n">
-        <v>484</v>
+        <v>560</v>
       </c>
       <c r="J191" s="7" t="n"/>
       <c r="K191" s="7" t="n"/>
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
       <c r="N191" s="7" t="n">
-        <v>13860</v>
+        <v>14176</v>
       </c>
       <c r="O191" s="7" t="n">
         <v>0</v>
@@ -15092,12 +15092,12 @@
       <c r="P191" s="7" t="n"/>
       <c r="Q191" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="R191" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Xeno Property, Bristol</t>
         </is>
       </c>
       <c r="S191" s="8" t="inlineStr"/>
@@ -15114,7 +15114,7 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
-          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
+          <t>b526d218fc0af31831d0b254c61f84941a655cb3</t>
         </is>
       </c>
     </row>
@@ -15128,13 +15128,13 @@
         </is>
       </c>
       <c r="C192" s="9" t="n">
-        <v>2010</v>
+        <v>1450</v>
       </c>
       <c r="D192" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E192" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F192" s="7" t="inlineStr">
         <is>
@@ -15143,7 +15143,7 @@
       </c>
       <c r="G192" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Welsh Back, Bristol</t>
         </is>
       </c>
       <c r="H192" s="7" t="inlineStr">
@@ -15151,15 +15151,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I192" s="7" t="n">
-        <v>722</v>
-      </c>
+      <c r="I192" s="7" t="n"/>
       <c r="J192" s="7" t="n"/>
       <c r="K192" s="7" t="n"/>
       <c r="L192" s="7" t="n"/>
       <c r="M192" s="7" t="n"/>
       <c r="N192" s="7" t="n">
-        <v>13860</v>
+        <v>13668</v>
       </c>
       <c r="O192" s="7" t="n">
         <v>0</v>
@@ -15167,12 +15165,12 @@
       <c r="P192" s="7" t="n"/>
       <c r="Q192" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="R192" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Wildheart Residential Management Limited, Epsom</t>
         </is>
       </c>
       <c r="S192" s="8" t="inlineStr"/>
@@ -15189,7 +15187,7 @@
       <c r="V192" s="6" t="inlineStr"/>
       <c r="W192" s="7" t="inlineStr">
         <is>
-          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
+          <t>56c3b85a936dabb2f3efed3e60f35a531f889f74</t>
         </is>
       </c>
     </row>
@@ -15203,7 +15201,7 @@
         </is>
       </c>
       <c r="C193" s="9" t="n">
-        <v>1635</v>
+        <v>1605</v>
       </c>
       <c r="D193" s="7" t="n">
         <v>1</v>
@@ -15218,7 +15216,7 @@
       </c>
       <c r="G193" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H193" s="7" t="inlineStr">
@@ -15227,14 +15225,14 @@
         </is>
       </c>
       <c r="I193" s="7" t="n">
-        <v>560</v>
+        <v>487</v>
       </c>
       <c r="J193" s="7" t="n"/>
       <c r="K193" s="7" t="n"/>
       <c r="L193" s="7" t="n"/>
       <c r="M193" s="7" t="n"/>
       <c r="N193" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O193" s="7" t="n">
         <v>0</v>
@@ -15242,12 +15240,12 @@
       <c r="P193" s="7" t="n"/>
       <c r="Q193" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R193" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S193" s="8" t="inlineStr"/>
@@ -15264,7 +15262,7 @@
       <c r="V193" s="6" t="inlineStr"/>
       <c r="W193" s="7" t="inlineStr">
         <is>
-          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
+          <t>06c878ecc0a558c1e3d410c222e6a75daefc54fc</t>
         </is>
       </c>
     </row>
@@ -15278,13 +15276,13 @@
         </is>
       </c>
       <c r="C194" s="9" t="n">
-        <v>1665</v>
+        <v>2185</v>
       </c>
       <c r="D194" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E194" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F194" s="7" t="inlineStr">
         <is>
@@ -15293,7 +15291,7 @@
       </c>
       <c r="G194" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H194" s="7" t="inlineStr">
@@ -15302,14 +15300,14 @@
         </is>
       </c>
       <c r="I194" s="7" t="n">
-        <v>434</v>
+        <v>721</v>
       </c>
       <c r="J194" s="7" t="n"/>
       <c r="K194" s="7" t="n"/>
       <c r="L194" s="7" t="n"/>
       <c r="M194" s="7" t="n"/>
       <c r="N194" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O194" s="7" t="n">
         <v>0</v>
@@ -15317,12 +15315,12 @@
       <c r="P194" s="7" t="n"/>
       <c r="Q194" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R194" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S194" s="8" t="inlineStr"/>
@@ -15339,7 +15337,7 @@
       <c r="V194" s="6" t="inlineStr"/>
       <c r="W194" s="7" t="inlineStr">
         <is>
-          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
+          <t>02c577529005afd814fcc1ab2e5183817f6527d1</t>
         </is>
       </c>
     </row>
@@ -15353,13 +15351,13 @@
         </is>
       </c>
       <c r="C195" s="9" t="n">
-        <v>1990</v>
+        <v>1640</v>
       </c>
       <c r="D195" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E195" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F195" s="7" t="inlineStr">
         <is>
@@ -15368,7 +15366,7 @@
       </c>
       <c r="G195" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H195" s="7" t="inlineStr">
@@ -15377,27 +15375,27 @@
         </is>
       </c>
       <c r="I195" s="7" t="n">
-        <v>682</v>
+        <v>484</v>
       </c>
       <c r="J195" s="7" t="n"/>
       <c r="K195" s="7" t="n"/>
       <c r="L195" s="7" t="n"/>
       <c r="M195" s="7" t="n"/>
       <c r="N195" s="7" t="n">
-        <v>13964</v>
+        <v>13860</v>
       </c>
       <c r="O195" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P195" s="7" t="n"/>
       <c r="Q195" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R195" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S195" s="8" t="inlineStr"/>
@@ -15414,7 +15412,7 @@
       <c r="V195" s="6" t="inlineStr"/>
       <c r="W195" s="7" t="inlineStr">
         <is>
-          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
+          <t>2e7bf1eca2181a0e6b62530ab26aa17e90afdfaf</t>
         </is>
       </c>
     </row>
@@ -15428,13 +15426,13 @@
         </is>
       </c>
       <c r="C196" s="9" t="n">
-        <v>1480</v>
+        <v>2010</v>
       </c>
       <c r="D196" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E196" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F196" s="7" t="inlineStr">
         <is>
@@ -15443,7 +15441,7 @@
       </c>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H196" s="7" t="inlineStr">
@@ -15452,27 +15450,27 @@
         </is>
       </c>
       <c r="I196" s="7" t="n">
-        <v>417</v>
+        <v>722</v>
       </c>
       <c r="J196" s="7" t="n"/>
       <c r="K196" s="7" t="n"/>
       <c r="L196" s="7" t="n"/>
       <c r="M196" s="7" t="n"/>
       <c r="N196" s="7" t="n">
-        <v>13356</v>
+        <v>13860</v>
       </c>
       <c r="O196" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P196" s="7" t="n"/>
       <c r="Q196" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R196" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S196" s="8" t="inlineStr"/>
@@ -15489,7 +15487,7 @@
       <c r="V196" s="6" t="inlineStr"/>
       <c r="W196" s="7" t="inlineStr">
         <is>
-          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
+          <t>f4a874ba03e08902e44080c4b06dac76fa620312</t>
         </is>
       </c>
     </row>
@@ -15503,13 +15501,13 @@
         </is>
       </c>
       <c r="C197" s="9" t="n">
-        <v>1750</v>
+        <v>1635</v>
       </c>
       <c r="D197" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E197" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F197" s="7" t="inlineStr">
         <is>
@@ -15518,7 +15516,7 @@
       </c>
       <c r="G197" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H197" s="7" t="inlineStr">
@@ -15526,13 +15524,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I197" s="7" t="n"/>
+      <c r="I197" s="7" t="n">
+        <v>560</v>
+      </c>
       <c r="J197" s="7" t="n"/>
       <c r="K197" s="7" t="n"/>
       <c r="L197" s="7" t="n"/>
       <c r="M197" s="7" t="n"/>
       <c r="N197" s="7" t="n">
-        <v>20828</v>
+        <v>13356</v>
       </c>
       <c r="O197" s="7" t="n">
         <v>0</v>
@@ -15540,12 +15540,12 @@
       <c r="P197" s="7" t="n"/>
       <c r="Q197" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R197" s="7" t="inlineStr">
         <is>
-          <t>Abode Property Management, Bristol</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S197" s="8" t="inlineStr"/>
@@ -15562,7 +15562,7 @@
       <c r="V197" s="6" t="inlineStr"/>
       <c r="W197" s="7" t="inlineStr">
         <is>
-          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
+          <t>3edbe2fd3855f2202c71293aa8818bf5f27e9dfb</t>
         </is>
       </c>
     </row>
@@ -15576,13 +15576,13 @@
         </is>
       </c>
       <c r="C198" s="9" t="n">
-        <v>2080</v>
+        <v>1665</v>
       </c>
       <c r="D198" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E198" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F198" s="7" t="inlineStr">
         <is>
@@ -15591,7 +15591,7 @@
       </c>
       <c r="G198" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H198" s="7" t="inlineStr">
@@ -15600,27 +15600,27 @@
         </is>
       </c>
       <c r="I198" s="7" t="n">
-        <v>705</v>
+        <v>434</v>
       </c>
       <c r="J198" s="7" t="n"/>
       <c r="K198" s="7" t="n"/>
       <c r="L198" s="7" t="n"/>
       <c r="M198" s="7" t="n"/>
       <c r="N198" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O198" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P198" s="7" t="n"/>
       <c r="Q198" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R198" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S198" s="8" t="inlineStr"/>
@@ -15637,7 +15637,7 @@
       <c r="V198" s="6" t="inlineStr"/>
       <c r="W198" s="7" t="inlineStr">
         <is>
-          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
+          <t>23bbeac14b986015996b87d2bc4409bbcd03dd21</t>
         </is>
       </c>
     </row>
@@ -15651,13 +15651,13 @@
         </is>
       </c>
       <c r="C199" s="9" t="n">
-        <v>1680</v>
+        <v>1990</v>
       </c>
       <c r="D199" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E199" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F199" s="7" t="inlineStr">
         <is>
@@ -15666,7 +15666,7 @@
       </c>
       <c r="G199" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H199" s="7" t="inlineStr">
@@ -15675,14 +15675,14 @@
         </is>
       </c>
       <c r="I199" s="7" t="n">
-        <v>487</v>
+        <v>682</v>
       </c>
       <c r="J199" s="7" t="n"/>
       <c r="K199" s="7" t="n"/>
       <c r="L199" s="7" t="n"/>
       <c r="M199" s="7" t="n"/>
       <c r="N199" s="7" t="n">
-        <v>13356</v>
+        <v>13964</v>
       </c>
       <c r="O199" s="7" t="n">
         <v>1</v>
@@ -15690,12 +15690,12 @@
       <c r="P199" s="7" t="n"/>
       <c r="Q199" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R199" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S199" s="8" t="inlineStr"/>
@@ -15712,7 +15712,7 @@
       <c r="V199" s="6" t="inlineStr"/>
       <c r="W199" s="7" t="inlineStr">
         <is>
-          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
+          <t>1e33a956a54226127b9170d4f9dc9bdae5d71f2b</t>
         </is>
       </c>
     </row>
@@ -15726,13 +15726,13 @@
         </is>
       </c>
       <c r="C200" s="9" t="n">
-        <v>1845</v>
+        <v>1480</v>
       </c>
       <c r="D200" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E200" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F200" s="7" t="inlineStr">
         <is>
@@ -15741,7 +15741,7 @@
       </c>
       <c r="G200" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H200" s="7" t="inlineStr">
@@ -15750,27 +15750,27 @@
         </is>
       </c>
       <c r="I200" s="7" t="n">
-        <v>641</v>
+        <v>417</v>
       </c>
       <c r="J200" s="7" t="n"/>
       <c r="K200" s="7" t="n"/>
       <c r="L200" s="7" t="n"/>
       <c r="M200" s="7" t="n"/>
       <c r="N200" s="7" t="n">
-        <v>21476</v>
+        <v>13356</v>
       </c>
       <c r="O200" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P200" s="7" t="n"/>
       <c r="Q200" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R200" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S200" s="8" t="inlineStr"/>
@@ -15787,7 +15787,7 @@
       <c r="V200" s="6" t="inlineStr"/>
       <c r="W200" s="7" t="inlineStr">
         <is>
-          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
+          <t>5f50ca74d058f8ccfbe36f2ca51454ee30e84558</t>
         </is>
       </c>
     </row>
@@ -15801,13 +15801,13 @@
         </is>
       </c>
       <c r="C201" s="9" t="n">
-        <v>1685</v>
+        <v>1750</v>
       </c>
       <c r="D201" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E201" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F201" s="7" t="inlineStr">
         <is>
@@ -15816,7 +15816,7 @@
       </c>
       <c r="G201" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Anchorage, Gaol Ferry Steps, Harbourside, Bristol, BS1</t>
         </is>
       </c>
       <c r="H201" s="7" t="inlineStr">
@@ -15824,28 +15824,26 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I201" s="7" t="n">
-        <v>578</v>
-      </c>
+      <c r="I201" s="7" t="n"/>
       <c r="J201" s="7" t="n"/>
       <c r="K201" s="7" t="n"/>
       <c r="L201" s="7" t="n"/>
       <c r="M201" s="7" t="n"/>
       <c r="N201" s="7" t="n">
-        <v>13356</v>
+        <v>20828</v>
       </c>
       <c r="O201" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P201" s="7" t="n"/>
       <c r="Q201" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R201" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Abode Property Management, Bristol</t>
         </is>
       </c>
       <c r="S201" s="8" t="inlineStr"/>
@@ -15862,7 +15860,7 @@
       <c r="V201" s="6" t="inlineStr"/>
       <c r="W201" s="7" t="inlineStr">
         <is>
-          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
+          <t>321eb82323a5ee8dac3345dc3e9d704334b46eb6</t>
         </is>
       </c>
     </row>
@@ -15876,13 +15874,13 @@
         </is>
       </c>
       <c r="C202" s="9" t="n">
-        <v>1765</v>
+        <v>2080</v>
       </c>
       <c r="D202" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E202" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F202" s="7" t="inlineStr">
         <is>
@@ -15900,7 +15898,7 @@
         </is>
       </c>
       <c r="I202" s="7" t="n">
-        <v>641</v>
+        <v>705</v>
       </c>
       <c r="J202" s="7" t="n"/>
       <c r="K202" s="7" t="n"/>
@@ -15915,7 +15913,7 @@
       <c r="P202" s="7" t="n"/>
       <c r="Q202" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R202" s="7" t="inlineStr">
@@ -15937,7 +15935,7 @@
       <c r="V202" s="6" t="inlineStr"/>
       <c r="W202" s="7" t="inlineStr">
         <is>
-          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
+          <t>8e9e150b544061deed77a670ebc8193048c31be8</t>
         </is>
       </c>
     </row>
@@ -15951,13 +15949,13 @@
         </is>
       </c>
       <c r="C203" s="9" t="n">
-        <v>2240</v>
+        <v>1680</v>
       </c>
       <c r="D203" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E203" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F203" s="7" t="inlineStr">
         <is>
@@ -15975,22 +15973,22 @@
         </is>
       </c>
       <c r="I203" s="7" t="n">
-        <v>884</v>
+        <v>487</v>
       </c>
       <c r="J203" s="7" t="n"/>
       <c r="K203" s="7" t="n"/>
       <c r="L203" s="7" t="n"/>
       <c r="M203" s="7" t="n"/>
       <c r="N203" s="7" t="n">
-        <v>13388</v>
+        <v>13356</v>
       </c>
       <c r="O203" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P203" s="7" t="n"/>
       <c r="Q203" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R203" s="7" t="inlineStr">
@@ -16012,7 +16010,7 @@
       <c r="V203" s="6" t="inlineStr"/>
       <c r="W203" s="7" t="inlineStr">
         <is>
-          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
+          <t>9bfa7ba1ffd022b6ee7ac21ebffea804fb1f14d2</t>
         </is>
       </c>
     </row>
@@ -16026,13 +16024,13 @@
         </is>
       </c>
       <c r="C204" s="9" t="n">
-        <v>1150</v>
+        <v>1845</v>
       </c>
       <c r="D204" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E204" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F204" s="7" t="inlineStr">
         <is>
@@ -16041,7 +16039,7 @@
       </c>
       <c r="G204" s="8" t="inlineStr">
         <is>
-          <t>John Street, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H204" s="7" t="inlineStr">
@@ -16050,25 +16048,27 @@
         </is>
       </c>
       <c r="I204" s="7" t="n">
-        <v>248</v>
+        <v>641</v>
       </c>
       <c r="J204" s="7" t="n"/>
       <c r="K204" s="7" t="n"/>
       <c r="L204" s="7" t="n"/>
       <c r="M204" s="7" t="n"/>
-      <c r="N204" s="7" t="n"/>
+      <c r="N204" s="7" t="n">
+        <v>21476</v>
+      </c>
       <c r="O204" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P204" s="7" t="n"/>
       <c r="Q204" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R204" s="7" t="inlineStr">
         <is>
-          <t>Bristol Property Centre, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S204" s="8" t="inlineStr"/>
@@ -16085,14 +16085,312 @@
       <c r="V204" s="6" t="inlineStr"/>
       <c r="W204" s="7" t="inlineStr">
         <is>
+          <t>5f23a97541727a3abb0e11b01c3494b28988b4c8</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B205" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C205" s="9" t="n">
+        <v>1685</v>
+      </c>
+      <c r="D205" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E205" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F205" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G205" s="8" t="inlineStr">
+        <is>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
+        </is>
+      </c>
+      <c r="H205" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I205" s="7" t="n">
+        <v>578</v>
+      </c>
+      <c r="J205" s="7" t="n"/>
+      <c r="K205" s="7" t="n"/>
+      <c r="L205" s="7" t="n"/>
+      <c r="M205" s="7" t="n"/>
+      <c r="N205" s="7" t="n">
+        <v>13356</v>
+      </c>
+      <c r="O205" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P205" s="7" t="n"/>
+      <c r="Q205" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R205" s="7" t="inlineStr">
+        <is>
+          <t>Grainger, Glasshouse Square</t>
+        </is>
+      </c>
+      <c r="S205" s="8" t="inlineStr"/>
+      <c r="T205" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V205" s="6" t="inlineStr"/>
+      <c r="W205" s="7" t="inlineStr">
+        <is>
+          <t>29a2267eb063b1d16ef2b902aa3a5e4c2001b9d6</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B206" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C206" s="9" t="n">
+        <v>1765</v>
+      </c>
+      <c r="D206" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E206" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F206" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G206" s="8" t="inlineStr">
+        <is>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
+        </is>
+      </c>
+      <c r="H206" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I206" s="7" t="n">
+        <v>641</v>
+      </c>
+      <c r="J206" s="7" t="n"/>
+      <c r="K206" s="7" t="n"/>
+      <c r="L206" s="7" t="n"/>
+      <c r="M206" s="7" t="n"/>
+      <c r="N206" s="7" t="n">
+        <v>13356</v>
+      </c>
+      <c r="O206" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P206" s="7" t="n"/>
+      <c r="Q206" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="R206" s="7" t="inlineStr">
+        <is>
+          <t>Grainger, Glasshouse Square</t>
+        </is>
+      </c>
+      <c r="S206" s="8" t="inlineStr"/>
+      <c r="T206" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V206" s="6" t="inlineStr"/>
+      <c r="W206" s="7" t="inlineStr">
+        <is>
+          <t>4628ab90345cbce8fdec89e9fef92e37b1ed2f77</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B207" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C207" s="9" t="n">
+        <v>2240</v>
+      </c>
+      <c r="D207" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E207" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F207" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G207" s="8" t="inlineStr">
+        <is>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
+        </is>
+      </c>
+      <c r="H207" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I207" s="7" t="n">
+        <v>884</v>
+      </c>
+      <c r="J207" s="7" t="n"/>
+      <c r="K207" s="7" t="n"/>
+      <c r="L207" s="7" t="n"/>
+      <c r="M207" s="7" t="n"/>
+      <c r="N207" s="7" t="n">
+        <v>13388</v>
+      </c>
+      <c r="O207" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P207" s="7" t="n"/>
+      <c r="Q207" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="R207" s="7" t="inlineStr">
+        <is>
+          <t>Grainger, Glasshouse Square</t>
+        </is>
+      </c>
+      <c r="S207" s="8" t="inlineStr"/>
+      <c r="T207" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V207" s="6" t="inlineStr"/>
+      <c r="W207" s="7" t="inlineStr">
+        <is>
+          <t>21df863778ecb1f94df8dba393d9ccaa180a560d</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B208" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C208" s="9" t="n">
+        <v>1150</v>
+      </c>
+      <c r="D208" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E208" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F208" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G208" s="8" t="inlineStr">
+        <is>
+          <t>John Street, BS1</t>
+        </is>
+      </c>
+      <c r="H208" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I208" s="7" t="n">
+        <v>248</v>
+      </c>
+      <c r="J208" s="7" t="n"/>
+      <c r="K208" s="7" t="n"/>
+      <c r="L208" s="7" t="n"/>
+      <c r="M208" s="7" t="n"/>
+      <c r="N208" s="7" t="n"/>
+      <c r="O208" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P208" s="7" t="n"/>
+      <c r="Q208" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="R208" s="7" t="inlineStr">
+        <is>
+          <t>Bristol Property Centre, Bristol</t>
+        </is>
+      </c>
+      <c r="S208" s="8" t="inlineStr"/>
+      <c r="T208" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V208" s="6" t="inlineStr"/>
+      <c r="W208" s="7" t="inlineStr">
+        <is>
           <t>08b26f667fbc84f6b5abfe87a96caaf90fa4070b</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W204"/>
+  <autoFilter ref="A1:W208"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204 U205 U206 U207 U208" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16300,6 +16598,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T202" r:id="rId201"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T203" r:id="rId202"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T208" r:id="rId207"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 176
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$194</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W191"/>
+  <dimension ref="A1:W194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8188,7 +8188,7 @@
         <v>17004</v>
       </c>
       <c r="O98" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P98" s="7" t="n"/>
       <c r="Q98" s="7" t="inlineStr">
@@ -8825,7 +8825,7 @@
         </is>
       </c>
       <c r="C107" s="9" t="n">
-        <v>1600</v>
+        <v>1550</v>
       </c>
       <c r="D107" s="7" t="n">
         <v>1</v>
@@ -10601,7 +10601,7 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="D131" s="7" t="n">
         <v>2</v>
@@ -10824,13 +10824,13 @@
         </is>
       </c>
       <c r="C134" s="9" t="n">
-        <v>1300</v>
+        <v>2040</v>
       </c>
       <c r="D134" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E134" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
@@ -10839,23 +10839,23 @@
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t>Chimney Steps, Bristol, BS2</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H134" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I134" s="7" t="n">
-        <v>452</v>
+        <v>873</v>
       </c>
       <c r="J134" s="7" t="n"/>
       <c r="K134" s="7" t="n"/>
       <c r="L134" s="7" t="n"/>
       <c r="M134" s="7" t="n"/>
       <c r="N134" s="7" t="n">
-        <v>19996</v>
+        <v>21740</v>
       </c>
       <c r="O134" s="7" t="n">
         <v>0</v>
@@ -10863,12 +10863,12 @@
       <c r="P134" s="7" t="n"/>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S134" s="8" t="inlineStr"/>
@@ -10885,7 +10885,7 @@
       <c r="V134" s="6" t="inlineStr"/>
       <c r="W134" s="7" t="inlineStr">
         <is>
-          <t>b0804dcb3dae15dea73fb6b7320023ee0cc5e93a</t>
+          <t>71c0c04e367fed20ae4d5f7b68c6919d921a50a1</t>
         </is>
       </c>
     </row>
@@ -10899,7 +10899,7 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1400</v>
+        <v>1485</v>
       </c>
       <c r="D135" s="7" t="n">
         <v>1</v>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Taylors Bank, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
@@ -10922,13 +10922,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I135" s="7" t="n"/>
+      <c r="I135" s="7" t="n">
+        <v>470</v>
+      </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="7" t="n">
-        <v>21996</v>
+        <v>21740</v>
       </c>
       <c r="O135" s="7" t="n">
         <v>0</v>
@@ -10936,12 +10938,12 @@
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S135" s="8" t="inlineStr"/>
@@ -10958,7 +10960,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>464a8221babcd58554ee30417192b0a25eacccb0</t>
+          <t>6a8e5c401e5404f7710ff0be94ae72acde00ee84</t>
         </is>
       </c>
     </row>
@@ -10972,7 +10974,7 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>1400</v>
+        <v>1350</v>
       </c>
       <c r="D136" s="7" t="n">
         <v>1</v>
@@ -10987,36 +10989,34 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The General, BS1</t>
+          <t>Wilder House, Wilder Street, St Pauls, Bristol, BS2</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I136" s="7" t="n">
-        <v>604</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I136" s="7" t="n"/>
       <c r="J136" s="7" t="n"/>
       <c r="K136" s="7" t="n"/>
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>19076</v>
+        <v>22132</v>
       </c>
       <c r="O136" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>CJ Hole, Southville</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11033,7 +11033,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>adaa31d271a8abff25dafaf34aa54eb1f22dd072</t>
+          <t>b2d9778ecb79a49e6e9293b16d6e5677835f9ce6</t>
         </is>
       </c>
     </row>
@@ -11047,13 +11047,13 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>2400</v>
+        <v>1300</v>
       </c>
       <c r="D137" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E137" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
@@ -11062,7 +11062,7 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>Chimney Steps, Bristol, BS2</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
@@ -11070,13 +11070,15 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I137" s="7" t="n"/>
+      <c r="I137" s="7" t="n">
+        <v>452</v>
+      </c>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="7" t="n">
-        <v>21360</v>
+        <v>19996</v>
       </c>
       <c r="O137" s="7" t="n">
         <v>0</v>
@@ -11084,12 +11086,12 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S137" s="8" t="inlineStr"/>
@@ -11106,7 +11108,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>0b6e19cc97b73c7e581c5f306902c64d0c59b226</t>
+          <t>b0804dcb3dae15dea73fb6b7320023ee0cc5e93a</t>
         </is>
       </c>
     </row>
@@ -11120,7 +11122,7 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1600</v>
+        <v>1400</v>
       </c>
       <c r="D138" s="7" t="n">
         <v>1</v>
@@ -11135,7 +11137,7 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Taylors Bank, Bristol, BS1</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
@@ -11157,12 +11159,12 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11179,7 +11181,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
+          <t>464a8221babcd58554ee30417192b0a25eacccb0</t>
         </is>
       </c>
     </row>
@@ -11193,7 +11195,7 @@
         </is>
       </c>
       <c r="C139" s="9" t="n">
-        <v>1560</v>
+        <v>1400</v>
       </c>
       <c r="D139" s="7" t="n">
         <v>1</v>
@@ -11208,7 +11210,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>City Centre, The General, BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11217,14 +11219,14 @@
         </is>
       </c>
       <c r="I139" s="7" t="n">
-        <v>472</v>
+        <v>604</v>
       </c>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>20984</v>
+        <v>19076</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11232,12 +11234,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11254,7 +11256,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
+          <t>adaa31d271a8abff25dafaf34aa54eb1f22dd072</t>
         </is>
       </c>
     </row>
@@ -11268,13 +11270,13 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>1660</v>
+        <v>2400</v>
       </c>
       <c r="D140" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E140" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
@@ -11283,23 +11285,21 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I140" s="7" t="n">
-        <v>558</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I140" s="7" t="n"/>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>20984</v>
+        <v>21360</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11307,12 +11307,12 @@
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11329,7 +11329,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
+          <t>0b6e19cc97b73c7e581c5f306902c64d0c59b226</t>
         </is>
       </c>
     </row>
@@ -11343,13 +11343,13 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1860</v>
+        <v>1600</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E141" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
@@ -11358,7 +11358,7 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
@@ -11366,15 +11366,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I141" s="7" t="n">
-        <v>647</v>
-      </c>
+      <c r="I141" s="7" t="n"/>
       <c r="J141" s="7" t="n"/>
       <c r="K141" s="7" t="n"/>
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>21740</v>
+        <v>21996</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11382,12 +11380,12 @@
       <c r="P141" s="7" t="n"/>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11404,7 +11402,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
+          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
         </is>
       </c>
     </row>
@@ -11418,7 +11416,7 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>1600</v>
+        <v>1560</v>
       </c>
       <c r="D142" s="7" t="n">
         <v>1</v>
@@ -11433,7 +11431,7 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
@@ -11442,14 +11440,14 @@
         </is>
       </c>
       <c r="I142" s="7" t="n">
-        <v>549</v>
+        <v>472</v>
       </c>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>21816</v>
+        <v>20984</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11457,12 +11455,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11479,7 +11477,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
+          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
         </is>
       </c>
     </row>
@@ -11493,13 +11491,13 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1900</v>
+        <v>1660</v>
       </c>
       <c r="D143" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E143" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
@@ -11508,7 +11506,7 @@
       </c>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H143" s="7" t="inlineStr">
@@ -11517,14 +11515,14 @@
         </is>
       </c>
       <c r="I143" s="7" t="n">
-        <v>624</v>
+        <v>558</v>
       </c>
       <c r="J143" s="7" t="n"/>
       <c r="K143" s="7" t="n"/>
       <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="n"/>
       <c r="N143" s="7" t="n">
-        <v>21740</v>
+        <v>20984</v>
       </c>
       <c r="O143" s="7" t="n">
         <v>0</v>
@@ -11532,12 +11530,12 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S143" s="8" t="inlineStr"/>
@@ -11554,7 +11552,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
+          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
         </is>
       </c>
     </row>
@@ -11568,13 +11566,13 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1530</v>
+        <v>1860</v>
       </c>
       <c r="D144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E144" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
@@ -11592,7 +11590,7 @@
         </is>
       </c>
       <c r="I144" s="7" t="n">
-        <v>548</v>
+        <v>647</v>
       </c>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
@@ -11607,7 +11605,7 @@
       <c r="P144" s="7" t="n"/>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
@@ -11629,7 +11627,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
+          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
         </is>
       </c>
     </row>
@@ -11643,13 +11641,13 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>2110</v>
+        <v>1600</v>
       </c>
       <c r="D145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E145" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
@@ -11667,14 +11665,14 @@
         </is>
       </c>
       <c r="I145" s="7" t="n">
-        <v>624</v>
+        <v>549</v>
       </c>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>21740</v>
+        <v>21816</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11682,7 +11680,7 @@
       <c r="P145" s="7" t="n"/>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
@@ -11704,7 +11702,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
+          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
         </is>
       </c>
     </row>
@@ -11718,13 +11716,13 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>1530</v>
+        <v>1900</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E146" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
@@ -11742,7 +11740,7 @@
         </is>
       </c>
       <c r="I146" s="7" t="n">
-        <v>544</v>
+        <v>624</v>
       </c>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
@@ -11757,7 +11755,7 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
@@ -11779,7 +11777,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
+          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
         </is>
       </c>
     </row>
@@ -11793,13 +11791,13 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>1600</v>
+        <v>1530</v>
       </c>
       <c r="D147" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E147" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F147" s="7" t="inlineStr">
         <is>
@@ -11808,7 +11806,7 @@
       </c>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H147" s="7" t="inlineStr">
@@ -11816,13 +11814,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I147" s="7" t="n"/>
+      <c r="I147" s="7" t="n">
+        <v>548</v>
+      </c>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
       <c r="L147" s="7" t="n"/>
       <c r="M147" s="7" t="n"/>
       <c r="N147" s="7" t="n">
-        <v>20880</v>
+        <v>21740</v>
       </c>
       <c r="O147" s="7" t="n">
         <v>0</v>
@@ -11830,12 +11830,12 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S147" s="8" t="inlineStr"/>
@@ -11852,7 +11852,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
+          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
         </is>
       </c>
     </row>
@@ -11866,7 +11866,7 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>1800</v>
+        <v>2110</v>
       </c>
       <c r="D148" s="7" t="n">
         <v>2</v>
@@ -11881,7 +11881,7 @@
       </c>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H148" s="7" t="inlineStr">
@@ -11890,14 +11890,14 @@
         </is>
       </c>
       <c r="I148" s="7" t="n">
-        <v>980</v>
+        <v>624</v>
       </c>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
       <c r="L148" s="7" t="n"/>
       <c r="M148" s="7" t="n"/>
       <c r="N148" s="7" t="n">
-        <v>21316</v>
+        <v>21740</v>
       </c>
       <c r="O148" s="7" t="n">
         <v>0</v>
@@ -11905,12 +11905,12 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S148" s="8" t="inlineStr"/>
@@ -11927,7 +11927,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
+          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
         </is>
       </c>
     </row>
@@ -11941,7 +11941,7 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>1995</v>
+        <v>1530</v>
       </c>
       <c r="D149" s="7" t="n">
         <v>1</v>
@@ -11956,7 +11956,7 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H149" s="7" t="inlineStr">
@@ -11964,13 +11964,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I149" s="7" t="n"/>
+      <c r="I149" s="7" t="n">
+        <v>544</v>
+      </c>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
       <c r="L149" s="7" t="n"/>
       <c r="M149" s="7" t="n"/>
       <c r="N149" s="7" t="n">
-        <v>21196</v>
+        <v>21740</v>
       </c>
       <c r="O149" s="7" t="n">
         <v>0</v>
@@ -11978,12 +11980,12 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S149" s="8" t="inlineStr"/>
@@ -12000,7 +12002,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
+          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
         </is>
       </c>
     </row>
@@ -12014,7 +12016,7 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1750</v>
+        <v>1600</v>
       </c>
       <c r="D150" s="7" t="n">
         <v>2</v>
@@ -12029,7 +12031,7 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
@@ -12037,15 +12039,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I150" s="7" t="n">
-        <v>849</v>
-      </c>
+      <c r="I150" s="7" t="n"/>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>21028</v>
+        <v>20880</v>
       </c>
       <c r="O150" s="7" t="n">
         <v>0</v>
@@ -12053,12 +12053,12 @@
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12075,7 +12075,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
+          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
         </is>
       </c>
     </row>
@@ -12089,7 +12089,7 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1550</v>
+        <v>1800</v>
       </c>
       <c r="D151" s="7" t="n">
         <v>2</v>
@@ -12104,21 +12104,23 @@
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t>Portland Heights - St. Pauls</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H151" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I151" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I151" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>21420</v>
+        <v>21316</v>
       </c>
       <c r="O151" s="7" t="n">
         <v>0</v>
@@ -12126,12 +12128,12 @@
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Bishopston</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12148,7 +12150,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
+          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
         </is>
       </c>
     </row>
@@ -12162,7 +12164,7 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1400</v>
+        <v>1995</v>
       </c>
       <c r="D152" s="7" t="n">
         <v>1</v>
@@ -12177,7 +12179,7 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>The Atrium, Redcliffe Street, BS1</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
@@ -12191,7 +12193,7 @@
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>20292</v>
+        <v>21196</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12199,12 +12201,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12221,7 +12223,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
+          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
         </is>
       </c>
     </row>
@@ -12235,13 +12237,13 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>1150</v>
+        <v>1750</v>
       </c>
       <c r="D153" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E153" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
@@ -12250,21 +12252,23 @@
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
+          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I153" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I153" s="7" t="n">
+        <v>849</v>
+      </c>
       <c r="J153" s="7" t="n"/>
       <c r="K153" s="7" t="n"/>
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>15376</v>
+        <v>21028</v>
       </c>
       <c r="O153" s="7" t="n">
         <v>0</v>
@@ -12272,12 +12276,12 @@
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12294,7 +12298,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
+          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
         </is>
       </c>
     </row>
@@ -12308,13 +12312,13 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1300</v>
+        <v>1550</v>
       </c>
       <c r="D154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E154" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
@@ -12323,23 +12327,21 @@
       </c>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The Milliners, BS1 6WU</t>
+          <t>Portland Heights - St. Pauls</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I154" s="7" t="n">
-        <v>463</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I154" s="7" t="n"/>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="7" t="n">
-        <v>21440</v>
+        <v>21420</v>
       </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
@@ -12347,12 +12349,12 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Ocean, Bishopston</t>
         </is>
       </c>
       <c r="S154" s="8" t="inlineStr"/>
@@ -12369,7 +12371,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
+          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
         </is>
       </c>
     </row>
@@ -12383,7 +12385,7 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>1150</v>
+        <v>1400</v>
       </c>
       <c r="D155" s="7" t="n">
         <v>1</v>
@@ -12398,23 +12400,21 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Century Place, St. Paul Street, BS2 8AN</t>
+          <t>The Atrium, Redcliffe Street, BS1</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I155" s="7" t="n">
-        <v>344</v>
-      </c>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I155" s="7" t="n"/>
       <c r="J155" s="7" t="n"/>
       <c r="K155" s="7" t="n"/>
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="7" t="n">
-        <v>21792</v>
+        <v>20292</v>
       </c>
       <c r="O155" s="7" t="n">
         <v>0</v>
@@ -12422,12 +12422,12 @@
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12444,7 +12444,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
+          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
         </is>
       </c>
     </row>
@@ -12458,13 +12458,13 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>1800</v>
+        <v>1150</v>
       </c>
       <c r="D156" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E156" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F156" s="7" t="inlineStr">
         <is>
@@ -12473,12 +12473,12 @@
       </c>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>Waverley House, BS1</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS3</t>
         </is>
       </c>
       <c r="I156" s="7" t="n"/>
@@ -12487,7 +12487,7 @@
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="7" t="n">
-        <v>17956</v>
+        <v>15376</v>
       </c>
       <c r="O156" s="7" t="n">
         <v>0</v>
@@ -12495,12 +12495,12 @@
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S156" s="8" t="inlineStr"/>
@@ -12517,7 +12517,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
+          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
         </is>
       </c>
     </row>
@@ -12531,13 +12531,13 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>2170</v>
+        <v>1300</v>
       </c>
       <c r="D157" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E157" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
@@ -12546,7 +12546,7 @@
       </c>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>City Centre, The Milliners, BS1 6WU</t>
         </is>
       </c>
       <c r="H157" s="7" t="inlineStr">
@@ -12555,14 +12555,14 @@
         </is>
       </c>
       <c r="I157" s="7" t="n">
-        <v>721</v>
+        <v>463</v>
       </c>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="7" t="n">
-        <v>21732</v>
+        <v>21440</v>
       </c>
       <c r="O157" s="7" t="n">
         <v>0</v>
@@ -12570,12 +12570,12 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S157" s="8" t="inlineStr"/>
@@ -12592,7 +12592,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
+          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
         </is>
       </c>
     </row>
@@ -12606,13 +12606,13 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>1965</v>
+        <v>1150</v>
       </c>
       <c r="D158" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E158" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F158" s="7" t="inlineStr">
         <is>
@@ -12621,23 +12621,23 @@
       </c>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Century Place, St. Paul Street, BS2 8AN</t>
         </is>
       </c>
       <c r="H158" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I158" s="7" t="n">
-        <v>771</v>
+        <v>344</v>
       </c>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>21740</v>
+        <v>21792</v>
       </c>
       <c r="O158" s="7" t="n">
         <v>0</v>
@@ -12645,12 +12645,12 @@
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S158" s="8" t="inlineStr"/>
@@ -12667,7 +12667,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
+          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
         </is>
       </c>
     </row>
@@ -12681,13 +12681,13 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1680</v>
+        <v>1800</v>
       </c>
       <c r="D159" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E159" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F159" s="7" t="inlineStr">
         <is>
@@ -12696,7 +12696,7 @@
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Waverley House, BS1</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
@@ -12710,7 +12710,7 @@
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="7" t="n">
-        <v>20628</v>
+        <v>17956</v>
       </c>
       <c r="O159" s="7" t="n">
         <v>0</v>
@@ -12718,12 +12718,12 @@
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12740,7 +12740,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
+          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
         </is>
       </c>
     </row>
@@ -12754,13 +12754,13 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>1625</v>
+        <v>2170</v>
       </c>
       <c r="D160" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E160" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F160" s="7" t="inlineStr">
         <is>
@@ -12778,7 +12778,7 @@
         </is>
       </c>
       <c r="I160" s="7" t="n">
-        <v>486</v>
+        <v>721</v>
       </c>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
@@ -12793,7 +12793,7 @@
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
@@ -12815,7 +12815,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
+          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
         </is>
       </c>
     </row>
@@ -12829,7 +12829,7 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>1940</v>
+        <v>1965</v>
       </c>
       <c r="D161" s="7" t="n">
         <v>2</v>
@@ -12853,7 +12853,7 @@
         </is>
       </c>
       <c r="I161" s="7" t="n">
-        <v>607</v>
+        <v>771</v>
       </c>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
@@ -12868,7 +12868,7 @@
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
@@ -12890,7 +12890,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
+          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
         </is>
       </c>
     </row>
@@ -12904,10 +12904,10 @@
         </is>
       </c>
       <c r="C162" s="9" t="n">
-        <v>1465</v>
+        <v>1680</v>
       </c>
       <c r="D162" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E162" s="7" t="n">
         <v>1</v>
@@ -12919,7 +12919,7 @@
       </c>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
@@ -12927,15 +12927,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I162" s="7" t="n">
-        <v>505</v>
-      </c>
+      <c r="I162" s="7" t="n"/>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
       <c r="N162" s="7" t="n">
-        <v>21816</v>
+        <v>20628</v>
       </c>
       <c r="O162" s="7" t="n">
         <v>0</v>
@@ -12948,7 +12946,7 @@
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S162" s="8" t="inlineStr"/>
@@ -12965,7 +12963,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>e86143466441bbbf802706245b19ef679ec29055</t>
+          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
         </is>
       </c>
     </row>
@@ -12979,7 +12977,7 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1150</v>
+        <v>1625</v>
       </c>
       <c r="D163" s="7" t="n">
         <v>1</v>
@@ -12994,21 +12992,23 @@
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>St. Philips, Bristol, BS2</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I163" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I163" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="7" t="n">
-        <v>20784</v>
+        <v>21732</v>
       </c>
       <c r="O163" s="7" t="n">
         <v>0</v>
@@ -13016,12 +13016,12 @@
       <c r="P163" s="7" t="n"/>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13038,7 +13038,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
+          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
         </is>
       </c>
     </row>
@@ -13052,13 +13052,13 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>1685</v>
+        <v>1940</v>
       </c>
       <c r="D164" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E164" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F164" s="7" t="inlineStr">
         <is>
@@ -13067,7 +13067,7 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
@@ -13076,14 +13076,14 @@
         </is>
       </c>
       <c r="I164" s="7" t="n">
-        <v>545</v>
+        <v>607</v>
       </c>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="7" t="n">
-        <v>21024</v>
+        <v>21740</v>
       </c>
       <c r="O164" s="7" t="n">
         <v>0</v>
@@ -13091,12 +13091,12 @@
       <c r="P164" s="7" t="n"/>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13113,7 +13113,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
+          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
         </is>
       </c>
     </row>
@@ -13127,36 +13127,38 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1700</v>
+        <v>1465</v>
       </c>
       <c r="D165" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E165" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F165" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Dunkerry Road - Windmill Hill</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H165" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I165" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I165" s="7" t="n">
+        <v>505</v>
+      </c>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>8448</v>
+        <v>21816</v>
       </c>
       <c r="O165" s="7" t="n">
         <v>0</v>
@@ -13164,12 +13166,12 @@
       <c r="P165" s="7" t="n"/>
       <c r="Q165" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R165" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S165" s="8" t="inlineStr"/>
@@ -13186,7 +13188,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
+          <t>e86143466441bbbf802706245b19ef679ec29055</t>
         </is>
       </c>
     </row>
@@ -13200,7 +13202,7 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>1460</v>
+        <v>1150</v>
       </c>
       <c r="D166" s="7" t="n">
         <v>1</v>
@@ -13215,23 +13217,21 @@
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>St. Philips, Bristol, BS2</t>
         </is>
       </c>
       <c r="H166" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I166" s="7" t="n">
-        <v>473</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I166" s="7" t="n"/>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="7" t="n">
-        <v>13840</v>
+        <v>20784</v>
       </c>
       <c r="O166" s="7" t="n">
         <v>0</v>
@@ -13239,12 +13239,12 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
@@ -13261,7 +13261,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
+          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
         </is>
       </c>
     </row>
@@ -13275,7 +13275,7 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>1630</v>
+        <v>1685</v>
       </c>
       <c r="D167" s="7" t="n">
         <v>1</v>
@@ -13290,7 +13290,7 @@
       </c>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H167" s="7" t="inlineStr">
@@ -13299,27 +13299,27 @@
         </is>
       </c>
       <c r="I167" s="7" t="n">
-        <v>486</v>
+        <v>545</v>
       </c>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="7" t="n">
-        <v>13860</v>
+        <v>21024</v>
       </c>
       <c r="O167" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S167" s="8" t="inlineStr"/>
@@ -13336,7 +13336,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
+          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
         </is>
       </c>
     </row>
@@ -13350,38 +13350,36 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1625</v>
+        <v>1700</v>
       </c>
       <c r="D168" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E168" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F168" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Dunkerry Road - Windmill Hill</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I168" s="7" t="n">
-        <v>486</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I168" s="7" t="n"/>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="7" t="n">
-        <v>21732</v>
+        <v>8448</v>
       </c>
       <c r="O168" s="7" t="n">
         <v>0</v>
@@ -13389,12 +13387,12 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13411,7 +13409,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
+          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
         </is>
       </c>
     </row>
@@ -13425,13 +13423,13 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1650</v>
+        <v>1460</v>
       </c>
       <c r="D169" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E169" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
@@ -13440,7 +13438,7 @@
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Harris Lofts, BS1 4BB</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
@@ -13449,14 +13447,14 @@
         </is>
       </c>
       <c r="I169" s="7" t="n">
-        <v>667</v>
+        <v>473</v>
       </c>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>20088</v>
+        <v>13840</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13464,12 +13462,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13486,7 +13484,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
+          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
         </is>
       </c>
     </row>
@@ -13500,7 +13498,7 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>1650</v>
+        <v>1630</v>
       </c>
       <c r="D170" s="7" t="n">
         <v>1</v>
@@ -13515,7 +13513,7 @@
       </c>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t>Central Quey North, Broad Quay, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H170" s="7" t="inlineStr">
@@ -13523,26 +13521,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I170" s="7" t="n"/>
+      <c r="I170" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
       <c r="L170" s="7" t="n"/>
       <c r="M170" s="7" t="n"/>
       <c r="N170" s="7" t="n">
-        <v>20768</v>
+        <v>13860</v>
       </c>
       <c r="O170" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -13559,7 +13559,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
+          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
         </is>
       </c>
     </row>
@@ -13573,7 +13573,7 @@
         </is>
       </c>
       <c r="C171" s="9" t="n">
-        <v>1550</v>
+        <v>1625</v>
       </c>
       <c r="D171" s="7" t="n">
         <v>1</v>
@@ -13588,7 +13588,7 @@
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H171" s="7" t="inlineStr">
@@ -13596,13 +13596,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I171" s="7" t="n"/>
+      <c r="I171" s="7" t="n">
+        <v>486</v>
+      </c>
       <c r="J171" s="7" t="n"/>
       <c r="K171" s="7" t="n"/>
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="7" t="n">
-        <v>21100</v>
+        <v>21732</v>
       </c>
       <c r="O171" s="7" t="n">
         <v>0</v>
@@ -13610,12 +13612,12 @@
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S171" s="8" t="inlineStr"/>
@@ -13632,7 +13634,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
+          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
         </is>
       </c>
     </row>
@@ -13646,13 +13648,13 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1390</v>
+        <v>1650</v>
       </c>
       <c r="D172" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E172" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F172" s="7" t="inlineStr">
         <is>
@@ -13661,7 +13663,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Harbourside, Harris Lofts, BS1 4BB</t>
         </is>
       </c>
       <c r="H172" s="7" t="inlineStr">
@@ -13669,24 +13671,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I172" s="7" t="n"/>
+      <c r="I172" s="7" t="n">
+        <v>667</v>
+      </c>
       <c r="J172" s="7" t="n"/>
       <c r="K172" s="7" t="n"/>
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
-      <c r="N172" s="7" t="n"/>
+      <c r="N172" s="7" t="n">
+        <v>20088</v>
+      </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -13703,7 +13709,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
+          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
         </is>
       </c>
     </row>
@@ -13717,7 +13723,7 @@
         </is>
       </c>
       <c r="C173" s="9" t="n">
-        <v>1485</v>
+        <v>1650</v>
       </c>
       <c r="D173" s="7" t="n">
         <v>1</v>
@@ -13732,7 +13738,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Central Quey North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
@@ -13740,15 +13746,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I173" s="7" t="n">
-        <v>470</v>
-      </c>
+      <c r="I173" s="7" t="n"/>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>21740</v>
+        <v>20768</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13756,12 +13760,12 @@
       <c r="P173" s="7" t="n"/>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -13778,7 +13782,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
+          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
         </is>
       </c>
     </row>
@@ -13792,7 +13796,7 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1635</v>
+        <v>1550</v>
       </c>
       <c r="D174" s="7" t="n">
         <v>1</v>
@@ -13807,7 +13811,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
@@ -13815,15 +13819,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I174" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I174" s="7" t="n"/>
       <c r="J174" s="7" t="n"/>
       <c r="K174" s="7" t="n"/>
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>21732</v>
+        <v>21100</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13831,12 +13833,12 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S174" s="8" t="inlineStr"/>
@@ -13853,7 +13855,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
+          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
         </is>
       </c>
     </row>
@@ -13867,13 +13869,13 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>2060</v>
+        <v>1390</v>
       </c>
       <c r="D175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E175" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
@@ -13882,7 +13884,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
@@ -13890,28 +13892,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I175" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I175" s="7" t="n"/>
       <c r="J175" s="7" t="n"/>
       <c r="K175" s="7" t="n"/>
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
-      <c r="N175" s="7" t="n">
-        <v>21732</v>
-      </c>
+      <c r="N175" s="7" t="n"/>
       <c r="O175" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -13928,7 +13926,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
+          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
         </is>
       </c>
     </row>
@@ -13942,7 +13940,7 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>1545</v>
+        <v>1485</v>
       </c>
       <c r="D176" s="7" t="n">
         <v>1</v>
@@ -13966,7 +13964,7 @@
         </is>
       </c>
       <c r="I176" s="7" t="n">
-        <v>548</v>
+        <v>470</v>
       </c>
       <c r="J176" s="7" t="n"/>
       <c r="K176" s="7" t="n"/>
@@ -13981,7 +13979,7 @@
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
@@ -14003,7 +14001,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
+          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
         </is>
       </c>
     </row>
@@ -14017,7 +14015,7 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>1640</v>
+        <v>1635</v>
       </c>
       <c r="D177" s="7" t="n">
         <v>1</v>
@@ -14056,7 +14054,7 @@
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
@@ -14078,7 +14076,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
+          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
         </is>
       </c>
     </row>
@@ -14092,13 +14090,13 @@
         </is>
       </c>
       <c r="C178" s="9" t="n">
-        <v>2115</v>
+        <v>2060</v>
       </c>
       <c r="D178" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E178" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F178" s="7" t="inlineStr">
         <is>
@@ -14116,7 +14114,7 @@
         </is>
       </c>
       <c r="I178" s="7" t="n">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
@@ -14131,7 +14129,7 @@
       <c r="P178" s="7" t="n"/>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
@@ -14153,7 +14151,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
+          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
         </is>
       </c>
     </row>
@@ -14167,13 +14165,13 @@
         </is>
       </c>
       <c r="C179" s="9" t="n">
-        <v>1970</v>
+        <v>1545</v>
       </c>
       <c r="D179" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E179" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
@@ -14191,7 +14189,7 @@
         </is>
       </c>
       <c r="I179" s="7" t="n">
-        <v>750</v>
+        <v>548</v>
       </c>
       <c r="J179" s="7" t="n"/>
       <c r="K179" s="7" t="n"/>
@@ -14206,7 +14204,7 @@
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
@@ -14228,7 +14226,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
+          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
         </is>
       </c>
     </row>
@@ -14242,7 +14240,7 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>1575</v>
+        <v>1640</v>
       </c>
       <c r="D180" s="7" t="n">
         <v>1</v>
@@ -14257,7 +14255,7 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
@@ -14266,14 +14264,14 @@
         </is>
       </c>
       <c r="I180" s="7" t="n">
-        <v>430</v>
+        <v>486</v>
       </c>
       <c r="J180" s="7" t="n"/>
       <c r="K180" s="7" t="n"/>
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="7" t="n">
-        <v>21816</v>
+        <v>21732</v>
       </c>
       <c r="O180" s="7" t="n">
         <v>0</v>
@@ -14281,12 +14279,12 @@
       <c r="P180" s="7" t="n"/>
       <c r="Q180" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14303,7 +14301,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
+          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
         </is>
       </c>
     </row>
@@ -14317,10 +14315,10 @@
         </is>
       </c>
       <c r="C181" s="9" t="n">
-        <v>1350</v>
+        <v>2115</v>
       </c>
       <c r="D181" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E181" s="7" t="n">
         <v>1</v>
@@ -14332,7 +14330,7 @@
       </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t>Invicta, Millenium Promenade, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H181" s="7" t="inlineStr">
@@ -14340,13 +14338,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I181" s="7" t="n"/>
+      <c r="I181" s="7" t="n">
+        <v>722</v>
+      </c>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
       <c r="L181" s="7" t="n"/>
       <c r="M181" s="7" t="n"/>
       <c r="N181" s="7" t="n">
-        <v>17344</v>
+        <v>21732</v>
       </c>
       <c r="O181" s="7" t="n">
         <v>0</v>
@@ -14354,12 +14354,12 @@
       <c r="P181" s="7" t="n"/>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S181" s="8" t="inlineStr"/>
@@ -14376,7 +14376,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
+          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
         </is>
       </c>
     </row>
@@ -14390,13 +14390,13 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>1600</v>
+        <v>1970</v>
       </c>
       <c r="D182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E182" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
@@ -14405,7 +14405,7 @@
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
@@ -14413,13 +14413,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I182" s="7" t="n"/>
+      <c r="I182" s="7" t="n">
+        <v>750</v>
+      </c>
       <c r="J182" s="7" t="n"/>
       <c r="K182" s="7" t="n"/>
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>13404</v>
+        <v>21740</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14427,12 +14429,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14449,7 +14451,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
+          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
         </is>
       </c>
     </row>
@@ -14463,10 +14465,10 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>1700</v>
+        <v>1575</v>
       </c>
       <c r="D183" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E183" s="7" t="n">
         <v>1</v>
@@ -14478,7 +14480,7 @@
       </c>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H183" s="7" t="inlineStr">
@@ -14487,14 +14489,14 @@
         </is>
       </c>
       <c r="I183" s="7" t="n">
-        <v>646</v>
+        <v>430</v>
       </c>
       <c r="J183" s="7" t="n"/>
       <c r="K183" s="7" t="n"/>
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="7" t="n">
-        <v>20928</v>
+        <v>21816</v>
       </c>
       <c r="O183" s="7" t="n">
         <v>0</v>
@@ -14502,12 +14504,12 @@
       <c r="P183" s="7" t="n"/>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S183" s="8" t="inlineStr"/>
@@ -14524,7 +14526,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
+          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
         </is>
       </c>
     </row>
@@ -14538,13 +14540,13 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>2105</v>
+        <v>1350</v>
       </c>
       <c r="D184" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E184" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F184" s="7" t="inlineStr">
         <is>
@@ -14553,7 +14555,7 @@
       </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Invicta, Millenium Promenade, BS1</t>
         </is>
       </c>
       <c r="H184" s="7" t="inlineStr">
@@ -14561,15 +14563,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I184" s="7" t="n">
-        <v>745</v>
-      </c>
+      <c r="I184" s="7" t="n"/>
       <c r="J184" s="7" t="n"/>
       <c r="K184" s="7" t="n"/>
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
       <c r="N184" s="7" t="n">
-        <v>20984</v>
+        <v>17344</v>
       </c>
       <c r="O184" s="7" t="n">
         <v>0</v>
@@ -14577,12 +14577,12 @@
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S184" s="8" t="inlineStr"/>
@@ -14599,7 +14599,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
+          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
         </is>
       </c>
     </row>
@@ -14613,7 +14613,7 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>1595</v>
+        <v>1600</v>
       </c>
       <c r="D185" s="7" t="n">
         <v>1</v>
@@ -14628,7 +14628,7 @@
       </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Central Quay North, Bristol, BS1</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
@@ -14636,15 +14636,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I185" s="7" t="n">
-        <v>484</v>
-      </c>
+      <c r="I185" s="7" t="n"/>
       <c r="J185" s="7" t="n"/>
       <c r="K185" s="7" t="n"/>
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="7" t="n">
-        <v>21732</v>
+        <v>13404</v>
       </c>
       <c r="O185" s="7" t="n">
         <v>0</v>
@@ -14652,12 +14650,12 @@
       <c r="P185" s="7" t="n"/>
       <c r="Q185" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S185" s="8" t="inlineStr"/>
@@ -14674,7 +14672,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
+          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14686,7 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>1999</v>
+        <v>1700</v>
       </c>
       <c r="D186" s="7" t="n">
         <v>2</v>
@@ -14703,21 +14701,23 @@
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I186" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I186" s="7" t="n">
+        <v>646</v>
+      </c>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>21736</v>
+        <v>20928</v>
       </c>
       <c r="O186" s="7" t="n">
         <v>0</v>
@@ -14725,12 +14725,12 @@
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14747,7 +14747,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
+          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
         </is>
       </c>
     </row>
@@ -14761,13 +14761,13 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>1605</v>
+        <v>2105</v>
       </c>
       <c r="D187" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E187" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F187" s="7" t="inlineStr">
         <is>
@@ -14776,7 +14776,7 @@
       </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
@@ -14785,14 +14785,14 @@
         </is>
       </c>
       <c r="I187" s="7" t="n">
-        <v>487</v>
+        <v>745</v>
       </c>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>21732</v>
+        <v>20984</v>
       </c>
       <c r="O187" s="7" t="n">
         <v>0</v>
@@ -14800,12 +14800,12 @@
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S187" s="8" t="inlineStr"/>
@@ -14822,7 +14822,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
+          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
         </is>
       </c>
     </row>
@@ -14836,7 +14836,7 @@
         </is>
       </c>
       <c r="C188" s="9" t="n">
-        <v>1390</v>
+        <v>1595</v>
       </c>
       <c r="D188" s="7" t="n">
         <v>1</v>
@@ -14851,7 +14851,7 @@
       </c>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
@@ -14859,24 +14859,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I188" s="7" t="n"/>
+      <c r="I188" s="7" t="n">
+        <v>484</v>
+      </c>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
       <c r="L188" s="7" t="n"/>
       <c r="M188" s="7" t="n"/>
-      <c r="N188" s="7" t="n"/>
+      <c r="N188" s="7" t="n">
+        <v>21732</v>
+      </c>
       <c r="O188" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S188" s="8" t="inlineStr"/>
@@ -14893,7 +14897,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
         </is>
       </c>
     </row>
@@ -14907,10 +14911,10 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>1395</v>
+        <v>1999</v>
       </c>
       <c r="D189" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E189" s="7" t="n">
         <v>1</v>
@@ -14922,12 +14926,12 @@
       </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I189" s="7" t="n"/>
@@ -14936,7 +14940,7 @@
       <c r="L189" s="7" t="n"/>
       <c r="M189" s="7" t="n"/>
       <c r="N189" s="7" t="n">
-        <v>20524</v>
+        <v>21736</v>
       </c>
       <c r="O189" s="7" t="n">
         <v>0</v>
@@ -14944,7 +14948,7 @@
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="R189" s="7" t="inlineStr">
@@ -14966,7 +14970,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
         </is>
       </c>
     </row>
@@ -14980,7 +14984,7 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>1200</v>
+        <v>1605</v>
       </c>
       <c r="D190" s="7" t="n">
         <v>1</v>
@@ -14990,28 +14994,28 @@
       </c>
       <c r="F190" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>Sweetman Place, Bristol, BS2 0JN</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I190" s="7" t="n">
-        <v>452</v>
+        <v>487</v>
       </c>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="7" t="n">
-        <v>20472</v>
+        <v>21732</v>
       </c>
       <c r="O190" s="7" t="n">
         <v>0</v>
@@ -15019,12 +15023,12 @@
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S190" s="8" t="inlineStr"/>
@@ -15041,7 +15045,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
+          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
         </is>
       </c>
     </row>
@@ -15055,7 +15059,7 @@
         </is>
       </c>
       <c r="C191" s="9" t="n">
-        <v>1450</v>
+        <v>1390</v>
       </c>
       <c r="D191" s="7" t="n">
         <v>1</v>
@@ -15070,7 +15074,7 @@
       </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H191" s="7" t="inlineStr">
@@ -15083,21 +15087,19 @@
       <c r="K191" s="7" t="n"/>
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
-      <c r="N191" s="7" t="n">
-        <v>16664</v>
-      </c>
+      <c r="N191" s="7" t="n"/>
       <c r="O191" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P191" s="7" t="n"/>
       <c r="Q191" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R191" s="7" t="inlineStr">
         <is>
-          <t>Howard, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S191" s="8" t="inlineStr"/>
@@ -15114,14 +15116,235 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
+          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B192" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C192" s="9" t="n">
+        <v>1395</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F192" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G192" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Court, Bristol, BS1</t>
+        </is>
+      </c>
+      <c r="H192" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I192" s="7" t="n"/>
+      <c r="J192" s="7" t="n"/>
+      <c r="K192" s="7" t="n"/>
+      <c r="L192" s="7" t="n"/>
+      <c r="M192" s="7" t="n"/>
+      <c r="N192" s="7" t="n">
+        <v>20524</v>
+      </c>
+      <c r="O192" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P192" s="7" t="n"/>
+      <c r="Q192" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="R192" s="7" t="inlineStr">
+        <is>
+          <t>OpenRent, London</t>
+        </is>
+      </c>
+      <c r="S192" s="8" t="inlineStr"/>
+      <c r="T192" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V192" s="6" t="inlineStr"/>
+      <c r="W192" s="7" t="inlineStr">
+        <is>
+          <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B193" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C193" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D193" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E193" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F193" s="7" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G193" s="8" t="inlineStr">
+        <is>
+          <t>Sweetman Place, Bristol, BS2 0JN</t>
+        </is>
+      </c>
+      <c r="H193" s="7" t="inlineStr">
+        <is>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I193" s="7" t="n">
+        <v>452</v>
+      </c>
+      <c r="J193" s="7" t="n"/>
+      <c r="K193" s="7" t="n"/>
+      <c r="L193" s="7" t="n"/>
+      <c r="M193" s="7" t="n"/>
+      <c r="N193" s="7" t="n">
+        <v>20472</v>
+      </c>
+      <c r="O193" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P193" s="7" t="n"/>
+      <c r="Q193" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="R193" s="7" t="inlineStr">
+        <is>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
+        </is>
+      </c>
+      <c r="S193" s="8" t="inlineStr"/>
+      <c r="T193" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V193" s="6" t="inlineStr"/>
+      <c r="W193" s="7" t="inlineStr">
+        <is>
+          <t>44a00b698c6b5a317e09685fde82a32c1c765361</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B194" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C194" s="9" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E194" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F194" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G194" s="8" t="inlineStr">
+        <is>
+          <t>Anchorage, Gaol Ferry Steps, Bristol, BS1</t>
+        </is>
+      </c>
+      <c r="H194" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I194" s="7" t="n"/>
+      <c r="J194" s="7" t="n"/>
+      <c r="K194" s="7" t="n"/>
+      <c r="L194" s="7" t="n"/>
+      <c r="M194" s="7" t="n"/>
+      <c r="N194" s="7" t="n">
+        <v>16664</v>
+      </c>
+      <c r="O194" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P194" s="7" t="n"/>
+      <c r="Q194" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R194" s="7" t="inlineStr">
+        <is>
+          <t>Howard, Bristol</t>
+        </is>
+      </c>
+      <c r="S194" s="8" t="inlineStr"/>
+      <c r="T194" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V194" s="6" t="inlineStr"/>
+      <c r="W194" s="7" t="inlineStr">
+        <is>
           <t>1ac36e9c91a77dd147c6577e08dbb37440366bb9</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W191"/>
+  <autoFilter ref="A1:W194"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15316,6 +15539,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T189" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T190" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T194" r:id="rId193"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 178
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -12,7 +12,7 @@
     <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'To Rent'!$A$1:$W$193</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -625,7 +625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W192"/>
+  <dimension ref="A1:W193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10887,7 +10887,7 @@
         </is>
       </c>
       <c r="C135" s="9" t="n">
-        <v>1100</v>
+        <v>1680</v>
       </c>
       <c r="D135" s="7" t="n">
         <v>1</v>
@@ -10902,21 +10902,23 @@
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t>Bath Road - Arnos Vale</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>BS4</t>
-        </is>
-      </c>
-      <c r="I135" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I135" s="7" t="n">
+        <v>558</v>
+      </c>
       <c r="J135" s="7" t="n"/>
       <c r="K135" s="7" t="n"/>
       <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="n"/>
       <c r="N135" s="7" t="n">
-        <v>6248</v>
+        <v>20984</v>
       </c>
       <c r="O135" s="7" t="n">
         <v>0</v>
@@ -10924,12 +10926,12 @@
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S135" s="8" t="inlineStr"/>
@@ -10946,7 +10948,7 @@
       <c r="V135" s="6" t="inlineStr"/>
       <c r="W135" s="7" t="inlineStr">
         <is>
-          <t>e63386a22f0ffb4baee6b24143f47a42221ce776</t>
+          <t>6ffc2ba688d7b5956d85534872c157a0d524f2f3</t>
         </is>
       </c>
     </row>
@@ -10960,7 +10962,7 @@
         </is>
       </c>
       <c r="C136" s="9" t="n">
-        <v>1400</v>
+        <v>1100</v>
       </c>
       <c r="D136" s="7" t="n">
         <v>1</v>
@@ -10975,12 +10977,12 @@
       </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t>Redcross Village, Bristol, BS2</t>
+          <t>Bath Road - Arnos Vale</t>
         </is>
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS4</t>
         </is>
       </c>
       <c r="I136" s="7" t="n"/>
@@ -10989,7 +10991,7 @@
       <c r="L136" s="7" t="n"/>
       <c r="M136" s="7" t="n"/>
       <c r="N136" s="7" t="n">
-        <v>21520</v>
+        <v>6248</v>
       </c>
       <c r="O136" s="7" t="n">
         <v>0</v>
@@ -10997,12 +10999,12 @@
       <c r="P136" s="7" t="n"/>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
         <is>
-          <t>The Letting Game, Redland</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S136" s="8" t="inlineStr"/>
@@ -11019,7 +11021,7 @@
       <c r="V136" s="6" t="inlineStr"/>
       <c r="W136" s="7" t="inlineStr">
         <is>
-          <t>811a7931cecb689888c03706aa5821a875281cb2</t>
+          <t>e63386a22f0ffb4baee6b24143f47a42221ce776</t>
         </is>
       </c>
     </row>
@@ -11033,7 +11035,7 @@
         </is>
       </c>
       <c r="C137" s="9" t="n">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="D137" s="7" t="n">
         <v>1</v>
@@ -11048,7 +11050,7 @@
       </c>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t>Chimney Steps, Bristol, BS2</t>
+          <t>Redcross Village, Bristol, BS2</t>
         </is>
       </c>
       <c r="H137" s="7" t="inlineStr">
@@ -11056,15 +11058,13 @@
           <t>BS2</t>
         </is>
       </c>
-      <c r="I137" s="7" t="n">
-        <v>452</v>
-      </c>
+      <c r="I137" s="7" t="n"/>
       <c r="J137" s="7" t="n"/>
       <c r="K137" s="7" t="n"/>
       <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="n"/>
       <c r="N137" s="7" t="n">
-        <v>19996</v>
+        <v>21520</v>
       </c>
       <c r="O137" s="7" t="n">
         <v>0</v>
@@ -11072,12 +11072,12 @@
       <c r="P137" s="7" t="n"/>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>Nook Lettings, Bristol</t>
+          <t>The Letting Game, Redland</t>
         </is>
       </c>
       <c r="S137" s="8" t="inlineStr"/>
@@ -11094,7 +11094,7 @@
       <c r="V137" s="6" t="inlineStr"/>
       <c r="W137" s="7" t="inlineStr">
         <is>
-          <t>b0804dcb3dae15dea73fb6b7320023ee0cc5e93a</t>
+          <t>811a7931cecb689888c03706aa5821a875281cb2</t>
         </is>
       </c>
     </row>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="C138" s="9" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
       <c r="D138" s="7" t="n">
         <v>1</v>
@@ -11123,21 +11123,23 @@
       </c>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t>Taylors Bank, Bristol, BS1</t>
+          <t>Chimney Steps, Bristol, BS2</t>
         </is>
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I138" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I138" s="7" t="n">
+        <v>452</v>
+      </c>
       <c r="J138" s="7" t="n"/>
       <c r="K138" s="7" t="n"/>
       <c r="L138" s="7" t="n"/>
       <c r="M138" s="7" t="n"/>
       <c r="N138" s="7" t="n">
-        <v>21996</v>
+        <v>19996</v>
       </c>
       <c r="O138" s="7" t="n">
         <v>0</v>
@@ -11145,12 +11147,12 @@
       <c r="P138" s="7" t="n"/>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Nook Lettings, Bristol</t>
         </is>
       </c>
       <c r="S138" s="8" t="inlineStr"/>
@@ -11167,7 +11169,7 @@
       <c r="V138" s="6" t="inlineStr"/>
       <c r="W138" s="7" t="inlineStr">
         <is>
-          <t>464a8221babcd58554ee30417192b0a25eacccb0</t>
+          <t>b0804dcb3dae15dea73fb6b7320023ee0cc5e93a</t>
         </is>
       </c>
     </row>
@@ -11196,7 +11198,7 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The General, BS1</t>
+          <t>Taylors Bank, Bristol, BS1</t>
         </is>
       </c>
       <c r="H139" s="7" t="inlineStr">
@@ -11204,15 +11206,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I139" s="7" t="n">
-        <v>604</v>
-      </c>
+      <c r="I139" s="7" t="n"/>
       <c r="J139" s="7" t="n"/>
       <c r="K139" s="7" t="n"/>
       <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="n"/>
       <c r="N139" s="7" t="n">
-        <v>19076</v>
+        <v>21996</v>
       </c>
       <c r="O139" s="7" t="n">
         <v>0</v>
@@ -11220,12 +11220,12 @@
       <c r="P139" s="7" t="n"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr"/>
@@ -11242,7 +11242,7 @@
       <c r="V139" s="6" t="inlineStr"/>
       <c r="W139" s="7" t="inlineStr">
         <is>
-          <t>adaa31d271a8abff25dafaf34aa54eb1f22dd072</t>
+          <t>464a8221babcd58554ee30417192b0a25eacccb0</t>
         </is>
       </c>
     </row>
@@ -11256,13 +11256,13 @@
         </is>
       </c>
       <c r="C140" s="9" t="n">
-        <v>2400</v>
+        <v>1400</v>
       </c>
       <c r="D140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E140" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
@@ -11271,21 +11271,23 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Portland Square, Bristol, BS2</t>
+          <t>City Centre, The General, BS1</t>
         </is>
       </c>
       <c r="H140" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I140" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I140" s="7" t="n">
+        <v>604</v>
+      </c>
       <c r="J140" s="7" t="n"/>
       <c r="K140" s="7" t="n"/>
       <c r="L140" s="7" t="n"/>
       <c r="M140" s="7" t="n"/>
       <c r="N140" s="7" t="n">
-        <v>21360</v>
+        <v>19076</v>
       </c>
       <c r="O140" s="7" t="n">
         <v>0</v>
@@ -11293,12 +11295,12 @@
       <c r="P140" s="7" t="n"/>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>Just Lets, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S140" s="8" t="inlineStr"/>
@@ -11315,7 +11317,7 @@
       <c r="V140" s="6" t="inlineStr"/>
       <c r="W140" s="7" t="inlineStr">
         <is>
-          <t>0b6e19cc97b73c7e581c5f306902c64d0c59b226</t>
+          <t>adaa31d271a8abff25dafaf34aa54eb1f22dd072</t>
         </is>
       </c>
     </row>
@@ -11329,13 +11331,13 @@
         </is>
       </c>
       <c r="C141" s="9" t="n">
-        <v>1600</v>
+        <v>2400</v>
       </c>
       <c r="D141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E141" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
@@ -11344,12 +11346,12 @@
       </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t>Horizon, Broad Weir, BS1</t>
+          <t>Portland Square, Bristol, BS2</t>
         </is>
       </c>
       <c r="H141" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I141" s="7" t="n"/>
@@ -11358,7 +11360,7 @@
       <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="n"/>
       <c r="N141" s="7" t="n">
-        <v>21996</v>
+        <v>21360</v>
       </c>
       <c r="O141" s="7" t="n">
         <v>0</v>
@@ -11371,7 +11373,7 @@
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Just Lets, Bristol</t>
         </is>
       </c>
       <c r="S141" s="8" t="inlineStr"/>
@@ -11388,7 +11390,7 @@
       <c r="V141" s="6" t="inlineStr"/>
       <c r="W141" s="7" t="inlineStr">
         <is>
-          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
+          <t>0b6e19cc97b73c7e581c5f306902c64d0c59b226</t>
         </is>
       </c>
     </row>
@@ -11402,7 +11404,7 @@
         </is>
       </c>
       <c r="C142" s="9" t="n">
-        <v>1560</v>
+        <v>1600</v>
       </c>
       <c r="D142" s="7" t="n">
         <v>1</v>
@@ -11417,7 +11419,7 @@
       </c>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Horizon, Broad Weir, BS1</t>
         </is>
       </c>
       <c r="H142" s="7" t="inlineStr">
@@ -11425,15 +11427,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I142" s="7" t="n">
-        <v>472</v>
-      </c>
+      <c r="I142" s="7" t="n"/>
       <c r="J142" s="7" t="n"/>
       <c r="K142" s="7" t="n"/>
       <c r="L142" s="7" t="n"/>
       <c r="M142" s="7" t="n"/>
       <c r="N142" s="7" t="n">
-        <v>20984</v>
+        <v>21996</v>
       </c>
       <c r="O142" s="7" t="n">
         <v>0</v>
@@ -11441,12 +11441,12 @@
       <c r="P142" s="7" t="n"/>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S142" s="8" t="inlineStr"/>
@@ -11463,7 +11463,7 @@
       <c r="V142" s="6" t="inlineStr"/>
       <c r="W142" s="7" t="inlineStr">
         <is>
-          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
+          <t>f2976928ca2581a4e6e81561eba91cddb2dc839a</t>
         </is>
       </c>
     </row>
@@ -11477,7 +11477,7 @@
         </is>
       </c>
       <c r="C143" s="9" t="n">
-        <v>1660</v>
+        <v>1560</v>
       </c>
       <c r="D143" s="7" t="n">
         <v>1</v>
@@ -11501,7 +11501,7 @@
         </is>
       </c>
       <c r="I143" s="7" t="n">
-        <v>558</v>
+        <v>472</v>
       </c>
       <c r="J143" s="7" t="n"/>
       <c r="K143" s="7" t="n"/>
@@ -11516,7 +11516,7 @@
       <c r="P143" s="7" t="n"/>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R143" s="7" t="inlineStr">
@@ -11538,7 +11538,7 @@
       <c r="V143" s="6" t="inlineStr"/>
       <c r="W143" s="7" t="inlineStr">
         <is>
-          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
+          <t>55d26f5321b390d578ce33d45d67e2026995aa77</t>
         </is>
       </c>
     </row>
@@ -11552,13 +11552,13 @@
         </is>
       </c>
       <c r="C144" s="9" t="n">
-        <v>1860</v>
+        <v>1660</v>
       </c>
       <c r="D144" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E144" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
@@ -11567,7 +11567,7 @@
       </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
@@ -11576,14 +11576,14 @@
         </is>
       </c>
       <c r="I144" s="7" t="n">
-        <v>647</v>
+        <v>558</v>
       </c>
       <c r="J144" s="7" t="n"/>
       <c r="K144" s="7" t="n"/>
       <c r="L144" s="7" t="n"/>
       <c r="M144" s="7" t="n"/>
       <c r="N144" s="7" t="n">
-        <v>21740</v>
+        <v>20984</v>
       </c>
       <c r="O144" s="7" t="n">
         <v>0</v>
@@ -11596,7 +11596,7 @@
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S144" s="8" t="inlineStr"/>
@@ -11613,7 +11613,7 @@
       <c r="V144" s="6" t="inlineStr"/>
       <c r="W144" s="7" t="inlineStr">
         <is>
-          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
+          <t>f0f860bf519ea51e7817dad01af0d01e6f68d6eb</t>
         </is>
       </c>
     </row>
@@ -11627,13 +11627,13 @@
         </is>
       </c>
       <c r="C145" s="9" t="n">
-        <v>1600</v>
+        <v>1860</v>
       </c>
       <c r="D145" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E145" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
@@ -11651,14 +11651,14 @@
         </is>
       </c>
       <c r="I145" s="7" t="n">
-        <v>549</v>
+        <v>647</v>
       </c>
       <c r="J145" s="7" t="n"/>
       <c r="K145" s="7" t="n"/>
       <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="n"/>
       <c r="N145" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O145" s="7" t="n">
         <v>0</v>
@@ -11688,7 +11688,7 @@
       <c r="V145" s="6" t="inlineStr"/>
       <c r="W145" s="7" t="inlineStr">
         <is>
-          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
+          <t>b46dee44dc68b52ae3cb0b9e014ec37873dac6e1</t>
         </is>
       </c>
     </row>
@@ -11702,13 +11702,13 @@
         </is>
       </c>
       <c r="C146" s="9" t="n">
-        <v>1900</v>
+        <v>1600</v>
       </c>
       <c r="D146" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E146" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
@@ -11726,14 +11726,14 @@
         </is>
       </c>
       <c r="I146" s="7" t="n">
-        <v>624</v>
+        <v>549</v>
       </c>
       <c r="J146" s="7" t="n"/>
       <c r="K146" s="7" t="n"/>
       <c r="L146" s="7" t="n"/>
       <c r="M146" s="7" t="n"/>
       <c r="N146" s="7" t="n">
-        <v>21740</v>
+        <v>21816</v>
       </c>
       <c r="O146" s="7" t="n">
         <v>0</v>
@@ -11741,7 +11741,7 @@
       <c r="P146" s="7" t="n"/>
       <c r="Q146" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R146" s="7" t="inlineStr">
@@ -11763,7 +11763,7 @@
       <c r="V146" s="6" t="inlineStr"/>
       <c r="W146" s="7" t="inlineStr">
         <is>
-          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
+          <t>48fce3ef8f4dc68d39b439b7f0740ed05fe5ae26</t>
         </is>
       </c>
     </row>
@@ -11777,13 +11777,13 @@
         </is>
       </c>
       <c r="C147" s="9" t="n">
-        <v>1530</v>
+        <v>1900</v>
       </c>
       <c r="D147" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E147" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F147" s="7" t="inlineStr">
         <is>
@@ -11801,7 +11801,7 @@
         </is>
       </c>
       <c r="I147" s="7" t="n">
-        <v>548</v>
+        <v>624</v>
       </c>
       <c r="J147" s="7" t="n"/>
       <c r="K147" s="7" t="n"/>
@@ -11816,7 +11816,7 @@
       <c r="P147" s="7" t="n"/>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
@@ -11838,7 +11838,7 @@
       <c r="V147" s="6" t="inlineStr"/>
       <c r="W147" s="7" t="inlineStr">
         <is>
-          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
+          <t>656f78f15f4e6c8f81d012d47b0373306bd9e49e</t>
         </is>
       </c>
     </row>
@@ -11852,13 +11852,13 @@
         </is>
       </c>
       <c r="C148" s="9" t="n">
-        <v>2110</v>
+        <v>1530</v>
       </c>
       <c r="D148" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E148" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
@@ -11876,7 +11876,7 @@
         </is>
       </c>
       <c r="I148" s="7" t="n">
-        <v>624</v>
+        <v>548</v>
       </c>
       <c r="J148" s="7" t="n"/>
       <c r="K148" s="7" t="n"/>
@@ -11891,7 +11891,7 @@
       <c r="P148" s="7" t="n"/>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
@@ -11913,7 +11913,7 @@
       <c r="V148" s="6" t="inlineStr"/>
       <c r="W148" s="7" t="inlineStr">
         <is>
-          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
+          <t>f6b585f60dfa2832d9a44ad01d0fe12ed82f08ec</t>
         </is>
       </c>
     </row>
@@ -11927,13 +11927,13 @@
         </is>
       </c>
       <c r="C149" s="9" t="n">
-        <v>1530</v>
+        <v>2110</v>
       </c>
       <c r="D149" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E149" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F149" s="7" t="inlineStr">
         <is>
@@ -11951,7 +11951,7 @@
         </is>
       </c>
       <c r="I149" s="7" t="n">
-        <v>544</v>
+        <v>624</v>
       </c>
       <c r="J149" s="7" t="n"/>
       <c r="K149" s="7" t="n"/>
@@ -11966,7 +11966,7 @@
       <c r="P149" s="7" t="n"/>
       <c r="Q149" s="7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R149" s="7" t="inlineStr">
@@ -11988,7 +11988,7 @@
       <c r="V149" s="6" t="inlineStr"/>
       <c r="W149" s="7" t="inlineStr">
         <is>
-          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
+          <t>fe9077839a5f7ef2de3e82f388dbe3557051b1f9</t>
         </is>
       </c>
     </row>
@@ -12002,13 +12002,13 @@
         </is>
       </c>
       <c r="C150" s="9" t="n">
-        <v>1600</v>
+        <v>1530</v>
       </c>
       <c r="D150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E150" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
@@ -12017,7 +12017,7 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Marsh Street, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H150" s="7" t="inlineStr">
@@ -12025,13 +12025,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I150" s="7" t="n"/>
+      <c r="I150" s="7" t="n">
+        <v>544</v>
+      </c>
       <c r="J150" s="7" t="n"/>
       <c r="K150" s="7" t="n"/>
       <c r="L150" s="7" t="n"/>
       <c r="M150" s="7" t="n"/>
       <c r="N150" s="7" t="n">
-        <v>20880</v>
+        <v>21740</v>
       </c>
       <c r="O150" s="7" t="n">
         <v>0</v>
@@ -12039,12 +12041,12 @@
       <c r="P150" s="7" t="n"/>
       <c r="Q150" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S150" s="8" t="inlineStr"/>
@@ -12061,7 +12063,7 @@
       <c r="V150" s="6" t="inlineStr"/>
       <c r="W150" s="7" t="inlineStr">
         <is>
-          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
+          <t>f1ca53e6417e96bb53391d4a81dd88d4e56206bd</t>
         </is>
       </c>
     </row>
@@ -12075,7 +12077,7 @@
         </is>
       </c>
       <c r="C151" s="9" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="D151" s="7" t="n">
         <v>2</v>
@@ -12098,15 +12100,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I151" s="7" t="n">
-        <v>980</v>
-      </c>
+      <c r="I151" s="7" t="n"/>
       <c r="J151" s="7" t="n"/>
       <c r="K151" s="7" t="n"/>
       <c r="L151" s="7" t="n"/>
       <c r="M151" s="7" t="n"/>
       <c r="N151" s="7" t="n">
-        <v>21316</v>
+        <v>20880</v>
       </c>
       <c r="O151" s="7" t="n">
         <v>0</v>
@@ -12114,12 +12114,12 @@
       <c r="P151" s="7" t="n"/>
       <c r="Q151" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R151" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S151" s="8" t="inlineStr"/>
@@ -12136,7 +12136,7 @@
       <c r="V151" s="6" t="inlineStr"/>
       <c r="W151" s="7" t="inlineStr">
         <is>
-          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
+          <t>62f337c2d4b593d0a8a7316b73657bc80bea27f5</t>
         </is>
       </c>
     </row>
@@ -12150,13 +12150,13 @@
         </is>
       </c>
       <c r="C152" s="9" t="n">
-        <v>1995</v>
+        <v>1800</v>
       </c>
       <c r="D152" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E152" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
@@ -12165,7 +12165,7 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>Baldwin St, Bristol, BS1</t>
+          <t>Marsh Street, Bristol, BS1</t>
         </is>
       </c>
       <c r="H152" s="7" t="inlineStr">
@@ -12173,13 +12173,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I152" s="7" t="n"/>
+      <c r="I152" s="7" t="n">
+        <v>980</v>
+      </c>
       <c r="J152" s="7" t="n"/>
       <c r="K152" s="7" t="n"/>
       <c r="L152" s="7" t="n"/>
       <c r="M152" s="7" t="n"/>
       <c r="N152" s="7" t="n">
-        <v>21196</v>
+        <v>21316</v>
       </c>
       <c r="O152" s="7" t="n">
         <v>0</v>
@@ -12187,12 +12189,12 @@
       <c r="P152" s="7" t="n"/>
       <c r="Q152" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S152" s="8" t="inlineStr"/>
@@ -12209,7 +12211,7 @@
       <c r="V152" s="6" t="inlineStr"/>
       <c r="W152" s="7" t="inlineStr">
         <is>
-          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
+          <t>1bd9cb1b7942915b74ae0cb79e84a122906aeee7</t>
         </is>
       </c>
     </row>
@@ -12223,13 +12225,13 @@
         </is>
       </c>
       <c r="C153" s="9" t="n">
-        <v>1750</v>
+        <v>1995</v>
       </c>
       <c r="D153" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E153" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
@@ -12238,7 +12240,7 @@
       </c>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
+          <t>Baldwin St, Bristol, BS1</t>
         </is>
       </c>
       <c r="H153" s="7" t="inlineStr">
@@ -12246,15 +12248,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I153" s="7" t="n">
-        <v>849</v>
-      </c>
+      <c r="I153" s="7" t="n"/>
       <c r="J153" s="7" t="n"/>
       <c r="K153" s="7" t="n"/>
       <c r="L153" s="7" t="n"/>
       <c r="M153" s="7" t="n"/>
       <c r="N153" s="7" t="n">
-        <v>21028</v>
+        <v>21196</v>
       </c>
       <c r="O153" s="7" t="n">
         <v>0</v>
@@ -12262,12 +12262,12 @@
       <c r="P153" s="7" t="n"/>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>A2Dominion Group, A2Dominion Lettings</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S153" s="8" t="inlineStr"/>
@@ -12284,7 +12284,7 @@
       <c r="V153" s="6" t="inlineStr"/>
       <c r="W153" s="7" t="inlineStr">
         <is>
-          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
+          <t>afeb98753462ccfb5528732e6cdc31bdc6ce9666</t>
         </is>
       </c>
     </row>
@@ -12298,7 +12298,7 @@
         </is>
       </c>
       <c r="C154" s="9" t="n">
-        <v>1550</v>
+        <v>1750</v>
       </c>
       <c r="D154" s="7" t="n">
         <v>2</v>
@@ -12313,21 +12313,23 @@
       </c>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t>Portland Heights - St. Pauls</t>
+          <t>Kiln House, St Thomas Street, Redcliff, Bristol, Bristol City</t>
         </is>
       </c>
       <c r="H154" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I154" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I154" s="7" t="n">
+        <v>849</v>
+      </c>
       <c r="J154" s="7" t="n"/>
       <c r="K154" s="7" t="n"/>
       <c r="L154" s="7" t="n"/>
       <c r="M154" s="7" t="n"/>
       <c r="N154" s="7" t="n">
-        <v>21420</v>
+        <v>21028</v>
       </c>
       <c r="O154" s="7" t="n">
         <v>0</v>
@@ -12335,12 +12337,12 @@
       <c r="P154" s="7" t="n"/>
       <c r="Q154" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R154" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Bishopston</t>
+          <t>A2Dominion Group, A2Dominion Lettings</t>
         </is>
       </c>
       <c r="S154" s="8" t="inlineStr"/>
@@ -12357,7 +12359,7 @@
       <c r="V154" s="6" t="inlineStr"/>
       <c r="W154" s="7" t="inlineStr">
         <is>
-          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
+          <t>f3200b5929e6da684c280ffd6afc184efbe2ebf1</t>
         </is>
       </c>
     </row>
@@ -12371,13 +12373,13 @@
         </is>
       </c>
       <c r="C155" s="9" t="n">
-        <v>1400</v>
+        <v>1550</v>
       </c>
       <c r="D155" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E155" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F155" s="7" t="inlineStr">
         <is>
@@ -12386,12 +12388,12 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>The Atrium, Redcliffe Street, BS1</t>
+          <t>Portland Heights - St. Pauls</t>
         </is>
       </c>
       <c r="H155" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
+          <t>BS2</t>
         </is>
       </c>
       <c r="I155" s="7" t="n"/>
@@ -12400,7 +12402,7 @@
       <c r="L155" s="7" t="n"/>
       <c r="M155" s="7" t="n"/>
       <c r="N155" s="7" t="n">
-        <v>20292</v>
+        <v>21420</v>
       </c>
       <c r="O155" s="7" t="n">
         <v>0</v>
@@ -12408,12 +12410,12 @@
       <c r="P155" s="7" t="n"/>
       <c r="Q155" s="7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Ocean, Bishopston</t>
         </is>
       </c>
       <c r="S155" s="8" t="inlineStr"/>
@@ -12430,7 +12432,7 @@
       <c r="V155" s="6" t="inlineStr"/>
       <c r="W155" s="7" t="inlineStr">
         <is>
-          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
+          <t>99fe3e39d0594e7d8193a0c484efbe85d08f3e40</t>
         </is>
       </c>
     </row>
@@ -12444,7 +12446,7 @@
         </is>
       </c>
       <c r="C156" s="9" t="n">
-        <v>1150</v>
+        <v>1400</v>
       </c>
       <c r="D156" s="7" t="n">
         <v>1</v>
@@ -12459,12 +12461,12 @@
       </c>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
+          <t>The Atrium, Redcliffe Street, BS1</t>
         </is>
       </c>
       <c r="H156" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I156" s="7" t="n"/>
@@ -12473,7 +12475,7 @@
       <c r="L156" s="7" t="n"/>
       <c r="M156" s="7" t="n"/>
       <c r="N156" s="7" t="n">
-        <v>15376</v>
+        <v>20292</v>
       </c>
       <c r="O156" s="7" t="n">
         <v>0</v>
@@ -12481,12 +12483,12 @@
       <c r="P156" s="7" t="n"/>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Accommodation Unlimited, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S156" s="8" t="inlineStr"/>
@@ -12503,7 +12505,7 @@
       <c r="V156" s="6" t="inlineStr"/>
       <c r="W156" s="7" t="inlineStr">
         <is>
-          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
+          <t>7dcd9ae5ed03dcc4ea3bf2f5256469c38d345fd0</t>
         </is>
       </c>
     </row>
@@ -12517,7 +12519,7 @@
         </is>
       </c>
       <c r="C157" s="9" t="n">
-        <v>1300</v>
+        <v>1150</v>
       </c>
       <c r="D157" s="7" t="n">
         <v>1</v>
@@ -12532,23 +12534,21 @@
       </c>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t>City Centre, The Milliners, BS1 6WU</t>
+          <t>Bedminster Parade Bedminster, Bristol, BS3</t>
         </is>
       </c>
       <c r="H157" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I157" s="7" t="n">
-        <v>463</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I157" s="7" t="n"/>
       <c r="J157" s="7" t="n"/>
       <c r="K157" s="7" t="n"/>
       <c r="L157" s="7" t="n"/>
       <c r="M157" s="7" t="n"/>
       <c r="N157" s="7" t="n">
-        <v>21440</v>
+        <v>15376</v>
       </c>
       <c r="O157" s="7" t="n">
         <v>0</v>
@@ -12556,12 +12556,12 @@
       <c r="P157" s="7" t="n"/>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Bishopston</t>
+          <t>Accommodation Unlimited, Bristol</t>
         </is>
       </c>
       <c r="S157" s="8" t="inlineStr"/>
@@ -12578,7 +12578,7 @@
       <c r="V157" s="6" t="inlineStr"/>
       <c r="W157" s="7" t="inlineStr">
         <is>
-          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
+          <t>8e4a3728fef6aff0c3fc6c809fa86ad0a6d1e193</t>
         </is>
       </c>
     </row>
@@ -12592,7 +12592,7 @@
         </is>
       </c>
       <c r="C158" s="9" t="n">
-        <v>1150</v>
+        <v>1300</v>
       </c>
       <c r="D158" s="7" t="n">
         <v>1</v>
@@ -12607,23 +12607,23 @@
       </c>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t>Century Place, St. Paul Street, BS2 8AN</t>
+          <t>City Centre, The Milliners, BS1 6WU</t>
         </is>
       </c>
       <c r="H158" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
+          <t>BS1</t>
         </is>
       </c>
       <c r="I158" s="7" t="n">
-        <v>344</v>
+        <v>463</v>
       </c>
       <c r="J158" s="7" t="n"/>
       <c r="K158" s="7" t="n"/>
       <c r="L158" s="7" t="n"/>
       <c r="M158" s="7" t="n"/>
       <c r="N158" s="7" t="n">
-        <v>21792</v>
+        <v>21440</v>
       </c>
       <c r="O158" s="7" t="n">
         <v>0</v>
@@ -12631,7 +12631,7 @@
       <c r="P158" s="7" t="n"/>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
@@ -12653,7 +12653,7 @@
       <c r="V158" s="6" t="inlineStr"/>
       <c r="W158" s="7" t="inlineStr">
         <is>
-          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
+          <t>85e83e18f3b71ba14944d2208c25cef593680450</t>
         </is>
       </c>
     </row>
@@ -12667,13 +12667,13 @@
         </is>
       </c>
       <c r="C159" s="9" t="n">
-        <v>1800</v>
+        <v>1150</v>
       </c>
       <c r="D159" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E159" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F159" s="7" t="inlineStr">
         <is>
@@ -12682,21 +12682,23 @@
       </c>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t>Waverley House, BS1</t>
+          <t>Century Place, St. Paul Street, BS2 8AN</t>
         </is>
       </c>
       <c r="H159" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I159" s="7" t="n"/>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I159" s="7" t="n">
+        <v>344</v>
+      </c>
       <c r="J159" s="7" t="n"/>
       <c r="K159" s="7" t="n"/>
       <c r="L159" s="7" t="n"/>
       <c r="M159" s="7" t="n"/>
       <c r="N159" s="7" t="n">
-        <v>17956</v>
+        <v>21792</v>
       </c>
       <c r="O159" s="7" t="n">
         <v>0</v>
@@ -12704,12 +12706,12 @@
       <c r="P159" s="7" t="n"/>
       <c r="Q159" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>Hopewell, Bristol</t>
+          <t>The Bristol Residential Letting Co, Bishopston</t>
         </is>
       </c>
       <c r="S159" s="8" t="inlineStr"/>
@@ -12726,7 +12728,7 @@
       <c r="V159" s="6" t="inlineStr"/>
       <c r="W159" s="7" t="inlineStr">
         <is>
-          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
+          <t>beaef6433448786c8bfa366d8b2005048a7e4e0d</t>
         </is>
       </c>
     </row>
@@ -12740,7 +12742,7 @@
         </is>
       </c>
       <c r="C160" s="9" t="n">
-        <v>2170</v>
+        <v>1800</v>
       </c>
       <c r="D160" s="7" t="n">
         <v>2</v>
@@ -12755,7 +12757,7 @@
       </c>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Waverley House, BS1</t>
         </is>
       </c>
       <c r="H160" s="7" t="inlineStr">
@@ -12763,15 +12765,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I160" s="7" t="n">
-        <v>721</v>
-      </c>
+      <c r="I160" s="7" t="n"/>
       <c r="J160" s="7" t="n"/>
       <c r="K160" s="7" t="n"/>
       <c r="L160" s="7" t="n"/>
       <c r="M160" s="7" t="n"/>
       <c r="N160" s="7" t="n">
-        <v>21732</v>
+        <v>17956</v>
       </c>
       <c r="O160" s="7" t="n">
         <v>0</v>
@@ -12779,12 +12779,12 @@
       <c r="P160" s="7" t="n"/>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Hopewell, Bristol</t>
         </is>
       </c>
       <c r="S160" s="8" t="inlineStr"/>
@@ -12801,7 +12801,7 @@
       <c r="V160" s="6" t="inlineStr"/>
       <c r="W160" s="7" t="inlineStr">
         <is>
-          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
+          <t>ed824d85d8a0fb2062456afe35c84587307518cf</t>
         </is>
       </c>
     </row>
@@ -12815,7 +12815,7 @@
         </is>
       </c>
       <c r="C161" s="9" t="n">
-        <v>1965</v>
+        <v>2170</v>
       </c>
       <c r="D161" s="7" t="n">
         <v>2</v>
@@ -12830,7 +12830,7 @@
       </c>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H161" s="7" t="inlineStr">
@@ -12839,14 +12839,14 @@
         </is>
       </c>
       <c r="I161" s="7" t="n">
-        <v>771</v>
+        <v>721</v>
       </c>
       <c r="J161" s="7" t="n"/>
       <c r="K161" s="7" t="n"/>
       <c r="L161" s="7" t="n"/>
       <c r="M161" s="7" t="n"/>
       <c r="N161" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O161" s="7" t="n">
         <v>0</v>
@@ -12854,12 +12854,12 @@
       <c r="P161" s="7" t="n"/>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S161" s="8" t="inlineStr"/>
@@ -12876,7 +12876,7 @@
       <c r="V161" s="6" t="inlineStr"/>
       <c r="W161" s="7" t="inlineStr">
         <is>
-          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
+          <t>83f93fd8b52dd9181939537e43bdc4dc966f1618</t>
         </is>
       </c>
     </row>
@@ -12890,13 +12890,13 @@
         </is>
       </c>
       <c r="C162" s="9" t="n">
-        <v>1680</v>
+        <v>1965</v>
       </c>
       <c r="D162" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E162" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F162" s="7" t="inlineStr">
         <is>
@@ -12905,7 +12905,7 @@
       </c>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
@@ -12913,13 +12913,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I162" s="7" t="n"/>
+      <c r="I162" s="7" t="n">
+        <v>771</v>
+      </c>
       <c r="J162" s="7" t="n"/>
       <c r="K162" s="7" t="n"/>
       <c r="L162" s="7" t="n"/>
       <c r="M162" s="7" t="n"/>
       <c r="N162" s="7" t="n">
-        <v>20628</v>
+        <v>21740</v>
       </c>
       <c r="O162" s="7" t="n">
         <v>0</v>
@@ -12927,12 +12929,12 @@
       <c r="P162" s="7" t="n"/>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S162" s="8" t="inlineStr"/>
@@ -12949,7 +12951,7 @@
       <c r="V162" s="6" t="inlineStr"/>
       <c r="W162" s="7" t="inlineStr">
         <is>
-          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
+          <t>265e1ae108b921246faaa42d95608312a5d45dfa</t>
         </is>
       </c>
     </row>
@@ -12963,10 +12965,10 @@
         </is>
       </c>
       <c r="C163" s="9" t="n">
-        <v>1625</v>
+        <v>1680</v>
       </c>
       <c r="D163" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E163" s="7" t="n">
         <v>1</v>
@@ -12978,7 +12980,7 @@
       </c>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H163" s="7" t="inlineStr">
@@ -12986,15 +12988,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I163" s="7" t="n">
-        <v>486</v>
-      </c>
+      <c r="I163" s="7" t="n"/>
       <c r="J163" s="7" t="n"/>
       <c r="K163" s="7" t="n"/>
       <c r="L163" s="7" t="n"/>
       <c r="M163" s="7" t="n"/>
       <c r="N163" s="7" t="n">
-        <v>21732</v>
+        <v>20628</v>
       </c>
       <c r="O163" s="7" t="n">
         <v>0</v>
@@ -13007,7 +13007,7 @@
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S163" s="8" t="inlineStr"/>
@@ -13024,7 +13024,7 @@
       <c r="V163" s="6" t="inlineStr"/>
       <c r="W163" s="7" t="inlineStr">
         <is>
-          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
+          <t>4b0bc4fd5ee58a799bcf549a536a60817abe078f</t>
         </is>
       </c>
     </row>
@@ -13038,13 +13038,13 @@
         </is>
       </c>
       <c r="C164" s="9" t="n">
-        <v>1940</v>
+        <v>1625</v>
       </c>
       <c r="D164" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E164" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F164" s="7" t="inlineStr">
         <is>
@@ -13053,7 +13053,7 @@
       </c>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H164" s="7" t="inlineStr">
@@ -13062,14 +13062,14 @@
         </is>
       </c>
       <c r="I164" s="7" t="n">
-        <v>607</v>
+        <v>486</v>
       </c>
       <c r="J164" s="7" t="n"/>
       <c r="K164" s="7" t="n"/>
       <c r="L164" s="7" t="n"/>
       <c r="M164" s="7" t="n"/>
       <c r="N164" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O164" s="7" t="n">
         <v>0</v>
@@ -13082,7 +13082,7 @@
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S164" s="8" t="inlineStr"/>
@@ -13099,7 +13099,7 @@
       <c r="V164" s="6" t="inlineStr"/>
       <c r="W164" s="7" t="inlineStr">
         <is>
-          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
+          <t>c1a887bef4786a41ce2750be0a6d2734258545b3</t>
         </is>
       </c>
     </row>
@@ -13113,13 +13113,13 @@
         </is>
       </c>
       <c r="C165" s="9" t="n">
-        <v>1465</v>
+        <v>1940</v>
       </c>
       <c r="D165" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E165" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F165" s="7" t="inlineStr">
         <is>
@@ -13137,14 +13137,14 @@
         </is>
       </c>
       <c r="I165" s="7" t="n">
-        <v>505</v>
+        <v>607</v>
       </c>
       <c r="J165" s="7" t="n"/>
       <c r="K165" s="7" t="n"/>
       <c r="L165" s="7" t="n"/>
       <c r="M165" s="7" t="n"/>
       <c r="N165" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O165" s="7" t="n">
         <v>0</v>
@@ -13174,7 +13174,7 @@
       <c r="V165" s="6" t="inlineStr"/>
       <c r="W165" s="7" t="inlineStr">
         <is>
-          <t>e86143466441bbbf802706245b19ef679ec29055</t>
+          <t>570a52f857d184562592fd86d2a0345a2e353ffb</t>
         </is>
       </c>
     </row>
@@ -13188,7 +13188,7 @@
         </is>
       </c>
       <c r="C166" s="9" t="n">
-        <v>1150</v>
+        <v>1465</v>
       </c>
       <c r="D166" s="7" t="n">
         <v>1</v>
@@ -13203,21 +13203,23 @@
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>St. Philips, Bristol, BS2</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H166" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I166" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I166" s="7" t="n">
+        <v>505</v>
+      </c>
       <c r="J166" s="7" t="n"/>
       <c r="K166" s="7" t="n"/>
       <c r="L166" s="7" t="n"/>
       <c r="M166" s="7" t="n"/>
       <c r="N166" s="7" t="n">
-        <v>20784</v>
+        <v>21816</v>
       </c>
       <c r="O166" s="7" t="n">
         <v>0</v>
@@ -13225,12 +13227,12 @@
       <c r="P166" s="7" t="n"/>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S166" s="8" t="inlineStr"/>
@@ -13247,7 +13249,7 @@
       <c r="V166" s="6" t="inlineStr"/>
       <c r="W166" s="7" t="inlineStr">
         <is>
-          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
+          <t>e86143466441bbbf802706245b19ef679ec29055</t>
         </is>
       </c>
     </row>
@@ -13261,7 +13263,7 @@
         </is>
       </c>
       <c r="C167" s="9" t="n">
-        <v>1685</v>
+        <v>1150</v>
       </c>
       <c r="D167" s="7" t="n">
         <v>1</v>
@@ -13276,23 +13278,21 @@
       </c>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>St. Philips, Bristol, BS2</t>
         </is>
       </c>
       <c r="H167" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I167" s="7" t="n">
-        <v>545</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I167" s="7" t="n"/>
       <c r="J167" s="7" t="n"/>
       <c r="K167" s="7" t="n"/>
       <c r="L167" s="7" t="n"/>
       <c r="M167" s="7" t="n"/>
       <c r="N167" s="7" t="n">
-        <v>21024</v>
+        <v>20784</v>
       </c>
       <c r="O167" s="7" t="n">
         <v>0</v>
@@ -13300,12 +13300,12 @@
       <c r="P167" s="7" t="n"/>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S167" s="8" t="inlineStr"/>
@@ -13322,7 +13322,7 @@
       <c r="V167" s="6" t="inlineStr"/>
       <c r="W167" s="7" t="inlineStr">
         <is>
-          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
+          <t>9a9d98f3d39c0afd7b5ee46e6be85f7b4ea3b1c4</t>
         </is>
       </c>
     </row>
@@ -13336,36 +13336,38 @@
         </is>
       </c>
       <c r="C168" s="9" t="n">
-        <v>1700</v>
+        <v>1685</v>
       </c>
       <c r="D168" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E168" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F168" s="7" t="inlineStr">
         <is>
-          <t>terraced</t>
+          <t>flat</t>
         </is>
       </c>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t>Dunkerry Road - Windmill Hill</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H168" s="7" t="inlineStr">
         <is>
-          <t>BS3</t>
-        </is>
-      </c>
-      <c r="I168" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I168" s="7" t="n">
+        <v>545</v>
+      </c>
       <c r="J168" s="7" t="n"/>
       <c r="K168" s="7" t="n"/>
       <c r="L168" s="7" t="n"/>
       <c r="M168" s="7" t="n"/>
       <c r="N168" s="7" t="n">
-        <v>8448</v>
+        <v>21024</v>
       </c>
       <c r="O168" s="7" t="n">
         <v>0</v>
@@ -13373,12 +13375,12 @@
       <c r="P168" s="7" t="n"/>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Ocean, Southville</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S168" s="8" t="inlineStr"/>
@@ -13395,7 +13397,7 @@
       <c r="V168" s="6" t="inlineStr"/>
       <c r="W168" s="7" t="inlineStr">
         <is>
-          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
+          <t>88ed4e2977aedcdc89320a99485a8fe083efdc12</t>
         </is>
       </c>
     </row>
@@ -13409,38 +13411,36 @@
         </is>
       </c>
       <c r="C169" s="9" t="n">
-        <v>1460</v>
+        <v>1700</v>
       </c>
       <c r="D169" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E169" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
-          <t>flat</t>
+          <t>terraced</t>
         </is>
       </c>
       <c r="G169" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Dunkerry Road - Windmill Hill</t>
         </is>
       </c>
       <c r="H169" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I169" s="7" t="n">
-        <v>473</v>
-      </c>
+          <t>BS3</t>
+        </is>
+      </c>
+      <c r="I169" s="7" t="n"/>
       <c r="J169" s="7" t="n"/>
       <c r="K169" s="7" t="n"/>
       <c r="L169" s="7" t="n"/>
       <c r="M169" s="7" t="n"/>
       <c r="N169" s="7" t="n">
-        <v>13840</v>
+        <v>8448</v>
       </c>
       <c r="O169" s="7" t="n">
         <v>0</v>
@@ -13448,12 +13448,12 @@
       <c r="P169" s="7" t="n"/>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Ocean, Southville</t>
         </is>
       </c>
       <c r="S169" s="8" t="inlineStr"/>
@@ -13470,7 +13470,7 @@
       <c r="V169" s="6" t="inlineStr"/>
       <c r="W169" s="7" t="inlineStr">
         <is>
-          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
+          <t>032764f4b044e7950437eeca48af4c24f53cf56e</t>
         </is>
       </c>
     </row>
@@ -13484,7 +13484,7 @@
         </is>
       </c>
       <c r="C170" s="9" t="n">
-        <v>1630</v>
+        <v>1460</v>
       </c>
       <c r="D170" s="7" t="n">
         <v>1</v>
@@ -13499,7 +13499,7 @@
       </c>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H170" s="7" t="inlineStr">
@@ -13508,27 +13508,27 @@
         </is>
       </c>
       <c r="I170" s="7" t="n">
-        <v>486</v>
+        <v>473</v>
       </c>
       <c r="J170" s="7" t="n"/>
       <c r="K170" s="7" t="n"/>
       <c r="L170" s="7" t="n"/>
       <c r="M170" s="7" t="n"/>
       <c r="N170" s="7" t="n">
-        <v>13860</v>
+        <v>13840</v>
       </c>
       <c r="O170" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P170" s="7" t="n"/>
       <c r="Q170" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R170" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S170" s="8" t="inlineStr"/>
@@ -13545,7 +13545,7 @@
       <c r="V170" s="6" t="inlineStr"/>
       <c r="W170" s="7" t="inlineStr">
         <is>
-          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
+          <t>485437aa3b2824e3aa6c5c511c6509e65e53b5b1</t>
         </is>
       </c>
     </row>
@@ -13559,7 +13559,7 @@
         </is>
       </c>
       <c r="C171" s="9" t="n">
-        <v>1625</v>
+        <v>1630</v>
       </c>
       <c r="D171" s="7" t="n">
         <v>1</v>
@@ -13590,15 +13590,15 @@
       <c r="L171" s="7" t="n"/>
       <c r="M171" s="7" t="n"/>
       <c r="N171" s="7" t="n">
-        <v>21732</v>
+        <v>13860</v>
       </c>
       <c r="O171" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P171" s="7" t="n"/>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
@@ -13620,7 +13620,7 @@
       <c r="V171" s="6" t="inlineStr"/>
       <c r="W171" s="7" t="inlineStr">
         <is>
-          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
+          <t>f169402d820a88e32d1253b9b548e48e8ad1fd01</t>
         </is>
       </c>
     </row>
@@ -13634,13 +13634,13 @@
         </is>
       </c>
       <c r="C172" s="9" t="n">
-        <v>1650</v>
+        <v>1625</v>
       </c>
       <c r="D172" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E172" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F172" s="7" t="inlineStr">
         <is>
@@ -13649,7 +13649,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>Harbourside, Harris Lofts, BS1 4BB</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H172" s="7" t="inlineStr">
@@ -13658,14 +13658,14 @@
         </is>
       </c>
       <c r="I172" s="7" t="n">
-        <v>667</v>
+        <v>486</v>
       </c>
       <c r="J172" s="7" t="n"/>
       <c r="K172" s="7" t="n"/>
       <c r="L172" s="7" t="n"/>
       <c r="M172" s="7" t="n"/>
       <c r="N172" s="7" t="n">
-        <v>20088</v>
+        <v>21732</v>
       </c>
       <c r="O172" s="7" t="n">
         <v>0</v>
@@ -13673,12 +13673,12 @@
       <c r="P172" s="7" t="n"/>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
         <is>
-          <t>The Bristol Residential Letting Co, Southville</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S172" s="8" t="inlineStr"/>
@@ -13695,7 +13695,7 @@
       <c r="V172" s="6" t="inlineStr"/>
       <c r="W172" s="7" t="inlineStr">
         <is>
-          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
+          <t>e8fa2bba98a0740c1a1c463dee19d50ba8e557a4</t>
         </is>
       </c>
     </row>
@@ -13712,10 +13712,10 @@
         <v>1650</v>
       </c>
       <c r="D173" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E173" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
@@ -13724,7 +13724,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>Central Quey North, Broad Quay, BS1</t>
+          <t>Harbourside, Harris Lofts, BS1 4BB</t>
         </is>
       </c>
       <c r="H173" s="7" t="inlineStr">
@@ -13732,13 +13732,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I173" s="7" t="n"/>
+      <c r="I173" s="7" t="n">
+        <v>667</v>
+      </c>
       <c r="J173" s="7" t="n"/>
       <c r="K173" s="7" t="n"/>
       <c r="L173" s="7" t="n"/>
       <c r="M173" s="7" t="n"/>
       <c r="N173" s="7" t="n">
-        <v>20768</v>
+        <v>20088</v>
       </c>
       <c r="O173" s="7" t="n">
         <v>0</v>
@@ -13751,7 +13753,7 @@
       </c>
       <c r="R173" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>The Bristol Residential Letting Co, Southville</t>
         </is>
       </c>
       <c r="S173" s="8" t="inlineStr"/>
@@ -13768,7 +13770,7 @@
       <c r="V173" s="6" t="inlineStr"/>
       <c r="W173" s="7" t="inlineStr">
         <is>
-          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
+          <t>570bd2fefe4b7b6f9264eaec3bfac939c790af6b</t>
         </is>
       </c>
     </row>
@@ -13782,7 +13784,7 @@
         </is>
       </c>
       <c r="C174" s="9" t="n">
-        <v>1550</v>
+        <v>1650</v>
       </c>
       <c r="D174" s="7" t="n">
         <v>1</v>
@@ -13797,7 +13799,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
+          <t>Central Quey North, Broad Quay, BS1</t>
         </is>
       </c>
       <c r="H174" s="7" t="inlineStr">
@@ -13811,7 +13813,7 @@
       <c r="L174" s="7" t="n"/>
       <c r="M174" s="7" t="n"/>
       <c r="N174" s="7" t="n">
-        <v>21100</v>
+        <v>20768</v>
       </c>
       <c r="O174" s="7" t="n">
         <v>0</v>
@@ -13819,7 +13821,7 @@
       <c r="P174" s="7" t="n"/>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
@@ -13841,7 +13843,7 @@
       <c r="V174" s="6" t="inlineStr"/>
       <c r="W174" s="7" t="inlineStr">
         <is>
-          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
+          <t>c1e93efa9291a4139a482181ff6c71d0bd2130ca</t>
         </is>
       </c>
     </row>
@@ -13855,7 +13857,7 @@
         </is>
       </c>
       <c r="C175" s="9" t="n">
-        <v>1390</v>
+        <v>1550</v>
       </c>
       <c r="D175" s="7" t="n">
         <v>1</v>
@@ -13870,7 +13872,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Central Quay North, Broad Quay, Bristol, BS1</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
@@ -13883,19 +13885,21 @@
       <c r="K175" s="7" t="n"/>
       <c r="L175" s="7" t="n"/>
       <c r="M175" s="7" t="n"/>
-      <c r="N175" s="7" t="n"/>
+      <c r="N175" s="7" t="n">
+        <v>21100</v>
+      </c>
       <c r="O175" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P175" s="7" t="n"/>
       <c r="Q175" s="7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R175" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S175" s="8" t="inlineStr"/>
@@ -13912,7 +13916,7 @@
       <c r="V175" s="6" t="inlineStr"/>
       <c r="W175" s="7" t="inlineStr">
         <is>
-          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
+          <t>918e6ace72d6470be4290d6aa465e702ae049b38</t>
         </is>
       </c>
     </row>
@@ -13926,7 +13930,7 @@
         </is>
       </c>
       <c r="C176" s="9" t="n">
-        <v>1485</v>
+        <v>1390</v>
       </c>
       <c r="D176" s="7" t="n">
         <v>1</v>
@@ -13941,7 +13945,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Thomas Court, Bristol, BS1</t>
         </is>
       </c>
       <c r="H176" s="7" t="inlineStr">
@@ -13949,28 +13953,24 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I176" s="7" t="n">
-        <v>470</v>
-      </c>
+      <c r="I176" s="7" t="n"/>
       <c r="J176" s="7" t="n"/>
       <c r="K176" s="7" t="n"/>
       <c r="L176" s="7" t="n"/>
       <c r="M176" s="7" t="n"/>
-      <c r="N176" s="7" t="n">
-        <v>21740</v>
-      </c>
+      <c r="N176" s="7" t="n"/>
       <c r="O176" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P176" s="7" t="n"/>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S176" s="8" t="inlineStr"/>
@@ -13987,7 +13987,7 @@
       <c r="V176" s="6" t="inlineStr"/>
       <c r="W176" s="7" t="inlineStr">
         <is>
-          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
+          <t>d059b7e0cd5c97ed00a5cc8d6548c29896f2f756</t>
         </is>
       </c>
     </row>
@@ -14001,7 +14001,7 @@
         </is>
       </c>
       <c r="C177" s="9" t="n">
-        <v>1635</v>
+        <v>1485</v>
       </c>
       <c r="D177" s="7" t="n">
         <v>1</v>
@@ -14016,7 +14016,7 @@
       </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H177" s="7" t="inlineStr">
@@ -14025,14 +14025,14 @@
         </is>
       </c>
       <c r="I177" s="7" t="n">
-        <v>486</v>
+        <v>470</v>
       </c>
       <c r="J177" s="7" t="n"/>
       <c r="K177" s="7" t="n"/>
       <c r="L177" s="7" t="n"/>
       <c r="M177" s="7" t="n"/>
       <c r="N177" s="7" t="n">
-        <v>21732</v>
+        <v>21740</v>
       </c>
       <c r="O177" s="7" t="n">
         <v>0</v>
@@ -14040,12 +14040,12 @@
       <c r="P177" s="7" t="n"/>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S177" s="8" t="inlineStr"/>
@@ -14062,7 +14062,7 @@
       <c r="V177" s="6" t="inlineStr"/>
       <c r="W177" s="7" t="inlineStr">
         <is>
-          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
+          <t>bfd77b1d5efb83c8ea40f8fbb1a6e0ce80968090</t>
         </is>
       </c>
     </row>
@@ -14076,13 +14076,13 @@
         </is>
       </c>
       <c r="C178" s="9" t="n">
-        <v>2060</v>
+        <v>1635</v>
       </c>
       <c r="D178" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E178" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F178" s="7" t="inlineStr">
         <is>
@@ -14100,7 +14100,7 @@
         </is>
       </c>
       <c r="I178" s="7" t="n">
-        <v>721</v>
+        <v>486</v>
       </c>
       <c r="J178" s="7" t="n"/>
       <c r="K178" s="7" t="n"/>
@@ -14137,7 +14137,7 @@
       <c r="V178" s="6" t="inlineStr"/>
       <c r="W178" s="7" t="inlineStr">
         <is>
-          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
+          <t>d656d10a3343db70bfb31489c5c46b84dd3d751a</t>
         </is>
       </c>
     </row>
@@ -14151,13 +14151,13 @@
         </is>
       </c>
       <c r="C179" s="9" t="n">
-        <v>1545</v>
+        <v>2060</v>
       </c>
       <c r="D179" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E179" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
@@ -14166,7 +14166,7 @@
       </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H179" s="7" t="inlineStr">
@@ -14175,14 +14175,14 @@
         </is>
       </c>
       <c r="I179" s="7" t="n">
-        <v>548</v>
+        <v>721</v>
       </c>
       <c r="J179" s="7" t="n"/>
       <c r="K179" s="7" t="n"/>
       <c r="L179" s="7" t="n"/>
       <c r="M179" s="7" t="n"/>
       <c r="N179" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O179" s="7" t="n">
         <v>0</v>
@@ -14190,12 +14190,12 @@
       <c r="P179" s="7" t="n"/>
       <c r="Q179" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R179" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S179" s="8" t="inlineStr"/>
@@ -14212,7 +14212,7 @@
       <c r="V179" s="6" t="inlineStr"/>
       <c r="W179" s="7" t="inlineStr">
         <is>
-          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
+          <t>a8b050f5ece745a07a49c045a6b3de9ab3d906f0</t>
         </is>
       </c>
     </row>
@@ -14226,7 +14226,7 @@
         </is>
       </c>
       <c r="C180" s="9" t="n">
-        <v>1640</v>
+        <v>1545</v>
       </c>
       <c r="D180" s="7" t="n">
         <v>1</v>
@@ -14241,7 +14241,7 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H180" s="7" t="inlineStr">
@@ -14250,14 +14250,14 @@
         </is>
       </c>
       <c r="I180" s="7" t="n">
-        <v>486</v>
+        <v>548</v>
       </c>
       <c r="J180" s="7" t="n"/>
       <c r="K180" s="7" t="n"/>
       <c r="L180" s="7" t="n"/>
       <c r="M180" s="7" t="n"/>
       <c r="N180" s="7" t="n">
-        <v>21732</v>
+        <v>21740</v>
       </c>
       <c r="O180" s="7" t="n">
         <v>0</v>
@@ -14270,7 +14270,7 @@
       </c>
       <c r="R180" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S180" s="8" t="inlineStr"/>
@@ -14287,7 +14287,7 @@
       <c r="V180" s="6" t="inlineStr"/>
       <c r="W180" s="7" t="inlineStr">
         <is>
-          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
+          <t>4e1b7003002888c7ea87cca695d7e3d5b841b634</t>
         </is>
       </c>
     </row>
@@ -14301,10 +14301,10 @@
         </is>
       </c>
       <c r="C181" s="9" t="n">
-        <v>2115</v>
+        <v>1640</v>
       </c>
       <c r="D181" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E181" s="7" t="n">
         <v>1</v>
@@ -14325,7 +14325,7 @@
         </is>
       </c>
       <c r="I181" s="7" t="n">
-        <v>722</v>
+        <v>486</v>
       </c>
       <c r="J181" s="7" t="n"/>
       <c r="K181" s="7" t="n"/>
@@ -14362,7 +14362,7 @@
       <c r="V181" s="6" t="inlineStr"/>
       <c r="W181" s="7" t="inlineStr">
         <is>
-          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
+          <t>b42c1abfa69fcb3c8fcdee14c8cc621e4bc97c5f</t>
         </is>
       </c>
     </row>
@@ -14376,13 +14376,13 @@
         </is>
       </c>
       <c r="C182" s="9" t="n">
-        <v>1970</v>
+        <v>2115</v>
       </c>
       <c r="D182" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E182" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
@@ -14391,7 +14391,7 @@
       </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H182" s="7" t="inlineStr">
@@ -14400,14 +14400,14 @@
         </is>
       </c>
       <c r="I182" s="7" t="n">
-        <v>750</v>
+        <v>722</v>
       </c>
       <c r="J182" s="7" t="n"/>
       <c r="K182" s="7" t="n"/>
       <c r="L182" s="7" t="n"/>
       <c r="M182" s="7" t="n"/>
       <c r="N182" s="7" t="n">
-        <v>21740</v>
+        <v>21732</v>
       </c>
       <c r="O182" s="7" t="n">
         <v>0</v>
@@ -14415,12 +14415,12 @@
       <c r="P182" s="7" t="n"/>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Hawkins &amp; George</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S182" s="8" t="inlineStr"/>
@@ -14437,7 +14437,7 @@
       <c r="V182" s="6" t="inlineStr"/>
       <c r="W182" s="7" t="inlineStr">
         <is>
-          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
+          <t>d76d2b4a5abe7b7b6a980b6fed901da22fe62faa</t>
         </is>
       </c>
     </row>
@@ -14451,13 +14451,13 @@
         </is>
       </c>
       <c r="C183" s="9" t="n">
-        <v>1575</v>
+        <v>1970</v>
       </c>
       <c r="D183" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E183" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F183" s="7" t="inlineStr">
         <is>
@@ -14475,14 +14475,14 @@
         </is>
       </c>
       <c r="I183" s="7" t="n">
-        <v>430</v>
+        <v>750</v>
       </c>
       <c r="J183" s="7" t="n"/>
       <c r="K183" s="7" t="n"/>
       <c r="L183" s="7" t="n"/>
       <c r="M183" s="7" t="n"/>
       <c r="N183" s="7" t="n">
-        <v>21816</v>
+        <v>21740</v>
       </c>
       <c r="O183" s="7" t="n">
         <v>0</v>
@@ -14512,7 +14512,7 @@
       <c r="V183" s="6" t="inlineStr"/>
       <c r="W183" s="7" t="inlineStr">
         <is>
-          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
+          <t>fcbcb7d449a675f163e3bc230f20ce82b99fd6fb</t>
         </is>
       </c>
     </row>
@@ -14526,7 +14526,7 @@
         </is>
       </c>
       <c r="C184" s="9" t="n">
-        <v>1350</v>
+        <v>1575</v>
       </c>
       <c r="D184" s="7" t="n">
         <v>1</v>
@@ -14541,7 +14541,7 @@
       </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t>Invicta, Millenium Promenade, BS1</t>
+          <t>Hawkins &amp; George, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H184" s="7" t="inlineStr">
@@ -14549,13 +14549,15 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I184" s="7" t="n"/>
+      <c r="I184" s="7" t="n">
+        <v>430</v>
+      </c>
       <c r="J184" s="7" t="n"/>
       <c r="K184" s="7" t="n"/>
       <c r="L184" s="7" t="n"/>
       <c r="M184" s="7" t="n"/>
       <c r="N184" s="7" t="n">
-        <v>17344</v>
+        <v>21816</v>
       </c>
       <c r="O184" s="7" t="n">
         <v>0</v>
@@ -14563,12 +14565,12 @@
       <c r="P184" s="7" t="n"/>
       <c r="Q184" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R184" s="7" t="inlineStr">
         <is>
-          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
+          <t>Grainger, Hawkins &amp; George</t>
         </is>
       </c>
       <c r="S184" s="8" t="inlineStr"/>
@@ -14585,7 +14587,7 @@
       <c r="V184" s="6" t="inlineStr"/>
       <c r="W184" s="7" t="inlineStr">
         <is>
-          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
+          <t>a6f51a67f600a115794110dbb08b353e3b7b57af</t>
         </is>
       </c>
     </row>
@@ -14599,7 +14601,7 @@
         </is>
       </c>
       <c r="C185" s="9" t="n">
-        <v>1600</v>
+        <v>1350</v>
       </c>
       <c r="D185" s="7" t="n">
         <v>1</v>
@@ -14614,7 +14616,7 @@
       </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t>Central Quay North, Bristol, BS1</t>
+          <t>Invicta, Millenium Promenade, BS1</t>
         </is>
       </c>
       <c r="H185" s="7" t="inlineStr">
@@ -14628,7 +14630,7 @@
       <c r="L185" s="7" t="n"/>
       <c r="M185" s="7" t="n"/>
       <c r="N185" s="7" t="n">
-        <v>13404</v>
+        <v>17344</v>
       </c>
       <c r="O185" s="7" t="n">
         <v>0</v>
@@ -14641,7 +14643,7 @@
       </c>
       <c r="R185" s="7" t="inlineStr">
         <is>
-          <t>HPG, Bristol</t>
+          <t>Chappell &amp; Matthews Lettings, Bristol Harbourside</t>
         </is>
       </c>
       <c r="S185" s="8" t="inlineStr"/>
@@ -14658,7 +14660,7 @@
       <c r="V185" s="6" t="inlineStr"/>
       <c r="W185" s="7" t="inlineStr">
         <is>
-          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
+          <t>6f98ebba772b361fb92441f7aac7e0b11d4baf99</t>
         </is>
       </c>
     </row>
@@ -14672,10 +14674,10 @@
         </is>
       </c>
       <c r="C186" s="9" t="n">
-        <v>1700</v>
+        <v>1600</v>
       </c>
       <c r="D186" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E186" s="7" t="n">
         <v>1</v>
@@ -14687,7 +14689,7 @@
       </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
+          <t>Central Quay North, Bristol, BS1</t>
         </is>
       </c>
       <c r="H186" s="7" t="inlineStr">
@@ -14695,15 +14697,13 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I186" s="7" t="n">
-        <v>646</v>
-      </c>
+      <c r="I186" s="7" t="n"/>
       <c r="J186" s="7" t="n"/>
       <c r="K186" s="7" t="n"/>
       <c r="L186" s="7" t="n"/>
       <c r="M186" s="7" t="n"/>
       <c r="N186" s="7" t="n">
-        <v>20928</v>
+        <v>13404</v>
       </c>
       <c r="O186" s="7" t="n">
         <v>0</v>
@@ -14711,12 +14711,12 @@
       <c r="P186" s="7" t="n"/>
       <c r="Q186" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R186" s="7" t="inlineStr">
         <is>
-          <t>Acen Properties, Bristol</t>
+          <t>HPG, Bristol</t>
         </is>
       </c>
       <c r="S186" s="8" t="inlineStr"/>
@@ -14733,7 +14733,7 @@
       <c r="V186" s="6" t="inlineStr"/>
       <c r="W186" s="7" t="inlineStr">
         <is>
-          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
+          <t>fa2a6e8bc7e80262181907e1f2aec4309ba73bfe</t>
         </is>
       </c>
     </row>
@@ -14747,13 +14747,13 @@
         </is>
       </c>
       <c r="C187" s="9" t="n">
-        <v>2105</v>
+        <v>1700</v>
       </c>
       <c r="D187" s="7" t="n">
         <v>2</v>
       </c>
       <c r="E187" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F187" s="7" t="inlineStr">
         <is>
@@ -14762,7 +14762,7 @@
       </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t>Glasshouse Square, Bristol Bristol BS1</t>
+          <t>Welsh Back, Riverside House Welsh Back, BS1</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
@@ -14771,14 +14771,14 @@
         </is>
       </c>
       <c r="I187" s="7" t="n">
-        <v>745</v>
+        <v>646</v>
       </c>
       <c r="J187" s="7" t="n"/>
       <c r="K187" s="7" t="n"/>
       <c r="L187" s="7" t="n"/>
       <c r="M187" s="7" t="n"/>
       <c r="N187" s="7" t="n">
-        <v>20984</v>
+        <v>20928</v>
       </c>
       <c r="O187" s="7" t="n">
         <v>0</v>
@@ -14786,12 +14786,12 @@
       <c r="P187" s="7" t="n"/>
       <c r="Q187" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R187" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Glasshouse Square</t>
+          <t>Acen Properties, Bristol</t>
         </is>
       </c>
       <c r="S187" s="8" t="inlineStr"/>
@@ -14808,7 +14808,7 @@
       <c r="V187" s="6" t="inlineStr"/>
       <c r="W187" s="7" t="inlineStr">
         <is>
-          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
+          <t>c7893e602f95d149c07e9736c029eea7a1363cb3</t>
         </is>
       </c>
     </row>
@@ -14822,13 +14822,13 @@
         </is>
       </c>
       <c r="C188" s="9" t="n">
-        <v>1595</v>
+        <v>2105</v>
       </c>
       <c r="D188" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E188" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F188" s="7" t="inlineStr">
         <is>
@@ -14837,7 +14837,7 @@
       </c>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Glasshouse Square, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
@@ -14846,14 +14846,14 @@
         </is>
       </c>
       <c r="I188" s="7" t="n">
-        <v>484</v>
+        <v>745</v>
       </c>
       <c r="J188" s="7" t="n"/>
       <c r="K188" s="7" t="n"/>
       <c r="L188" s="7" t="n"/>
       <c r="M188" s="7" t="n"/>
       <c r="N188" s="7" t="n">
-        <v>21732</v>
+        <v>20984</v>
       </c>
       <c r="O188" s="7" t="n">
         <v>0</v>
@@ -14861,12 +14861,12 @@
       <c r="P188" s="7" t="n"/>
       <c r="Q188" s="7" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R188" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>Grainger, Glasshouse Square</t>
         </is>
       </c>
       <c r="S188" s="8" t="inlineStr"/>
@@ -14883,7 +14883,7 @@
       <c r="V188" s="6" t="inlineStr"/>
       <c r="W188" s="7" t="inlineStr">
         <is>
-          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
+          <t>8146130a32a1e09821b810718fe41303e6e3e932</t>
         </is>
       </c>
     </row>
@@ -14897,10 +14897,10 @@
         </is>
       </c>
       <c r="C189" s="9" t="n">
-        <v>1999</v>
+        <v>1595</v>
       </c>
       <c r="D189" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E189" s="7" t="n">
         <v>1</v>
@@ -14912,21 +14912,23 @@
       </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t>Hamilton Court, Bristol, BS2</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
         <is>
-          <t>BS2</t>
-        </is>
-      </c>
-      <c r="I189" s="7" t="n"/>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I189" s="7" t="n">
+        <v>484</v>
+      </c>
       <c r="J189" s="7" t="n"/>
       <c r="K189" s="7" t="n"/>
       <c r="L189" s="7" t="n"/>
       <c r="M189" s="7" t="n"/>
       <c r="N189" s="7" t="n">
-        <v>21736</v>
+        <v>21732</v>
       </c>
       <c r="O189" s="7" t="n">
         <v>0</v>
@@ -14934,12 +14936,12 @@
       <c r="P189" s="7" t="n"/>
       <c r="Q189" s="7" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R189" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S189" s="8" t="inlineStr"/>
@@ -14956,7 +14958,7 @@
       <c r="V189" s="6" t="inlineStr"/>
       <c r="W189" s="7" t="inlineStr">
         <is>
-          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
+          <t>5a12c308e2cd7ae303f48b5e82bd930cb8733969</t>
         </is>
       </c>
     </row>
@@ -14970,10 +14972,10 @@
         </is>
       </c>
       <c r="C190" s="9" t="n">
-        <v>1605</v>
+        <v>1999</v>
       </c>
       <c r="D190" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E190" s="7" t="n">
         <v>1</v>
@@ -14985,23 +14987,21 @@
       </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t>Millwrights Place, Bristol Bristol BS1</t>
+          <t>Hamilton Court, Bristol, BS2</t>
         </is>
       </c>
       <c r="H190" s="7" t="inlineStr">
         <is>
-          <t>BS1</t>
-        </is>
-      </c>
-      <c r="I190" s="7" t="n">
-        <v>487</v>
-      </c>
+          <t>BS2</t>
+        </is>
+      </c>
+      <c r="I190" s="7" t="n"/>
       <c r="J190" s="7" t="n"/>
       <c r="K190" s="7" t="n"/>
       <c r="L190" s="7" t="n"/>
       <c r="M190" s="7" t="n"/>
       <c r="N190" s="7" t="n">
-        <v>21732</v>
+        <v>21736</v>
       </c>
       <c r="O190" s="7" t="n">
         <v>0</v>
@@ -15009,12 +15009,12 @@
       <c r="P190" s="7" t="n"/>
       <c r="Q190" s="7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="R190" s="7" t="inlineStr">
         <is>
-          <t>Grainger, Millwrights Place</t>
+          <t>OpenRent, London</t>
         </is>
       </c>
       <c r="S190" s="8" t="inlineStr"/>
@@ -15031,7 +15031,7 @@
       <c r="V190" s="6" t="inlineStr"/>
       <c r="W190" s="7" t="inlineStr">
         <is>
-          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
+          <t>7e84be8b1496e4e7c3f30b44557f5fdc8c97aed3</t>
         </is>
       </c>
     </row>
@@ -15045,7 +15045,7 @@
         </is>
       </c>
       <c r="C191" s="9" t="n">
-        <v>1390</v>
+        <v>1605</v>
       </c>
       <c r="D191" s="7" t="n">
         <v>1</v>
@@ -15060,7 +15060,7 @@
       </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t>Thomas Court, Bristol, BS1</t>
+          <t>Millwrights Place, Bristol Bristol BS1</t>
         </is>
       </c>
       <c r="H191" s="7" t="inlineStr">
@@ -15068,24 +15068,28 @@
           <t>BS1</t>
         </is>
       </c>
-      <c r="I191" s="7" t="n"/>
+      <c r="I191" s="7" t="n">
+        <v>487</v>
+      </c>
       <c r="J191" s="7" t="n"/>
       <c r="K191" s="7" t="n"/>
       <c r="L191" s="7" t="n"/>
       <c r="M191" s="7" t="n"/>
-      <c r="N191" s="7" t="n"/>
+      <c r="N191" s="7" t="n">
+        <v>21732</v>
+      </c>
       <c r="O191" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P191" s="7" t="n"/>
       <c r="Q191" s="7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R191" s="7" t="inlineStr">
         <is>
-          <t>OpenRent, London</t>
+          <t>Grainger, Millwrights Place</t>
         </is>
       </c>
       <c r="S191" s="8" t="inlineStr"/>
@@ -15102,7 +15106,7 @@
       <c r="V191" s="6" t="inlineStr"/>
       <c r="W191" s="7" t="inlineStr">
         <is>
-          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+          <t>d7d47054224ca2dacb0503f012c570e02407997c</t>
         </is>
       </c>
     </row>
@@ -15116,7 +15120,7 @@
         </is>
       </c>
       <c r="C192" s="9" t="n">
-        <v>1395</v>
+        <v>1390</v>
       </c>
       <c r="D192" s="7" t="n">
         <v>1</v>
@@ -15144,16 +15148,14 @@
       <c r="K192" s="7" t="n"/>
       <c r="L192" s="7" t="n"/>
       <c r="M192" s="7" t="n"/>
-      <c r="N192" s="7" t="n">
-        <v>20524</v>
-      </c>
+      <c r="N192" s="7" t="n"/>
       <c r="O192" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P192" s="7" t="n"/>
       <c r="Q192" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R192" s="7" t="inlineStr">
@@ -15175,14 +15177,87 @@
       <c r="V192" s="6" t="inlineStr"/>
       <c r="W192" s="7" t="inlineStr">
         <is>
+          <t>e7c74b862a265c230fbaaabb92ed08e50d85632a</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B193" s="8" t="inlineStr">
+        <is>
+          <t>Keyword match only (no API key configured for full scoring).</t>
+        </is>
+      </c>
+      <c r="C193" s="9" t="n">
+        <v>1395</v>
+      </c>
+      <c r="D193" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E193" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F193" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="G193" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Court, Bristol, BS1</t>
+        </is>
+      </c>
+      <c r="H193" s="7" t="inlineStr">
+        <is>
+          <t>BS1</t>
+        </is>
+      </c>
+      <c r="I193" s="7" t="n"/>
+      <c r="J193" s="7" t="n"/>
+      <c r="K193" s="7" t="n"/>
+      <c r="L193" s="7" t="n"/>
+      <c r="M193" s="7" t="n"/>
+      <c r="N193" s="7" t="n">
+        <v>20524</v>
+      </c>
+      <c r="O193" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P193" s="7" t="n"/>
+      <c r="Q193" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="R193" s="7" t="inlineStr">
+        <is>
+          <t>OpenRent, London</t>
+        </is>
+      </c>
+      <c r="S193" s="8" t="inlineStr"/>
+      <c r="T193" s="10" t="inlineStr">
+        <is>
+          <t>View listing</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="V193" s="6" t="inlineStr"/>
+      <c r="W193" s="7" t="inlineStr">
+        <is>
           <t>f0aa9fb55fbecd943fa3b5e0649d09b0565b441f</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W192"/>
+  <autoFilter ref="A1:W193"/>
   <dataValidations count="1">
-    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2 U3 U4 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"new,interested,viewing_booked,viewed,offer_made,offer_accepted,rejected,sold_stc,withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15378,6 +15453,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T190" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T191" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T193" r:id="rId192"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
House search data from run 180
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>1475</v>
+        <v>1450</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>1</v>
@@ -9656,7 +9656,7 @@
         <v>21736</v>
       </c>
       <c r="O118" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P118" s="7" t="n"/>
       <c r="Q118" s="7" t="inlineStr">
@@ -10593,7 +10593,7 @@
         </is>
       </c>
       <c r="C131" s="9" t="n">
-        <v>1350</v>
+        <v>1300</v>
       </c>
       <c r="D131" s="7" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
House search data from run 182
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>1250</v>
+        <v>1200</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>1</v>
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="C64" s="9" t="n">
-        <v>1450</v>
+        <v>1395</v>
       </c>
       <c r="D64" s="7" t="n">
         <v>1</v>
@@ -8659,7 +8659,7 @@
         </is>
       </c>
       <c r="C105" s="9" t="n">
-        <v>1550</v>
+        <v>1500</v>
       </c>
       <c r="D105" s="7" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
House search data from run 184
</commit_message>
<xml_diff>
--- a/data/houses.xlsx
+++ b/data/houses.xlsx
@@ -5829,7 +5829,7 @@
         </is>
       </c>
       <c r="C67" s="9" t="n">
-        <v>1350</v>
+        <v>1300</v>
       </c>
       <c r="D67" s="7" t="n">
         <v>1</v>
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="C123" s="9" t="n">
-        <v>1350</v>
+        <v>1250</v>
       </c>
       <c r="D123" s="7" t="n">
         <v>1</v>

</xml_diff>